<commit_message>
[dnn-library] [SW-3233] automatize generation of non-inline header files definition in LibNodes.h (function declarations, extern template...)
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -5,10 +5,11 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Instances" sheetId="2" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="153">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -232,7 +233,7 @@
     <t xml:space="preserve">MaxPool</t>
   </si>
   <si>
-    <t xml:space="preserve">ETSOCMaxSplat</t>
+    <t xml:space="preserve">MaxSplat</t>
   </si>
   <si>
     <t xml:space="preserve">Value</t>
@@ -314,6 +315,171 @@
   </si>
   <si>
     <t xml:space="preserve">Shuffle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int16QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy, FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty, Float16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int8QTy,Int8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UInt8QTy,Int8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int8QTy,UInt8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UInt8QTy,UInt8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int64Ty,Int64Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,FloatTy,FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,Float16Ty,Float16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int8Qty,Int8Qty,Int8Qty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int8Qty,Int8Qty,Int32QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int16QTy,Int16QTy,Int16Qty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int16QTy,Int16QTy,Int32QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,Float16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32ITy,Float16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32ITy,FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32ITy,Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int64ITy,Float16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int64ITy,FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int64ITy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int8QTy,Int8QTy,Int8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int16QTy,Int16QTy,Int16QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,Int8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,UInt8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,Int16QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,Int32QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,Int8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,UInt8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,Int16QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,Int32QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32ITy,Int32ITy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int64ITy,Int64ITy,Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,Float16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32ITy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int64ITy,Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int8QTy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UInt8QTy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int16QTy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int8QTy,Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UInt8QTy,Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int16QTy,Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UInt8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32QTy</t>
   </si>
 </sst>
 </file>
@@ -494,7 +660,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="8" style="0" width="8.67"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1773,4 +1939,2181 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:P70"/>
+  <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="19.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="21.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="24.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="24.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="24.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="0" width="17.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="16.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="16.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="14.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="15.06"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="str">
+        <f aca="false">LibManager!A2</f>
+        <v>AdaptiveAvgPool</v>
+      </c>
+      <c r="B2" s="0" t="n">
+        <f aca="false">LibManager!B2</f>
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="n">
+        <f aca="false">LibManager!C2</f>
+        <v>1</v>
+      </c>
+      <c r="D2" s="0" t="n">
+        <f aca="false">LibManager!E2</f>
+        <v>1</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F2" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G2" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H2" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I2" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J2" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="str">
+        <f aca="false">LibManager!A3</f>
+        <v>ArgMax</v>
+      </c>
+      <c r="B3" s="0" t="n">
+        <f aca="false">LibManager!B3</f>
+        <v>1</v>
+      </c>
+      <c r="C3" s="0" t="n">
+        <f aca="false">LibManager!C3</f>
+        <v>1</v>
+      </c>
+      <c r="D3" s="0" t="n">
+        <f aca="false">LibManager!E3</f>
+        <v>1</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F3" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G3" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H3" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I3" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J3" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="str">
+        <f aca="false">LibManager!A4</f>
+        <v>AvgPool</v>
+      </c>
+      <c r="B4" s="0" t="n">
+        <f aca="false">LibManager!B4</f>
+        <v>1</v>
+      </c>
+      <c r="C4" s="0" t="n">
+        <f aca="false">LibManager!C4</f>
+        <v>1</v>
+      </c>
+      <c r="D4" s="0" t="str">
+        <f aca="false">LibManager!E4</f>
+        <v>0,1</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="F4" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="G4" s="0" t="s">
+        <v>106</v>
+      </c>
+      <c r="H4" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="I4" s="0" t="s">
+        <v>108</v>
+      </c>
+      <c r="J4" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="K4" s="0" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="str">
+        <f aca="false">LibManager!A5</f>
+        <v>BatchOneHot</v>
+      </c>
+      <c r="B5" s="0" t="n">
+        <f aca="false">LibManager!B5</f>
+        <v>1</v>
+      </c>
+      <c r="C5" s="0" t="n">
+        <f aca="false">LibManager!C5</f>
+        <v>3</v>
+      </c>
+      <c r="D5" s="0" t="n">
+        <f aca="false">LibManager!E5</f>
+        <v>0</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F5" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G5" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H5" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I5" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J5" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="str">
+        <f aca="false">LibManager!A6</f>
+        <v>BatchedAdd</v>
+      </c>
+      <c r="B6" s="0" t="n">
+        <f aca="false">LibManager!B6</f>
+        <v>1</v>
+      </c>
+      <c r="C6" s="0" t="n">
+        <f aca="false">LibManager!C6</f>
+        <v>2</v>
+      </c>
+      <c r="D6" s="0" t="str">
+        <f aca="false">LibManager!E6</f>
+        <v>0,1,2</v>
+      </c>
+      <c r="E6" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="F6" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="G6" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="H6" s="0" t="s">
+        <v>114</v>
+      </c>
+      <c r="I6" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="J6" s="0" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="str">
+        <f aca="false">LibManager!A7</f>
+        <v>BatchedReduceAdd</v>
+      </c>
+      <c r="B7" s="0" t="n">
+        <f aca="false">LibManager!B7</f>
+        <v>1</v>
+      </c>
+      <c r="C7" s="0" t="n">
+        <f aca="false">LibManager!C7</f>
+        <v>1</v>
+      </c>
+      <c r="D7" s="0" t="n">
+        <f aca="false">LibManager!E7</f>
+        <v>1</v>
+      </c>
+      <c r="E7" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F7" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G7" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H7" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I7" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J7" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="str">
+        <f aca="false">LibManager!A8</f>
+        <v>Checksum</v>
+      </c>
+      <c r="B8" s="0" t="n">
+        <f aca="false">LibManager!B8</f>
+        <v>0</v>
+      </c>
+      <c r="C8" s="0" t="n">
+        <f aca="false">LibManager!C8</f>
+        <v>1</v>
+      </c>
+      <c r="D8" s="0" t="n">
+        <f aca="false">LibManager!E8</f>
+        <v>0</v>
+      </c>
+      <c r="E8" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F8" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G8" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H8" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I8" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J8" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="str">
+        <f aca="false">LibManager!A9</f>
+        <v>ConvertTo</v>
+      </c>
+      <c r="B9" s="0" t="n">
+        <f aca="false">LibManager!B9</f>
+        <v>1</v>
+      </c>
+      <c r="C9" s="0" t="n">
+        <f aca="false">LibManager!C9</f>
+        <v>1</v>
+      </c>
+      <c r="D9" s="0" t="str">
+        <f aca="false">LibManager!E9</f>
+        <v>0,1</v>
+      </c>
+      <c r="E9" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="F9" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="G9" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="H9" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="I9" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="J9" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="K9" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="L9" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="M9" s="0" t="s">
+        <v>125</v>
+      </c>
+      <c r="N9" s="0" t="s">
+        <v>126</v>
+      </c>
+      <c r="O9" s="0" t="s">
+        <v>127</v>
+      </c>
+      <c r="P9" s="0" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="str">
+        <f aca="false">LibManager!A10</f>
+        <v>Convolution</v>
+      </c>
+      <c r="B10" s="0" t="n">
+        <f aca="false">LibManager!B10</f>
+        <v>1</v>
+      </c>
+      <c r="C10" s="0" t="n">
+        <f aca="false">LibManager!C10</f>
+        <v>3</v>
+      </c>
+      <c r="D10" s="0" t="str">
+        <f aca="false">LibManager!E10</f>
+        <v>0,1,2</v>
+      </c>
+      <c r="E10" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="F10" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="G10" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="H10" s="0" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="str">
+        <f aca="false">LibManager!A11</f>
+        <v>Convolution3D</v>
+      </c>
+      <c r="B11" s="0" t="n">
+        <f aca="false">LibManager!B11</f>
+        <v>1</v>
+      </c>
+      <c r="C11" s="0" t="n">
+        <f aca="false">LibManager!C11</f>
+        <v>3</v>
+      </c>
+      <c r="D11" s="0" t="n">
+        <f aca="false">LibManager!E11</f>
+        <v>0</v>
+      </c>
+      <c r="E11" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F11" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G11" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H11" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I11" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J11" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="str">
+        <f aca="false">LibManager!A12</f>
+        <v>Copy</v>
+      </c>
+      <c r="B12" s="0" t="n">
+        <f aca="false">LibManager!B12</f>
+        <v>1</v>
+      </c>
+      <c r="C12" s="0" t="n">
+        <f aca="false">LibManager!C12</f>
+        <v>1</v>
+      </c>
+      <c r="D12" s="0" t="n">
+        <f aca="false">LibManager!E12</f>
+        <v>0</v>
+      </c>
+      <c r="E12" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F12" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G12" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H12" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I12" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J12" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="str">
+        <f aca="false">LibManager!A13</f>
+        <v>CrossEntropyLoss</v>
+      </c>
+      <c r="B13" s="0" t="n">
+        <f aca="false">LibManager!B13</f>
+        <v>1</v>
+      </c>
+      <c r="C13" s="0" t="n">
+        <f aca="false">LibManager!C13</f>
+        <v>2</v>
+      </c>
+      <c r="D13" s="0" t="n">
+        <f aca="false">LibManager!E13</f>
+        <v>1</v>
+      </c>
+      <c r="E13" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F13" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G13" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H13" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I13" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J13" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="str">
+        <f aca="false">LibManager!A14</f>
+        <v>Dequantize</v>
+      </c>
+      <c r="B14" s="0" t="n">
+        <f aca="false">LibManager!B14</f>
+        <v>1</v>
+      </c>
+      <c r="C14" s="0" t="n">
+        <f aca="false">LibManager!C14</f>
+        <v>1</v>
+      </c>
+      <c r="D14" s="0" t="n">
+        <f aca="false">LibManager!E14</f>
+        <v>1</v>
+      </c>
+      <c r="E14" s="0" t="s">
+        <v>131</v>
+      </c>
+      <c r="F14" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="G14" s="0" t="s">
+        <v>133</v>
+      </c>
+      <c r="H14" s="0" t="s">
+        <v>134</v>
+      </c>
+      <c r="I14" s="0" t="s">
+        <v>135</v>
+      </c>
+      <c r="J14" s="0" t="s">
+        <v>136</v>
+      </c>
+      <c r="K14" s="0" t="s">
+        <v>137</v>
+      </c>
+      <c r="L14" s="0" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="str">
+        <f aca="false">LibManager!A15</f>
+        <v>ElementAdd</v>
+      </c>
+      <c r="B15" s="0" t="n">
+        <f aca="false">LibManager!B15</f>
+        <v>1</v>
+      </c>
+      <c r="C15" s="0" t="n">
+        <f aca="false">LibManager!C15</f>
+        <v>2</v>
+      </c>
+      <c r="D15" s="0" t="str">
+        <f aca="false">LibManager!E15</f>
+        <v>0,1,2</v>
+      </c>
+      <c r="E15" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="F15" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="G15" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="H15" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="I15" s="0" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0" t="str">
+        <f aca="false">LibManager!A16</f>
+        <v>ElementCmpEQ</v>
+      </c>
+      <c r="B16" s="0" t="n">
+        <f aca="false">LibManager!B16</f>
+        <v>1</v>
+      </c>
+      <c r="C16" s="0" t="n">
+        <f aca="false">LibManager!C16</f>
+        <v>2</v>
+      </c>
+      <c r="D16" s="0" t="str">
+        <f aca="false">LibManager!E16</f>
+        <v>1,2</v>
+      </c>
+      <c r="E16" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="F16" s="0" t="s">
+        <v>142</v>
+      </c>
+      <c r="G16" s="0" t="s">
+        <v>106</v>
+      </c>
+      <c r="H16" s="0" t="s">
+        <v>143</v>
+      </c>
+      <c r="I16" s="0" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="0" t="str">
+        <f aca="false">LibManager!A17</f>
+        <v>ElementCmpLT</v>
+      </c>
+      <c r="B17" s="0" t="n">
+        <f aca="false">LibManager!B17</f>
+        <v>1</v>
+      </c>
+      <c r="C17" s="0" t="n">
+        <f aca="false">LibManager!C17</f>
+        <v>2</v>
+      </c>
+      <c r="D17" s="0" t="str">
+        <f aca="false">LibManager!E17</f>
+        <v>1,2</v>
+      </c>
+      <c r="E17" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="F17" s="0" t="s">
+        <v>142</v>
+      </c>
+      <c r="G17" s="0" t="s">
+        <v>106</v>
+      </c>
+      <c r="H17" s="0" t="s">
+        <v>143</v>
+      </c>
+      <c r="I17" s="0" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0" t="str">
+        <f aca="false">LibManager!A18</f>
+        <v>ElementCmpLTE</v>
+      </c>
+      <c r="B18" s="0" t="n">
+        <f aca="false">LibManager!B18</f>
+        <v>1</v>
+      </c>
+      <c r="C18" s="0" t="n">
+        <f aca="false">LibManager!C18</f>
+        <v>2</v>
+      </c>
+      <c r="D18" s="0" t="str">
+        <f aca="false">LibManager!E18</f>
+        <v>1,2</v>
+      </c>
+      <c r="E18" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="F18" s="0" t="s">
+        <v>142</v>
+      </c>
+      <c r="G18" s="0" t="s">
+        <v>106</v>
+      </c>
+      <c r="H18" s="0" t="s">
+        <v>143</v>
+      </c>
+      <c r="I18" s="0" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="0" t="str">
+        <f aca="false">LibManager!A19</f>
+        <v>ElementDiv</v>
+      </c>
+      <c r="B19" s="0" t="n">
+        <f aca="false">LibManager!B19</f>
+        <v>1</v>
+      </c>
+      <c r="C19" s="0" t="n">
+        <f aca="false">LibManager!C19</f>
+        <v>2</v>
+      </c>
+      <c r="D19" s="0" t="str">
+        <f aca="false">LibManager!E19</f>
+        <v>0,1,2</v>
+      </c>
+      <c r="E19" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="F19" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="G19" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="H19" s="0" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="0" t="str">
+        <f aca="false">LibManager!A20</f>
+        <v>ElementExp</v>
+      </c>
+      <c r="B20" s="0" t="n">
+        <f aca="false">LibManager!B20</f>
+        <v>1</v>
+      </c>
+      <c r="C20" s="0" t="n">
+        <f aca="false">LibManager!C20</f>
+        <v>1</v>
+      </c>
+      <c r="D20" s="0" t="n">
+        <f aca="false">LibManager!E20</f>
+        <v>1</v>
+      </c>
+      <c r="E20" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F20" s="0" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0" t="str">
+        <f aca="false">LibManager!A21</f>
+        <v>ElementIsNaN</v>
+      </c>
+      <c r="B21" s="0" t="n">
+        <f aca="false">LibManager!B21</f>
+        <v>1</v>
+      </c>
+      <c r="C21" s="0" t="n">
+        <f aca="false">LibManager!C21</f>
+        <v>1</v>
+      </c>
+      <c r="D21" s="0" t="n">
+        <f aca="false">LibManager!E21</f>
+        <v>1</v>
+      </c>
+      <c r="E21" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F21" s="0" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="0" t="str">
+        <f aca="false">LibManager!A22</f>
+        <v>ElementLog</v>
+      </c>
+      <c r="B22" s="0" t="n">
+        <f aca="false">LibManager!B22</f>
+        <v>1</v>
+      </c>
+      <c r="C22" s="0" t="n">
+        <f aca="false">LibManager!C22</f>
+        <v>1</v>
+      </c>
+      <c r="D22" s="0" t="str">
+        <f aca="false">LibManager!E22</f>
+        <v>0,1</v>
+      </c>
+      <c r="E22" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="F22" s="0" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="0" t="str">
+        <f aca="false">LibManager!A23</f>
+        <v>ElementMax</v>
+      </c>
+      <c r="B23" s="0" t="n">
+        <f aca="false">LibManager!B23</f>
+        <v>1</v>
+      </c>
+      <c r="C23" s="0" t="n">
+        <f aca="false">LibManager!C23</f>
+        <v>2</v>
+      </c>
+      <c r="D23" s="0" t="str">
+        <f aca="false">LibManager!E23</f>
+        <v>0,1,2</v>
+      </c>
+      <c r="E23" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="F23" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="G23" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="H23" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="I23" s="0" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="0" t="str">
+        <f aca="false">LibManager!A24</f>
+        <v>ElementMin</v>
+      </c>
+      <c r="B24" s="0" t="n">
+        <f aca="false">LibManager!B24</f>
+        <v>1</v>
+      </c>
+      <c r="C24" s="0" t="n">
+        <f aca="false">LibManager!C24</f>
+        <v>2</v>
+      </c>
+      <c r="D24" s="0" t="str">
+        <f aca="false">LibManager!E24</f>
+        <v>0,1,2</v>
+      </c>
+      <c r="E24" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="F24" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="G24" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="H24" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="I24" s="0" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="0" t="str">
+        <f aca="false">LibManager!A25</f>
+        <v>ElementMul</v>
+      </c>
+      <c r="B25" s="0" t="n">
+        <f aca="false">LibManager!B25</f>
+        <v>1</v>
+      </c>
+      <c r="C25" s="0" t="n">
+        <f aca="false">LibManager!C25</f>
+        <v>2</v>
+      </c>
+      <c r="D25" s="0" t="str">
+        <f aca="false">LibManager!E25</f>
+        <v>0,1,2</v>
+      </c>
+      <c r="E25" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="F25" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="G25" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="H25" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="I25" s="0" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="0" t="str">
+        <f aca="false">LibManager!A26</f>
+        <v>ElementPow</v>
+      </c>
+      <c r="B26" s="0" t="n">
+        <f aca="false">LibManager!B26</f>
+        <v>1</v>
+      </c>
+      <c r="C26" s="0" t="n">
+        <f aca="false">LibManager!C26</f>
+        <v>2</v>
+      </c>
+      <c r="D26" s="0" t="str">
+        <f aca="false">LibManager!E26</f>
+        <v>0,1,2</v>
+      </c>
+      <c r="E26" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="F26" s="0" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="0" t="str">
+        <f aca="false">LibManager!A27</f>
+        <v>ElementSelect</v>
+      </c>
+      <c r="B27" s="0" t="n">
+        <f aca="false">LibManager!B27</f>
+        <v>1</v>
+      </c>
+      <c r="C27" s="0" t="n">
+        <f aca="false">LibManager!C27</f>
+        <v>3</v>
+      </c>
+      <c r="D27" s="0" t="n">
+        <f aca="false">LibManager!E27</f>
+        <v>1</v>
+      </c>
+      <c r="E27" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F27" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G27" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H27" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I27" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J27" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0" t="str">
+        <f aca="false">LibManager!A28</f>
+        <v>ElementSub</v>
+      </c>
+      <c r="B28" s="0" t="n">
+        <f aca="false">LibManager!B28</f>
+        <v>1</v>
+      </c>
+      <c r="C28" s="0" t="n">
+        <f aca="false">LibManager!C28</f>
+        <v>2</v>
+      </c>
+      <c r="D28" s="0" t="str">
+        <f aca="false">LibManager!E28</f>
+        <v>0,1,2</v>
+      </c>
+      <c r="E28" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="F28" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="G28" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="H28" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="I28" s="0" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="0" t="str">
+        <f aca="false">LibManager!A29</f>
+        <v>EmbeddingBag</v>
+      </c>
+      <c r="B29" s="0" t="n">
+        <f aca="false">LibManager!B29</f>
+        <v>1</v>
+      </c>
+      <c r="C29" s="0" t="n">
+        <f aca="false">LibManager!C29</f>
+        <v>4</v>
+      </c>
+      <c r="D29" s="0" t="str">
+        <f aca="false">LibManager!E29</f>
+        <v>NONE</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0" t="str">
+        <f aca="false">LibManager!A30</f>
+        <v>ExtractTensor</v>
+      </c>
+      <c r="B30" s="0" t="n">
+        <f aca="false">LibManager!B30</f>
+        <v>1</v>
+      </c>
+      <c r="C30" s="0" t="n">
+        <f aca="false">LibManager!C30</f>
+        <v>1</v>
+      </c>
+      <c r="D30" s="0" t="n">
+        <f aca="false">LibManager!E30</f>
+        <v>1</v>
+      </c>
+      <c r="E30" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F30" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G30" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H30" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I30" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J30" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="0" t="str">
+        <f aca="false">LibManager!A31</f>
+        <v>Flip</v>
+      </c>
+      <c r="B31" s="0" t="n">
+        <f aca="false">LibManager!B31</f>
+        <v>1</v>
+      </c>
+      <c r="C31" s="0" t="n">
+        <f aca="false">LibManager!C31</f>
+        <v>1</v>
+      </c>
+      <c r="D31" s="0" t="n">
+        <f aca="false">LibManager!E31</f>
+        <v>1</v>
+      </c>
+      <c r="E31" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F31" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G31" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H31" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I31" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J31" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="0" t="str">
+        <f aca="false">LibManager!A32</f>
+        <v>FullyConnected</v>
+      </c>
+      <c r="B32" s="0" t="n">
+        <f aca="false">LibManager!B32</f>
+        <v>1</v>
+      </c>
+      <c r="C32" s="0" t="n">
+        <f aca="false">LibManager!C32</f>
+        <v>3</v>
+      </c>
+      <c r="D32" s="0" t="str">
+        <f aca="false">LibManager!E32</f>
+        <v>0,1,2</v>
+      </c>
+      <c r="E32" s="0" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="0" t="str">
+        <f aca="false">LibManager!A33</f>
+        <v>FusedRowwiseQuantizedSparseLengthsSum</v>
+      </c>
+      <c r="B33" s="0" t="n">
+        <f aca="false">LibManager!B33</f>
+        <v>1</v>
+      </c>
+      <c r="C33" s="0" t="n">
+        <f aca="false">LibManager!C33</f>
+        <v>3</v>
+      </c>
+      <c r="D33" s="0" t="n">
+        <f aca="false">LibManager!E33</f>
+        <v>0</v>
+      </c>
+      <c r="E33" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F33" s="0" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="0" t="str">
+        <f aca="false">LibManager!A34</f>
+        <v>FusedRowwiseQuantizedSparseLengthsWeightedSum</v>
+      </c>
+      <c r="B34" s="0" t="n">
+        <f aca="false">LibManager!B34</f>
+        <v>1</v>
+      </c>
+      <c r="C34" s="0" t="n">
+        <f aca="false">LibManager!C34</f>
+        <v>4</v>
+      </c>
+      <c r="D34" s="0" t="n">
+        <f aca="false">LibManager!E34</f>
+        <v>0</v>
+      </c>
+      <c r="E34" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F34" s="0" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="0" t="str">
+        <f aca="false">LibManager!A35</f>
+        <v>Gather</v>
+      </c>
+      <c r="B35" s="0" t="n">
+        <f aca="false">LibManager!B35</f>
+        <v>1</v>
+      </c>
+      <c r="C35" s="0" t="n">
+        <f aca="false">LibManager!C35</f>
+        <v>2</v>
+      </c>
+      <c r="D35" s="0" t="str">
+        <f aca="false">LibManager!E35</f>
+        <v>1,2</v>
+      </c>
+      <c r="E35" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="F35" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="G35" s="0" t="s">
+        <v>145</v>
+      </c>
+      <c r="H35" s="0" t="s">
+        <v>146</v>
+      </c>
+      <c r="I35" s="0" t="s">
+        <v>147</v>
+      </c>
+      <c r="J35" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="K35" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="L35" s="0" t="s">
+        <v>148</v>
+      </c>
+      <c r="M35" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="N35" s="0" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="0" t="str">
+        <f aca="false">LibManager!A36</f>
+        <v>GatherRanges</v>
+      </c>
+      <c r="B36" s="0" t="n">
+        <f aca="false">LibManager!B36</f>
+        <v>2</v>
+      </c>
+      <c r="C36" s="0" t="n">
+        <f aca="false">LibManager!C36</f>
+        <v>2</v>
+      </c>
+      <c r="D36" s="0" t="str">
+        <f aca="false">LibManager!E36</f>
+        <v>2,3</v>
+      </c>
+      <c r="E36" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="F36" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="G36" s="0" t="s">
+        <v>145</v>
+      </c>
+      <c r="H36" s="0" t="s">
+        <v>146</v>
+      </c>
+      <c r="I36" s="0" t="s">
+        <v>147</v>
+      </c>
+      <c r="J36" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="K36" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="L36" s="0" t="s">
+        <v>148</v>
+      </c>
+      <c r="M36" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="N36" s="0" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="0" t="str">
+        <f aca="false">LibManager!A37</f>
+        <v>InsertTensor</v>
+      </c>
+      <c r="B37" s="0" t="n">
+        <f aca="false">LibManager!B37</f>
+        <v>1</v>
+      </c>
+      <c r="C37" s="0" t="n">
+        <f aca="false">LibManager!C37</f>
+        <v>1</v>
+      </c>
+      <c r="D37" s="0" t="n">
+        <f aca="false">LibManager!E37</f>
+        <v>1</v>
+      </c>
+      <c r="E37" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F37" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G37" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H37" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I37" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J37" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="0" t="str">
+        <f aca="false">LibManager!A38</f>
+        <v>Int8Converter</v>
+      </c>
+      <c r="B38" s="0" t="n">
+        <f aca="false">LibManager!B38</f>
+        <v>1</v>
+      </c>
+      <c r="C38" s="0" t="n">
+        <f aca="false">LibManager!C38</f>
+        <v>1</v>
+      </c>
+      <c r="D38" s="0" t="n">
+        <f aca="false">LibManager!E38</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="0" t="str">
+        <f aca="false">LibManager!A39</f>
+        <v>IntLookupTable</v>
+      </c>
+      <c r="B39" s="0" t="n">
+        <f aca="false">LibManager!B39</f>
+        <v>1</v>
+      </c>
+      <c r="C39" s="0" t="n">
+        <f aca="false">LibManager!C39</f>
+        <v>2</v>
+      </c>
+      <c r="D39" s="0" t="str">
+        <f aca="false">LibManager!E39</f>
+        <v>NONE</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="0" t="str">
+        <f aca="false">LibManager!A40</f>
+        <v>LengthsSum</v>
+      </c>
+      <c r="B40" s="0" t="n">
+        <f aca="false">LibManager!B40</f>
+        <v>1</v>
+      </c>
+      <c r="C40" s="0" t="n">
+        <f aca="false">LibManager!C40</f>
+        <v>2</v>
+      </c>
+      <c r="D40" s="0" t="n">
+        <f aca="false">LibManager!E40</f>
+        <v>1</v>
+      </c>
+      <c r="E40" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F40" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G40" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H40" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I40" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J40" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="0" t="str">
+        <f aca="false">LibManager!A41</f>
+        <v>LengthsToRanges</v>
+      </c>
+      <c r="B41" s="0" t="n">
+        <f aca="false">LibManager!B41</f>
+        <v>1</v>
+      </c>
+      <c r="C41" s="0" t="n">
+        <f aca="false">LibManager!C41</f>
+        <v>1</v>
+      </c>
+      <c r="D41" s="0" t="n">
+        <f aca="false">LibManager!E41</f>
+        <v>1</v>
+      </c>
+      <c r="E41" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F41" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G41" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H41" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I41" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J41" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="0" t="str">
+        <f aca="false">LibManager!A42</f>
+        <v>LocalResponseNormalization</v>
+      </c>
+      <c r="B42" s="0" t="n">
+        <f aca="false">LibManager!B42</f>
+        <v>2</v>
+      </c>
+      <c r="C42" s="0" t="n">
+        <f aca="false">LibManager!C42</f>
+        <v>1</v>
+      </c>
+      <c r="D42" s="0" t="n">
+        <f aca="false">LibManager!E42</f>
+        <v>1</v>
+      </c>
+      <c r="E42" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F42" s="0" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="0" t="str">
+        <f aca="false">LibManager!A43</f>
+        <v>MatMul</v>
+      </c>
+      <c r="B43" s="0" t="n">
+        <f aca="false">LibManager!B43</f>
+        <v>1</v>
+      </c>
+      <c r="C43" s="0" t="n">
+        <f aca="false">LibManager!C43</f>
+        <v>2</v>
+      </c>
+      <c r="D43" s="0" t="n">
+        <f aca="false">LibManager!E43</f>
+        <v>1</v>
+      </c>
+      <c r="E43" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F43" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G43" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H43" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I43" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J43" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="0" t="str">
+        <f aca="false">LibManager!A44</f>
+        <v>MaxPool</v>
+      </c>
+      <c r="B44" s="0" t="n">
+        <f aca="false">LibManager!B44</f>
+        <v>1</v>
+      </c>
+      <c r="C44" s="0" t="n">
+        <f aca="false">LibManager!C44</f>
+        <v>1</v>
+      </c>
+      <c r="D44" s="0" t="str">
+        <f aca="false">LibManager!E44</f>
+        <v>0,1</v>
+      </c>
+      <c r="E44" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="F44" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="G44" s="0" t="s">
+        <v>106</v>
+      </c>
+      <c r="H44" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="I44" s="0" t="s">
+        <v>108</v>
+      </c>
+      <c r="J44" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="K44" s="0" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="0" t="str">
+        <f aca="false">LibManager!A45</f>
+        <v>MaxSplat</v>
+      </c>
+      <c r="B45" s="0" t="n">
+        <f aca="false">LibManager!B45</f>
+        <v>1</v>
+      </c>
+      <c r="C45" s="0" t="n">
+        <f aca="false">LibManager!C45</f>
+        <v>1</v>
+      </c>
+      <c r="D45" s="0" t="n">
+        <f aca="false">LibManager!E45</f>
+        <v>1</v>
+      </c>
+      <c r="E45" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F45" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G45" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H45" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I45" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J45" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="0" t="str">
+        <f aca="false">LibManager!A46</f>
+        <v>Modulo</v>
+      </c>
+      <c r="B46" s="0" t="n">
+        <f aca="false">LibManager!B46</f>
+        <v>1</v>
+      </c>
+      <c r="C46" s="0" t="n">
+        <f aca="false">LibManager!C46</f>
+        <v>1</v>
+      </c>
+      <c r="D46" s="0" t="n">
+        <f aca="false">LibManager!E46</f>
+        <v>1</v>
+      </c>
+      <c r="E46" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="F46" s="0" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="0" t="str">
+        <f aca="false">LibManager!A47</f>
+        <v>Quantize</v>
+      </c>
+      <c r="B47" s="0" t="n">
+        <f aca="false">LibManager!B47</f>
+        <v>1</v>
+      </c>
+      <c r="C47" s="0" t="n">
+        <f aca="false">LibManager!C47</f>
+        <v>1</v>
+      </c>
+      <c r="D47" s="0" t="n">
+        <f aca="false">LibManager!E47</f>
+        <v>0</v>
+      </c>
+      <c r="E47" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="F47" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="G47" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="H47" s="0" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="0" t="str">
+        <f aca="false">LibManager!A48</f>
+        <v>RescaleQuantized</v>
+      </c>
+      <c r="B48" s="0" t="n">
+        <f aca="false">LibManager!B48</f>
+        <v>1</v>
+      </c>
+      <c r="C48" s="0" t="n">
+        <f aca="false">LibManager!C48</f>
+        <v>1</v>
+      </c>
+      <c r="D48" s="0" t="n">
+        <f aca="false">LibManager!E48</f>
+        <v>1</v>
+      </c>
+      <c r="E48" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="F48" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="G48" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="H48" s="0" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="0" t="str">
+        <f aca="false">LibManager!A49</f>
+        <v>RowwiseQuantizedFullyConnected</v>
+      </c>
+      <c r="B49" s="0" t="n">
+        <f aca="false">LibManager!B49</f>
+        <v>1</v>
+      </c>
+      <c r="C49" s="0" t="n">
+        <f aca="false">LibManager!C49</f>
+        <v>5</v>
+      </c>
+      <c r="D49" s="0" t="str">
+        <f aca="false">LibManager!E49</f>
+        <v>NONE</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="0" t="str">
+        <f aca="false">LibManager!A50</f>
+        <v>RowwiseQuantizedSparseLengthsWeightedSum</v>
+      </c>
+      <c r="B50" s="0" t="n">
+        <f aca="false">LibManager!B50</f>
+        <v>1</v>
+      </c>
+      <c r="C50" s="0" t="n">
+        <f aca="false">LibManager!C50</f>
+        <v>6</v>
+      </c>
+      <c r="D50" s="0" t="str">
+        <f aca="false">LibManager!E50</f>
+        <v>0,1</v>
+      </c>
+      <c r="E50" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="F50" s="0" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="0" t="str">
+        <f aca="false">LibManager!A51</f>
+        <v>ScatterData</v>
+      </c>
+      <c r="B51" s="0" t="n">
+        <f aca="false">LibManager!B51</f>
+        <v>1</v>
+      </c>
+      <c r="C51" s="0" t="n">
+        <f aca="false">LibManager!C51</f>
+        <v>2</v>
+      </c>
+      <c r="D51" s="0" t="n">
+        <f aca="false">LibManager!E51</f>
+        <v>1</v>
+      </c>
+      <c r="E51" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F51" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G51" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H51" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I51" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J51" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="0" t="str">
+        <f aca="false">LibManager!A52</f>
+        <v>Sigmoid</v>
+      </c>
+      <c r="B52" s="0" t="n">
+        <f aca="false">LibManager!B52</f>
+        <v>1</v>
+      </c>
+      <c r="C52" s="0" t="n">
+        <f aca="false">LibManager!C52</f>
+        <v>1</v>
+      </c>
+      <c r="D52" s="0" t="n">
+        <f aca="false">LibManager!E52</f>
+        <v>1</v>
+      </c>
+      <c r="E52" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F52" s="0" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="0" t="str">
+        <f aca="false">LibManager!A53</f>
+        <v>SoftMax</v>
+      </c>
+      <c r="B53" s="0" t="n">
+        <f aca="false">LibManager!B53</f>
+        <v>1</v>
+      </c>
+      <c r="C53" s="0" t="n">
+        <f aca="false">LibManager!C53</f>
+        <v>1</v>
+      </c>
+      <c r="D53" s="0" t="n">
+        <f aca="false">LibManager!E53</f>
+        <v>1</v>
+      </c>
+      <c r="E53" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F53" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G53" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H53" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I53" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J53" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="0" t="str">
+        <f aca="false">LibManager!A54</f>
+        <v>SparseLengthsWeightedSum</v>
+      </c>
+      <c r="B54" s="0" t="n">
+        <f aca="false">LibManager!B54</f>
+        <v>1</v>
+      </c>
+      <c r="C54" s="0" t="n">
+        <f aca="false">LibManager!C54</f>
+        <v>4</v>
+      </c>
+      <c r="D54" s="0" t="n">
+        <f aca="false">LibManager!E54</f>
+        <v>1</v>
+      </c>
+      <c r="E54" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F54" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G54" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H54" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I54" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J54" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="0" t="str">
+        <f aca="false">LibManager!A55</f>
+        <v>SparseToDense</v>
+      </c>
+      <c r="B55" s="0" t="n">
+        <f aca="false">LibManager!B55</f>
+        <v>1</v>
+      </c>
+      <c r="C55" s="0" t="n">
+        <f aca="false">LibManager!C55</f>
+        <v>2</v>
+      </c>
+      <c r="D55" s="0" t="n">
+        <f aca="false">LibManager!E55</f>
+        <v>1</v>
+      </c>
+      <c r="E55" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F55" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G55" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H55" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I55" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J55" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="0" t="str">
+        <f aca="false">LibManager!A56</f>
+        <v>SparseToDenseMask</v>
+      </c>
+      <c r="B56" s="0" t="n">
+        <f aca="false">LibManager!B56</f>
+        <v>1</v>
+      </c>
+      <c r="C56" s="0" t="n">
+        <f aca="false">LibManager!C56</f>
+        <v>4</v>
+      </c>
+      <c r="D56" s="0" t="n">
+        <f aca="false">LibManager!E56</f>
+        <v>1</v>
+      </c>
+      <c r="E56" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F56" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G56" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H56" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I56" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J56" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="0" t="str">
+        <f aca="false">LibManager!A57</f>
+        <v>Splat</v>
+      </c>
+      <c r="B57" s="0" t="n">
+        <f aca="false">LibManager!B57</f>
+        <v>1</v>
+      </c>
+      <c r="C57" s="0" t="n">
+        <f aca="false">LibManager!C57</f>
+        <v>0</v>
+      </c>
+      <c r="D57" s="0" t="n">
+        <f aca="false">LibManager!E57</f>
+        <v>0</v>
+      </c>
+      <c r="E57" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F57" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G57" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H57" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I57" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J57" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="0" t="str">
+        <f aca="false">LibManager!A58</f>
+        <v>Syncopy</v>
+      </c>
+      <c r="B58" s="0" t="n">
+        <f aca="false">LibManager!B58</f>
+        <v>1</v>
+      </c>
+      <c r="C58" s="0" t="n">
+        <f aca="false">LibManager!C58</f>
+        <v>1</v>
+      </c>
+      <c r="D58" s="0" t="n">
+        <f aca="false">LibManager!E58</f>
+        <v>1</v>
+      </c>
+      <c r="E58" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F58" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G58" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H58" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I58" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J58" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="0" t="str">
+        <f aca="false">LibManager!A59</f>
+        <v>Tanh</v>
+      </c>
+      <c r="B59" s="0" t="n">
+        <f aca="false">LibManager!B59</f>
+        <v>1</v>
+      </c>
+      <c r="C59" s="0" t="n">
+        <f aca="false">LibManager!C59</f>
+        <v>1</v>
+      </c>
+      <c r="D59" s="0" t="n">
+        <f aca="false">LibManager!E59</f>
+        <v>1</v>
+      </c>
+      <c r="E59" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F59" s="0" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="0" t="str">
+        <f aca="false">LibManager!A60</f>
+        <v>TensorView</v>
+      </c>
+      <c r="B60" s="0" t="n">
+        <f aca="false">LibManager!B60</f>
+        <v>0</v>
+      </c>
+      <c r="C60" s="0" t="n">
+        <f aca="false">LibManager!C60</f>
+        <v>1</v>
+      </c>
+      <c r="D60" s="0" t="n">
+        <f aca="false">LibManager!E60</f>
+        <v>0</v>
+      </c>
+      <c r="E60" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F60" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G60" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H60" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I60" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J60" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="0" t="str">
+        <f aca="false">LibManager!A61</f>
+        <v>TopK</v>
+      </c>
+      <c r="B61" s="0" t="n">
+        <f aca="false">LibManager!B61</f>
+        <v>2</v>
+      </c>
+      <c r="C61" s="0" t="n">
+        <f aca="false">LibManager!C61</f>
+        <v>1</v>
+      </c>
+      <c r="D61" s="0" t="n">
+        <f aca="false">LibManager!E61</f>
+        <v>2</v>
+      </c>
+      <c r="E61" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F61" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G61" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H61" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I61" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J61" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="0" t="str">
+        <f aca="false">LibManager!A62</f>
+        <v>Transpose</v>
+      </c>
+      <c r="B62" s="0" t="n">
+        <f aca="false">LibManager!B62</f>
+        <v>1</v>
+      </c>
+      <c r="C62" s="0" t="n">
+        <f aca="false">LibManager!C62</f>
+        <v>1</v>
+      </c>
+      <c r="D62" s="0" t="n">
+        <f aca="false">LibManager!E62</f>
+        <v>1</v>
+      </c>
+      <c r="E62" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F62" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G62" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="H62" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I62" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="J62" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="0" t="n">
+        <f aca="false">LibManager!A63</f>
+        <v>0</v>
+      </c>
+      <c r="B63" s="0" t="n">
+        <f aca="false">LibManager!B63</f>
+        <v>0</v>
+      </c>
+      <c r="C63" s="0" t="n">
+        <f aca="false">LibManager!C63</f>
+        <v>0</v>
+      </c>
+      <c r="D63" s="0" t="n">
+        <f aca="false">LibManager!E63</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="0" t="n">
+        <f aca="false">LibManager!A64</f>
+        <v>0</v>
+      </c>
+      <c r="B64" s="0" t="n">
+        <f aca="false">LibManager!B64</f>
+        <v>0</v>
+      </c>
+      <c r="C64" s="0" t="n">
+        <f aca="false">LibManager!C64</f>
+        <v>0</v>
+      </c>
+      <c r="D64" s="0" t="n">
+        <f aca="false">LibManager!E64</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="0" t="n">
+        <f aca="false">LibManager!A65</f>
+        <v>0</v>
+      </c>
+      <c r="B65" s="0" t="n">
+        <f aca="false">LibManager!B65</f>
+        <v>0</v>
+      </c>
+      <c r="C65" s="0" t="n">
+        <f aca="false">LibManager!C65</f>
+        <v>0</v>
+      </c>
+      <c r="D65" s="0" t="n">
+        <f aca="false">LibManager!E65</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="0" t="n">
+        <f aca="false">LibManager!A66</f>
+        <v>0</v>
+      </c>
+      <c r="B66" s="0" t="n">
+        <f aca="false">LibManager!B66</f>
+        <v>0</v>
+      </c>
+      <c r="C66" s="0" t="n">
+        <f aca="false">LibManager!C66</f>
+        <v>0</v>
+      </c>
+      <c r="D66" s="0" t="n">
+        <f aca="false">LibManager!E66</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="0" t="n">
+        <f aca="false">LibManager!A67</f>
+        <v>0</v>
+      </c>
+      <c r="B67" s="0" t="n">
+        <f aca="false">LibManager!B67</f>
+        <v>0</v>
+      </c>
+      <c r="C67" s="0" t="n">
+        <f aca="false">LibManager!C67</f>
+        <v>0</v>
+      </c>
+      <c r="D67" s="0" t="n">
+        <f aca="false">LibManager!E67</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="0" t="n">
+        <f aca="false">LibManager!A68</f>
+        <v>0</v>
+      </c>
+      <c r="B68" s="0" t="n">
+        <f aca="false">LibManager!B68</f>
+        <v>0</v>
+      </c>
+      <c r="C68" s="0" t="n">
+        <f aca="false">LibManager!C68</f>
+        <v>0</v>
+      </c>
+      <c r="D68" s="0" t="n">
+        <f aca="false">LibManager!E68</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="0" t="n">
+        <f aca="false">LibManager!A69</f>
+        <v>0</v>
+      </c>
+      <c r="B69" s="0" t="n">
+        <f aca="false">LibManager!B69</f>
+        <v>0</v>
+      </c>
+      <c r="C69" s="0" t="n">
+        <f aca="false">LibManager!C69</f>
+        <v>0</v>
+      </c>
+      <c r="D69" s="0" t="n">
+        <f aca="false">LibManager!E69</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="0" t="n">
+        <f aca="false">LibManager!A70</f>
+        <v>0</v>
+      </c>
+      <c r="B70" s="0" t="n">
+        <f aca="false">LibManager!B70</f>
+        <v>0</v>
+      </c>
+      <c r="C70" s="0" t="n">
+        <f aca="false">LibManager!C70</f>
+        <v>0</v>
+      </c>
+      <c r="D70" s="0" t="n">
+        <f aca="false">LibManager!E70</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
[dnn-library] [SW-3233] Fixing compilation errors debugging script output
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="150">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -353,7 +353,7 @@
     <t xml:space="preserve">UInt8QTy,UInt8QTy</t>
   </si>
   <si>
-    <t xml:space="preserve">Int64Ty,Int64Ty</t>
+    <t xml:space="preserve">Int64ITy,Int64ITy</t>
   </si>
   <si>
     <t xml:space="preserve">FloatTy,FloatTy,FloatTy</t>
@@ -362,13 +362,13 @@
     <t xml:space="preserve">Float16Ty,Float16Ty,Float16Ty</t>
   </si>
   <si>
-    <t xml:space="preserve">Int8Qty,Int8Qty,Int8Qty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int8Qty,Int8Qty,Int32QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int16QTy,Int16QTy,Int16Qty</t>
+    <t xml:space="preserve">Int8QTy,Int8QTy,Int8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int8QTy,Int8QTy,Int32QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int16QTy,Int16QTy,Int16QTy</t>
   </si>
   <si>
     <t xml:space="preserve">Int16QTy,Int16QTy,Int32QTy</t>
@@ -410,12 +410,6 @@
     <t xml:space="preserve">Int64ITy,Int32ITy</t>
   </si>
   <si>
-    <t xml:space="preserve">Int8QTy,Int8QTy,Int8QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int16QTy,Int16QTy,Int16QTy</t>
-  </si>
-  <si>
     <t xml:space="preserve">FloatTy,Int8QTy</t>
   </si>
   <si>
@@ -453,9 +447,6 @@
   </si>
   <si>
     <t xml:space="preserve">Int32ITy,Int32ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int64ITy,Int64ITy</t>
   </si>
   <si>
     <t xml:space="preserve">Int8QTy,Int32ITy</t>
@@ -2313,10 +2304,10 @@
         <v>112</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>129</v>
+        <v>113</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>130</v>
+        <v>115</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2445,28 +2436,28 @@
         <v>1</v>
       </c>
       <c r="E14" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="F14" s="0" t="s">
+        <v>130</v>
+      </c>
+      <c r="G14" s="0" t="s">
         <v>131</v>
       </c>
-      <c r="F14" s="0" t="s">
+      <c r="H14" s="0" t="s">
         <v>132</v>
       </c>
-      <c r="G14" s="0" t="s">
+      <c r="I14" s="0" t="s">
         <v>133</v>
       </c>
-      <c r="H14" s="0" t="s">
+      <c r="J14" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="I14" s="0" t="s">
+      <c r="K14" s="0" t="s">
         <v>135</v>
       </c>
-      <c r="J14" s="0" t="s">
+      <c r="L14" s="0" t="s">
         <v>136</v>
-      </c>
-      <c r="K14" s="0" t="s">
-        <v>137</v>
-      </c>
-      <c r="L14" s="0" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2493,13 +2484,13 @@
         <v>112</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>129</v>
+        <v>113</v>
       </c>
       <c r="H15" s="0" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="I15" s="0" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2520,19 +2511,19 @@
         <v>1,2</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F16" s="0" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="G16" s="0" t="s">
         <v>106</v>
       </c>
       <c r="H16" s="0" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="I16" s="0" t="s">
-        <v>144</v>
+        <v>110</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2553,19 +2544,19 @@
         <v>1,2</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F17" s="0" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="G17" s="0" t="s">
         <v>106</v>
       </c>
       <c r="H17" s="0" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="I17" s="0" t="s">
-        <v>144</v>
+        <v>110</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2586,19 +2577,19 @@
         <v>1,2</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="G18" s="0" t="s">
         <v>106</v>
       </c>
       <c r="H18" s="0" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="I18" s="0" t="s">
-        <v>144</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2625,10 +2616,10 @@
         <v>112</v>
       </c>
       <c r="G19" s="0" t="s">
-        <v>129</v>
+        <v>113</v>
       </c>
       <c r="H19" s="0" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2697,10 +2688,10 @@
         <v>0,1</v>
       </c>
       <c r="E22" s="0" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F22" s="0" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2727,13 +2718,13 @@
         <v>112</v>
       </c>
       <c r="G23" s="0" t="s">
-        <v>129</v>
+        <v>113</v>
       </c>
       <c r="H23" s="0" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="I23" s="0" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2760,13 +2751,13 @@
         <v>112</v>
       </c>
       <c r="G24" s="0" t="s">
-        <v>129</v>
+        <v>113</v>
       </c>
       <c r="H24" s="0" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="I24" s="0" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2793,13 +2784,13 @@
         <v>112</v>
       </c>
       <c r="G25" s="0" t="s">
-        <v>129</v>
+        <v>113</v>
       </c>
       <c r="H25" s="0" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="I25" s="0" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2886,13 +2877,13 @@
         <v>112</v>
       </c>
       <c r="G28" s="0" t="s">
-        <v>129</v>
+        <v>113</v>
       </c>
       <c r="H28" s="0" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="I28" s="0" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3078,13 +3069,13 @@
         <v>118</v>
       </c>
       <c r="G35" s="0" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="H35" s="0" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="I35" s="0" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="J35" s="0" t="s">
         <v>122</v>
@@ -3093,13 +3084,13 @@
         <v>119</v>
       </c>
       <c r="L35" s="0" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="M35" s="0" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="N35" s="0" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3126,13 +3117,13 @@
         <v>118</v>
       </c>
       <c r="G36" s="0" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="H36" s="0" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="I36" s="0" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="J36" s="0" t="s">
         <v>122</v>
@@ -3141,13 +3132,13 @@
         <v>119</v>
       </c>
       <c r="L36" s="0" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="M36" s="0" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="N36" s="0" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3474,13 +3465,13 @@
         <v>100</v>
       </c>
       <c r="F47" s="0" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="G47" s="0" t="s">
         <v>103</v>
       </c>
       <c r="H47" s="0" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3504,13 +3495,13 @@
         <v>100</v>
       </c>
       <c r="F48" s="0" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="G48" s="0" t="s">
         <v>103</v>
       </c>
       <c r="H48" s="0" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3549,10 +3540,10 @@
         <v>0,1</v>
       </c>
       <c r="E50" s="0" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="F50" s="0" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] piecing all previous changes together  * fixing generator script issues  * fixing compilation problems
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="150">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -930,8 +930,8 @@
       <c r="C14" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="E14" s="0" t="n">
-        <v>1</v>
+      <c r="E14" s="0" t="s">
+        <v>13</v>
       </c>
       <c r="F14" s="0" t="s">
         <v>14</v>
@@ -2431,9 +2431,9 @@
         <f aca="false">LibManager!C14</f>
         <v>1</v>
       </c>
-      <c r="D14" s="0" t="n">
+      <c r="D14" s="0" t="str">
         <f aca="false">LibManager!E14</f>
-        <v>1</v>
+        <v>0,1</v>
       </c>
       <c r="E14" s="0" t="s">
         <v>129</v>
@@ -2994,7 +2994,7 @@
         <v>0,1,2</v>
       </c>
       <c r="E32" s="0" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3193,6 +3193,12 @@
       <c r="D38" s="0" t="n">
         <f aca="false">LibManager!E38</f>
         <v>1</v>
+      </c>
+      <c r="E38" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="F38" s="0" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] more "glue" to put all the changes in place
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="153">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -83,9 +83,6 @@
     <t xml:space="preserve">Axis</t>
   </si>
   <si>
-    <t xml:space="preserve">Threaded, Int8, Int8Threaded</t>
-  </si>
-  <si>
     <t xml:space="preserve">Checksum</t>
   </si>
   <si>
@@ -188,9 +185,6 @@
     <t xml:space="preserve">FusedRowwiseQuantizedSparseLengthsWeightedSum</t>
   </si>
   <si>
-    <t xml:space="preserve">FloatTy, FloatTyThreaded, FloatTyVectorized, FloatTyVectorized</t>
-  </si>
-  <si>
     <t xml:space="preserve">Gather</t>
   </si>
   <si>
@@ -290,7 +284,7 @@
     <t xml:space="preserve">Splat</t>
   </si>
   <si>
-    <t xml:space="preserve">Syncopy</t>
+    <t xml:space="preserve">#Syncopy =&gt; commented out (special case)</t>
   </si>
   <si>
     <t xml:space="preserve">SyncOffset</t>
@@ -305,18 +299,18 @@
     <t xml:space="preserve">TopK</t>
   </si>
   <si>
-    <t xml:space="preserve">K</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Threaded_all, Threaded_k4, Threaded_k4, Threaded_k8</t>
-  </si>
-  <si>
     <t xml:space="preserve">Transpose</t>
   </si>
   <si>
     <t xml:space="preserve">Shuffle</t>
   </si>
   <si>
+    <t xml:space="preserve">MaxPoolWithArgMax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,2</t>
+  </si>
+  <si>
     <t xml:space="preserve">FloatTy</t>
   </si>
   <si>
@@ -377,87 +371,99 @@
     <t xml:space="preserve">Float16Ty,FloatTy</t>
   </si>
   <si>
+    <t xml:space="preserve">#Float16Ty,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#Float16Ty,Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,Float16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#FloatTy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#Int32ITy,Float16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#Int32ITy,FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#Int32ITy,Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#Int64ITy,Float16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int64ITy,FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#Int64ITy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,Int8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,UInt8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,Int16QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,Int32QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,Int8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,UInt8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,Int16QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,Int32QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32ITy,Int32ITy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int64ITy,Int64ITy,Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,Float16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32ITy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#Float16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,Int32ITy</t>
+  </si>
+  <si>
     <t xml:space="preserve">Float16Ty,Int32ITy</t>
   </si>
   <si>
+    <t xml:space="preserve">Int8QTy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UInt8QTy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int16QTy,Int32ITy</t>
+  </si>
+  <si>
     <t xml:space="preserve">Float16Ty,Int64ITy</t>
   </si>
   <si>
-    <t xml:space="preserve">FloatTy,Float16Ty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FloatTy,Int32ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FloatTy,Int64ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int32ITy,Float16Ty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int32ITy,FloatTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int32ITy,Int64ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int64ITy,Float16Ty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int64ITy,FloatTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int64ITy,Int32ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FloatTy,Int8QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FloatTy,UInt8QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FloatTy,Int16QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FloatTy,Int32QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Float16Ty,Int8QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Float16Ty,UInt8QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Float16Ty,Int16QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Float16Ty,Int32QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int32ITy,Int32ITy,Int32ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int64ITy,Int64ITy,Int64ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FloatTy,FloatTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Float16Ty,Float16Ty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int32ITy,Int32ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int8QTy,Int32ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UInt8QTy,Int32ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int16QTy,Int32ITy</t>
-  </si>
-  <si>
     <t xml:space="preserve">Int8QTy,Int64ITy</t>
   </si>
   <si>
@@ -471,6 +477,9 @@
   </si>
   <si>
     <t xml:space="preserve">Int32QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#Float16Ty,UInt8QTy</t>
   </si>
 </sst>
 </file>
@@ -638,16 +647,16 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:G63"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="70"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="79.98"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="27.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="51.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="7.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="8" style="0" width="8.67"/>
   </cols>
   <sheetData>
@@ -791,7 +800,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="G7" s="0" t="s">
         <v>8</v>
@@ -799,7 +808,7 @@
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B8" s="0" t="n">
         <v>0</v>
@@ -816,7 +825,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B9" s="0" t="n">
         <v>1</v>
@@ -828,7 +837,7 @@
         <v>13</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G9" s="0" t="s">
         <v>8</v>
@@ -836,7 +845,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B10" s="0" t="n">
         <v>1</v>
@@ -845,13 +854,13 @@
         <v>3</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E10" s="0" t="s">
         <v>17</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G10" s="0" t="s">
         <v>8</v>
@@ -859,7 +868,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B11" s="0" t="n">
         <v>1</v>
@@ -868,7 +877,7 @@
         <v>3</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E11" s="0" t="n">
         <v>0</v>
@@ -882,19 +891,19 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="0" t="s">
         <v>27</v>
-      </c>
-      <c r="B12" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="0" t="s">
-        <v>28</v>
       </c>
       <c r="G12" s="0" t="s">
         <v>8</v>
@@ -902,7 +911,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B13" s="0" t="n">
         <v>1</v>
@@ -922,7 +931,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B14" s="0" t="n">
         <v>1</v>
@@ -942,7 +951,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B15" s="0" t="n">
         <v>1</v>
@@ -954,7 +963,7 @@
         <v>17</v>
       </c>
       <c r="F15" s="0" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G15" s="0" t="s">
         <v>8</v>
@@ -962,19 +971,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" s="0" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C16" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="E16" s="0" t="s">
-        <v>33</v>
-      </c>
       <c r="F16" s="0" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G16" s="0" t="s">
         <v>8</v>
@@ -982,7 +991,7 @@
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B17" s="0" t="n">
         <v>1</v>
@@ -991,10 +1000,10 @@
         <v>2</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F17" s="0" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G17" s="0" t="s">
         <v>8</v>
@@ -1002,7 +1011,7 @@
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B18" s="0" t="n">
         <v>1</v>
@@ -1011,10 +1020,10 @@
         <v>2</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G18" s="0" t="s">
         <v>8</v>
@@ -1022,7 +1031,7 @@
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B19" s="0" t="n">
         <v>1</v>
@@ -1034,7 +1043,7 @@
         <v>17</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G19" s="0" t="s">
         <v>8</v>
@@ -1042,7 +1051,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B20" s="0" t="n">
         <v>1</v>
@@ -1059,7 +1068,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B21" s="0" t="n">
         <v>1</v>
@@ -1079,7 +1088,7 @@
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B22" s="0" t="n">
         <v>1</v>
@@ -1091,7 +1100,7 @@
         <v>13</v>
       </c>
       <c r="F22" s="0" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G22" s="0" t="s">
         <v>8</v>
@@ -1099,7 +1108,7 @@
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B23" s="0" t="n">
         <v>1</v>
@@ -1111,7 +1120,7 @@
         <v>17</v>
       </c>
       <c r="F23" s="0" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G23" s="0" t="s">
         <v>8</v>
@@ -1119,7 +1128,7 @@
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B24" s="0" t="n">
         <v>1</v>
@@ -1131,7 +1140,7 @@
         <v>17</v>
       </c>
       <c r="F24" s="0" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G24" s="0" t="s">
         <v>8</v>
@@ -1139,7 +1148,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B25" s="0" t="n">
         <v>1</v>
@@ -1151,7 +1160,7 @@
         <v>17</v>
       </c>
       <c r="F25" s="0" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G25" s="0" t="s">
         <v>8</v>
@@ -1159,7 +1168,7 @@
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B26" s="0" t="n">
         <v>1</v>
@@ -1171,7 +1180,7 @@
         <v>17</v>
       </c>
       <c r="F26" s="0" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G26" s="0" t="s">
         <v>8</v>
@@ -1179,7 +1188,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B27" s="0" t="n">
         <v>1</v>
@@ -1199,7 +1208,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B28" s="0" t="n">
         <v>1</v>
@@ -1211,7 +1220,7 @@
         <v>17</v>
       </c>
       <c r="F28" s="0" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G28" s="0" t="s">
         <v>8</v>
@@ -1219,7 +1228,7 @@
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B29" s="0" t="n">
         <v>1</v>
@@ -1228,7 +1237,7 @@
         <v>4</v>
       </c>
       <c r="E29" s="0" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G29" s="0" t="s">
         <v>8</v>
@@ -1236,16 +1245,16 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="0" t="s">
         <v>48</v>
-      </c>
-      <c r="B30" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C30" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="0" t="s">
-        <v>49</v>
       </c>
       <c r="E30" s="0" t="n">
         <v>1</v>
@@ -1259,7 +1268,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B31" s="0" t="n">
         <v>1</v>
@@ -1279,7 +1288,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B32" s="0" t="n">
         <v>1</v>
@@ -1291,7 +1300,7 @@
         <v>17</v>
       </c>
       <c r="F32" s="0" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G32" s="0" t="s">
         <v>8</v>
@@ -1299,7 +1308,7 @@
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B33" s="0" t="n">
         <v>1</v>
@@ -1311,7 +1320,7 @@
         <v>0</v>
       </c>
       <c r="F33" s="0" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G33" s="0" t="s">
         <v>8</v>
@@ -1319,7 +1328,7 @@
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B34" s="0" t="n">
         <v>1</v>
@@ -1331,7 +1340,7 @@
         <v>0</v>
       </c>
       <c r="F34" s="0" t="s">
-        <v>55</v>
+        <v>22</v>
       </c>
       <c r="G34" s="0" t="s">
         <v>8</v>
@@ -1339,7 +1348,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B35" s="0" t="n">
         <v>1</v>
@@ -1348,10 +1357,10 @@
         <v>2</v>
       </c>
       <c r="D35" s="0" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F35" s="0" t="s">
         <v>14</v>
@@ -1362,7 +1371,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B36" s="0" t="n">
         <v>2</v>
@@ -1371,7 +1380,7 @@
         <v>2</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F36" s="0" t="s">
         <v>14</v>
@@ -1382,7 +1391,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B37" s="0" t="n">
         <v>1</v>
@@ -1391,7 +1400,7 @@
         <v>1</v>
       </c>
       <c r="D37" s="0" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E37" s="0" t="n">
         <v>1</v>
@@ -1405,7 +1414,7 @@
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B38" s="0" t="n">
         <v>1</v>
@@ -1422,7 +1431,7 @@
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B39" s="0" t="n">
         <v>1</v>
@@ -1431,7 +1440,7 @@
         <v>2</v>
       </c>
       <c r="E39" s="0" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F39" s="0" t="s">
         <v>14</v>
@@ -1442,7 +1451,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B40" s="0" t="n">
         <v>1</v>
@@ -1462,7 +1471,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B41" s="0" t="n">
         <v>1</v>
@@ -1482,7 +1491,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B42" s="0" t="n">
         <v>2</v>
@@ -1491,13 +1500,13 @@
         <v>1</v>
       </c>
       <c r="D42" s="0" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E42" s="0" t="n">
         <v>1</v>
       </c>
       <c r="F42" s="0" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G42" s="0" t="s">
         <v>8</v>
@@ -1505,7 +1514,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B43" s="0" t="n">
         <v>1</v>
@@ -1517,7 +1526,7 @@
         <v>1</v>
       </c>
       <c r="F43" s="0" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G43" s="0" t="s">
         <v>8</v>
@@ -1525,7 +1534,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B44" s="0" t="n">
         <v>1</v>
@@ -1548,22 +1557,22 @@
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="E45" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F45" s="0" t="s">
         <v>70</v>
-      </c>
-      <c r="B45" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C45" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D45" s="0" t="s">
-        <v>71</v>
-      </c>
-      <c r="E45" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="F45" s="0" t="s">
-        <v>72</v>
       </c>
       <c r="G45" s="0" t="s">
         <v>8</v>
@@ -1571,7 +1580,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B46" s="0" t="n">
         <v>1</v>
@@ -1580,7 +1589,7 @@
         <v>1</v>
       </c>
       <c r="D46" s="0" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E46" s="0" t="n">
         <v>1</v>
@@ -1594,7 +1603,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B47" s="0" t="n">
         <v>1</v>
@@ -1614,7 +1623,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B48" s="0" t="n">
         <v>1</v>
@@ -1634,7 +1643,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B49" s="0" t="n">
         <v>1</v>
@@ -1643,10 +1652,10 @@
         <v>5</v>
       </c>
       <c r="E49" s="0" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F49" s="0" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G49" s="0" t="s">
         <v>8</v>
@@ -1654,7 +1663,7 @@
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B50" s="0" t="n">
         <v>1</v>
@@ -1666,7 +1675,7 @@
         <v>13</v>
       </c>
       <c r="F50" s="0" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G50" s="0" t="s">
         <v>8</v>
@@ -1674,7 +1683,7 @@
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B51" s="0" t="n">
         <v>1</v>
@@ -1691,7 +1700,7 @@
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B52" s="0" t="n">
         <v>1</v>
@@ -1711,7 +1720,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B53" s="0" t="n">
         <v>1</v>
@@ -1723,7 +1732,7 @@
         <v>1</v>
       </c>
       <c r="F53" s="0" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G53" s="0" t="s">
         <v>8</v>
@@ -1731,7 +1740,7 @@
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B54" s="0" t="n">
         <v>1</v>
@@ -1751,7 +1760,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B55" s="0" t="n">
         <v>1</v>
@@ -1763,7 +1772,7 @@
         <v>1</v>
       </c>
       <c r="F55" s="0" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G55" s="0" t="s">
         <v>8</v>
@@ -1771,7 +1780,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="0" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B56" s="0" t="n">
         <v>1</v>
@@ -1780,7 +1789,7 @@
         <v>4</v>
       </c>
       <c r="D56" s="0" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E56" s="0" t="n">
         <v>1</v>
@@ -1794,7 +1803,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="0" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B57" s="0" t="n">
         <v>1</v>
@@ -1803,13 +1812,13 @@
         <v>0</v>
       </c>
       <c r="D57" s="0" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E57" s="0" t="n">
         <v>0</v>
       </c>
       <c r="F57" s="0" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G57" s="0" t="s">
         <v>8</v>
@@ -1817,7 +1826,7 @@
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B58" s="0" t="n">
         <v>1</v>
@@ -1826,7 +1835,7 @@
         <v>1</v>
       </c>
       <c r="D58" s="0" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E58" s="0" t="n">
         <v>1</v>
@@ -1834,7 +1843,7 @@
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B59" s="0" t="n">
         <v>1</v>
@@ -1854,22 +1863,22 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B60" s="0" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C60" s="0" t="n">
         <v>1</v>
       </c>
       <c r="D60" s="0" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E60" s="0" t="n">
         <v>0</v>
       </c>
       <c r="F60" s="0" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G60" s="0" t="s">
         <v>8</v>
@@ -1877,7 +1886,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B61" s="0" t="n">
         <v>2</v>
@@ -1886,13 +1895,13 @@
         <v>1</v>
       </c>
       <c r="D61" s="0" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="E61" s="0" t="n">
         <v>2</v>
       </c>
       <c r="F61" s="0" t="s">
-        <v>95</v>
+        <v>14</v>
       </c>
       <c r="G61" s="0" t="s">
         <v>8</v>
@@ -1900,7 +1909,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="0" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B62" s="0" t="n">
         <v>1</v>
@@ -1909,15 +1918,38 @@
         <v>1</v>
       </c>
       <c r="D62" s="0" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="E62" s="0" t="n">
         <v>1</v>
       </c>
       <c r="F62" s="0" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G62" s="0" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="B63" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C63" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D63" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E63" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="F63" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G63" s="0" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1989,22 +2021,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F2" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G2" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="H2" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="I2" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H2" s="0" t="s">
+      <c r="J2" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="I2" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J2" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2025,22 +2057,22 @@
         <v>1</v>
       </c>
       <c r="E3" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F3" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G3" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="H3" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="I3" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H3" s="0" t="s">
+      <c r="J3" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="I3" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J3" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2061,25 +2093,25 @@
         <v>0,1</v>
       </c>
       <c r="E4" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="F4" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="G4" s="0" t="s">
         <v>104</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="H4" s="0" t="s">
         <v>105</v>
       </c>
-      <c r="G4" s="0" t="s">
+      <c r="I4" s="0" t="s">
         <v>106</v>
       </c>
-      <c r="H4" s="0" t="s">
+      <c r="J4" s="0" t="s">
         <v>107</v>
       </c>
-      <c r="I4" s="0" t="s">
+      <c r="K4" s="0" t="s">
         <v>108</v>
-      </c>
-      <c r="J4" s="0" t="s">
-        <v>109</v>
-      </c>
-      <c r="K4" s="0" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2100,22 +2132,22 @@
         <v>0</v>
       </c>
       <c r="E5" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F5" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G5" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="H5" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G5" s="0" t="s">
+      <c r="I5" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H5" s="0" t="s">
+      <c r="J5" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="I5" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J5" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2136,22 +2168,22 @@
         <v>0,1,2</v>
       </c>
       <c r="E6" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="F6" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="G6" s="0" t="s">
         <v>111</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="H6" s="0" t="s">
         <v>112</v>
       </c>
-      <c r="G6" s="0" t="s">
+      <c r="I6" s="0" t="s">
         <v>113</v>
       </c>
-      <c r="H6" s="0" t="s">
+      <c r="J6" s="0" t="s">
         <v>114</v>
-      </c>
-      <c r="I6" s="0" t="s">
-        <v>115</v>
-      </c>
-      <c r="J6" s="0" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2172,22 +2204,22 @@
         <v>1</v>
       </c>
       <c r="E7" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F7" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G7" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F7" s="0" t="s">
+      <c r="H7" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G7" s="0" t="s">
+      <c r="I7" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H7" s="0" t="s">
+      <c r="J7" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="I7" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J7" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2208,22 +2240,22 @@
         <v>0</v>
       </c>
       <c r="E8" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F8" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G8" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F8" s="0" t="s">
+      <c r="H8" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G8" s="0" t="s">
+      <c r="I8" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H8" s="0" t="s">
+      <c r="J8" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="I8" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J8" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2244,40 +2276,40 @@
         <v>0,1</v>
       </c>
       <c r="E9" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="F9" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="G9" s="0" t="s">
         <v>117</v>
       </c>
-      <c r="F9" s="0" t="s">
+      <c r="H9" s="0" t="s">
         <v>118</v>
       </c>
-      <c r="G9" s="0" t="s">
+      <c r="I9" s="0" t="s">
         <v>119</v>
       </c>
-      <c r="H9" s="0" t="s">
+      <c r="J9" s="0" t="s">
         <v>120</v>
       </c>
-      <c r="I9" s="0" t="s">
+      <c r="K9" s="0" t="s">
         <v>121</v>
       </c>
-      <c r="J9" s="0" t="s">
+      <c r="L9" s="0" t="s">
         <v>122</v>
       </c>
-      <c r="K9" s="0" t="s">
+      <c r="M9" s="0" t="s">
         <v>123</v>
       </c>
-      <c r="L9" s="0" t="s">
+      <c r="N9" s="0" t="s">
         <v>124</v>
       </c>
-      <c r="M9" s="0" t="s">
+      <c r="O9" s="0" t="s">
         <v>125</v>
       </c>
-      <c r="N9" s="0" t="s">
+      <c r="P9" s="0" t="s">
         <v>126</v>
-      </c>
-      <c r="O9" s="0" t="s">
-        <v>127</v>
-      </c>
-      <c r="P9" s="0" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2298,16 +2330,16 @@
         <v>0,1,2</v>
       </c>
       <c r="E10" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="F10" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="G10" s="0" t="s">
         <v>111</v>
       </c>
-      <c r="F10" s="0" t="s">
-        <v>112</v>
-      </c>
-      <c r="G10" s="0" t="s">
+      <c r="H10" s="0" t="s">
         <v>113</v>
-      </c>
-      <c r="H10" s="0" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2328,22 +2360,22 @@
         <v>0</v>
       </c>
       <c r="E11" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F11" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G11" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F11" s="0" t="s">
+      <c r="H11" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G11" s="0" t="s">
+      <c r="I11" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H11" s="0" t="s">
+      <c r="J11" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="I11" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J11" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2364,22 +2396,22 @@
         <v>0</v>
       </c>
       <c r="E12" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F12" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G12" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F12" s="0" t="s">
+      <c r="H12" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G12" s="0" t="s">
+      <c r="I12" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H12" s="0" t="s">
+      <c r="J12" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="I12" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J12" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2400,22 +2432,22 @@
         <v>1</v>
       </c>
       <c r="E13" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F13" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G13" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F13" s="0" t="s">
+      <c r="H13" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G13" s="0" t="s">
+      <c r="I13" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H13" s="0" t="s">
+      <c r="J13" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="I13" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J13" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2436,28 +2468,28 @@
         <v>0,1</v>
       </c>
       <c r="E14" s="0" t="s">
+        <v>127</v>
+      </c>
+      <c r="F14" s="0" t="s">
+        <v>128</v>
+      </c>
+      <c r="G14" s="0" t="s">
         <v>129</v>
       </c>
-      <c r="F14" s="0" t="s">
+      <c r="H14" s="0" t="s">
         <v>130</v>
       </c>
-      <c r="G14" s="0" t="s">
+      <c r="I14" s="0" t="s">
         <v>131</v>
       </c>
-      <c r="H14" s="0" t="s">
+      <c r="J14" s="0" t="s">
         <v>132</v>
       </c>
-      <c r="I14" s="0" t="s">
+      <c r="K14" s="0" t="s">
         <v>133</v>
       </c>
-      <c r="J14" s="0" t="s">
+      <c r="L14" s="0" t="s">
         <v>134</v>
-      </c>
-      <c r="K14" s="0" t="s">
-        <v>135</v>
-      </c>
-      <c r="L14" s="0" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2478,19 +2510,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E15" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="F15" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="G15" s="0" t="s">
         <v>111</v>
       </c>
-      <c r="F15" s="0" t="s">
-        <v>112</v>
-      </c>
-      <c r="G15" s="0" t="s">
-        <v>113</v>
-      </c>
       <c r="H15" s="0" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="I15" s="0" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2511,19 +2543,19 @@
         <v>1,2</v>
       </c>
       <c r="E16" s="0" t="s">
+        <v>137</v>
+      </c>
+      <c r="F16" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="G16" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="H16" s="0" t="s">
         <v>139</v>
       </c>
-      <c r="F16" s="0" t="s">
-        <v>140</v>
-      </c>
-      <c r="G16" s="0" t="s">
-        <v>106</v>
-      </c>
-      <c r="H16" s="0" t="s">
-        <v>141</v>
-      </c>
       <c r="I16" s="0" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2544,19 +2576,19 @@
         <v>1,2</v>
       </c>
       <c r="E17" s="0" t="s">
+        <v>137</v>
+      </c>
+      <c r="F17" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="G17" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="H17" s="0" t="s">
         <v>139</v>
       </c>
-      <c r="F17" s="0" t="s">
-        <v>140</v>
-      </c>
-      <c r="G17" s="0" t="s">
-        <v>106</v>
-      </c>
-      <c r="H17" s="0" t="s">
-        <v>141</v>
-      </c>
       <c r="I17" s="0" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2577,19 +2609,19 @@
         <v>1,2</v>
       </c>
       <c r="E18" s="0" t="s">
+        <v>137</v>
+      </c>
+      <c r="F18" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="G18" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="H18" s="0" t="s">
         <v>139</v>
       </c>
-      <c r="F18" s="0" t="s">
-        <v>140</v>
-      </c>
-      <c r="G18" s="0" t="s">
-        <v>106</v>
-      </c>
-      <c r="H18" s="0" t="s">
-        <v>141</v>
-      </c>
       <c r="I18" s="0" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2610,16 +2642,16 @@
         <v>0,1,2</v>
       </c>
       <c r="E19" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="F19" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="G19" s="0" t="s">
         <v>111</v>
       </c>
-      <c r="F19" s="0" t="s">
-        <v>112</v>
-      </c>
-      <c r="G19" s="0" t="s">
-        <v>113</v>
-      </c>
       <c r="H19" s="0" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2640,10 +2672,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="0" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F20" s="0" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2664,10 +2696,10 @@
         <v>1</v>
       </c>
       <c r="E21" s="0" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F21" s="0" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2688,10 +2720,10 @@
         <v>0,1</v>
       </c>
       <c r="E22" s="0" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F22" s="0" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2712,19 +2744,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E23" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="F23" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="G23" s="0" t="s">
         <v>111</v>
       </c>
-      <c r="F23" s="0" t="s">
-        <v>112</v>
-      </c>
-      <c r="G23" s="0" t="s">
-        <v>113</v>
-      </c>
       <c r="H23" s="0" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="I23" s="0" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2745,19 +2777,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E24" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="F24" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="G24" s="0" t="s">
         <v>111</v>
       </c>
-      <c r="F24" s="0" t="s">
-        <v>112</v>
-      </c>
-      <c r="G24" s="0" t="s">
-        <v>113</v>
-      </c>
       <c r="H24" s="0" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="I24" s="0" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2778,19 +2810,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E25" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="F25" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="G25" s="0" t="s">
         <v>111</v>
       </c>
-      <c r="F25" s="0" t="s">
-        <v>112</v>
-      </c>
-      <c r="G25" s="0" t="s">
-        <v>113</v>
-      </c>
       <c r="H25" s="0" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="I25" s="0" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2811,10 +2843,10 @@
         <v>0,1,2</v>
       </c>
       <c r="E26" s="0" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F26" s="0" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2835,22 +2867,22 @@
         <v>1</v>
       </c>
       <c r="E27" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F27" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G27" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F27" s="0" t="s">
+      <c r="H27" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G27" s="0" t="s">
+      <c r="I27" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H27" s="0" t="s">
+      <c r="J27" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="I27" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J27" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2871,19 +2903,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E28" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="F28" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="G28" s="0" t="s">
         <v>111</v>
       </c>
-      <c r="F28" s="0" t="s">
-        <v>112</v>
-      </c>
-      <c r="G28" s="0" t="s">
-        <v>113</v>
-      </c>
       <c r="H28" s="0" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="I28" s="0" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2922,22 +2954,22 @@
         <v>1</v>
       </c>
       <c r="E30" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F30" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G30" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F30" s="0" t="s">
+      <c r="H30" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G30" s="0" t="s">
+      <c r="I30" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H30" s="0" t="s">
+      <c r="J30" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="I30" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J30" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2958,22 +2990,22 @@
         <v>1</v>
       </c>
       <c r="E31" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F31" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G31" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F31" s="0" t="s">
+      <c r="H31" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G31" s="0" t="s">
+      <c r="I31" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H31" s="0" t="s">
+      <c r="J31" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="I31" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J31" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2994,7 +3026,7 @@
         <v>0,1,2</v>
       </c>
       <c r="E32" s="0" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3015,10 +3047,10 @@
         <v>0</v>
       </c>
       <c r="E33" s="0" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F33" s="0" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3039,10 +3071,10 @@
         <v>0</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F34" s="0" t="s">
-        <v>99</v>
+        <v>140</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3063,34 +3095,34 @@
         <v>1,2</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>121</v>
+        <v>141</v>
       </c>
       <c r="F35" s="0" t="s">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="G35" s="0" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H35" s="0" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I35" s="0" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J35" s="0" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="K35" s="0" t="s">
-        <v>119</v>
+        <v>146</v>
       </c>
       <c r="L35" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="M35" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="N35" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3111,34 +3143,34 @@
         <v>2,3</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>121</v>
+        <v>141</v>
       </c>
       <c r="F36" s="0" t="s">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="G36" s="0" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H36" s="0" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I36" s="0" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J36" s="0" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="K36" s="0" t="s">
-        <v>119</v>
+        <v>146</v>
       </c>
       <c r="L36" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="M36" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="N36" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3159,22 +3191,22 @@
         <v>1</v>
       </c>
       <c r="E37" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F37" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G37" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F37" s="0" t="s">
+      <c r="H37" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G37" s="0" t="s">
+      <c r="I37" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H37" s="0" t="s">
+      <c r="J37" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="I37" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J37" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3195,10 +3227,10 @@
         <v>1</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F38" s="0" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3237,22 +3269,22 @@
         <v>1</v>
       </c>
       <c r="E40" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F40" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G40" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F40" s="0" t="s">
+      <c r="H40" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G40" s="0" t="s">
+      <c r="I40" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H40" s="0" t="s">
+      <c r="J40" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="I40" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J40" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3273,22 +3305,22 @@
         <v>1</v>
       </c>
       <c r="E41" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F41" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G41" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F41" s="0" t="s">
+      <c r="H41" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G41" s="0" t="s">
+      <c r="I41" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H41" s="0" t="s">
+      <c r="J41" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="I41" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J41" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3309,10 +3341,10 @@
         <v>1</v>
       </c>
       <c r="E42" s="0" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F42" s="0" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3333,22 +3365,22 @@
         <v>1</v>
       </c>
       <c r="E43" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F43" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G43" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F43" s="0" t="s">
+      <c r="H43" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G43" s="0" t="s">
+      <c r="I43" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H43" s="0" t="s">
+      <c r="J43" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="I43" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J43" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3369,25 +3401,25 @@
         <v>0,1</v>
       </c>
       <c r="E44" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="F44" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="G44" s="0" t="s">
         <v>104</v>
       </c>
-      <c r="F44" s="0" t="s">
+      <c r="H44" s="0" t="s">
         <v>105</v>
       </c>
-      <c r="G44" s="0" t="s">
+      <c r="I44" s="0" t="s">
         <v>106</v>
       </c>
-      <c r="H44" s="0" t="s">
+      <c r="J44" s="0" t="s">
         <v>107</v>
       </c>
-      <c r="I44" s="0" t="s">
+      <c r="K44" s="0" t="s">
         <v>108</v>
-      </c>
-      <c r="J44" s="0" t="s">
-        <v>109</v>
-      </c>
-      <c r="K44" s="0" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3408,22 +3440,22 @@
         <v>1</v>
       </c>
       <c r="E45" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F45" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G45" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F45" s="0" t="s">
+      <c r="H45" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G45" s="0" t="s">
+      <c r="I45" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H45" s="0" t="s">
+      <c r="J45" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="I45" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J45" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3444,10 +3476,10 @@
         <v>1</v>
       </c>
       <c r="E46" s="0" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F46" s="0" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3468,16 +3500,16 @@
         <v>0</v>
       </c>
       <c r="E47" s="0" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F47" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="G47" s="0" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="H47" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3498,16 +3530,16 @@
         <v>1</v>
       </c>
       <c r="E48" s="0" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F48" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="G48" s="0" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="H48" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3546,10 +3578,10 @@
         <v>0,1</v>
       </c>
       <c r="E50" s="0" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F50" s="0" t="s">
-        <v>134</v>
+        <v>152</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3570,22 +3602,22 @@
         <v>1</v>
       </c>
       <c r="E51" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F51" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G51" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F51" s="0" t="s">
+      <c r="H51" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G51" s="0" t="s">
+      <c r="I51" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H51" s="0" t="s">
+      <c r="J51" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="I51" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J51" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3606,10 +3638,10 @@
         <v>1</v>
       </c>
       <c r="E52" s="0" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F52" s="0" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3630,22 +3662,22 @@
         <v>1</v>
       </c>
       <c r="E53" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F53" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G53" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F53" s="0" t="s">
+      <c r="H53" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G53" s="0" t="s">
+      <c r="I53" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H53" s="0" t="s">
+      <c r="J53" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="I53" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J53" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3666,22 +3698,22 @@
         <v>1</v>
       </c>
       <c r="E54" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F54" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G54" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F54" s="0" t="s">
+      <c r="H54" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G54" s="0" t="s">
+      <c r="I54" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H54" s="0" t="s">
+      <c r="J54" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="I54" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J54" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3702,22 +3734,22 @@
         <v>1</v>
       </c>
       <c r="E55" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F55" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G55" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F55" s="0" t="s">
+      <c r="H55" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G55" s="0" t="s">
+      <c r="I55" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H55" s="0" t="s">
+      <c r="J55" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="I55" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J55" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3738,22 +3770,22 @@
         <v>1</v>
       </c>
       <c r="E56" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F56" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G56" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F56" s="0" t="s">
+      <c r="H56" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G56" s="0" t="s">
+      <c r="I56" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H56" s="0" t="s">
+      <c r="J56" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="I56" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J56" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3774,28 +3806,28 @@
         <v>0</v>
       </c>
       <c r="E57" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F57" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G57" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F57" s="0" t="s">
+      <c r="H57" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G57" s="0" t="s">
+      <c r="I57" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H57" s="0" t="s">
+      <c r="J57" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="I57" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J57" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="str">
         <f aca="false">LibManager!A58</f>
-        <v>Syncopy</v>
+        <v>#Syncopy =&gt; commented out (special case)</v>
       </c>
       <c r="B58" s="0" t="n">
         <f aca="false">LibManager!B58</f>
@@ -3810,22 +3842,22 @@
         <v>1</v>
       </c>
       <c r="E58" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F58" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G58" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F58" s="0" t="s">
+      <c r="H58" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G58" s="0" t="s">
+      <c r="I58" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H58" s="0" t="s">
+      <c r="J58" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="I58" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J58" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3846,10 +3878,10 @@
         <v>1</v>
       </c>
       <c r="E59" s="0" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F59" s="0" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3859,7 +3891,7 @@
       </c>
       <c r="B60" s="0" t="n">
         <f aca="false">LibManager!B60</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C60" s="0" t="n">
         <f aca="false">LibManager!C60</f>
@@ -3870,22 +3902,22 @@
         <v>0</v>
       </c>
       <c r="E60" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F60" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G60" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F60" s="0" t="s">
+      <c r="H60" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G60" s="0" t="s">
+      <c r="I60" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H60" s="0" t="s">
+      <c r="J60" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="I60" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J60" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3906,22 +3938,22 @@
         <v>2</v>
       </c>
       <c r="E61" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F61" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G61" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F61" s="0" t="s">
+      <c r="H61" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G61" s="0" t="s">
+      <c r="I61" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H61" s="0" t="s">
+      <c r="J61" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="I61" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J61" s="0" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3942,40 +3974,61 @@
         <v>1</v>
       </c>
       <c r="E62" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F62" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G62" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="F62" s="0" t="s">
+      <c r="H62" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="G62" s="0" t="s">
+      <c r="I62" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="H62" s="0" t="s">
+      <c r="J62" s="0" t="s">
         <v>101</v>
       </c>
-      <c r="I62" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="J62" s="0" t="s">
-        <v>103</v>
-      </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="0" t="n">
+      <c r="A63" s="0" t="str">
         <f aca="false">LibManager!A63</f>
-        <v>0</v>
+        <v>MaxPoolWithArgMax</v>
       </c>
       <c r="B63" s="0" t="n">
         <f aca="false">LibManager!B63</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C63" s="0" t="n">
         <f aca="false">LibManager!C63</f>
-        <v>0</v>
-      </c>
-      <c r="D63" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D63" s="0" t="str">
         <f aca="false">LibManager!E63</f>
-        <v>0</v>
+        <v>0,2</v>
+      </c>
+      <c r="E63" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="F63" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="G63" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="H63" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="I63" s="0" t="s">
+        <v>106</v>
+      </c>
+      <c r="J63" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="K63" s="0" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] adjustments after merge [SW-2982]
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="163">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -272,6 +272,9 @@
     <t xml:space="preserve">SparseLengthsWeightedSum</t>
   </si>
   <si>
+    <t xml:space="preserve">1,3</t>
+  </si>
+  <si>
     <t xml:space="preserve">SparseToDense</t>
   </si>
   <si>
@@ -311,6 +314,15 @@
     <t xml:space="preserve">0,2</t>
   </si>
   <si>
+    <t xml:space="preserve">BatchedReduceMin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CumSum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exclusive, Reverse</t>
+  </si>
+  <si>
     <t xml:space="preserve">FloatTy</t>
   </si>
   <si>
@@ -480,6 +492,24 @@
   </si>
   <si>
     <t xml:space="preserve">#Float16Ty,UInt8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy, Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty, Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int8QTy, Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int64ITy, Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32ITy, Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int16QTy, Int64ITy</t>
   </si>
 </sst>
 </file>
@@ -647,16 +677,16 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11.02"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="27.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="27.58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11.64"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="51.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="7.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="7.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="8" style="0" width="8.67"/>
   </cols>
   <sheetData>
@@ -1748,8 +1778,8 @@
       <c r="C54" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="E54" s="0" t="n">
-        <v>1</v>
+      <c r="E54" s="0" t="s">
+        <v>83</v>
       </c>
       <c r="F54" s="0" t="s">
         <v>14</v>
@@ -1760,7 +1790,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B55" s="0" t="n">
         <v>1</v>
@@ -1780,7 +1810,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B56" s="0" t="n">
         <v>1</v>
@@ -1789,7 +1819,7 @@
         <v>4</v>
       </c>
       <c r="D56" s="0" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E56" s="0" t="n">
         <v>1</v>
@@ -1803,7 +1833,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B57" s="0" t="n">
         <v>1</v>
@@ -1826,7 +1856,7 @@
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B58" s="0" t="n">
         <v>1</v>
@@ -1835,7 +1865,7 @@
         <v>1</v>
       </c>
       <c r="D58" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E58" s="0" t="n">
         <v>1</v>
@@ -1843,7 +1873,7 @@
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B59" s="0" t="n">
         <v>1</v>
@@ -1863,7 +1893,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B60" s="0" t="n">
         <v>1</v>
@@ -1886,7 +1916,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B61" s="0" t="n">
         <v>2</v>
@@ -1895,7 +1925,7 @@
         <v>1</v>
       </c>
       <c r="D61" s="0" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E61" s="0" t="n">
         <v>2</v>
@@ -1909,7 +1939,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B62" s="0" t="n">
         <v>1</v>
@@ -1918,7 +1948,7 @@
         <v>1</v>
       </c>
       <c r="D62" s="0" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E62" s="0" t="n">
         <v>1</v>
@@ -1932,7 +1962,7 @@
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="0" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B63" s="0" t="n">
         <v>2</v>
@@ -1944,13 +1974,53 @@
         <v>12</v>
       </c>
       <c r="E63" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F63" s="0" t="s">
         <v>14</v>
       </c>
       <c r="G63" s="0" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="B64" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C64" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="E64" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F64" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="G64" s="0" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="B65" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C65" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="E65" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1973,8 +2043,8 @@
   <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11.03"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11.64"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="19.99"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26.05"/>
@@ -1986,7 +2056,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="16.07"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="16.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="14.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="15.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="15.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="17" style="0" width="8.67"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2021,22 +2092,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J2" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2057,22 +2128,22 @@
         <v>1</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J3" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2093,25 +2164,25 @@
         <v>0,1</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="J4" s="0" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="K4" s="0" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2132,22 +2203,22 @@
         <v>0</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I5" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J5" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2168,22 +2239,22 @@
         <v>0,1,2</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="I6" s="0" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="J6" s="0" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2204,22 +2275,22 @@
         <v>1</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I7" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J7" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2240,22 +2311,22 @@
         <v>0</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I8" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J8" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2276,40 +2347,40 @@
         <v>0,1</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="I9" s="0" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="J9" s="0" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="K9" s="0" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="L9" s="0" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="M9" s="0" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="N9" s="0" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="O9" s="0" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="P9" s="0" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2330,16 +2401,16 @@
         <v>0,1,2</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2360,22 +2431,22 @@
         <v>0</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F11" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I11" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J11" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2396,22 +2467,22 @@
         <v>0</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I12" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J12" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2432,22 +2503,22 @@
         <v>1</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F13" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I13" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J13" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2468,28 +2539,28 @@
         <v>0,1</v>
       </c>
       <c r="E14" s="0" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="H14" s="0" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="I14" s="0" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="J14" s="0" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="K14" s="0" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="L14" s="0" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2510,19 +2581,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F15" s="0" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="H15" s="0" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="I15" s="0" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2543,19 +2614,19 @@
         <v>1,2</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="F16" s="0" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="H16" s="0" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="I16" s="0" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2576,19 +2647,19 @@
         <v>1,2</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="F17" s="0" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="H17" s="0" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="I17" s="0" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2609,19 +2680,19 @@
         <v>1,2</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="G18" s="0" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="H18" s="0" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="I18" s="0" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2642,16 +2713,16 @@
         <v>0,1,2</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="G19" s="0" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="H19" s="0" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2672,10 +2743,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F20" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2696,10 +2767,10 @@
         <v>1</v>
       </c>
       <c r="E21" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F21" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2720,10 +2791,10 @@
         <v>0,1</v>
       </c>
       <c r="E22" s="0" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="F22" s="0" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2744,19 +2815,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E23" s="0" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F23" s="0" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="G23" s="0" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="H23" s="0" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="I23" s="0" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2777,19 +2848,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E24" s="0" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F24" s="0" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="G24" s="0" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="H24" s="0" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="I24" s="0" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2810,19 +2881,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E25" s="0" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F25" s="0" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="G25" s="0" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="H25" s="0" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="I25" s="0" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2843,10 +2914,10 @@
         <v>0,1,2</v>
       </c>
       <c r="E26" s="0" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F26" s="0" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2867,22 +2938,22 @@
         <v>1</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F27" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G27" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H27" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I27" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J27" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2903,19 +2974,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E28" s="0" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F28" s="0" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="G28" s="0" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="H28" s="0" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="I28" s="0" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2954,22 +3025,22 @@
         <v>1</v>
       </c>
       <c r="E30" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F30" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G30" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H30" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I30" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J30" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2990,22 +3061,22 @@
         <v>1</v>
       </c>
       <c r="E31" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F31" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G31" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H31" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I31" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J31" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3026,7 +3097,7 @@
         <v>0,1,2</v>
       </c>
       <c r="E32" s="0" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3047,10 +3118,10 @@
         <v>0</v>
       </c>
       <c r="E33" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F33" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3071,10 +3142,10 @@
         <v>0</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F34" s="0" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3095,34 +3166,34 @@
         <v>1,2</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="F35" s="0" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="G35" s="0" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="H35" s="0" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="I35" s="0" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="J35" s="0" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="K35" s="0" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="L35" s="0" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="M35" s="0" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="N35" s="0" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3143,34 +3214,34 @@
         <v>2,3</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="F36" s="0" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="G36" s="0" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="H36" s="0" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="I36" s="0" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="J36" s="0" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="K36" s="0" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="L36" s="0" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="M36" s="0" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="N36" s="0" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3191,22 +3262,22 @@
         <v>1</v>
       </c>
       <c r="E37" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F37" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G37" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H37" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I37" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J37" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3227,10 +3298,10 @@
         <v>1</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="F38" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3269,22 +3340,22 @@
         <v>1</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F40" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G40" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H40" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I40" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J40" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3305,22 +3376,22 @@
         <v>1</v>
       </c>
       <c r="E41" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F41" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G41" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H41" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I41" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J41" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3341,10 +3412,10 @@
         <v>1</v>
       </c>
       <c r="E42" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F42" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3365,22 +3436,22 @@
         <v>1</v>
       </c>
       <c r="E43" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F43" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G43" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H43" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I43" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J43" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3401,25 +3472,25 @@
         <v>0,1</v>
       </c>
       <c r="E44" s="0" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="F44" s="0" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="G44" s="0" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="H44" s="0" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="I44" s="0" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="J44" s="0" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="K44" s="0" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3440,22 +3511,22 @@
         <v>1</v>
       </c>
       <c r="E45" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F45" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G45" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H45" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I45" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J45" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3476,10 +3547,10 @@
         <v>1</v>
       </c>
       <c r="E46" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="F46" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3500,16 +3571,16 @@
         <v>0</v>
       </c>
       <c r="E47" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="F47" s="0" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="G47" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="H47" s="0" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3530,16 +3601,16 @@
         <v>1</v>
       </c>
       <c r="E48" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="F48" s="0" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="G48" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="H48" s="0" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3578,10 +3649,10 @@
         <v>0,1</v>
       </c>
       <c r="E50" s="0" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="F50" s="0" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3602,22 +3673,22 @@
         <v>1</v>
       </c>
       <c r="E51" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F51" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G51" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H51" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I51" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J51" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3638,10 +3709,10 @@
         <v>1</v>
       </c>
       <c r="E52" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F52" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3662,22 +3733,22 @@
         <v>1</v>
       </c>
       <c r="E53" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F53" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G53" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H53" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I53" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J53" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3693,27 +3764,27 @@
         <f aca="false">LibManager!C54</f>
         <v>4</v>
       </c>
-      <c r="D54" s="0" t="n">
+      <c r="D54" s="0" t="str">
         <f aca="false">LibManager!E54</f>
-        <v>1</v>
+        <v>1,3</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>96</v>
+        <v>157</v>
       </c>
       <c r="F54" s="0" t="s">
-        <v>97</v>
+        <v>158</v>
       </c>
       <c r="G54" s="0" t="s">
-        <v>98</v>
+        <v>159</v>
       </c>
       <c r="H54" s="0" t="s">
-        <v>99</v>
+        <v>160</v>
       </c>
       <c r="I54" s="0" t="s">
-        <v>100</v>
+        <v>161</v>
       </c>
       <c r="J54" s="0" t="s">
-        <v>101</v>
+        <v>162</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3734,22 +3805,22 @@
         <v>1</v>
       </c>
       <c r="E55" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F55" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G55" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H55" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I55" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J55" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3770,22 +3841,22 @@
         <v>1</v>
       </c>
       <c r="E56" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F56" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G56" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H56" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I56" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J56" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3806,22 +3877,22 @@
         <v>0</v>
       </c>
       <c r="E57" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F57" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G57" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H57" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I57" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J57" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3842,22 +3913,22 @@
         <v>1</v>
       </c>
       <c r="E58" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F58" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G58" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H58" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I58" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J58" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3878,10 +3949,10 @@
         <v>1</v>
       </c>
       <c r="E59" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F59" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3902,22 +3973,22 @@
         <v>0</v>
       </c>
       <c r="E60" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F60" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G60" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H60" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I60" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J60" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3938,22 +4009,22 @@
         <v>2</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F61" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G61" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H61" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I61" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J61" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3974,22 +4045,22 @@
         <v>1</v>
       </c>
       <c r="E62" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F62" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G62" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H62" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I62" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J62" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4010,61 +4081,91 @@
         <v>0,2</v>
       </c>
       <c r="E63" s="0" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="F63" s="0" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="G63" s="0" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="H63" s="0" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="I63" s="0" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="J63" s="0" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="K63" s="0" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="0" t="n">
+      <c r="A64" s="0" t="str">
         <f aca="false">LibManager!A64</f>
-        <v>0</v>
+        <v>BatchedReduceMin</v>
       </c>
       <c r="B64" s="0" t="n">
         <f aca="false">LibManager!B64</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C64" s="0" t="n">
         <f aca="false">LibManager!C64</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D64" s="0" t="n">
         <f aca="false">LibManager!E64</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="E64" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="F64" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="G64" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="H64" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="I64" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="J64" s="0" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="0" t="n">
+      <c r="A65" s="0" t="str">
         <f aca="false">LibManager!A65</f>
-        <v>0</v>
+        <v>CumSum</v>
       </c>
       <c r="B65" s="0" t="n">
         <f aca="false">LibManager!B65</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C65" s="0" t="n">
         <f aca="false">LibManager!C65</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D65" s="0" t="n">
         <f aca="false">LibManager!E65</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="E65" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="F65" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="G65" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="H65" s="0" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] [SW-3320] missing axis param to insertTensor after merge
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
@@ -200,7 +200,7 @@
     <t xml:space="preserve">InsertTensor</t>
   </si>
   <si>
-    <t xml:space="preserve">Offsets, Count</t>
+    <t xml:space="preserve">Offsets, Count,Axis</t>
   </si>
   <si>
     <t xml:space="preserve">Int8Converter</t>

</xml_diff>

<commit_message>
[dnn-library] [SW-3325] misc Fixes for elementwise - fixing typo in elementwise instructions: div/mul and min/max where swapped - log wasn't working in the first place (swapped in and out tensor when generating the handles) - Select: using incorrect elemKind (from cond instead of out) and fixed error creating tensorBundle with BoolTy depending on dimensions and padding
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -1227,7 +1227,7 @@
         <v>3</v>
       </c>
       <c r="E27" s="0" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F27" s="0" t="s">
         <v>14</v>
@@ -2935,7 +2935,7 @@
       </c>
       <c r="D27" s="0" t="n">
         <f aca="false">LibManager!E27</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E27" s="0" t="s">
         <v>100</v>

</xml_diff>

<commit_message>
[dnn-library] making new operators BatchedReduceMin and CumSum compile
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="163">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -677,7 +677,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:G66"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.99"/>
@@ -1999,9 +1999,6 @@
       <c r="E64" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="F64" s="0" t="s">
-        <v>14</v>
-      </c>
       <c r="G64" s="0" t="s">
         <v>8</v>
       </c>
@@ -2023,6 +2020,7 @@
         <v>1</v>
       </c>
     </row>
+    <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
@@ -2039,7 +2037,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P70"/>
+  <dimension ref="A1:P71"/>
   <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.99"/>
@@ -4258,6 +4256,18 @@
         <v>0</v>
       </c>
     </row>
+    <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="75" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="76" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="77" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="80" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
[dnn-library] Add SpaceToDepth and ResizeNearest operands. Fix BatchedReduceMinInst.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="168">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -317,10 +317,25 @@
     <t xml:space="preserve">BatchedReduceMin</t>
   </si>
   <si>
+    <t xml:space="preserve">Axes</t>
+  </si>
+  <si>
     <t xml:space="preserve">CumSum</t>
   </si>
   <si>
     <t xml:space="preserve">Exclusive, Reverse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SpaceToDepth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BlockSize</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ResizeNearest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RszScale</t>
   </si>
   <si>
     <t xml:space="preserve">FloatTy</t>
@@ -677,12 +692,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G66"/>
+  <dimension ref="A1:G1048576"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11.04"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="27.58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11.64"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="51.19"/>
@@ -1994,7 +2009,7 @@
         <v>1</v>
       </c>
       <c r="D64" s="0" t="s">
-        <v>19</v>
+        <v>98</v>
       </c>
       <c r="E64" s="0" t="n">
         <v>1</v>
@@ -2005,7 +2020,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="0" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B65" s="0" t="n">
         <v>1</v>
@@ -2014,13 +2029,53 @@
         <v>1</v>
       </c>
       <c r="D65" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E65" s="0" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="B66" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C66" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="E66" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" s="0" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="B67" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C67" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="E67" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" s="0" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
@@ -2041,8 +2096,8 @@
   <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11.04"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11.64"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="19.99"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26.05"/>
@@ -2054,7 +2109,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="16.07"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="16.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="14.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="15.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="15.08"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="17" style="0" width="8.67"/>
   </cols>
   <sheetData>
@@ -2090,22 +2145,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J2" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2126,22 +2181,22 @@
         <v>1</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J3" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2162,25 +2217,25 @@
         <v>0,1</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="J4" s="0" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="K4" s="0" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2201,22 +2256,22 @@
         <v>0</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I5" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J5" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2237,22 +2292,22 @@
         <v>0,1,2</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="I6" s="0" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="J6" s="0" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2273,22 +2328,22 @@
         <v>1</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I7" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J7" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2309,22 +2364,22 @@
         <v>0</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I8" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J8" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2345,40 +2400,40 @@
         <v>0,1</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="I9" s="0" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="J9" s="0" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="K9" s="0" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="L9" s="0" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="M9" s="0" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="N9" s="0" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="O9" s="0" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="P9" s="0" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2399,16 +2454,16 @@
         <v>0,1,2</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2429,22 +2484,22 @@
         <v>0</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F11" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I11" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J11" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2465,22 +2520,22 @@
         <v>0</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I12" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J12" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2501,22 +2556,22 @@
         <v>1</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F13" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I13" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J13" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2537,28 +2592,28 @@
         <v>0,1</v>
       </c>
       <c r="E14" s="0" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="H14" s="0" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="I14" s="0" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="J14" s="0" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="K14" s="0" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="L14" s="0" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2579,19 +2634,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="F15" s="0" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="H15" s="0" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="I15" s="0" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2612,19 +2667,19 @@
         <v>1,2</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F16" s="0" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="H16" s="0" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="I16" s="0" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2645,19 +2700,19 @@
         <v>1,2</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F17" s="0" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="H17" s="0" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="I17" s="0" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2678,19 +2733,19 @@
         <v>1,2</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="G18" s="0" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="H18" s="0" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="I18" s="0" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2711,16 +2766,16 @@
         <v>0,1,2</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G19" s="0" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="H19" s="0" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2741,10 +2796,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F20" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2765,10 +2820,10 @@
         <v>1</v>
       </c>
       <c r="E21" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F21" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2789,10 +2844,10 @@
         <v>0,1</v>
       </c>
       <c r="E22" s="0" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F22" s="0" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2813,19 +2868,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E23" s="0" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="F23" s="0" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G23" s="0" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="H23" s="0" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="I23" s="0" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2846,19 +2901,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E24" s="0" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="F24" s="0" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G24" s="0" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="H24" s="0" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="I24" s="0" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2879,19 +2934,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E25" s="0" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="F25" s="0" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G25" s="0" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="H25" s="0" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="I25" s="0" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2912,10 +2967,10 @@
         <v>0,1,2</v>
       </c>
       <c r="E26" s="0" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="F26" s="0" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2936,22 +2991,22 @@
         <v>0</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F27" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G27" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H27" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I27" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J27" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2972,19 +3027,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E28" s="0" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="F28" s="0" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G28" s="0" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="H28" s="0" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="I28" s="0" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3023,22 +3078,22 @@
         <v>1</v>
       </c>
       <c r="E30" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F30" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G30" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H30" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I30" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J30" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3059,22 +3114,22 @@
         <v>1</v>
       </c>
       <c r="E31" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F31" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G31" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H31" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I31" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J31" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3095,7 +3150,7 @@
         <v>0,1,2</v>
       </c>
       <c r="E32" s="0" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3116,10 +3171,10 @@
         <v>0</v>
       </c>
       <c r="E33" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F33" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3140,10 +3195,10 @@
         <v>0</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F34" s="0" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3164,34 +3219,34 @@
         <v>1,2</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="F35" s="0" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="G35" s="0" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="H35" s="0" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="I35" s="0" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="J35" s="0" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="K35" s="0" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="L35" s="0" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="M35" s="0" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="N35" s="0" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3212,34 +3267,34 @@
         <v>2,3</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="F36" s="0" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="G36" s="0" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="H36" s="0" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="I36" s="0" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="J36" s="0" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="K36" s="0" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="L36" s="0" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="M36" s="0" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="N36" s="0" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3260,22 +3315,22 @@
         <v>1</v>
       </c>
       <c r="E37" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F37" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G37" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H37" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I37" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J37" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3296,10 +3351,10 @@
         <v>1</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="F38" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3338,22 +3393,22 @@
         <v>1</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F40" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G40" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H40" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I40" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J40" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3374,22 +3429,22 @@
         <v>1</v>
       </c>
       <c r="E41" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F41" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G41" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H41" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I41" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J41" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3410,10 +3465,10 @@
         <v>1</v>
       </c>
       <c r="E42" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F42" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3434,22 +3489,22 @@
         <v>1</v>
       </c>
       <c r="E43" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F43" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G43" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H43" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I43" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J43" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3470,25 +3525,25 @@
         <v>0,1</v>
       </c>
       <c r="E44" s="0" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="F44" s="0" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="G44" s="0" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="H44" s="0" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="I44" s="0" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="J44" s="0" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="K44" s="0" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3509,22 +3564,22 @@
         <v>1</v>
       </c>
       <c r="E45" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F45" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G45" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H45" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I45" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J45" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3545,10 +3600,10 @@
         <v>1</v>
       </c>
       <c r="E46" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="F46" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3569,16 +3624,16 @@
         <v>0</v>
       </c>
       <c r="E47" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="F47" s="0" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="G47" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="H47" s="0" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3599,16 +3654,16 @@
         <v>1</v>
       </c>
       <c r="E48" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="F48" s="0" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="G48" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="H48" s="0" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3647,10 +3702,10 @@
         <v>0,1</v>
       </c>
       <c r="E50" s="0" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="F50" s="0" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3671,22 +3726,22 @@
         <v>1</v>
       </c>
       <c r="E51" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F51" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G51" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H51" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I51" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J51" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3707,10 +3762,10 @@
         <v>1</v>
       </c>
       <c r="E52" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F52" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3731,22 +3786,22 @@
         <v>1</v>
       </c>
       <c r="E53" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F53" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G53" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H53" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I53" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J53" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3767,22 +3822,22 @@
         <v>1,3</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="F54" s="0" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="G54" s="0" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="H54" s="0" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="I54" s="0" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="J54" s="0" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3803,22 +3858,22 @@
         <v>1</v>
       </c>
       <c r="E55" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F55" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G55" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H55" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I55" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J55" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3839,22 +3894,22 @@
         <v>1</v>
       </c>
       <c r="E56" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F56" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G56" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H56" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I56" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J56" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3875,22 +3930,22 @@
         <v>0</v>
       </c>
       <c r="E57" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F57" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G57" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H57" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I57" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J57" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3911,22 +3966,22 @@
         <v>1</v>
       </c>
       <c r="E58" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F58" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G58" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H58" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I58" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J58" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3947,10 +4002,10 @@
         <v>1</v>
       </c>
       <c r="E59" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F59" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3971,22 +4026,22 @@
         <v>0</v>
       </c>
       <c r="E60" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F60" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G60" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H60" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I60" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J60" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4007,22 +4062,22 @@
         <v>2</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F61" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G61" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H61" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I61" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J61" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4043,22 +4098,22 @@
         <v>1</v>
       </c>
       <c r="E62" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F62" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G62" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H62" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I62" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J62" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4079,25 +4134,25 @@
         <v>0,2</v>
       </c>
       <c r="E63" s="0" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="F63" s="0" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="G63" s="0" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="H63" s="0" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="I63" s="0" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="J63" s="0" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="K63" s="0" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4118,22 +4173,22 @@
         <v>1</v>
       </c>
       <c r="E64" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F64" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G64" s="0" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H64" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I64" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J64" s="0" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4154,52 +4209,85 @@
         <v>1</v>
       </c>
       <c r="E65" s="0" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F65" s="0" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G65" s="0" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="H65" s="0" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="0" t="n">
+      <c r="A66" s="0" t="str">
         <f aca="false">LibManager!A66</f>
-        <v>0</v>
+        <v>SpaceToDepth</v>
       </c>
       <c r="B66" s="0" t="n">
         <f aca="false">LibManager!B66</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C66" s="0" t="n">
         <f aca="false">LibManager!C66</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D66" s="0" t="n">
         <f aca="false">LibManager!E66</f>
         <v>0</v>
       </c>
+      <c r="E66" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="F66" s="0" t="s">
+        <v>106</v>
+      </c>
+      <c r="G66" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="H66" s="0" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="0" t="n">
+      <c r="A67" s="0" t="str">
         <f aca="false">LibManager!A67</f>
-        <v>0</v>
+        <v>ResizeNearest</v>
       </c>
       <c r="B67" s="0" t="n">
         <f aca="false">LibManager!B67</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C67" s="0" t="n">
         <f aca="false">LibManager!C67</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D67" s="0" t="n">
         <f aca="false">LibManager!E67</f>
         <v>0</v>
+      </c>
+      <c r="E67" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="F67" s="0" t="s">
+        <v>106</v>
+      </c>
+      <c r="G67" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="H67" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="I67" s="0" t="s">
+        <v>160</v>
+      </c>
+      <c r="J67" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="K67" s="0" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] Fix EmbeddingBagInst. Fix LengthRangeFillInst.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="170">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -161,54 +161,57 @@
     <t xml:space="preserve">EmbeddingBag</t>
   </si>
   <si>
+    <t xml:space="preserve">HasEndOffset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ExtractTensor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Offsets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FullyConnected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FusedRowwiseQuantizedSparseLengthsSum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Threaded,Vectorized</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FusedRowwiseQuantizedSparseLengthsWeightedSum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gather</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BatchDims</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GatherRanges</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsertTensor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Offsets, Count,Axis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int8Converter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IntLookupTable</t>
+  </si>
+  <si>
     <t xml:space="preserve">NONE</t>
   </si>
   <si>
-    <t xml:space="preserve">ExtractTensor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Offsets</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flip</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FullyConnected</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FusedRowwiseQuantizedSparseLengthsSum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Threaded,Vectorized</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FusedRowwiseQuantizedSparseLengthsWeightedSum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gather</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BatchDims</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GatherRanges</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsertTensor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Offsets, Count,Axis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int8Converter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IntLookupTable</t>
-  </si>
-  <si>
     <t xml:space="preserve">LengthsSum</t>
   </si>
   <si>
@@ -336,6 +339,9 @@
   </si>
   <si>
     <t xml:space="preserve">RszScale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LengthsRangeFill</t>
   </si>
   <si>
     <t xml:space="preserve">FloatTy</t>
@@ -1281,8 +1287,11 @@
       <c r="C29" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="E29" s="0" t="s">
+      <c r="D29" s="0" t="s">
         <v>46</v>
+      </c>
+      <c r="E29" s="0" t="n">
+        <v>0</v>
       </c>
       <c r="G29" s="0" t="s">
         <v>8</v>
@@ -1485,7 +1494,7 @@
         <v>2</v>
       </c>
       <c r="E39" s="0" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="F39" s="0" t="s">
         <v>14</v>
@@ -1496,7 +1505,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B40" s="0" t="n">
         <v>1</v>
@@ -1516,7 +1525,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B41" s="0" t="n">
         <v>1</v>
@@ -1536,7 +1545,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B42" s="0" t="n">
         <v>2</v>
@@ -1545,7 +1554,7 @@
         <v>1</v>
       </c>
       <c r="D42" s="0" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E42" s="0" t="n">
         <v>1</v>
@@ -1559,7 +1568,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B43" s="0" t="n">
         <v>1</v>
@@ -1579,7 +1588,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B44" s="0" t="n">
         <v>1</v>
@@ -1602,7 +1611,7 @@
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B45" s="0" t="n">
         <v>1</v>
@@ -1611,13 +1620,13 @@
         <v>1</v>
       </c>
       <c r="D45" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E45" s="0" t="n">
         <v>1</v>
       </c>
       <c r="F45" s="0" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G45" s="0" t="s">
         <v>8</v>
@@ -1625,7 +1634,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B46" s="0" t="n">
         <v>1</v>
@@ -1634,7 +1643,7 @@
         <v>1</v>
       </c>
       <c r="D46" s="0" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E46" s="0" t="n">
         <v>1</v>
@@ -1648,7 +1657,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B47" s="0" t="n">
         <v>1</v>
@@ -1668,7 +1677,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B48" s="0" t="n">
         <v>1</v>
@@ -1688,7 +1697,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B49" s="0" t="n">
         <v>1</v>
@@ -1697,10 +1706,10 @@
         <v>5</v>
       </c>
       <c r="E49" s="0" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="F49" s="0" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G49" s="0" t="s">
         <v>8</v>
@@ -1708,7 +1717,7 @@
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B50" s="0" t="n">
         <v>1</v>
@@ -1728,7 +1737,7 @@
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B51" s="0" t="n">
         <v>1</v>
@@ -1745,7 +1754,7 @@
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B52" s="0" t="n">
         <v>1</v>
@@ -1765,7 +1774,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B53" s="0" t="n">
         <v>1</v>
@@ -1777,7 +1786,7 @@
         <v>1</v>
       </c>
       <c r="F53" s="0" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G53" s="0" t="s">
         <v>8</v>
@@ -1785,7 +1794,7 @@
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B54" s="0" t="n">
         <v>1</v>
@@ -1794,7 +1803,7 @@
         <v>4</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F54" s="0" t="s">
         <v>14</v>
@@ -1805,7 +1814,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B55" s="0" t="n">
         <v>1</v>
@@ -1825,7 +1834,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="0" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B56" s="0" t="n">
         <v>1</v>
@@ -1834,7 +1843,7 @@
         <v>4</v>
       </c>
       <c r="D56" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E56" s="0" t="n">
         <v>1</v>
@@ -1848,7 +1857,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B57" s="0" t="n">
         <v>1</v>
@@ -1857,7 +1866,7 @@
         <v>0</v>
       </c>
       <c r="D57" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E57" s="0" t="n">
         <v>0</v>
@@ -1871,7 +1880,7 @@
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B58" s="0" t="n">
         <v>1</v>
@@ -1880,7 +1889,7 @@
         <v>1</v>
       </c>
       <c r="D58" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E58" s="0" t="n">
         <v>1</v>
@@ -1888,7 +1897,7 @@
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B59" s="0" t="n">
         <v>1</v>
@@ -1908,7 +1917,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B60" s="0" t="n">
         <v>1</v>
@@ -1931,7 +1940,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B61" s="0" t="n">
         <v>2</v>
@@ -1940,7 +1949,7 @@
         <v>1</v>
       </c>
       <c r="D61" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E61" s="0" t="n">
         <v>2</v>
@@ -1954,7 +1963,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="0" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B62" s="0" t="n">
         <v>1</v>
@@ -1963,13 +1972,13 @@
         <v>1</v>
       </c>
       <c r="D62" s="0" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E62" s="0" t="n">
         <v>1</v>
       </c>
       <c r="F62" s="0" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G62" s="0" t="s">
         <v>8</v>
@@ -1977,7 +1986,7 @@
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B63" s="0" t="n">
         <v>2</v>
@@ -1989,7 +1998,7 @@
         <v>12</v>
       </c>
       <c r="E63" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F63" s="0" t="s">
         <v>14</v>
@@ -2000,7 +2009,7 @@
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B64" s="0" t="n">
         <v>1</v>
@@ -2009,7 +2018,7 @@
         <v>1</v>
       </c>
       <c r="D64" s="0" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E64" s="0" t="n">
         <v>1</v>
@@ -2020,7 +2029,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B65" s="0" t="n">
         <v>1</v>
@@ -2029,7 +2038,7 @@
         <v>1</v>
       </c>
       <c r="D65" s="0" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E65" s="0" t="n">
         <v>1</v>
@@ -2037,7 +2046,7 @@
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="0" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B66" s="0" t="n">
         <v>1</v>
@@ -2046,7 +2055,7 @@
         <v>1</v>
       </c>
       <c r="D66" s="0" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E66" s="0" t="n">
         <v>0</v>
@@ -2057,7 +2066,7 @@
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="0" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B67" s="0" t="n">
         <v>1</v>
@@ -2066,12 +2075,29 @@
         <v>1</v>
       </c>
       <c r="D67" s="0" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E67" s="0" t="n">
         <v>0</v>
       </c>
       <c r="G67" s="0" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="0" t="s">
+        <v>106</v>
+      </c>
+      <c r="B68" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C68" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E68" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" s="0" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2145,22 +2171,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J2" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2181,22 +2207,22 @@
         <v>1</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J3" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2217,25 +2243,25 @@
         <v>0,1</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="J4" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K4" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2256,22 +2282,22 @@
         <v>0</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I5" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J5" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2292,22 +2318,22 @@
         <v>0,1,2</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I6" s="0" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="J6" s="0" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2328,22 +2354,22 @@
         <v>1</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I7" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J7" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2364,22 +2390,22 @@
         <v>0</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I8" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J8" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2400,40 +2426,40 @@
         <v>0,1</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="I9" s="0" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="J9" s="0" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="K9" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="L9" s="0" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="M9" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="N9" s="0" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="O9" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="P9" s="0" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2454,16 +2480,16 @@
         <v>0,1,2</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2484,22 +2510,22 @@
         <v>0</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F11" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I11" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J11" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2520,22 +2546,22 @@
         <v>0</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I12" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J12" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2556,22 +2582,22 @@
         <v>1</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F13" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I13" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J13" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2592,28 +2618,28 @@
         <v>0,1</v>
       </c>
       <c r="E14" s="0" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="H14" s="0" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="I14" s="0" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="J14" s="0" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="K14" s="0" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="L14" s="0" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2634,19 +2660,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F15" s="0" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="H15" s="0" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="I15" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2667,19 +2693,19 @@
         <v>1,2</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F16" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H16" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I16" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2700,19 +2726,19 @@
         <v>1,2</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F17" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H17" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I17" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2733,19 +2759,19 @@
         <v>1,2</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G18" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H18" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I18" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2766,16 +2792,16 @@
         <v>0,1,2</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="G19" s="0" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="H19" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2796,10 +2822,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F20" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2820,10 +2846,10 @@
         <v>1</v>
       </c>
       <c r="E21" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F21" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2844,10 +2870,10 @@
         <v>0,1</v>
       </c>
       <c r="E22" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F22" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2868,19 +2894,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E23" s="0" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F23" s="0" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="G23" s="0" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="H23" s="0" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="I23" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2901,19 +2927,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E24" s="0" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F24" s="0" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="G24" s="0" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="H24" s="0" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="I24" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2934,19 +2960,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E25" s="0" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F25" s="0" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="G25" s="0" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="H25" s="0" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="I25" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2967,10 +2993,10 @@
         <v>0,1,2</v>
       </c>
       <c r="E26" s="0" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F26" s="0" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2991,22 +3017,22 @@
         <v>0</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F27" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G27" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H27" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I27" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J27" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3027,19 +3053,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E28" s="0" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F28" s="0" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="G28" s="0" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="H28" s="0" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="I28" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3055,9 +3081,15 @@
         <f aca="false">LibManager!C29</f>
         <v>4</v>
       </c>
-      <c r="D29" s="0" t="str">
+      <c r="D29" s="0" t="n">
         <f aca="false">LibManager!E29</f>
-        <v>NONE</v>
+        <v>0</v>
+      </c>
+      <c r="E29" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="F29" s="0" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3078,22 +3110,22 @@
         <v>1</v>
       </c>
       <c r="E30" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F30" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G30" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H30" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I30" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J30" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3114,22 +3146,22 @@
         <v>1</v>
       </c>
       <c r="E31" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F31" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G31" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H31" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I31" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J31" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3150,7 +3182,7 @@
         <v>0,1,2</v>
       </c>
       <c r="E32" s="0" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3171,10 +3203,10 @@
         <v>0</v>
       </c>
       <c r="E33" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F33" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3195,10 +3227,10 @@
         <v>0</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F34" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3219,34 +3251,34 @@
         <v>1,2</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F35" s="0" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G35" s="0" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H35" s="0" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="I35" s="0" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="J35" s="0" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="K35" s="0" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="L35" s="0" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="M35" s="0" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="N35" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3267,34 +3299,34 @@
         <v>2,3</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F36" s="0" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G36" s="0" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H36" s="0" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="I36" s="0" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="J36" s="0" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="K36" s="0" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="L36" s="0" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="M36" s="0" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="N36" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3315,22 +3347,22 @@
         <v>1</v>
       </c>
       <c r="E37" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F37" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G37" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H37" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I37" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J37" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3351,10 +3383,10 @@
         <v>1</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F38" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3393,22 +3425,22 @@
         <v>1</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F40" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G40" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H40" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I40" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J40" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3429,22 +3461,22 @@
         <v>1</v>
       </c>
       <c r="E41" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F41" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G41" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H41" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I41" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J41" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3465,10 +3497,10 @@
         <v>1</v>
       </c>
       <c r="E42" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F42" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3489,22 +3521,22 @@
         <v>1</v>
       </c>
       <c r="E43" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F43" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G43" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H43" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I43" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J43" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3525,25 +3557,25 @@
         <v>0,1</v>
       </c>
       <c r="E44" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F44" s="0" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G44" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H44" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="I44" s="0" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="J44" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K44" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3564,22 +3596,22 @@
         <v>1</v>
       </c>
       <c r="E45" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F45" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G45" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H45" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I45" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J45" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3600,10 +3632,10 @@
         <v>1</v>
       </c>
       <c r="E46" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F46" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3624,16 +3656,16 @@
         <v>0</v>
       </c>
       <c r="E47" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F47" s="0" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="G47" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="H47" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3654,16 +3686,16 @@
         <v>1</v>
       </c>
       <c r="E48" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F48" s="0" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="G48" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="H48" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3702,10 +3734,10 @@
         <v>0,1</v>
       </c>
       <c r="E50" s="0" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F50" s="0" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3726,22 +3758,22 @@
         <v>1</v>
       </c>
       <c r="E51" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F51" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G51" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H51" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I51" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J51" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3762,10 +3794,10 @@
         <v>1</v>
       </c>
       <c r="E52" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F52" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3786,22 +3818,22 @@
         <v>1</v>
       </c>
       <c r="E53" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F53" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G53" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H53" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I53" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J53" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3822,22 +3854,22 @@
         <v>1,3</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="F54" s="0" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="G54" s="0" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="H54" s="0" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="I54" s="0" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="J54" s="0" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3858,22 +3890,22 @@
         <v>1</v>
       </c>
       <c r="E55" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F55" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G55" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H55" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I55" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J55" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3894,22 +3926,22 @@
         <v>1</v>
       </c>
       <c r="E56" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F56" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G56" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H56" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I56" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J56" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3930,22 +3962,22 @@
         <v>0</v>
       </c>
       <c r="E57" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F57" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G57" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H57" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I57" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J57" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3966,22 +3998,22 @@
         <v>1</v>
       </c>
       <c r="E58" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F58" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G58" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H58" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I58" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J58" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4002,10 +4034,10 @@
         <v>1</v>
       </c>
       <c r="E59" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F59" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4026,22 +4058,22 @@
         <v>0</v>
       </c>
       <c r="E60" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F60" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G60" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H60" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I60" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J60" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4062,22 +4094,22 @@
         <v>2</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F61" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G61" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H61" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I61" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J61" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4098,22 +4130,22 @@
         <v>1</v>
       </c>
       <c r="E62" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F62" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G62" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H62" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I62" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J62" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4134,25 +4166,25 @@
         <v>0,2</v>
       </c>
       <c r="E63" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F63" s="0" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G63" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H63" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="I63" s="0" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="J63" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K63" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4173,22 +4205,22 @@
         <v>1</v>
       </c>
       <c r="E64" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F64" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G64" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H64" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I64" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J64" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4209,16 +4241,16 @@
         <v>1</v>
       </c>
       <c r="E65" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F65" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G65" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H65" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4239,16 +4271,16 @@
         <v>0</v>
       </c>
       <c r="E66" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F66" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G66" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H66" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4269,43 +4301,46 @@
         <v>0</v>
       </c>
       <c r="E67" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F67" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G67" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H67" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="I67" s="0" t="s">
+        <v>162</v>
+      </c>
+      <c r="J67" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="K67" s="0" t="s">
         <v>110</v>
       </c>
-      <c r="I67" s="0" t="s">
-        <v>160</v>
-      </c>
-      <c r="J67" s="0" t="s">
-        <v>109</v>
-      </c>
-      <c r="K67" s="0" t="s">
-        <v>108</v>
-      </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="0" t="n">
+      <c r="A68" s="0" t="str">
         <f aca="false">LibManager!A68</f>
-        <v>0</v>
+        <v>LengthsRangeFill</v>
       </c>
       <c r="B68" s="0" t="n">
         <f aca="false">LibManager!B68</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C68" s="0" t="n">
         <f aca="false">LibManager!C68</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D68" s="0" t="n">
         <f aca="false">LibManager!E68</f>
         <v>0</v>
+      </c>
+      <c r="E68" s="0" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] adjusting excel after merging with Rafa's changes
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="171">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -104,7 +104,7 @@
     <t xml:space="preserve">Copy</t>
   </si>
   <si>
-    <t xml:space="preserve">Threaded, Vectorized, Tensorized</t>
+    <t xml:space="preserve">TensorsAligned</t>
   </si>
   <si>
     <t xml:space="preserve">CrossEntropyLoss</t>
@@ -227,6 +227,9 @@
     <t xml:space="preserve">MatMul</t>
   </si>
   <si>
+    <t xml:space="preserve">Transposed</t>
+  </si>
+  <si>
     <t xml:space="preserve">MaxPool</t>
   </si>
   <si>
@@ -239,6 +242,9 @@
     <t xml:space="preserve">Threaded,Vectorized,Aligned32Bytes</t>
   </si>
   <si>
+    <t xml:space="preserve">custom</t>
+  </si>
+  <si>
     <t xml:space="preserve">Modulo</t>
   </si>
   <si>
@@ -269,9 +275,6 @@
     <t xml:space="preserve">SoftMax</t>
   </si>
   <si>
-    <t xml:space="preserve">Threaded, Vectorized, Threaded1, Vectorized1, 2, Threaded2</t>
-  </si>
-  <si>
     <t xml:space="preserve">SparseLengthsWeightedSum</t>
   </si>
   <si>
@@ -290,7 +293,7 @@
     <t xml:space="preserve">Splat</t>
   </si>
   <si>
-    <t xml:space="preserve">#Syncopy =&gt; commented out (special case)</t>
+    <t xml:space="preserve">Syncopy</t>
   </si>
   <si>
     <t xml:space="preserve">SyncOffset</t>
@@ -950,11 +953,14 @@
       <c r="C12" s="0" t="n">
         <v>1</v>
       </c>
+      <c r="D12" s="0" t="s">
+        <v>27</v>
+      </c>
       <c r="E12" s="0" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G12" s="0" t="s">
         <v>8</v>
@@ -1523,7 +1529,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
         <v>64</v>
       </c>
@@ -1566,7 +1572,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
         <v>67</v>
       </c>
@@ -1576,6 +1582,9 @@
       <c r="C43" s="0" t="n">
         <v>2</v>
       </c>
+      <c r="D43" s="0" t="s">
+        <v>68</v>
+      </c>
       <c r="E43" s="0" t="n">
         <v>1</v>
       </c>
@@ -1588,7 +1597,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B44" s="0" t="n">
         <v>1</v>
@@ -1611,7 +1620,7 @@
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B45" s="0" t="n">
         <v>1</v>
@@ -1620,21 +1629,21 @@
         <v>1</v>
       </c>
       <c r="D45" s="0" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E45" s="0" t="n">
         <v>1</v>
       </c>
       <c r="F45" s="0" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G45" s="0" t="s">
-        <v>8</v>
+        <v>73</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B46" s="0" t="n">
         <v>1</v>
@@ -1643,7 +1652,7 @@
         <v>1</v>
       </c>
       <c r="D46" s="0" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E46" s="0" t="n">
         <v>1</v>
@@ -1657,7 +1666,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B47" s="0" t="n">
         <v>1</v>
@@ -1677,7 +1686,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B48" s="0" t="n">
         <v>1</v>
@@ -1697,7 +1706,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B49" s="0" t="n">
         <v>1</v>
@@ -1709,15 +1718,15 @@
         <v>62</v>
       </c>
       <c r="F49" s="0" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G49" s="0" t="s">
-        <v>8</v>
+        <v>73</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B50" s="0" t="n">
         <v>1</v>
@@ -1737,7 +1746,7 @@
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B51" s="0" t="n">
         <v>1</v>
@@ -1754,7 +1763,7 @@
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B52" s="0" t="n">
         <v>1</v>
@@ -1774,7 +1783,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B53" s="0" t="n">
         <v>1</v>
@@ -1786,7 +1795,7 @@
         <v>1</v>
       </c>
       <c r="F53" s="0" t="s">
-        <v>82</v>
+        <v>22</v>
       </c>
       <c r="G53" s="0" t="s">
         <v>8</v>
@@ -1794,7 +1803,7 @@
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B54" s="0" t="n">
         <v>1</v>
@@ -1803,7 +1812,7 @@
         <v>4</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F54" s="0" t="s">
         <v>14</v>
@@ -1814,7 +1823,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B55" s="0" t="n">
         <v>1</v>
@@ -1834,7 +1843,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B56" s="0" t="n">
         <v>1</v>
@@ -1843,7 +1852,7 @@
         <v>4</v>
       </c>
       <c r="D56" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E56" s="0" t="n">
         <v>1</v>
@@ -1857,7 +1866,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B57" s="0" t="n">
         <v>1</v>
@@ -1866,7 +1875,7 @@
         <v>0</v>
       </c>
       <c r="D57" s="0" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E57" s="0" t="n">
         <v>0</v>
@@ -1880,7 +1889,7 @@
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B58" s="0" t="n">
         <v>1</v>
@@ -1889,15 +1898,18 @@
         <v>1</v>
       </c>
       <c r="D58" s="0" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E58" s="0" t="n">
         <v>1</v>
+      </c>
+      <c r="G58" s="0" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B59" s="0" t="n">
         <v>1</v>
@@ -1917,7 +1929,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B60" s="0" t="n">
         <v>1</v>
@@ -1940,7 +1952,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B61" s="0" t="n">
         <v>2</v>
@@ -1949,7 +1961,7 @@
         <v>1</v>
       </c>
       <c r="D61" s="0" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E61" s="0" t="n">
         <v>2</v>
@@ -1963,7 +1975,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="0" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B62" s="0" t="n">
         <v>1</v>
@@ -1972,13 +1984,13 @@
         <v>1</v>
       </c>
       <c r="D62" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E62" s="0" t="n">
         <v>1</v>
       </c>
       <c r="F62" s="0" t="s">
-        <v>77</v>
+        <v>22</v>
       </c>
       <c r="G62" s="0" t="s">
         <v>8</v>
@@ -1986,7 +1998,7 @@
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B63" s="0" t="n">
         <v>2</v>
@@ -1998,7 +2010,7 @@
         <v>12</v>
       </c>
       <c r="E63" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F63" s="0" t="s">
         <v>14</v>
@@ -2009,7 +2021,7 @@
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="0" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B64" s="0" t="n">
         <v>1</v>
@@ -2018,7 +2030,7 @@
         <v>1</v>
       </c>
       <c r="D64" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E64" s="0" t="n">
         <v>1</v>
@@ -2027,9 +2039,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="0" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B65" s="0" t="n">
         <v>1</v>
@@ -2038,15 +2050,18 @@
         <v>1</v>
       </c>
       <c r="D65" s="0" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E65" s="0" t="n">
         <v>1</v>
+      </c>
+      <c r="G65" s="0" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="0" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B66" s="0" t="n">
         <v>1</v>
@@ -2055,7 +2070,7 @@
         <v>1</v>
       </c>
       <c r="D66" s="0" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E66" s="0" t="n">
         <v>0</v>
@@ -2066,7 +2081,7 @@
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="0" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B67" s="0" t="n">
         <v>1</v>
@@ -2075,7 +2090,7 @@
         <v>1</v>
       </c>
       <c r="D67" s="0" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E67" s="0" t="n">
         <v>0</v>
@@ -2086,7 +2101,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="0" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B68" s="0" t="n">
         <v>1</v>
@@ -2118,7 +2133,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P71"/>
+  <dimension ref="A1:P82"/>
   <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.99"/>
@@ -2171,22 +2186,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J2" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2207,22 +2222,22 @@
         <v>1</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J3" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2243,25 +2258,25 @@
         <v>0,1</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="J4" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K4" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2282,22 +2297,22 @@
         <v>0</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I5" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J5" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2318,22 +2333,22 @@
         <v>0,1,2</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I6" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J6" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2354,22 +2369,22 @@
         <v>1</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I7" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J7" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2390,22 +2405,22 @@
         <v>0</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I8" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J8" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2426,40 +2441,40 @@
         <v>0,1</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I9" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="J9" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K9" s="0" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="L9" s="0" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="M9" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="N9" s="0" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="O9" s="0" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="P9" s="0" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2480,16 +2495,16 @@
         <v>0,1,2</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2510,22 +2525,22 @@
         <v>0</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F11" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I11" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J11" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2546,22 +2561,22 @@
         <v>0</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I12" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J12" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2582,22 +2597,22 @@
         <v>1</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F13" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I13" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J13" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2618,28 +2633,28 @@
         <v>0,1</v>
       </c>
       <c r="E14" s="0" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H14" s="0" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I14" s="0" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="J14" s="0" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="K14" s="0" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="L14" s="0" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2660,19 +2675,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F15" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H15" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I15" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2693,19 +2708,19 @@
         <v>1,2</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F16" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H16" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I16" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2726,19 +2741,19 @@
         <v>1,2</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F17" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H17" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I17" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2759,19 +2774,19 @@
         <v>1,2</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G18" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H18" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I18" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2792,16 +2807,16 @@
         <v>0,1,2</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G19" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H19" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2822,10 +2837,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F20" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2846,10 +2861,10 @@
         <v>1</v>
       </c>
       <c r="E21" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F21" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2870,10 +2885,10 @@
         <v>0,1</v>
       </c>
       <c r="E22" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F22" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2894,19 +2909,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E23" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F23" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G23" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H23" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I23" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2927,19 +2942,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E24" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F24" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G24" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H24" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I24" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2960,19 +2975,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E25" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F25" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G25" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H25" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I25" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2993,10 +3008,10 @@
         <v>0,1,2</v>
       </c>
       <c r="E26" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F26" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3017,22 +3032,22 @@
         <v>0</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F27" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G27" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H27" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I27" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J27" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3053,19 +3068,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E28" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F28" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G28" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H28" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I28" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3086,10 +3101,10 @@
         <v>0</v>
       </c>
       <c r="E29" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F29" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3110,22 +3125,22 @@
         <v>1</v>
       </c>
       <c r="E30" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F30" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G30" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H30" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I30" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J30" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3146,22 +3161,22 @@
         <v>1</v>
       </c>
       <c r="E31" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F31" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G31" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H31" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I31" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J31" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3182,7 +3197,7 @@
         <v>0,1,2</v>
       </c>
       <c r="E32" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3203,10 +3218,10 @@
         <v>0</v>
       </c>
       <c r="E33" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F33" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3227,10 +3242,10 @@
         <v>0</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F34" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3251,34 +3266,34 @@
         <v>1,2</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F35" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G35" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H35" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I35" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J35" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K35" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="L35" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M35" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N35" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3299,34 +3314,34 @@
         <v>2,3</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F36" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G36" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H36" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I36" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J36" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K36" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="L36" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M36" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N36" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3347,22 +3362,22 @@
         <v>1</v>
       </c>
       <c r="E37" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F37" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G37" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H37" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I37" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J37" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3383,10 +3398,10 @@
         <v>1</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F38" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3425,22 +3440,22 @@
         <v>1</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F40" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G40" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H40" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I40" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J40" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3461,22 +3476,22 @@
         <v>1</v>
       </c>
       <c r="E41" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F41" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G41" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H41" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I41" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J41" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3497,10 +3512,10 @@
         <v>1</v>
       </c>
       <c r="E42" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F42" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3521,22 +3536,22 @@
         <v>1</v>
       </c>
       <c r="E43" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F43" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G43" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H43" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I43" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J43" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3557,25 +3572,25 @@
         <v>0,1</v>
       </c>
       <c r="E44" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F44" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G44" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H44" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I44" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="J44" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K44" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3596,22 +3611,22 @@
         <v>1</v>
       </c>
       <c r="E45" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F45" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G45" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H45" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I45" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J45" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3632,10 +3647,10 @@
         <v>1</v>
       </c>
       <c r="E46" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F46" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3656,16 +3671,16 @@
         <v>0</v>
       </c>
       <c r="E47" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F47" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G47" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H47" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3686,16 +3701,16 @@
         <v>1</v>
       </c>
       <c r="E48" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F48" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G48" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H48" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3734,10 +3749,10 @@
         <v>0,1</v>
       </c>
       <c r="E50" s="0" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F50" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3758,22 +3773,22 @@
         <v>1</v>
       </c>
       <c r="E51" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F51" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G51" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H51" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I51" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J51" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3794,10 +3809,10 @@
         <v>1</v>
       </c>
       <c r="E52" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F52" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3818,22 +3833,22 @@
         <v>1</v>
       </c>
       <c r="E53" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F53" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G53" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H53" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I53" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J53" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3854,22 +3869,22 @@
         <v>1,3</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F54" s="0" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G54" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H54" s="0" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="I54" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J54" s="0" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3890,22 +3905,22 @@
         <v>1</v>
       </c>
       <c r="E55" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F55" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G55" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H55" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I55" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J55" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3926,22 +3941,22 @@
         <v>1</v>
       </c>
       <c r="E56" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F56" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G56" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H56" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I56" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J56" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3962,28 +3977,28 @@
         <v>0</v>
       </c>
       <c r="E57" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F57" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G57" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H57" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I57" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J57" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="str">
         <f aca="false">LibManager!A58</f>
-        <v>#Syncopy =&gt; commented out (special case)</v>
+        <v>Syncopy</v>
       </c>
       <c r="B58" s="0" t="n">
         <f aca="false">LibManager!B58</f>
@@ -3998,22 +4013,22 @@
         <v>1</v>
       </c>
       <c r="E58" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F58" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G58" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H58" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I58" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J58" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4034,10 +4049,10 @@
         <v>1</v>
       </c>
       <c r="E59" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F59" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4058,22 +4073,22 @@
         <v>0</v>
       </c>
       <c r="E60" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F60" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G60" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H60" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I60" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J60" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4094,22 +4109,22 @@
         <v>2</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F61" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G61" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H61" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I61" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J61" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4130,22 +4145,22 @@
         <v>1</v>
       </c>
       <c r="E62" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F62" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G62" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H62" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I62" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J62" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4166,25 +4181,25 @@
         <v>0,2</v>
       </c>
       <c r="E63" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F63" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G63" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H63" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I63" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="J63" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K63" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4205,22 +4220,22 @@
         <v>1</v>
       </c>
       <c r="E64" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F64" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G64" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H64" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I64" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J64" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4241,16 +4256,16 @@
         <v>1</v>
       </c>
       <c r="E65" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F65" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G65" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="H65" s="0" t="s">
         <v>111</v>
-      </c>
-      <c r="H65" s="0" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4271,16 +4286,16 @@
         <v>0</v>
       </c>
       <c r="E66" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F66" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G66" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H66" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4301,25 +4316,25 @@
         <v>0</v>
       </c>
       <c r="E67" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F67" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G67" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H67" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="I67" s="0" t="s">
+        <v>163</v>
+      </c>
+      <c r="J67" s="0" t="s">
         <v>112</v>
       </c>
-      <c r="I67" s="0" t="s">
-        <v>162</v>
-      </c>
-      <c r="J67" s="0" t="s">
+      <c r="K67" s="0" t="s">
         <v>111</v>
-      </c>
-      <c r="K67" s="0" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4340,7 +4355,7 @@
         <v>0</v>
       </c>
       <c r="E68" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4379,17 +4394,204 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="75" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="76" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="77" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="80" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="0" t="n">
+        <f aca="false">LibManager!A71</f>
+        <v>0</v>
+      </c>
+      <c r="B71" s="0" t="n">
+        <f aca="false">LibManager!B71</f>
+        <v>0</v>
+      </c>
+      <c r="C71" s="0" t="n">
+        <f aca="false">LibManager!C71</f>
+        <v>0</v>
+      </c>
+      <c r="D71" s="0" t="n">
+        <f aca="false">LibManager!E71</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="0" t="n">
+        <f aca="false">LibManager!A72</f>
+        <v>0</v>
+      </c>
+      <c r="B72" s="0" t="n">
+        <f aca="false">LibManager!B72</f>
+        <v>0</v>
+      </c>
+      <c r="C72" s="0" t="n">
+        <f aca="false">LibManager!C72</f>
+        <v>0</v>
+      </c>
+      <c r="D72" s="0" t="n">
+        <f aca="false">LibManager!E72</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="0" t="n">
+        <f aca="false">LibManager!A73</f>
+        <v>0</v>
+      </c>
+      <c r="B73" s="0" t="n">
+        <f aca="false">LibManager!B73</f>
+        <v>0</v>
+      </c>
+      <c r="C73" s="0" t="n">
+        <f aca="false">LibManager!C73</f>
+        <v>0</v>
+      </c>
+      <c r="D73" s="0" t="n">
+        <f aca="false">LibManager!E73</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="0" t="n">
+        <f aca="false">LibManager!A74</f>
+        <v>0</v>
+      </c>
+      <c r="B74" s="0" t="n">
+        <f aca="false">LibManager!B74</f>
+        <v>0</v>
+      </c>
+      <c r="C74" s="0" t="n">
+        <f aca="false">LibManager!C74</f>
+        <v>0</v>
+      </c>
+      <c r="D74" s="0" t="n">
+        <f aca="false">LibManager!E74</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="0" t="n">
+        <f aca="false">LibManager!A75</f>
+        <v>0</v>
+      </c>
+      <c r="B75" s="0" t="n">
+        <f aca="false">LibManager!B75</f>
+        <v>0</v>
+      </c>
+      <c r="C75" s="0" t="n">
+        <f aca="false">LibManager!C75</f>
+        <v>0</v>
+      </c>
+      <c r="D75" s="0" t="n">
+        <f aca="false">LibManager!E75</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="0" t="n">
+        <f aca="false">LibManager!A76</f>
+        <v>0</v>
+      </c>
+      <c r="B76" s="0" t="n">
+        <f aca="false">LibManager!B76</f>
+        <v>0</v>
+      </c>
+      <c r="C76" s="0" t="n">
+        <f aca="false">LibManager!C76</f>
+        <v>0</v>
+      </c>
+      <c r="D76" s="0" t="n">
+        <f aca="false">LibManager!E76</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="0" t="n">
+        <f aca="false">LibManager!A77</f>
+        <v>0</v>
+      </c>
+      <c r="B77" s="0" t="n">
+        <f aca="false">LibManager!B77</f>
+        <v>0</v>
+      </c>
+      <c r="C77" s="0" t="n">
+        <f aca="false">LibManager!C77</f>
+        <v>0</v>
+      </c>
+      <c r="D77" s="0" t="n">
+        <f aca="false">LibManager!E77</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="0" t="n">
+        <f aca="false">LibManager!A78</f>
+        <v>0</v>
+      </c>
+      <c r="B78" s="0" t="n">
+        <f aca="false">LibManager!B78</f>
+        <v>0</v>
+      </c>
+      <c r="C78" s="0" t="n">
+        <f aca="false">LibManager!C78</f>
+        <v>0</v>
+      </c>
+      <c r="D78" s="0" t="n">
+        <f aca="false">LibManager!E78</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="0" t="n">
+        <f aca="false">LibManager!A79</f>
+        <v>0</v>
+      </c>
+      <c r="B79" s="0" t="n">
+        <f aca="false">LibManager!B79</f>
+        <v>0</v>
+      </c>
+      <c r="C79" s="0" t="n">
+        <f aca="false">LibManager!C79</f>
+        <v>0</v>
+      </c>
+      <c r="D79" s="0" t="n">
+        <f aca="false">LibManager!E79</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="0" t="n">
+        <f aca="false">LibManager!A80</f>
+        <v>0</v>
+      </c>
+      <c r="B80" s="0" t="n">
+        <f aca="false">LibManager!B80</f>
+        <v>0</v>
+      </c>
+      <c r="C80" s="0" t="n">
+        <f aca="false">LibManager!C80</f>
+        <v>0</v>
+      </c>
+      <c r="D80" s="0" t="n">
+        <f aca="false">LibManager!E80</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="0" t="n">
+        <f aca="false">LibManager!A81</f>
+        <v>0</v>
+      </c>
+      <c r="B81" s="0" t="n">
+        <f aca="false">LibManager!B81</f>
+        <v>0</v>
+      </c>
+      <c r="C81" s="0" t="n">
+        <f aca="false">LibManager!C81</f>
+        <v>0</v>
+      </c>
+      <c r="D81" s="0" t="n">
+        <f aca="false">LibManager!E81</f>
+        <v>0</v>
+      </c>
+    </row>
     <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
[dnn-library] [SW-3346] Add version selector for elementwise because certain elemKinds don't work with vectorized
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -116,6 +116,9 @@
     <t xml:space="preserve">ElementAdd</t>
   </si>
   <si>
+    <t xml:space="preserve">custom</t>
+  </si>
+  <si>
     <t xml:space="preserve">ElementCmpEQ</t>
   </si>
   <si>
@@ -240,9 +243,6 @@
   </si>
   <si>
     <t xml:space="preserve">Threaded,Vectorized,Aligned32Bytes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">custom</t>
   </si>
   <si>
     <t xml:space="preserve">Modulo</t>
@@ -1023,12 +1023,12 @@
         <v>22</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B16" s="0" t="n">
         <v>1</v>
@@ -1037,7 +1037,7 @@
         <v>2</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F16" s="0" t="s">
         <v>22</v>
@@ -1048,16 +1048,16 @@
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="0" t="s">
         <v>33</v>
-      </c>
-      <c r="B17" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C17" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="E17" s="0" t="s">
-        <v>32</v>
       </c>
       <c r="F17" s="0" t="s">
         <v>22</v>
@@ -1068,7 +1068,7 @@
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B18" s="0" t="n">
         <v>1</v>
@@ -1077,7 +1077,7 @@
         <v>2</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F18" s="0" t="s">
         <v>22</v>
@@ -1088,7 +1088,7 @@
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B19" s="0" t="n">
         <v>1</v>
@@ -1103,12 +1103,12 @@
         <v>22</v>
       </c>
       <c r="G19" s="0" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B20" s="0" t="n">
         <v>1</v>
@@ -1125,7 +1125,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B21" s="0" t="n">
         <v>1</v>
@@ -1145,7 +1145,7 @@
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B22" s="0" t="n">
         <v>1</v>
@@ -1165,7 +1165,7 @@
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B23" s="0" t="n">
         <v>1</v>
@@ -1180,12 +1180,12 @@
         <v>22</v>
       </c>
       <c r="G23" s="0" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B24" s="0" t="n">
         <v>1</v>
@@ -1200,12 +1200,12 @@
         <v>22</v>
       </c>
       <c r="G24" s="0" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B25" s="0" t="n">
         <v>1</v>
@@ -1220,12 +1220,12 @@
         <v>22</v>
       </c>
       <c r="G25" s="0" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B26" s="0" t="n">
         <v>1</v>
@@ -1240,12 +1240,12 @@
         <v>22</v>
       </c>
       <c r="G26" s="0" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B27" s="0" t="n">
         <v>1</v>
@@ -1263,9 +1263,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B28" s="0" t="n">
         <v>1</v>
@@ -1280,12 +1280,12 @@
         <v>22</v>
       </c>
       <c r="G28" s="0" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B29" s="0" t="n">
         <v>1</v>
@@ -1294,7 +1294,7 @@
         <v>4</v>
       </c>
       <c r="D29" s="0" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E29" s="0" t="n">
         <v>0</v>
@@ -1305,7 +1305,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B30" s="0" t="n">
         <v>1</v>
@@ -1314,7 +1314,7 @@
         <v>1</v>
       </c>
       <c r="D30" s="0" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E30" s="0" t="n">
         <v>1</v>
@@ -1328,7 +1328,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B31" s="0" t="n">
         <v>1</v>
@@ -1348,7 +1348,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B32" s="0" t="n">
         <v>1</v>
@@ -1368,7 +1368,7 @@
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B33" s="0" t="n">
         <v>1</v>
@@ -1380,7 +1380,7 @@
         <v>0</v>
       </c>
       <c r="F33" s="0" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G33" s="0" t="s">
         <v>8</v>
@@ -1388,7 +1388,7 @@
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B34" s="0" t="n">
         <v>1</v>
@@ -1408,7 +1408,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B35" s="0" t="n">
         <v>1</v>
@@ -1417,10 +1417,10 @@
         <v>2</v>
       </c>
       <c r="D35" s="0" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F35" s="0" t="s">
         <v>14</v>
@@ -1431,7 +1431,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B36" s="0" t="n">
         <v>2</v>
@@ -1440,7 +1440,7 @@
         <v>2</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F36" s="0" t="s">
         <v>14</v>
@@ -1451,7 +1451,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B37" s="0" t="n">
         <v>1</v>
@@ -1460,7 +1460,7 @@
         <v>1</v>
       </c>
       <c r="D37" s="0" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E37" s="0" t="n">
         <v>1</v>
@@ -1474,7 +1474,7 @@
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B38" s="0" t="n">
         <v>1</v>
@@ -1491,7 +1491,7 @@
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B39" s="0" t="n">
         <v>1</v>
@@ -1500,7 +1500,7 @@
         <v>2</v>
       </c>
       <c r="E39" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F39" s="0" t="s">
         <v>14</v>
@@ -1511,7 +1511,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B40" s="0" t="n">
         <v>1</v>
@@ -1531,7 +1531,7 @@
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B41" s="0" t="n">
         <v>1</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B42" s="0" t="n">
         <v>2</v>
@@ -1560,7 +1560,7 @@
         <v>1</v>
       </c>
       <c r="D42" s="0" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E42" s="0" t="n">
         <v>1</v>
@@ -1574,7 +1574,7 @@
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B43" s="0" t="n">
         <v>1</v>
@@ -1583,7 +1583,7 @@
         <v>2</v>
       </c>
       <c r="D43" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E43" s="0" t="n">
         <v>1</v>
@@ -1597,7 +1597,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B44" s="0" t="n">
         <v>1</v>
@@ -1620,7 +1620,7 @@
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B45" s="0" t="n">
         <v>1</v>
@@ -1629,16 +1629,16 @@
         <v>1</v>
       </c>
       <c r="D45" s="0" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E45" s="0" t="n">
         <v>1</v>
       </c>
       <c r="F45" s="0" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G45" s="0" t="s">
-        <v>73</v>
+        <v>31</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1715,13 +1715,13 @@
         <v>5</v>
       </c>
       <c r="E49" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F49" s="0" t="s">
         <v>79</v>
       </c>
       <c r="G49" s="0" t="s">
-        <v>73</v>
+        <v>31</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1875,7 +1875,7 @@
         <v>0</v>
       </c>
       <c r="D57" s="0" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E57" s="0" t="n">
         <v>0</v>
@@ -1938,7 +1938,7 @@
         <v>1</v>
       </c>
       <c r="D60" s="0" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E60" s="0" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
[dnn-library] [SW-3347]  Vector version for logical compare insns not implemented for certain element types => add custom selector
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -1043,7 +1043,7 @@
         <v>22</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1063,7 +1063,7 @@
         <v>22</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1083,7 +1083,7 @@
         <v>22</v>
       </c>
       <c r="G18" s="0" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] [SW-3358] Using dst instead of idx elK for function template parameter
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -1755,7 +1755,7 @@
         <v>2</v>
       </c>
       <c r="E51" s="0" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G51" s="0" t="s">
         <v>8</v>
@@ -3770,7 +3770,7 @@
       </c>
       <c r="D51" s="0" t="n">
         <f aca="false">LibManager!E51</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E51" s="0" t="s">
         <v>108</v>

</xml_diff>

<commit_message>
[dnn-library] [SW-3359] wrong order of input tensor parameters in sparsetoDense
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -1832,7 +1832,7 @@
         <v>2</v>
       </c>
       <c r="E55" s="0" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F55" s="0" t="s">
         <v>22</v>
@@ -1841,7 +1841,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="0" t="s">
         <v>87</v>
       </c>
@@ -3902,7 +3902,7 @@
       </c>
       <c r="D55" s="0" t="n">
         <f aca="false">LibManager!E55</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E55" s="0" t="s">
         <v>108</v>

</xml_diff>

<commit_message>
[dnn-library] Fix SparseToDenseMask. Tensors are swapped and getting wrong elk template parameter.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
@@ -1855,7 +1855,7 @@
         <v>88</v>
       </c>
       <c r="E56" s="0" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F56" s="0" t="s">
         <v>14</v>
@@ -3938,7 +3938,7 @@
       </c>
       <c r="D56" s="0" t="n">
         <f aca="false">LibManager!E56</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E56" s="0" t="s">
         <v>108</v>

</xml_diff>

<commit_message>
[dnn-library] [SW-3380] Disabling sparseLenWeightedSum threaded implementation until Rafa fixes it
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="172">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -279,6 +279,9 @@
   </si>
   <si>
     <t xml:space="preserve">1,3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#Threaded</t>
   </si>
   <si>
     <t xml:space="preserve">SparseToDense</t>
@@ -1815,7 +1818,7 @@
         <v>85</v>
       </c>
       <c r="F54" s="0" t="s">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="G54" s="0" t="s">
         <v>8</v>
@@ -1823,7 +1826,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B55" s="0" t="n">
         <v>1</v>
@@ -1843,7 +1846,7 @@
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B56" s="0" t="n">
         <v>1</v>
@@ -1852,7 +1855,7 @@
         <v>4</v>
       </c>
       <c r="D56" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E56" s="0" t="n">
         <v>0</v>
@@ -1866,7 +1869,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B57" s="0" t="n">
         <v>1</v>
@@ -1889,7 +1892,7 @@
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B58" s="0" t="n">
         <v>1</v>
@@ -1898,7 +1901,7 @@
         <v>1</v>
       </c>
       <c r="D58" s="0" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E58" s="0" t="n">
         <v>1</v>
@@ -1909,7 +1912,7 @@
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B59" s="0" t="n">
         <v>1</v>
@@ -1929,7 +1932,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B60" s="0" t="n">
         <v>1</v>
@@ -1952,7 +1955,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B61" s="0" t="n">
         <v>2</v>
@@ -1961,7 +1964,7 @@
         <v>1</v>
       </c>
       <c r="D61" s="0" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E61" s="0" t="n">
         <v>2</v>
@@ -1975,7 +1978,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B62" s="0" t="n">
         <v>1</v>
@@ -1984,7 +1987,7 @@
         <v>1</v>
       </c>
       <c r="D62" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E62" s="0" t="n">
         <v>1</v>
@@ -1998,7 +2001,7 @@
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B63" s="0" t="n">
         <v>2</v>
@@ -2010,7 +2013,7 @@
         <v>12</v>
       </c>
       <c r="E63" s="0" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F63" s="0" t="s">
         <v>14</v>
@@ -2021,7 +2024,7 @@
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B64" s="0" t="n">
         <v>1</v>
@@ -2030,7 +2033,7 @@
         <v>1</v>
       </c>
       <c r="D64" s="0" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E64" s="0" t="n">
         <v>1</v>
@@ -2041,7 +2044,7 @@
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="0" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B65" s="0" t="n">
         <v>1</v>
@@ -2050,7 +2053,7 @@
         <v>1</v>
       </c>
       <c r="D65" s="0" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E65" s="0" t="n">
         <v>1</v>
@@ -2061,7 +2064,7 @@
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="0" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B66" s="0" t="n">
         <v>1</v>
@@ -2070,7 +2073,7 @@
         <v>1</v>
       </c>
       <c r="D66" s="0" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E66" s="0" t="n">
         <v>0</v>
@@ -2081,7 +2084,7 @@
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="0" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B67" s="0" t="n">
         <v>1</v>
@@ -2090,7 +2093,7 @@
         <v>1</v>
       </c>
       <c r="D67" s="0" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E67" s="0" t="n">
         <v>0</v>
@@ -2101,7 +2104,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B68" s="0" t="n">
         <v>1</v>
@@ -2186,22 +2189,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J2" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2222,22 +2225,22 @@
         <v>1</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J3" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2258,25 +2261,25 @@
         <v>0,1</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J4" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K4" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2297,22 +2300,22 @@
         <v>0</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I5" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J5" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2333,22 +2336,22 @@
         <v>0,1,2</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I6" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J6" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2369,22 +2372,22 @@
         <v>1</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I7" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J7" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2405,22 +2408,22 @@
         <v>0</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I8" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J8" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2441,40 +2444,40 @@
         <v>0,1</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I9" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="J9" s="0" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K9" s="0" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="L9" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="M9" s="0" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="N9" s="0" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="O9" s="0" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="P9" s="0" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2495,16 +2498,16 @@
         <v>0,1,2</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2525,22 +2528,22 @@
         <v>0</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F11" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I11" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J11" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2561,22 +2564,22 @@
         <v>0</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I12" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J12" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2597,22 +2600,22 @@
         <v>1</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F13" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I13" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J13" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2633,28 +2636,28 @@
         <v>0,1</v>
       </c>
       <c r="E14" s="0" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H14" s="0" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="I14" s="0" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="J14" s="0" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="K14" s="0" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="L14" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2675,19 +2678,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F15" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H15" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I15" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2708,19 +2711,19 @@
         <v>1,2</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F16" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H16" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="I16" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2741,19 +2744,19 @@
         <v>1,2</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F17" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H17" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="I17" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2774,19 +2777,19 @@
         <v>1,2</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G18" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H18" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="I18" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2807,16 +2810,16 @@
         <v>0,1,2</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G19" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H19" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2837,10 +2840,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F20" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2861,10 +2864,10 @@
         <v>1</v>
       </c>
       <c r="E21" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F21" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2885,10 +2888,10 @@
         <v>0,1</v>
       </c>
       <c r="E22" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F22" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2909,19 +2912,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E23" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F23" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G23" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H23" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I23" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2942,19 +2945,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E24" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F24" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G24" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H24" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I24" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2975,19 +2978,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E25" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F25" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G25" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H25" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I25" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3008,10 +3011,10 @@
         <v>0,1,2</v>
       </c>
       <c r="E26" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F26" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3032,22 +3035,22 @@
         <v>0</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F27" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G27" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H27" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I27" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J27" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3068,19 +3071,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E28" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F28" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G28" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H28" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I28" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3101,10 +3104,10 @@
         <v>0</v>
       </c>
       <c r="E29" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F29" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3125,22 +3128,22 @@
         <v>1</v>
       </c>
       <c r="E30" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F30" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G30" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H30" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I30" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J30" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3161,22 +3164,22 @@
         <v>1</v>
       </c>
       <c r="E31" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F31" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G31" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H31" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I31" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J31" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3197,7 +3200,7 @@
         <v>0,1,2</v>
       </c>
       <c r="E32" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3218,10 +3221,10 @@
         <v>0</v>
       </c>
       <c r="E33" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F33" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3242,10 +3245,10 @@
         <v>0</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F34" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3266,34 +3269,34 @@
         <v>1,2</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F35" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G35" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H35" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I35" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="J35" s="0" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K35" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="L35" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="M35" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="N35" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3314,34 +3317,34 @@
         <v>2,3</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F36" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G36" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H36" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I36" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="J36" s="0" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K36" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="L36" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="M36" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="N36" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3362,22 +3365,22 @@
         <v>1</v>
       </c>
       <c r="E37" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F37" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G37" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H37" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I37" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J37" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3398,10 +3401,10 @@
         <v>1</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F38" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3440,22 +3443,22 @@
         <v>1</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F40" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G40" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H40" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I40" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J40" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3476,22 +3479,22 @@
         <v>1</v>
       </c>
       <c r="E41" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F41" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G41" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H41" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I41" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J41" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3512,10 +3515,10 @@
         <v>1</v>
       </c>
       <c r="E42" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F42" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3536,22 +3539,22 @@
         <v>1</v>
       </c>
       <c r="E43" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F43" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G43" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H43" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I43" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J43" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3572,25 +3575,25 @@
         <v>0,1</v>
       </c>
       <c r="E44" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F44" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G44" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H44" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I44" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J44" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K44" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3611,22 +3614,22 @@
         <v>1</v>
       </c>
       <c r="E45" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F45" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G45" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H45" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I45" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J45" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3647,10 +3650,10 @@
         <v>1</v>
       </c>
       <c r="E46" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F46" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3671,16 +3674,16 @@
         <v>0</v>
       </c>
       <c r="E47" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F47" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G47" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H47" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3701,16 +3704,16 @@
         <v>1</v>
       </c>
       <c r="E48" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F48" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G48" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H48" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3749,10 +3752,10 @@
         <v>0,1</v>
       </c>
       <c r="E50" s="0" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F50" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3773,22 +3776,22 @@
         <v>0</v>
       </c>
       <c r="E51" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F51" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G51" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H51" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I51" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J51" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3809,10 +3812,10 @@
         <v>1</v>
       </c>
       <c r="E52" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F52" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3833,22 +3836,22 @@
         <v>1</v>
       </c>
       <c r="E53" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F53" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G53" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H53" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I53" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J53" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3869,22 +3872,22 @@
         <v>1,3</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F54" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G54" s="0" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H54" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I54" s="0" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J54" s="0" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3905,22 +3908,22 @@
         <v>0</v>
       </c>
       <c r="E55" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F55" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G55" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H55" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I55" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J55" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3941,22 +3944,22 @@
         <v>0</v>
       </c>
       <c r="E56" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F56" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G56" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H56" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I56" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J56" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3977,22 +3980,22 @@
         <v>0</v>
       </c>
       <c r="E57" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F57" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G57" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H57" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I57" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J57" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4013,22 +4016,22 @@
         <v>1</v>
       </c>
       <c r="E58" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F58" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G58" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H58" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I58" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J58" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4049,10 +4052,10 @@
         <v>1</v>
       </c>
       <c r="E59" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F59" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4073,22 +4076,22 @@
         <v>0</v>
       </c>
       <c r="E60" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F60" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G60" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H60" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I60" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J60" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4109,22 +4112,22 @@
         <v>2</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F61" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G61" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H61" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I61" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J61" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4145,22 +4148,22 @@
         <v>1</v>
       </c>
       <c r="E62" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F62" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G62" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H62" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I62" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J62" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4181,25 +4184,25 @@
         <v>0,2</v>
       </c>
       <c r="E63" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F63" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G63" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H63" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I63" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J63" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K63" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4220,22 +4223,22 @@
         <v>1</v>
       </c>
       <c r="E64" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F64" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G64" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H64" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I64" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J64" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4256,16 +4259,16 @@
         <v>1</v>
       </c>
       <c r="E65" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F65" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G65" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="H65" s="0" t="s">
         <v>112</v>
-      </c>
-      <c r="H65" s="0" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4286,16 +4289,16 @@
         <v>0</v>
       </c>
       <c r="E66" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F66" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G66" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H66" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4316,25 +4319,25 @@
         <v>0</v>
       </c>
       <c r="E67" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F67" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G67" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H67" s="0" t="s">
+        <v>114</v>
+      </c>
+      <c r="I67" s="0" t="s">
+        <v>164</v>
+      </c>
+      <c r="J67" s="0" t="s">
         <v>113</v>
       </c>
-      <c r="I67" s="0" t="s">
-        <v>163</v>
-      </c>
-      <c r="J67" s="0" t="s">
+      <c r="K67" s="0" t="s">
         <v>112</v>
-      </c>
-      <c r="K67" s="0" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4355,7 +4358,7 @@
         <v>0</v>
       </c>
       <c r="E68" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] SparseLengthsWeightedSum add more template arguments.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="581" uniqueCount="172">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -3889,6 +3889,15 @@
       <c r="J54" s="0" t="s">
         <v>171</v>
       </c>
+      <c r="K54" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="L54" s="0" t="s">
+        <v>155</v>
+      </c>
+      <c r="M54" s="0" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="str">

</xml_diff>

<commit_message>
[dnn-library] Fix almost all SparseLengthsSumInst test. Enable quantized modes for SparseLengthsWeightedSumInst
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="581" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="173">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -348,6 +348,9 @@
   </si>
   <si>
     <t xml:space="preserve">LengthsRangeFill</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SparseLengthsSum</t>
   </si>
   <si>
     <t xml:space="preserve">FloatTy</t>
@@ -2119,6 +2122,26 @@
         <v>8</v>
       </c>
     </row>
+    <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="B69" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C69" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="E69" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="F69" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="G69" s="0" t="s">
+        <v>8</v>
+      </c>
+    </row>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2189,22 +2212,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J2" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2225,22 +2248,22 @@
         <v>1</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J3" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2261,25 +2284,25 @@
         <v>0,1</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J4" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K4" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2300,22 +2323,22 @@
         <v>0</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I5" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J5" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2336,22 +2359,22 @@
         <v>0,1,2</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="I6" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J6" s="0" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2372,22 +2395,22 @@
         <v>1</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I7" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J7" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2408,22 +2431,22 @@
         <v>0</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I8" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J8" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2444,40 +2467,40 @@
         <v>0,1</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="I9" s="0" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="J9" s="0" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="K9" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="L9" s="0" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="M9" s="0" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="N9" s="0" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="O9" s="0" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="P9" s="0" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2498,16 +2521,16 @@
         <v>0,1,2</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2528,22 +2551,22 @@
         <v>0</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F11" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I11" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J11" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2564,22 +2587,22 @@
         <v>0</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I12" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J12" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2600,22 +2623,22 @@
         <v>1</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F13" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I13" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J13" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2636,28 +2659,28 @@
         <v>0,1</v>
       </c>
       <c r="E14" s="0" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H14" s="0" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I14" s="0" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J14" s="0" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="K14" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="L14" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2678,19 +2701,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F15" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H15" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="I15" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2711,19 +2734,19 @@
         <v>1,2</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F16" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H16" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I16" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2744,19 +2767,19 @@
         <v>1,2</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F17" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H17" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I17" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2777,19 +2800,19 @@
         <v>1,2</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G18" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H18" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I18" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2810,16 +2833,16 @@
         <v>0,1,2</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G19" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H19" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2840,10 +2863,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F20" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2864,10 +2887,10 @@
         <v>1</v>
       </c>
       <c r="E21" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F21" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2888,10 +2911,10 @@
         <v>0,1</v>
       </c>
       <c r="E22" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F22" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2912,19 +2935,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E23" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F23" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G23" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H23" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="I23" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2945,19 +2968,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E24" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F24" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G24" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H24" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="I24" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2978,19 +3001,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E25" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F25" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G25" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H25" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="I25" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3011,10 +3034,10 @@
         <v>0,1,2</v>
       </c>
       <c r="E26" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F26" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3035,22 +3058,22 @@
         <v>0</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F27" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G27" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H27" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I27" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J27" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3071,19 +3094,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E28" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F28" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G28" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H28" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="I28" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3104,10 +3127,10 @@
         <v>0</v>
       </c>
       <c r="E29" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F29" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3128,22 +3151,22 @@
         <v>1</v>
       </c>
       <c r="E30" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F30" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G30" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H30" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I30" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J30" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3164,22 +3187,22 @@
         <v>1</v>
       </c>
       <c r="E31" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F31" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G31" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H31" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I31" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J31" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3200,7 +3223,7 @@
         <v>0,1,2</v>
       </c>
       <c r="E32" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3221,10 +3244,10 @@
         <v>0</v>
       </c>
       <c r="E33" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F33" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3245,10 +3268,10 @@
         <v>0</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F34" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3269,34 +3292,34 @@
         <v>1,2</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F35" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G35" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H35" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="I35" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J35" s="0" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="K35" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="L35" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="M35" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="N35" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3317,34 +3340,34 @@
         <v>2,3</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F36" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G36" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H36" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="I36" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J36" s="0" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="K36" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="L36" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="M36" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="N36" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3365,22 +3388,22 @@
         <v>1</v>
       </c>
       <c r="E37" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F37" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G37" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H37" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I37" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J37" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3401,10 +3424,10 @@
         <v>1</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F38" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3443,22 +3466,22 @@
         <v>1</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F40" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G40" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H40" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I40" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J40" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3479,22 +3502,22 @@
         <v>1</v>
       </c>
       <c r="E41" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F41" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G41" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H41" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I41" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J41" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3515,10 +3538,10 @@
         <v>1</v>
       </c>
       <c r="E42" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F42" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3539,22 +3562,22 @@
         <v>1</v>
       </c>
       <c r="E43" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F43" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G43" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H43" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I43" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J43" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3575,25 +3598,25 @@
         <v>0,1</v>
       </c>
       <c r="E44" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F44" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G44" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H44" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I44" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J44" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K44" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3614,22 +3637,22 @@
         <v>1</v>
       </c>
       <c r="E45" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F45" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G45" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H45" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I45" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J45" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3650,10 +3673,10 @@
         <v>1</v>
       </c>
       <c r="E46" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F46" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3674,16 +3697,16 @@
         <v>0</v>
       </c>
       <c r="E47" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F47" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G47" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H47" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3704,16 +3727,16 @@
         <v>1</v>
       </c>
       <c r="E48" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F48" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G48" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H48" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3752,10 +3775,10 @@
         <v>0,1</v>
       </c>
       <c r="E50" s="0" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F50" s="0" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3776,22 +3799,22 @@
         <v>0</v>
       </c>
       <c r="E51" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F51" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G51" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H51" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I51" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J51" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3812,10 +3835,10 @@
         <v>1</v>
       </c>
       <c r="E52" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F52" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3836,22 +3859,22 @@
         <v>1</v>
       </c>
       <c r="E53" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F53" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G53" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H53" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I53" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J53" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3872,31 +3895,31 @@
         <v>1,3</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F54" s="0" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G54" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H54" s="0" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I54" s="0" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J54" s="0" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K54" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="L54" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="M54" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3917,22 +3940,22 @@
         <v>0</v>
       </c>
       <c r="E55" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F55" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G55" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H55" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I55" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J55" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3953,22 +3976,22 @@
         <v>0</v>
       </c>
       <c r="E56" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F56" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G56" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H56" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I56" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J56" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3989,22 +4012,22 @@
         <v>0</v>
       </c>
       <c r="E57" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F57" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G57" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H57" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I57" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J57" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4025,22 +4048,22 @@
         <v>1</v>
       </c>
       <c r="E58" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F58" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G58" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H58" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I58" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J58" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4061,10 +4084,10 @@
         <v>1</v>
       </c>
       <c r="E59" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F59" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4085,22 +4108,22 @@
         <v>0</v>
       </c>
       <c r="E60" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F60" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G60" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H60" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I60" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J60" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4121,22 +4144,22 @@
         <v>2</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F61" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G61" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H61" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I61" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J61" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4157,22 +4180,22 @@
         <v>1</v>
       </c>
       <c r="E62" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F62" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G62" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H62" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I62" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J62" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4193,25 +4216,25 @@
         <v>0,2</v>
       </c>
       <c r="E63" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F63" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G63" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H63" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I63" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J63" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K63" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4232,22 +4255,22 @@
         <v>1</v>
       </c>
       <c r="E64" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F64" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G64" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H64" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I64" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J64" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4268,16 +4291,16 @@
         <v>1</v>
       </c>
       <c r="E65" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F65" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G65" s="0" t="s">
+        <v>114</v>
+      </c>
+      <c r="H65" s="0" t="s">
         <v>113</v>
-      </c>
-      <c r="H65" s="0" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4298,16 +4321,16 @@
         <v>0</v>
       </c>
       <c r="E66" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F66" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G66" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H66" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4328,25 +4351,25 @@
         <v>0</v>
       </c>
       <c r="E67" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F67" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G67" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H67" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="I67" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="J67" s="0" t="s">
         <v>114</v>
       </c>
-      <c r="I67" s="0" t="s">
-        <v>164</v>
-      </c>
-      <c r="J67" s="0" t="s">
+      <c r="K67" s="0" t="s">
         <v>113</v>
-      </c>
-      <c r="K67" s="0" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4367,25 +4390,42 @@
         <v>0</v>
       </c>
       <c r="E68" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="0" t="n">
+      <c r="A69" s="0" t="str">
         <f aca="false">LibManager!A69</f>
-        <v>0</v>
+        <v>SparseLengthsSum</v>
       </c>
       <c r="B69" s="0" t="n">
         <f aca="false">LibManager!B69</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C69" s="0" t="n">
         <f aca="false">LibManager!C69</f>
-        <v>0</v>
-      </c>
-      <c r="D69" s="0" t="n">
-        <f aca="false">LibManager!E69</f>
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="D69" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="E69" s="0" t="s">
+        <v>155</v>
+      </c>
+      <c r="F69" s="0" t="s">
+        <v>134</v>
+      </c>
+      <c r="G69" s="0" t="s">
+        <v>156</v>
+      </c>
+      <c r="H69" s="0" t="s">
+        <v>160</v>
+      </c>
+      <c r="I69" s="0" t="s">
+        <v>161</v>
+      </c>
+      <c r="J69" s="0" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] Add int32 quantize template instation for Flip.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="173">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -485,6 +485,9 @@
     <t xml:space="preserve">Int32ITy,Int32ITy</t>
   </si>
   <si>
+    <t xml:space="preserve">Int32QTy</t>
+  </si>
+  <si>
     <t xml:space="preserve">#Float16Ty</t>
   </si>
   <si>
@@ -516,9 +519,6 @@
   </si>
   <si>
     <t xml:space="preserve">UInt8QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int32QTy</t>
   </si>
   <si>
     <t xml:space="preserve">#Float16Ty,UInt8QTy</t>
@@ -3204,6 +3204,9 @@
       <c r="J31" s="0" t="s">
         <v>115</v>
       </c>
+      <c r="K31" s="0" t="s">
+        <v>154</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="str">
@@ -3271,7 +3274,7 @@
         <v>110</v>
       </c>
       <c r="F34" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3292,34 +3295,34 @@
         <v>1,2</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F35" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G35" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H35" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I35" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J35" s="0" t="s">
         <v>134</v>
       </c>
       <c r="K35" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="L35" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="M35" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="N35" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3340,34 +3343,34 @@
         <v>2,3</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F36" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G36" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H36" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I36" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J36" s="0" t="s">
         <v>134</v>
       </c>
       <c r="K36" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="L36" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="M36" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="N36" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3700,13 +3703,13 @@
         <v>112</v>
       </c>
       <c r="F47" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="G47" s="0" t="s">
         <v>115</v>
       </c>
       <c r="H47" s="0" t="s">
-        <v>165</v>
+        <v>154</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3730,13 +3733,13 @@
         <v>112</v>
       </c>
       <c r="F48" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="G48" s="0" t="s">
         <v>115</v>
       </c>
       <c r="H48" s="0" t="s">
-        <v>165</v>
+        <v>154</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3913,13 +3916,13 @@
         <v>172</v>
       </c>
       <c r="K54" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L54" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="M54" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4363,7 +4366,7 @@
         <v>115</v>
       </c>
       <c r="I67" s="0" t="s">
-        <v>165</v>
+        <v>154</v>
       </c>
       <c r="J67" s="0" t="s">
         <v>114</v>
@@ -4410,22 +4413,22 @@
         <v>99</v>
       </c>
       <c r="E69" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F69" s="0" t="s">
         <v>134</v>
       </c>
       <c r="G69" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H69" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I69" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J69" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] [SW-3159] Quantize node in RN50 fails with --O0  - Quantize node in lib was assuming that input data is always float  - Changed source tensor to be templated, so it can be fp16 or float  - RN50 B1 INT8 quantize node unit test is now passing
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="598" uniqueCount="181">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -516,6 +516,30 @@
   </si>
   <si>
     <t xml:space="preserve">Int16QTy,Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int8QTy,FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UInt8QTy,FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int16QTy,FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32QTy,FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int8QTy,Float16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UInt8QTy,Float16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int16QTy,Float16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32QTy,Float16Ty</t>
   </si>
   <si>
     <t xml:space="preserve">UInt8QTy</t>
@@ -1680,8 +1704,8 @@
       <c r="C47" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="E47" s="0" t="n">
-        <v>0</v>
+      <c r="E47" s="0" t="s">
+        <v>13</v>
       </c>
       <c r="F47" s="0" t="s">
         <v>14</v>
@@ -3695,21 +3719,33 @@
         <f aca="false">LibManager!C47</f>
         <v>1</v>
       </c>
-      <c r="D47" s="0" t="n">
+      <c r="D47" s="0" t="str">
         <f aca="false">LibManager!E47</f>
-        <v>0</v>
+        <v>0,1</v>
       </c>
       <c r="E47" s="0" t="s">
-        <v>112</v>
+        <v>165</v>
       </c>
       <c r="F47" s="0" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G47" s="0" t="s">
-        <v>115</v>
+        <v>167</v>
       </c>
       <c r="H47" s="0" t="s">
-        <v>154</v>
+        <v>168</v>
+      </c>
+      <c r="I47" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="J47" s="0" t="s">
+        <v>170</v>
+      </c>
+      <c r="K47" s="0" t="s">
+        <v>171</v>
+      </c>
+      <c r="L47" s="0" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3733,7 +3769,7 @@
         <v>112</v>
       </c>
       <c r="F48" s="0" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="G48" s="0" t="s">
         <v>115</v>
@@ -3781,7 +3817,7 @@
         <v>142</v>
       </c>
       <c r="F50" s="0" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3898,22 +3934,22 @@
         <v>1,3</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="F54" s="0" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="G54" s="0" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="H54" s="0" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="I54" s="0" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="J54" s="0" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="K54" s="0" t="s">
         <v>156</v>

</xml_diff>

<commit_message>
[dnn-library] [SW-1561] Vectorized version of EmbeddingBag and cleanup of FRQSL*S.
Implemented threaded+vectorized version of Embedding Bag instruction.

Cleanup of the no longer required code for dual float32 and float16 output
for FusedRowwiseQuantizedSparseLengths[Weighted]Sum instructions.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="598" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="182">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -165,6 +165,9 @@
   </si>
   <si>
     <t xml:space="preserve">HasEndOffset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vectorized</t>
   </si>
   <si>
     <t xml:space="preserve">ExtractTensor</t>
@@ -1329,13 +1332,16 @@
       <c r="E29" s="0" t="n">
         <v>0</v>
       </c>
+      <c r="F29" s="0" t="s">
+        <v>48</v>
+      </c>
       <c r="G29" s="0" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B30" s="0" t="n">
         <v>1</v>
@@ -1344,7 +1350,7 @@
         <v>1</v>
       </c>
       <c r="D30" s="0" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E30" s="0" t="n">
         <v>1</v>
@@ -1358,7 +1364,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B31" s="0" t="n">
         <v>1</v>
@@ -1378,7 +1384,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B32" s="0" t="n">
         <v>1</v>
@@ -1398,7 +1404,7 @@
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B33" s="0" t="n">
         <v>1</v>
@@ -1410,7 +1416,7 @@
         <v>0</v>
       </c>
       <c r="F33" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G33" s="0" t="s">
         <v>8</v>
@@ -1418,7 +1424,7 @@
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B34" s="0" t="n">
         <v>1</v>
@@ -1438,7 +1444,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B35" s="0" t="n">
         <v>1</v>
@@ -1447,7 +1453,7 @@
         <v>2</v>
       </c>
       <c r="D35" s="0" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E35" s="0" t="s">
         <v>33</v>
@@ -1461,7 +1467,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B36" s="0" t="n">
         <v>2</v>
@@ -1470,7 +1476,7 @@
         <v>2</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F36" s="0" t="s">
         <v>14</v>
@@ -1481,7 +1487,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B37" s="0" t="n">
         <v>1</v>
@@ -1490,7 +1496,7 @@
         <v>1</v>
       </c>
       <c r="D37" s="0" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E37" s="0" t="n">
         <v>1</v>
@@ -1504,7 +1510,7 @@
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B38" s="0" t="n">
         <v>1</v>
@@ -1521,7 +1527,7 @@
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B39" s="0" t="n">
         <v>1</v>
@@ -1530,7 +1536,7 @@
         <v>2</v>
       </c>
       <c r="E39" s="0" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F39" s="0" t="s">
         <v>14</v>
@@ -1541,7 +1547,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B40" s="0" t="n">
         <v>1</v>
@@ -1561,7 +1567,7 @@
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B41" s="0" t="n">
         <v>1</v>
@@ -1581,7 +1587,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B42" s="0" t="n">
         <v>2</v>
@@ -1590,7 +1596,7 @@
         <v>1</v>
       </c>
       <c r="D42" s="0" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E42" s="0" t="n">
         <v>1</v>
@@ -1604,7 +1610,7 @@
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B43" s="0" t="n">
         <v>1</v>
@@ -1613,7 +1619,7 @@
         <v>2</v>
       </c>
       <c r="D43" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E43" s="0" t="n">
         <v>1</v>
@@ -1627,7 +1633,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B44" s="0" t="n">
         <v>1</v>
@@ -1650,7 +1656,7 @@
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B45" s="0" t="n">
         <v>1</v>
@@ -1659,13 +1665,13 @@
         <v>1</v>
       </c>
       <c r="D45" s="0" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E45" s="0" t="n">
         <v>1</v>
       </c>
       <c r="F45" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G45" s="0" t="s">
         <v>31</v>
@@ -1673,7 +1679,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B46" s="0" t="n">
         <v>1</v>
@@ -1682,7 +1688,7 @@
         <v>1</v>
       </c>
       <c r="D46" s="0" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E46" s="0" t="n">
         <v>1</v>
@@ -1696,7 +1702,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B47" s="0" t="n">
         <v>1</v>
@@ -1716,7 +1722,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B48" s="0" t="n">
         <v>1</v>
@@ -1736,7 +1742,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B49" s="0" t="n">
         <v>1</v>
@@ -1745,10 +1751,10 @@
         <v>5</v>
       </c>
       <c r="E49" s="0" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F49" s="0" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G49" s="0" t="s">
         <v>31</v>
@@ -1756,7 +1762,7 @@
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B50" s="0" t="n">
         <v>1</v>
@@ -1776,7 +1782,7 @@
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B51" s="0" t="n">
         <v>1</v>
@@ -1793,7 +1799,7 @@
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B52" s="0" t="n">
         <v>1</v>
@@ -1813,7 +1819,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B53" s="0" t="n">
         <v>1</v>
@@ -1833,7 +1839,7 @@
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B54" s="0" t="n">
         <v>1</v>
@@ -1842,10 +1848,10 @@
         <v>4</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F54" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G54" s="0" t="s">
         <v>8</v>
@@ -1853,7 +1859,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B55" s="0" t="n">
         <v>1</v>
@@ -1873,7 +1879,7 @@
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B56" s="0" t="n">
         <v>1</v>
@@ -1882,7 +1888,7 @@
         <v>4</v>
       </c>
       <c r="D56" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E56" s="0" t="n">
         <v>0</v>
@@ -1896,7 +1902,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="0" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B57" s="0" t="n">
         <v>1</v>
@@ -1905,7 +1911,7 @@
         <v>0</v>
       </c>
       <c r="D57" s="0" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E57" s="0" t="n">
         <v>0</v>
@@ -1919,7 +1925,7 @@
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B58" s="0" t="n">
         <v>1</v>
@@ -1928,7 +1934,7 @@
         <v>1</v>
       </c>
       <c r="D58" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E58" s="0" t="n">
         <v>1</v>
@@ -1939,7 +1945,7 @@
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B59" s="0" t="n">
         <v>1</v>
@@ -1959,7 +1965,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B60" s="0" t="n">
         <v>1</v>
@@ -1968,7 +1974,7 @@
         <v>1</v>
       </c>
       <c r="D60" s="0" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E60" s="0" t="n">
         <v>0</v>
@@ -1982,7 +1988,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B61" s="0" t="n">
         <v>2</v>
@@ -1991,7 +1997,7 @@
         <v>1</v>
       </c>
       <c r="D61" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E61" s="0" t="n">
         <v>2</v>
@@ -2005,7 +2011,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B62" s="0" t="n">
         <v>1</v>
@@ -2014,7 +2020,7 @@
         <v>1</v>
       </c>
       <c r="D62" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E62" s="0" t="n">
         <v>1</v>
@@ -2028,7 +2034,7 @@
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="0" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B63" s="0" t="n">
         <v>2</v>
@@ -2040,7 +2046,7 @@
         <v>12</v>
       </c>
       <c r="E63" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F63" s="0" t="s">
         <v>14</v>
@@ -2051,7 +2057,7 @@
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="0" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B64" s="0" t="n">
         <v>1</v>
@@ -2060,7 +2066,7 @@
         <v>1</v>
       </c>
       <c r="D64" s="0" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E64" s="0" t="n">
         <v>1</v>
@@ -2071,7 +2077,7 @@
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="0" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B65" s="0" t="n">
         <v>1</v>
@@ -2080,7 +2086,7 @@
         <v>1</v>
       </c>
       <c r="D65" s="0" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E65" s="0" t="n">
         <v>1</v>
@@ -2091,7 +2097,7 @@
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="0" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B66" s="0" t="n">
         <v>1</v>
@@ -2100,7 +2106,7 @@
         <v>1</v>
       </c>
       <c r="D66" s="0" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E66" s="0" t="n">
         <v>0</v>
@@ -2111,7 +2117,7 @@
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="0" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B67" s="0" t="n">
         <v>1</v>
@@ -2120,7 +2126,7 @@
         <v>1</v>
       </c>
       <c r="D67" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E67" s="0" t="n">
         <v>0</v>
@@ -2131,7 +2137,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B68" s="0" t="n">
         <v>1</v>
@@ -2148,7 +2154,7 @@
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B69" s="0" t="n">
         <v>1</v>
@@ -2157,10 +2163,10 @@
         <v>3</v>
       </c>
       <c r="E69" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F69" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G69" s="0" t="s">
         <v>8</v>
@@ -2236,22 +2242,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J2" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2272,22 +2278,22 @@
         <v>1</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J3" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2308,25 +2314,25 @@
         <v>0,1</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J4" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="K4" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2347,22 +2353,22 @@
         <v>0</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I5" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J5" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2383,22 +2389,22 @@
         <v>0,1,2</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="I6" s="0" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="J6" s="0" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2419,22 +2425,22 @@
         <v>1</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I7" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J7" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2455,22 +2461,22 @@
         <v>0</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I8" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J8" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2491,40 +2497,40 @@
         <v>0,1</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I9" s="0" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="J9" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="K9" s="0" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="L9" s="0" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="M9" s="0" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="N9" s="0" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="O9" s="0" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="P9" s="0" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2545,16 +2551,16 @@
         <v>0,1,2</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2575,22 +2581,22 @@
         <v>0</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F11" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I11" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J11" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2611,22 +2617,22 @@
         <v>0</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I12" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J12" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2647,22 +2653,22 @@
         <v>1</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F13" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I13" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J13" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2683,28 +2689,28 @@
         <v>0,1</v>
       </c>
       <c r="E14" s="0" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H14" s="0" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="I14" s="0" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="J14" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="K14" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="L14" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2725,19 +2731,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F15" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H15" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I15" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2758,19 +2764,19 @@
         <v>1,2</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F16" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H16" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I16" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2791,19 +2797,19 @@
         <v>1,2</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F17" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H17" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I17" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2824,19 +2830,19 @@
         <v>1,2</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G18" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H18" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I18" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2857,16 +2863,16 @@
         <v>0,1,2</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G19" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H19" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2887,10 +2893,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F20" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2911,10 +2917,10 @@
         <v>1</v>
       </c>
       <c r="E21" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F21" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2935,10 +2941,10 @@
         <v>0,1</v>
       </c>
       <c r="E22" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F22" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2959,19 +2965,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E23" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F23" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G23" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H23" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I23" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2992,19 +2998,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E24" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F24" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G24" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H24" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I24" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3025,19 +3031,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E25" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F25" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G25" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H25" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I25" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3058,10 +3064,10 @@
         <v>0,1,2</v>
       </c>
       <c r="E26" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F26" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3082,22 +3088,22 @@
         <v>0</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F27" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G27" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H27" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I27" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J27" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3118,19 +3124,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E28" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F28" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G28" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H28" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I28" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3151,10 +3157,10 @@
         <v>0</v>
       </c>
       <c r="E29" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F29" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3175,22 +3181,22 @@
         <v>1</v>
       </c>
       <c r="E30" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F30" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G30" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H30" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I30" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J30" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3211,25 +3217,25 @@
         <v>1</v>
       </c>
       <c r="E31" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F31" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G31" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H31" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I31" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J31" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K31" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3250,7 +3256,7 @@
         <v>0,1,2</v>
       </c>
       <c r="E32" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3271,10 +3277,10 @@
         <v>0</v>
       </c>
       <c r="E33" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F33" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3295,10 +3301,10 @@
         <v>0</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F34" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3319,34 +3325,34 @@
         <v>1,2</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F35" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G35" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H35" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="I35" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J35" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="K35" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="L35" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="M35" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="N35" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3367,34 +3373,34 @@
         <v>2,3</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F36" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G36" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H36" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="I36" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J36" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="K36" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="L36" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="M36" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="N36" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3415,22 +3421,22 @@
         <v>1</v>
       </c>
       <c r="E37" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F37" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G37" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H37" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I37" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J37" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3451,10 +3457,10 @@
         <v>1</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F38" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3493,22 +3499,22 @@
         <v>1</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F40" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G40" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H40" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I40" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J40" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3529,22 +3535,22 @@
         <v>1</v>
       </c>
       <c r="E41" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F41" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G41" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H41" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I41" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J41" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3565,10 +3571,10 @@
         <v>1</v>
       </c>
       <c r="E42" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F42" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3589,22 +3595,22 @@
         <v>1</v>
       </c>
       <c r="E43" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F43" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G43" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H43" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I43" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J43" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3625,25 +3631,25 @@
         <v>0,1</v>
       </c>
       <c r="E44" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F44" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G44" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H44" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I44" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J44" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="K44" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3664,22 +3670,22 @@
         <v>1</v>
       </c>
       <c r="E45" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F45" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G45" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H45" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I45" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J45" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3700,10 +3706,10 @@
         <v>1</v>
       </c>
       <c r="E46" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F46" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3724,28 +3730,28 @@
         <v>0,1</v>
       </c>
       <c r="E47" s="0" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F47" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G47" s="0" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H47" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I47" s="0" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J47" s="0" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K47" s="0" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="L47" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3766,16 +3772,16 @@
         <v>1</v>
       </c>
       <c r="E48" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F48" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="G48" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H48" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3814,10 +3820,10 @@
         <v>0,1</v>
       </c>
       <c r="E50" s="0" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F50" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3838,22 +3844,22 @@
         <v>0</v>
       </c>
       <c r="E51" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F51" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G51" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H51" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I51" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J51" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3874,10 +3880,10 @@
         <v>1</v>
       </c>
       <c r="E52" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F52" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3898,22 +3904,22 @@
         <v>1</v>
       </c>
       <c r="E53" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F53" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G53" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H53" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I53" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J53" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3934,31 +3940,31 @@
         <v>1,3</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F54" s="0" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="G54" s="0" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="H54" s="0" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I54" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J54" s="0" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K54" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="L54" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="M54" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3979,22 +3985,22 @@
         <v>0</v>
       </c>
       <c r="E55" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F55" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G55" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H55" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I55" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J55" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4015,22 +4021,22 @@
         <v>0</v>
       </c>
       <c r="E56" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F56" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G56" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H56" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I56" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J56" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4051,22 +4057,22 @@
         <v>0</v>
       </c>
       <c r="E57" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F57" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G57" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H57" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I57" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J57" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4087,22 +4093,22 @@
         <v>1</v>
       </c>
       <c r="E58" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F58" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G58" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H58" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I58" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J58" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4123,10 +4129,10 @@
         <v>1</v>
       </c>
       <c r="E59" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F59" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4147,22 +4153,22 @@
         <v>0</v>
       </c>
       <c r="E60" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F60" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G60" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H60" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I60" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J60" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4183,22 +4189,22 @@
         <v>2</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F61" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G61" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H61" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I61" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J61" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4219,22 +4225,22 @@
         <v>1</v>
       </c>
       <c r="E62" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F62" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G62" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H62" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I62" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J62" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4255,25 +4261,25 @@
         <v>0,2</v>
       </c>
       <c r="E63" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F63" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G63" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H63" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I63" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J63" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="K63" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4294,22 +4300,22 @@
         <v>1</v>
       </c>
       <c r="E64" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F64" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G64" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H64" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I64" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J64" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4330,16 +4336,16 @@
         <v>1</v>
       </c>
       <c r="E65" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F65" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G65" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="H65" s="0" t="s">
         <v>114</v>
-      </c>
-      <c r="H65" s="0" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4360,16 +4366,16 @@
         <v>0</v>
       </c>
       <c r="E66" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F66" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G66" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H66" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4390,25 +4396,25 @@
         <v>0</v>
       </c>
       <c r="E67" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F67" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G67" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H67" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="I67" s="0" t="s">
+        <v>155</v>
+      </c>
+      <c r="J67" s="0" t="s">
         <v>115</v>
       </c>
-      <c r="I67" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="J67" s="0" t="s">
+      <c r="K67" s="0" t="s">
         <v>114</v>
-      </c>
-      <c r="K67" s="0" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4429,7 +4435,7 @@
         <v>0</v>
       </c>
       <c r="E68" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4446,25 +4452,25 @@
         <v>3</v>
       </c>
       <c r="D69" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E69" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F69" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G69" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H69" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="I69" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J69" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] Make ConvertTo and EmbeddingBag operators fall back to single thread when destination tensor has untouchable padding attribute set
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -92,6 +92,9 @@
     <t xml:space="preserve">Threaded, Vectorized</t>
   </si>
   <si>
+    <t xml:space="preserve">custom</t>
+  </si>
+  <si>
     <t xml:space="preserve">Convolution</t>
   </si>
   <si>
@@ -114,9 +117,6 @@
   </si>
   <si>
     <t xml:space="preserve">ElementAdd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">custom</t>
   </si>
   <si>
     <t xml:space="preserve">ElementCmpEQ</t>
@@ -927,12 +927,12 @@
         <v>22</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>8</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B10" s="0" t="n">
         <v>1</v>
@@ -941,7 +941,7 @@
         <v>3</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E10" s="0" t="s">
         <v>17</v>
@@ -955,7 +955,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B11" s="0" t="n">
         <v>1</v>
@@ -964,7 +964,7 @@
         <v>3</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E11" s="0" t="n">
         <v>0</v>
@@ -978,7 +978,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B12" s="0" t="n">
         <v>1</v>
@@ -987,7 +987,7 @@
         <v>1</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E12" s="0" t="n">
         <v>0</v>
@@ -1001,7 +1001,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B13" s="0" t="n">
         <v>1</v>
@@ -1021,7 +1021,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B14" s="0" t="n">
         <v>1</v>
@@ -1041,7 +1041,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B15" s="0" t="n">
         <v>1</v>
@@ -1056,7 +1056,7 @@
         <v>22</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1076,7 +1076,7 @@
         <v>22</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1096,7 +1096,7 @@
         <v>22</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1116,7 +1116,7 @@
         <v>22</v>
       </c>
       <c r="G18" s="0" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1136,7 +1136,7 @@
         <v>22</v>
       </c>
       <c r="G19" s="0" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1213,7 +1213,7 @@
         <v>22</v>
       </c>
       <c r="G23" s="0" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1233,7 +1233,7 @@
         <v>22</v>
       </c>
       <c r="G24" s="0" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1253,7 +1253,7 @@
         <v>22</v>
       </c>
       <c r="G25" s="0" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1273,7 +1273,7 @@
         <v>22</v>
       </c>
       <c r="G26" s="0" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1313,7 +1313,7 @@
         <v>22</v>
       </c>
       <c r="G28" s="0" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1336,7 +1336,7 @@
         <v>48</v>
       </c>
       <c r="G29" s="0" t="s">
-        <v>8</v>
+        <v>23</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1674,7 +1674,7 @@
         <v>74</v>
       </c>
       <c r="G45" s="0" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1757,7 +1757,7 @@
         <v>80</v>
       </c>
       <c r="G49" s="0" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] [SW-3678] Lib Convolution quantized is not correctly getting bias numbers  - Bias was always consumed as float, but it might be int32 quantized and    is a template  - Updated the function to have the bias type as a template and created    and addresser instead of a regular array to read the bias  - Updated the lib spreadsheet to correctly send the new template and    updated the files generated automatically  - TensorTransformer was incorrectly dequantizing the tensors of int32    and storing the dequantize result as an int. It should simply copy    the original value coming from glow  - Moved bias in fully connected to be template instead of always float
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -5,12 +5,15 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
     <sheet name="Instances" sheetId="2" state="visible" r:id="rId3"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId4"/>
+  </externalReferences>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -21,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="187">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -101,6 +104,9 @@
     <t xml:space="preserve">Kernels, Strides, Pads, Group</t>
   </si>
   <si>
+    <t xml:space="preserve">0,1,2,3</t>
+  </si>
+  <si>
     <t xml:space="preserve">Convolution3D</t>
   </si>
   <si>
@@ -447,6 +453,18 @@
   </si>
   <si>
     <t xml:space="preserve">#Int64ITy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,FloatTy,FloatTy,FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,Float16Ty,Float16Ty,FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int8QTy,Int8QTy,Int8QTy,Int32QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int16QTy,Int16QTy,Int16QTy,Int32QTy</t>
   </si>
   <si>
     <t xml:space="preserve">FloatTy,Int8QTy</t>
@@ -729,6 +747,38 @@
 </styleSheet>
 </file>
 
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="LibManager"/>
+      <sheetName val="Instances"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="10">
+          <cell r="A10" t="str">
+            <v>Convolution</v>
+          </cell>
+          <cell r="B10">
+            <v>1</v>
+          </cell>
+          <cell r="C10">
+            <v>3</v>
+          </cell>
+        </row>
+        <row r="10">
+          <cell r="E10" t="str">
+            <v>0,1,2,3</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="1"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
@@ -930,7 +980,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
         <v>24</v>
       </c>
@@ -944,7 +994,7 @@
         <v>25</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="F10" s="0" t="s">
         <v>22</v>
@@ -955,7 +1005,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B11" s="0" t="n">
         <v>1</v>
@@ -978,7 +1028,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B12" s="0" t="n">
         <v>1</v>
@@ -987,7 +1037,7 @@
         <v>1</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E12" s="0" t="n">
         <v>0</v>
@@ -1001,7 +1051,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B13" s="0" t="n">
         <v>1</v>
@@ -1021,7 +1071,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B14" s="0" t="n">
         <v>1</v>
@@ -1041,7 +1091,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B15" s="0" t="n">
         <v>1</v>
@@ -1061,7 +1111,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B16" s="0" t="n">
         <v>1</v>
@@ -1070,7 +1120,7 @@
         <v>2</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F16" s="0" t="s">
         <v>22</v>
@@ -1081,16 +1131,16 @@
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="0" t="s">
         <v>34</v>
-      </c>
-      <c r="B17" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C17" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="E17" s="0" t="s">
-        <v>33</v>
       </c>
       <c r="F17" s="0" t="s">
         <v>22</v>
@@ -1101,7 +1151,7 @@
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B18" s="0" t="n">
         <v>1</v>
@@ -1110,7 +1160,7 @@
         <v>2</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F18" s="0" t="s">
         <v>22</v>
@@ -1121,7 +1171,7 @@
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B19" s="0" t="n">
         <v>1</v>
@@ -1141,7 +1191,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B20" s="0" t="n">
         <v>1</v>
@@ -1158,7 +1208,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B21" s="0" t="n">
         <v>1</v>
@@ -1178,7 +1228,7 @@
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B22" s="0" t="n">
         <v>1</v>
@@ -1198,7 +1248,7 @@
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B23" s="0" t="n">
         <v>1</v>
@@ -1218,7 +1268,7 @@
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B24" s="0" t="n">
         <v>1</v>
@@ -1238,7 +1288,7 @@
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B25" s="0" t="n">
         <v>1</v>
@@ -1258,7 +1308,7 @@
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B26" s="0" t="n">
         <v>1</v>
@@ -1278,7 +1328,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B27" s="0" t="n">
         <v>1</v>
@@ -1298,7 +1348,7 @@
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B28" s="0" t="n">
         <v>1</v>
@@ -1318,7 +1368,7 @@
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B29" s="0" t="n">
         <v>1</v>
@@ -1327,13 +1377,13 @@
         <v>4</v>
       </c>
       <c r="D29" s="0" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E29" s="0" t="n">
         <v>0</v>
       </c>
       <c r="F29" s="0" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G29" s="0" t="s">
         <v>23</v>
@@ -1341,7 +1391,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B30" s="0" t="n">
         <v>1</v>
@@ -1350,7 +1400,7 @@
         <v>1</v>
       </c>
       <c r="D30" s="0" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E30" s="0" t="n">
         <v>1</v>
@@ -1364,7 +1414,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B31" s="0" t="n">
         <v>1</v>
@@ -1384,7 +1434,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B32" s="0" t="n">
         <v>1</v>
@@ -1393,7 +1443,7 @@
         <v>3</v>
       </c>
       <c r="E32" s="0" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="F32" s="0" t="s">
         <v>22</v>
@@ -1404,7 +1454,7 @@
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B33" s="0" t="n">
         <v>1</v>
@@ -1416,7 +1466,7 @@
         <v>0</v>
       </c>
       <c r="F33" s="0" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G33" s="0" t="s">
         <v>8</v>
@@ -1424,7 +1474,7 @@
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B34" s="0" t="n">
         <v>1</v>
@@ -1444,7 +1494,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B35" s="0" t="n">
         <v>1</v>
@@ -1453,10 +1503,10 @@
         <v>2</v>
       </c>
       <c r="D35" s="0" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F35" s="0" t="s">
         <v>14</v>
@@ -1467,7 +1517,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B36" s="0" t="n">
         <v>2</v>
@@ -1476,7 +1526,7 @@
         <v>2</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F36" s="0" t="s">
         <v>14</v>
@@ -1487,7 +1537,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B37" s="0" t="n">
         <v>1</v>
@@ -1496,7 +1546,7 @@
         <v>1</v>
       </c>
       <c r="D37" s="0" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E37" s="0" t="n">
         <v>1</v>
@@ -1510,7 +1560,7 @@
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B38" s="0" t="n">
         <v>1</v>
@@ -1527,7 +1577,7 @@
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B39" s="0" t="n">
         <v>1</v>
@@ -1536,7 +1586,7 @@
         <v>2</v>
       </c>
       <c r="E39" s="0" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F39" s="0" t="s">
         <v>14</v>
@@ -1547,7 +1597,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B40" s="0" t="n">
         <v>1</v>
@@ -1567,7 +1617,7 @@
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B41" s="0" t="n">
         <v>1</v>
@@ -1587,7 +1637,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B42" s="0" t="n">
         <v>2</v>
@@ -1596,7 +1646,7 @@
         <v>1</v>
       </c>
       <c r="D42" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E42" s="0" t="n">
         <v>1</v>
@@ -1610,7 +1660,7 @@
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B43" s="0" t="n">
         <v>1</v>
@@ -1619,7 +1669,7 @@
         <v>2</v>
       </c>
       <c r="D43" s="0" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E43" s="0" t="n">
         <v>1</v>
@@ -1633,7 +1683,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B44" s="0" t="n">
         <v>1</v>
@@ -1656,7 +1706,7 @@
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B45" s="0" t="n">
         <v>1</v>
@@ -1665,13 +1715,13 @@
         <v>1</v>
       </c>
       <c r="D45" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E45" s="0" t="n">
         <v>1</v>
       </c>
       <c r="F45" s="0" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G45" s="0" t="s">
         <v>23</v>
@@ -1679,7 +1729,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B46" s="0" t="n">
         <v>1</v>
@@ -1688,7 +1738,7 @@
         <v>1</v>
       </c>
       <c r="D46" s="0" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E46" s="0" t="n">
         <v>1</v>
@@ -1702,7 +1752,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B47" s="0" t="n">
         <v>1</v>
@@ -1722,7 +1772,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B48" s="0" t="n">
         <v>1</v>
@@ -1742,7 +1792,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B49" s="0" t="n">
         <v>1</v>
@@ -1751,10 +1801,10 @@
         <v>5</v>
       </c>
       <c r="E49" s="0" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F49" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G49" s="0" t="s">
         <v>23</v>
@@ -1762,7 +1812,7 @@
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B50" s="0" t="n">
         <v>1</v>
@@ -1782,7 +1832,7 @@
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B51" s="0" t="n">
         <v>1</v>
@@ -1799,7 +1849,7 @@
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B52" s="0" t="n">
         <v>1</v>
@@ -1819,7 +1869,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B53" s="0" t="n">
         <v>1</v>
@@ -1839,7 +1889,7 @@
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B54" s="0" t="n">
         <v>1</v>
@@ -1848,10 +1898,10 @@
         <v>4</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F54" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G54" s="0" t="s">
         <v>8</v>
@@ -1859,7 +1909,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B55" s="0" t="n">
         <v>1</v>
@@ -1879,7 +1929,7 @@
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B56" s="0" t="n">
         <v>1</v>
@@ -1888,7 +1938,7 @@
         <v>4</v>
       </c>
       <c r="D56" s="0" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E56" s="0" t="n">
         <v>0</v>
@@ -1902,7 +1952,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="0" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B57" s="0" t="n">
         <v>1</v>
@@ -1911,7 +1961,7 @@
         <v>0</v>
       </c>
       <c r="D57" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E57" s="0" t="n">
         <v>0</v>
@@ -1925,7 +1975,7 @@
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B58" s="0" t="n">
         <v>1</v>
@@ -1934,7 +1984,7 @@
         <v>1</v>
       </c>
       <c r="D58" s="0" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E58" s="0" t="n">
         <v>1</v>
@@ -1945,7 +1995,7 @@
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B59" s="0" t="n">
         <v>1</v>
@@ -1965,7 +2015,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B60" s="0" t="n">
         <v>1</v>
@@ -1974,7 +2024,7 @@
         <v>1</v>
       </c>
       <c r="D60" s="0" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E60" s="0" t="n">
         <v>0</v>
@@ -1988,7 +2038,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B61" s="0" t="n">
         <v>2</v>
@@ -1997,7 +2047,7 @@
         <v>1</v>
       </c>
       <c r="D61" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E61" s="0" t="n">
         <v>2</v>
@@ -2011,7 +2061,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B62" s="0" t="n">
         <v>1</v>
@@ -2020,7 +2070,7 @@
         <v>1</v>
       </c>
       <c r="D62" s="0" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E62" s="0" t="n">
         <v>1</v>
@@ -2034,7 +2084,7 @@
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B63" s="0" t="n">
         <v>2</v>
@@ -2046,7 +2096,7 @@
         <v>12</v>
       </c>
       <c r="E63" s="0" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F63" s="0" t="s">
         <v>14</v>
@@ -2057,7 +2107,7 @@
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="0" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B64" s="0" t="n">
         <v>1</v>
@@ -2066,7 +2116,7 @@
         <v>1</v>
       </c>
       <c r="D64" s="0" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E64" s="0" t="n">
         <v>1</v>
@@ -2077,7 +2127,7 @@
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="0" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B65" s="0" t="n">
         <v>1</v>
@@ -2086,7 +2136,7 @@
         <v>1</v>
       </c>
       <c r="D65" s="0" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E65" s="0" t="n">
         <v>1</v>
@@ -2097,7 +2147,7 @@
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="0" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B66" s="0" t="n">
         <v>1</v>
@@ -2106,7 +2156,7 @@
         <v>1</v>
       </c>
       <c r="D66" s="0" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E66" s="0" t="n">
         <v>0</v>
@@ -2117,7 +2167,7 @@
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B67" s="0" t="n">
         <v>1</v>
@@ -2126,7 +2176,7 @@
         <v>1</v>
       </c>
       <c r="D67" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E67" s="0" t="n">
         <v>0</v>
@@ -2137,7 +2187,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B68" s="0" t="n">
         <v>1</v>
@@ -2154,7 +2204,7 @@
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B69" s="0" t="n">
         <v>1</v>
@@ -2163,10 +2213,10 @@
         <v>3</v>
       </c>
       <c r="E69" s="0" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F69" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G69" s="0" t="s">
         <v>8</v>
@@ -2242,22 +2292,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J2" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2278,22 +2328,22 @@
         <v>1</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J3" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2314,25 +2364,25 @@
         <v>0,1</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J4" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K4" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2353,22 +2403,22 @@
         <v>0</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I5" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J5" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2389,22 +2439,22 @@
         <v>0,1,2</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="I6" s="0" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J6" s="0" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2425,22 +2475,22 @@
         <v>1</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I7" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J7" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2461,22 +2511,22 @@
         <v>0</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I8" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J8" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2497,70 +2547,70 @@
         <v>0,1</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I9" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J9" s="0" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="K9" s="0" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="L9" s="0" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="M9" s="0" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="N9" s="0" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O9" s="0" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="P9" s="0" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="str">
-        <f aca="false">LibManager!A10</f>
+        <f aca="false">[1]LibManager!A10</f>
         <v>Convolution</v>
       </c>
       <c r="B10" s="0" t="n">
-        <f aca="false">LibManager!B10</f>
+        <f aca="false">[1]LibManager!B10</f>
         <v>1</v>
       </c>
       <c r="C10" s="0" t="n">
-        <f aca="false">LibManager!C10</f>
+        <f aca="false">[1]LibManager!C10</f>
         <v>3</v>
       </c>
       <c r="D10" s="0" t="str">
-        <f aca="false">LibManager!E10</f>
-        <v>0,1,2</v>
+        <f aca="false">[1]LibManager!E10</f>
+        <v>0,1,2,3</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>125</v>
+        <v>144</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>128</v>
+        <v>146</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2581,22 +2631,22 @@
         <v>0</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F11" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I11" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J11" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2617,22 +2667,22 @@
         <v>0</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I12" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J12" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2653,22 +2703,22 @@
         <v>1</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F13" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I13" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J13" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2689,28 +2739,28 @@
         <v>0,1</v>
       </c>
       <c r="E14" s="0" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="H14" s="0" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="I14" s="0" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="J14" s="0" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="K14" s="0" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="L14" s="0" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2731,19 +2781,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F15" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H15" s="0" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="I15" s="0" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2764,19 +2814,19 @@
         <v>1,2</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="F16" s="0" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H16" s="0" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="I16" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2797,19 +2847,19 @@
         <v>1,2</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="F17" s="0" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H17" s="0" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="I17" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2830,19 +2880,19 @@
         <v>1,2</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="G18" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H18" s="0" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="I18" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2863,16 +2913,16 @@
         <v>0,1,2</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G19" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H19" s="0" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2893,10 +2943,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F20" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2917,10 +2967,10 @@
         <v>1</v>
       </c>
       <c r="E21" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F21" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2941,10 +2991,10 @@
         <v>0,1</v>
       </c>
       <c r="E22" s="0" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="F22" s="0" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2965,19 +3015,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E23" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F23" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G23" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H23" s="0" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="I23" s="0" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2998,19 +3048,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E24" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F24" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G24" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H24" s="0" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="I24" s="0" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3031,19 +3081,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E25" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F25" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G25" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H25" s="0" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="I25" s="0" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3064,10 +3114,10 @@
         <v>0,1,2</v>
       </c>
       <c r="E26" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F26" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3088,22 +3138,22 @@
         <v>0</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F27" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G27" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H27" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I27" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J27" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3124,19 +3174,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E28" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F28" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G28" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H28" s="0" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="I28" s="0" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3157,10 +3207,10 @@
         <v>0</v>
       </c>
       <c r="E29" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F29" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3181,22 +3231,22 @@
         <v>1</v>
       </c>
       <c r="E30" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F30" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G30" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H30" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I30" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J30" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3217,25 +3267,25 @@
         <v>1</v>
       </c>
       <c r="E31" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F31" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G31" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H31" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I31" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J31" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="K31" s="0" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3253,10 +3303,10 @@
       </c>
       <c r="D32" s="0" t="str">
         <f aca="false">LibManager!E32</f>
-        <v>0,1,2</v>
+        <v>0,1,2,3</v>
       </c>
       <c r="E32" s="0" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3277,10 +3327,10 @@
         <v>0</v>
       </c>
       <c r="E33" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F33" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3301,10 +3351,10 @@
         <v>0</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F34" s="0" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3325,34 +3375,34 @@
         <v>1,2</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="F35" s="0" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="G35" s="0" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="H35" s="0" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="I35" s="0" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="J35" s="0" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="K35" s="0" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="L35" s="0" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="M35" s="0" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="N35" s="0" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3373,34 +3423,34 @@
         <v>2,3</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="F36" s="0" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="G36" s="0" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="H36" s="0" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="I36" s="0" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="J36" s="0" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="K36" s="0" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="L36" s="0" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="M36" s="0" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="N36" s="0" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3421,22 +3471,22 @@
         <v>1</v>
       </c>
       <c r="E37" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F37" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G37" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H37" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I37" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J37" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3457,10 +3507,10 @@
         <v>1</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F38" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3499,22 +3549,22 @@
         <v>1</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F40" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G40" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H40" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I40" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J40" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3535,22 +3585,22 @@
         <v>1</v>
       </c>
       <c r="E41" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F41" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G41" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H41" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I41" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J41" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3571,10 +3621,10 @@
         <v>1</v>
       </c>
       <c r="E42" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F42" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3595,22 +3645,22 @@
         <v>1</v>
       </c>
       <c r="E43" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F43" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G43" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H43" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I43" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J43" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3631,25 +3681,25 @@
         <v>0,1</v>
       </c>
       <c r="E44" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F44" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G44" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H44" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I44" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J44" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K44" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3670,22 +3720,22 @@
         <v>1</v>
       </c>
       <c r="E45" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F45" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G45" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H45" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I45" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J45" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3706,10 +3756,10 @@
         <v>1</v>
       </c>
       <c r="E46" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F46" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3730,28 +3780,28 @@
         <v>0,1</v>
       </c>
       <c r="E47" s="0" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="F47" s="0" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="G47" s="0" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="H47" s="0" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="I47" s="0" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="J47" s="0" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="K47" s="0" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="L47" s="0" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3772,16 +3822,16 @@
         <v>1</v>
       </c>
       <c r="E48" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F48" s="0" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="G48" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H48" s="0" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3820,10 +3870,10 @@
         <v>0,1</v>
       </c>
       <c r="E50" s="0" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="F50" s="0" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3844,22 +3894,22 @@
         <v>0</v>
       </c>
       <c r="E51" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F51" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G51" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H51" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I51" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J51" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3880,10 +3930,10 @@
         <v>1</v>
       </c>
       <c r="E52" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F52" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3904,22 +3954,22 @@
         <v>1</v>
       </c>
       <c r="E53" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F53" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G53" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H53" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I53" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J53" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3940,31 +3990,31 @@
         <v>1,3</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="F54" s="0" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="G54" s="0" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="H54" s="0" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="I54" s="0" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="J54" s="0" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="K54" s="0" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="L54" s="0" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="M54" s="0" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3985,22 +4035,22 @@
         <v>0</v>
       </c>
       <c r="E55" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F55" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G55" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H55" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I55" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J55" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4021,22 +4071,22 @@
         <v>0</v>
       </c>
       <c r="E56" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F56" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G56" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H56" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I56" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J56" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4057,22 +4107,22 @@
         <v>0</v>
       </c>
       <c r="E57" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F57" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G57" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H57" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I57" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J57" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4093,22 +4143,22 @@
         <v>1</v>
       </c>
       <c r="E58" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F58" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G58" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H58" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I58" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J58" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4129,10 +4179,10 @@
         <v>1</v>
       </c>
       <c r="E59" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F59" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4153,22 +4203,22 @@
         <v>0</v>
       </c>
       <c r="E60" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F60" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G60" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H60" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I60" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J60" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4189,22 +4239,22 @@
         <v>2</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F61" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G61" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H61" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I61" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J61" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4225,22 +4275,22 @@
         <v>1</v>
       </c>
       <c r="E62" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F62" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G62" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H62" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I62" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J62" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4261,25 +4311,25 @@
         <v>0,2</v>
       </c>
       <c r="E63" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F63" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G63" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H63" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I63" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J63" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K63" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4300,22 +4350,22 @@
         <v>1</v>
       </c>
       <c r="E64" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F64" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G64" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H64" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I64" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J64" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4336,16 +4386,16 @@
         <v>1</v>
       </c>
       <c r="E65" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F65" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G65" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="H65" s="0" t="s">
         <v>115</v>
-      </c>
-      <c r="H65" s="0" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4366,16 +4416,16 @@
         <v>0</v>
       </c>
       <c r="E66" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F66" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G66" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H66" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4396,25 +4446,25 @@
         <v>0</v>
       </c>
       <c r="E67" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F67" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G67" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H67" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="I67" s="0" t="s">
+        <v>160</v>
+      </c>
+      <c r="J67" s="0" t="s">
         <v>116</v>
       </c>
-      <c r="I67" s="0" t="s">
-        <v>155</v>
-      </c>
-      <c r="J67" s="0" t="s">
+      <c r="K67" s="0" t="s">
         <v>115</v>
-      </c>
-      <c r="K67" s="0" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4435,7 +4485,7 @@
         <v>0</v>
       </c>
       <c r="E68" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4452,25 +4502,25 @@
         <v>3</v>
       </c>
       <c r="D69" s="0" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E69" s="0" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="F69" s="0" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G69" s="0" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="H69" s="0" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="I69" s="0" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="J69" s="0" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] [SW-3726] Moving implementation selection logic for ConvertTo from libManager to lib itself
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -92,6 +92,9 @@
     <t xml:space="preserve">Threaded, Vectorized</t>
   </si>
   <si>
+    <t xml:space="preserve">custom</t>
+  </si>
+  <si>
     <t xml:space="preserve">Convolution</t>
   </si>
   <si>
@@ -114,9 +117,6 @@
   </si>
   <si>
     <t xml:space="preserve">ElementAdd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">custom</t>
   </si>
   <si>
     <t xml:space="preserve">ElementCmpEQ</t>
@@ -927,12 +927,12 @@
         <v>22</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>8</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B10" s="0" t="n">
         <v>1</v>
@@ -941,7 +941,7 @@
         <v>3</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E10" s="0" t="s">
         <v>17</v>
@@ -955,7 +955,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B11" s="0" t="n">
         <v>1</v>
@@ -964,7 +964,7 @@
         <v>3</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E11" s="0" t="n">
         <v>0</v>
@@ -978,7 +978,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B12" s="0" t="n">
         <v>1</v>
@@ -987,7 +987,7 @@
         <v>1</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E12" s="0" t="n">
         <v>0</v>
@@ -1001,7 +1001,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B13" s="0" t="n">
         <v>1</v>
@@ -1021,7 +1021,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B14" s="0" t="n">
         <v>1</v>
@@ -1041,7 +1041,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B15" s="0" t="n">
         <v>1</v>
@@ -1056,7 +1056,7 @@
         <v>22</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1076,7 +1076,7 @@
         <v>22</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1096,7 +1096,7 @@
         <v>22</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1116,7 +1116,7 @@
         <v>22</v>
       </c>
       <c r="G18" s="0" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1136,7 +1136,7 @@
         <v>22</v>
       </c>
       <c r="G19" s="0" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1213,7 +1213,7 @@
         <v>22</v>
       </c>
       <c r="G23" s="0" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1233,7 +1233,7 @@
         <v>22</v>
       </c>
       <c r="G24" s="0" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1253,7 +1253,7 @@
         <v>22</v>
       </c>
       <c r="G25" s="0" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1273,7 +1273,7 @@
         <v>22</v>
       </c>
       <c r="G26" s="0" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1313,7 +1313,7 @@
         <v>22</v>
       </c>
       <c r="G28" s="0" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1674,7 +1674,7 @@
         <v>74</v>
       </c>
       <c r="G45" s="0" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1757,7 +1757,7 @@
         <v>80</v>
       </c>
       <c r="G49" s="0" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] Add New Operators. SW-684 ConvertTo add all combinations. SW-817 Add ChannelwiseQuantizedConvolution operand. sw-1967 Add ConvTransposeInst  operand. SW-2863 ResizeBilinear. SW-1358 Convolution currently works with dilation parameter. SW-2340 Support for Int32ITy indices type.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="200">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -101,93 +101,99 @@
     <t xml:space="preserve">Convolution</t>
   </si>
   <si>
+    <t xml:space="preserve">Kernels, Strides, Pads, Group, Dilation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Convolution3D</t>
+  </si>
+  <si>
     <t xml:space="preserve">Kernels, Strides, Pads, Group</t>
   </si>
   <si>
+    <t xml:space="preserve">Copy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TensorsAligned</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CrossEntropyLoss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dequantize</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementAdd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementCmpEQ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementCmpLT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementCmpLTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementDiv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementExp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementIsNaN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementLog</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementMax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementMin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementMul</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementPow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementSelect</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementSub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EmbeddingBag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HasEndOffset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vectorized</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ExtractTensor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Offsets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FullyConnected</t>
+  </si>
+  <si>
     <t xml:space="preserve">0,1,2,3</t>
   </si>
   <si>
-    <t xml:space="preserve">Convolution3D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Copy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TensorsAligned</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CrossEntropyLoss</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dequantize</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementAdd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementCmpEQ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementCmpLT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementCmpLTE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementDiv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementExp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementIsNaN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementLog</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementMax</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementMin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementMul</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementPow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementSelect</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementSub</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EmbeddingBag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HasEndOffset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vectorized</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ExtractTensor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Offsets</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flip</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FullyConnected</t>
-  </si>
-  <si>
     <t xml:space="preserve">FusedRowwiseQuantizedSparseLengthsSum</t>
   </si>
   <si>
@@ -275,6 +281,9 @@
     <t xml:space="preserve">RowwiseQuantizedSparseLengthsWeightedSum</t>
   </si>
   <si>
+    <t xml:space="preserve">0,5</t>
+  </si>
+  <si>
     <t xml:space="preserve">ScatterData</t>
   </si>
   <si>
@@ -362,6 +371,21 @@
     <t xml:space="preserve">SparseLengthsSum</t>
   </si>
   <si>
+    <t xml:space="preserve">ResizeBilinear</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ChannelWiseQuantizedConvolution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ConvTranspose</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#NonMaxSuppression</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CenterPointBox, MaxOutputBoxesPerClass, IouThreshold, ScoreThreshold, IsTFVersion4</t>
+  </si>
+  <si>
     <t xml:space="preserve">FloatTy</t>
   </si>
   <si>
@@ -422,102 +446,123 @@
     <t xml:space="preserve">Float16Ty,FloatTy</t>
   </si>
   <si>
-    <t xml:space="preserve">#Float16Ty,Int32ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#Float16Ty,Int64ITy</t>
+    <t xml:space="preserve">Float16Ty,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,Int64ITy</t>
   </si>
   <si>
     <t xml:space="preserve">FloatTy,Float16Ty</t>
   </si>
   <si>
-    <t xml:space="preserve">#FloatTy,Int32ITy</t>
+    <t xml:space="preserve">FloatTy,Int32ITy</t>
   </si>
   <si>
     <t xml:space="preserve">FloatTy,Int64ITy</t>
   </si>
   <si>
-    <t xml:space="preserve">#Int32ITy,Float16Ty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#Int32ITy,FloatTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#Int32ITy,Int64ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#Int64ITy,Float16Ty</t>
+    <t xml:space="preserve">Int32ITy,Float16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32ITy,FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32ITy,Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int64ITy,Float16Ty</t>
   </si>
   <si>
     <t xml:space="preserve">Int64ITy,FloatTy</t>
   </si>
   <si>
-    <t xml:space="preserve">#Int64ITy,Int32ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FloatTy,FloatTy,FloatTy,FloatTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Float16Ty,Float16Ty,Float16Ty,FloatTy</t>
+    <t xml:space="preserve">Int64ITy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,BoolTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,BoolTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int64ITy,BoolTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32ITy,BoolTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BoolTy,FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BoolTy,Float16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BoolTy,Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BoolTy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BoolTy,BoolTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,Float16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int8QTy,Int32QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int16QTy,Int16QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int16QTy,Int32QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,Int8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,UInt8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,Int16QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,Int32QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,Int8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,UInt8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,Int16QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,Int32QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32ITy,Int32ITy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int64ITy,Int64ITy,Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32ITy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32QTy</t>
   </si>
   <si>
     <t xml:space="preserve">Int8QTy,Int8QTy,Int8QTy,Int32QTy</t>
   </si>
   <si>
-    <t xml:space="preserve">Int16QTy,Int16QTy,Int16QTy,Int32QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FloatTy,Int8QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FloatTy,UInt8QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FloatTy,Int16QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FloatTy,Int32QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Float16Ty,Int8QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Float16Ty,UInt8QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Float16Ty,Int16QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Float16Ty,Int32QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int32ITy,Int32ITy,Int32ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int64ITy,Int64ITy,Int64ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FloatTy,FloatTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Float16Ty,Float16Ty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int32ITy,Int32ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int32QTy</t>
-  </si>
-  <si>
     <t xml:space="preserve">#Float16Ty</t>
   </si>
   <si>
-    <t xml:space="preserve">FloatTy,Int32ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Float16Ty,Int32ITy</t>
-  </si>
-  <si>
     <t xml:space="preserve">Int8QTy,Int32ITy</t>
   </si>
   <si>
@@ -527,9 +572,6 @@
     <t xml:space="preserve">Int16QTy,Int32ITy</t>
   </si>
   <si>
-    <t xml:space="preserve">Float16Ty,Int64ITy</t>
-  </si>
-  <si>
     <t xml:space="preserve">Int8QTy,Int64ITy</t>
   </si>
   <si>
@@ -564,9 +606,6 @@
   </si>
   <si>
     <t xml:space="preserve">UInt8QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#Float16Ty,UInt8QTy</t>
   </si>
   <si>
     <t xml:space="preserve">FloatTy, Int64ITy</t>
@@ -767,11 +806,6 @@
             <v>3</v>
           </cell>
         </row>
-        <row r="10">
-          <cell r="E10" t="str">
-            <v>0,1,2,3</v>
-          </cell>
-        </row>
       </sheetData>
       <sheetData sheetId="1"/>
     </sheetDataSet>
@@ -790,7 +824,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.99"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="27.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="72.1"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11.64"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="51.19"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="7.87"/>
@@ -1014,7 +1048,7 @@
         <v>3</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E11" s="0" t="n">
         <v>0</v>
@@ -1028,7 +1062,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B12" s="0" t="n">
         <v>1</v>
@@ -1037,7 +1071,7 @@
         <v>1</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E12" s="0" t="n">
         <v>0</v>
@@ -1051,7 +1085,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B13" s="0" t="n">
         <v>1</v>
@@ -1071,7 +1105,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B14" s="0" t="n">
         <v>1</v>
@@ -1091,7 +1125,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B15" s="0" t="n">
         <v>1</v>
@@ -1111,7 +1145,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B16" s="0" t="n">
         <v>1</v>
@@ -1120,7 +1154,7 @@
         <v>2</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F16" s="0" t="s">
         <v>22</v>
@@ -1131,16 +1165,16 @@
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="0" t="s">
         <v>35</v>
-      </c>
-      <c r="B17" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C17" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="E17" s="0" t="s">
-        <v>34</v>
       </c>
       <c r="F17" s="0" t="s">
         <v>22</v>
@@ -1151,7 +1185,7 @@
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B18" s="0" t="n">
         <v>1</v>
@@ -1160,7 +1194,7 @@
         <v>2</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F18" s="0" t="s">
         <v>22</v>
@@ -1171,7 +1205,7 @@
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B19" s="0" t="n">
         <v>1</v>
@@ -1191,7 +1225,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B20" s="0" t="n">
         <v>1</v>
@@ -1208,7 +1242,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B21" s="0" t="n">
         <v>1</v>
@@ -1228,7 +1262,7 @@
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B22" s="0" t="n">
         <v>1</v>
@@ -1248,7 +1282,7 @@
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B23" s="0" t="n">
         <v>1</v>
@@ -1268,7 +1302,7 @@
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B24" s="0" t="n">
         <v>1</v>
@@ -1288,7 +1322,7 @@
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B25" s="0" t="n">
         <v>1</v>
@@ -1308,7 +1342,7 @@
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B26" s="0" t="n">
         <v>1</v>
@@ -1328,7 +1362,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B27" s="0" t="n">
         <v>1</v>
@@ -1348,7 +1382,7 @@
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B28" s="0" t="n">
         <v>1</v>
@@ -1368,7 +1402,7 @@
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B29" s="0" t="n">
         <v>1</v>
@@ -1377,13 +1411,13 @@
         <v>4</v>
       </c>
       <c r="D29" s="0" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E29" s="0" t="n">
         <v>0</v>
       </c>
       <c r="F29" s="0" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G29" s="0" t="s">
         <v>23</v>
@@ -1391,7 +1425,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B30" s="0" t="n">
         <v>1</v>
@@ -1400,7 +1434,7 @@
         <v>1</v>
       </c>
       <c r="D30" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E30" s="0" t="n">
         <v>1</v>
@@ -1414,7 +1448,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B31" s="0" t="n">
         <v>1</v>
@@ -1434,7 +1468,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B32" s="0" t="n">
         <v>1</v>
@@ -1443,7 +1477,7 @@
         <v>3</v>
       </c>
       <c r="E32" s="0" t="s">
-        <v>26</v>
+        <v>55</v>
       </c>
       <c r="F32" s="0" t="s">
         <v>22</v>
@@ -1454,7 +1488,7 @@
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B33" s="0" t="n">
         <v>1</v>
@@ -1466,7 +1500,7 @@
         <v>0</v>
       </c>
       <c r="F33" s="0" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="G33" s="0" t="s">
         <v>8</v>
@@ -1474,7 +1508,7 @@
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B34" s="0" t="n">
         <v>1</v>
@@ -1494,7 +1528,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B35" s="0" t="n">
         <v>1</v>
@@ -1503,10 +1537,10 @@
         <v>2</v>
       </c>
       <c r="D35" s="0" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F35" s="0" t="s">
         <v>14</v>
@@ -1517,7 +1551,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B36" s="0" t="n">
         <v>2</v>
@@ -1526,7 +1560,7 @@
         <v>2</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F36" s="0" t="s">
         <v>14</v>
@@ -1537,7 +1571,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B37" s="0" t="n">
         <v>1</v>
@@ -1546,7 +1580,7 @@
         <v>1</v>
       </c>
       <c r="D37" s="0" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E37" s="0" t="n">
         <v>1</v>
@@ -1560,7 +1594,7 @@
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B38" s="0" t="n">
         <v>1</v>
@@ -1577,7 +1611,7 @@
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B39" s="0" t="n">
         <v>1</v>
@@ -1586,7 +1620,7 @@
         <v>2</v>
       </c>
       <c r="E39" s="0" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F39" s="0" t="s">
         <v>14</v>
@@ -1597,7 +1631,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B40" s="0" t="n">
         <v>1</v>
@@ -1617,7 +1651,7 @@
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B41" s="0" t="n">
         <v>1</v>
@@ -1637,7 +1671,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B42" s="0" t="n">
         <v>2</v>
@@ -1646,7 +1680,7 @@
         <v>1</v>
       </c>
       <c r="D42" s="0" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E42" s="0" t="n">
         <v>1</v>
@@ -1660,7 +1694,7 @@
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B43" s="0" t="n">
         <v>1</v>
@@ -1669,7 +1703,7 @@
         <v>2</v>
       </c>
       <c r="D43" s="0" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E43" s="0" t="n">
         <v>1</v>
@@ -1683,7 +1717,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B44" s="0" t="n">
         <v>1</v>
@@ -1706,7 +1740,7 @@
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B45" s="0" t="n">
         <v>1</v>
@@ -1715,13 +1749,13 @@
         <v>1</v>
       </c>
       <c r="D45" s="0" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E45" s="0" t="n">
         <v>1</v>
       </c>
       <c r="F45" s="0" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G45" s="0" t="s">
         <v>23</v>
@@ -1729,7 +1763,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B46" s="0" t="n">
         <v>1</v>
@@ -1738,7 +1772,7 @@
         <v>1</v>
       </c>
       <c r="D46" s="0" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E46" s="0" t="n">
         <v>1</v>
@@ -1752,7 +1786,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B47" s="0" t="n">
         <v>1</v>
@@ -1772,7 +1806,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B48" s="0" t="n">
         <v>1</v>
@@ -1792,7 +1826,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B49" s="0" t="n">
         <v>1</v>
@@ -1801,10 +1835,10 @@
         <v>5</v>
       </c>
       <c r="E49" s="0" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F49" s="0" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="G49" s="0" t="s">
         <v>23</v>
@@ -1812,7 +1846,7 @@
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B50" s="0" t="n">
         <v>1</v>
@@ -1821,7 +1855,7 @@
         <v>6</v>
       </c>
       <c r="E50" s="0" t="s">
-        <v>13</v>
+        <v>85</v>
       </c>
       <c r="F50" s="0" t="s">
         <v>22</v>
@@ -1832,7 +1866,7 @@
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B51" s="0" t="n">
         <v>1</v>
@@ -1849,7 +1883,7 @@
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B52" s="0" t="n">
         <v>1</v>
@@ -1869,7 +1903,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B53" s="0" t="n">
         <v>1</v>
@@ -1889,7 +1923,7 @@
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B54" s="0" t="n">
         <v>1</v>
@@ -1898,10 +1932,10 @@
         <v>4</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="F54" s="0" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G54" s="0" t="s">
         <v>8</v>
@@ -1909,7 +1943,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B55" s="0" t="n">
         <v>1</v>
@@ -1929,7 +1963,7 @@
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="0" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B56" s="0" t="n">
         <v>1</v>
@@ -1938,7 +1972,7 @@
         <v>4</v>
       </c>
       <c r="D56" s="0" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="E56" s="0" t="n">
         <v>0</v>
@@ -1952,7 +1986,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="0" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B57" s="0" t="n">
         <v>1</v>
@@ -1961,7 +1995,7 @@
         <v>0</v>
       </c>
       <c r="D57" s="0" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E57" s="0" t="n">
         <v>0</v>
@@ -1975,7 +2009,7 @@
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B58" s="0" t="n">
         <v>1</v>
@@ -1984,7 +2018,7 @@
         <v>1</v>
       </c>
       <c r="D58" s="0" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E58" s="0" t="n">
         <v>1</v>
@@ -1995,7 +2029,7 @@
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B59" s="0" t="n">
         <v>1</v>
@@ -2015,7 +2049,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B60" s="0" t="n">
         <v>1</v>
@@ -2024,7 +2058,7 @@
         <v>1</v>
       </c>
       <c r="D60" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E60" s="0" t="n">
         <v>0</v>
@@ -2038,7 +2072,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B61" s="0" t="n">
         <v>2</v>
@@ -2047,7 +2081,7 @@
         <v>1</v>
       </c>
       <c r="D61" s="0" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="E61" s="0" t="n">
         <v>2</v>
@@ -2061,7 +2095,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="0" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B62" s="0" t="n">
         <v>1</v>
@@ -2070,7 +2104,7 @@
         <v>1</v>
       </c>
       <c r="D62" s="0" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="E62" s="0" t="n">
         <v>1</v>
@@ -2084,7 +2118,7 @@
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="0" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B63" s="0" t="n">
         <v>2</v>
@@ -2096,7 +2130,7 @@
         <v>12</v>
       </c>
       <c r="E63" s="0" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="F63" s="0" t="s">
         <v>14</v>
@@ -2107,7 +2141,7 @@
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="0" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B64" s="0" t="n">
         <v>1</v>
@@ -2116,7 +2150,7 @@
         <v>1</v>
       </c>
       <c r="D64" s="0" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="E64" s="0" t="n">
         <v>1</v>
@@ -2127,7 +2161,7 @@
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="0" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B65" s="0" t="n">
         <v>1</v>
@@ -2136,7 +2170,7 @@
         <v>1</v>
       </c>
       <c r="D65" s="0" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="E65" s="0" t="n">
         <v>1</v>
@@ -2147,7 +2181,7 @@
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="0" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B66" s="0" t="n">
         <v>1</v>
@@ -2156,7 +2190,7 @@
         <v>1</v>
       </c>
       <c r="D66" s="0" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="E66" s="0" t="n">
         <v>0</v>
@@ -2167,7 +2201,7 @@
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="0" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B67" s="0" t="n">
         <v>1</v>
@@ -2176,7 +2210,7 @@
         <v>1</v>
       </c>
       <c r="D67" s="0" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="E67" s="0" t="n">
         <v>0</v>
@@ -2187,7 +2221,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="0" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B68" s="0" t="n">
         <v>1</v>
@@ -2204,7 +2238,7 @@
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="0" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B69" s="0" t="n">
         <v>1</v>
@@ -2213,12 +2247,92 @@
         <v>3</v>
       </c>
       <c r="E69" s="0" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="F69" s="0" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G69" s="0" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="B70" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C70" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D70" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="E70" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" s="0" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="B71" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C71" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="D71" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="E71" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="G71" s="0" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="B72" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C72" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D72" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="E72" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G72" s="0" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="B73" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C73" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D73" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="E73" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" s="0" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2239,7 +2353,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P82"/>
+  <dimension ref="A1:Y82"/>
   <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.99"/>
@@ -2292,22 +2406,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J2" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2328,22 +2442,22 @@
         <v>1</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J3" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2364,25 +2478,25 @@
         <v>0,1</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="J4" s="0" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="K4" s="0" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2403,22 +2517,22 @@
         <v>0</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I5" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J5" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2439,22 +2553,22 @@
         <v>0,1,2</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="I6" s="0" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="J6" s="0" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2475,22 +2589,22 @@
         <v>1</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I7" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J7" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2511,22 +2625,22 @@
         <v>0</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I8" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J8" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2547,40 +2661,67 @@
         <v>0,1</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="I9" s="0" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="J9" s="0" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="K9" s="0" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="L9" s="0" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="M9" s="0" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="N9" s="0" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="O9" s="0" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="P9" s="0" t="s">
-        <v>142</v>
+        <v>150</v>
+      </c>
+      <c r="Q9" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="R9" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="S9" s="0" t="s">
+        <v>153</v>
+      </c>
+      <c r="T9" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="U9" s="0" t="s">
+        <v>155</v>
+      </c>
+      <c r="V9" s="0" t="s">
+        <v>156</v>
+      </c>
+      <c r="W9" s="0" t="s">
+        <v>157</v>
+      </c>
+      <c r="X9" s="0" t="s">
+        <v>158</v>
+      </c>
+      <c r="Y9" s="0" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2596,21 +2737,26 @@
         <f aca="false">[1]LibManager!C10</f>
         <v>3</v>
       </c>
-      <c r="D10" s="0" t="str">
-        <f aca="false">[1]LibManager!E10</f>
-        <v>0,1,2,3</v>
+      <c r="D10" s="0" t="s">
+        <v>26</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>143</v>
+        <v>160</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>144</v>
+        <v>161</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>145</v>
+        <v>128</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>146</v>
+        <v>162</v>
+      </c>
+      <c r="I10" s="0" t="s">
+        <v>163</v>
+      </c>
+      <c r="J10" s="0" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2631,22 +2777,22 @@
         <v>0</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F11" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I11" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J11" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2667,22 +2813,22 @@
         <v>0</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I12" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J12" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2703,22 +2849,22 @@
         <v>1</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F13" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I13" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J13" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2739,28 +2885,28 @@
         <v>0,1</v>
       </c>
       <c r="E14" s="0" t="s">
-        <v>147</v>
+        <v>165</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>148</v>
+        <v>166</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>149</v>
+        <v>167</v>
       </c>
       <c r="H14" s="0" t="s">
-        <v>150</v>
+        <v>168</v>
       </c>
       <c r="I14" s="0" t="s">
-        <v>151</v>
+        <v>169</v>
       </c>
       <c r="J14" s="0" t="s">
-        <v>152</v>
+        <v>170</v>
       </c>
       <c r="K14" s="0" t="s">
-        <v>153</v>
+        <v>171</v>
       </c>
       <c r="L14" s="0" t="s">
-        <v>154</v>
+        <v>172</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2781,19 +2927,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="F15" s="0" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="H15" s="0" t="s">
-        <v>155</v>
+        <v>173</v>
       </c>
       <c r="I15" s="0" t="s">
-        <v>156</v>
+        <v>174</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2814,19 +2960,19 @@
         <v>1,2</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="F16" s="0" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="H16" s="0" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
       <c r="I16" s="0" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2847,19 +2993,19 @@
         <v>1,2</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="F17" s="0" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="H17" s="0" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
       <c r="I17" s="0" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2880,19 +3026,19 @@
         <v>1,2</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="G18" s="0" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="H18" s="0" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
       <c r="I18" s="0" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2913,16 +3059,16 @@
         <v>0,1,2</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="G19" s="0" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="H19" s="0" t="s">
-        <v>156</v>
+        <v>174</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2943,10 +3089,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F20" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2967,10 +3113,10 @@
         <v>1</v>
       </c>
       <c r="E21" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F21" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2991,10 +3137,10 @@
         <v>0,1</v>
       </c>
       <c r="E22" s="0" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="F22" s="0" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3015,19 +3161,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E23" s="0" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="F23" s="0" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="G23" s="0" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="H23" s="0" t="s">
-        <v>155</v>
+        <v>173</v>
       </c>
       <c r="I23" s="0" t="s">
-        <v>156</v>
+        <v>174</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3048,19 +3194,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E24" s="0" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="F24" s="0" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="G24" s="0" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="H24" s="0" t="s">
-        <v>155</v>
+        <v>173</v>
       </c>
       <c r="I24" s="0" t="s">
-        <v>156</v>
+        <v>174</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3081,19 +3227,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E25" s="0" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="F25" s="0" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="G25" s="0" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="H25" s="0" t="s">
-        <v>155</v>
+        <v>173</v>
       </c>
       <c r="I25" s="0" t="s">
-        <v>156</v>
+        <v>174</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3114,10 +3260,10 @@
         <v>0,1,2</v>
       </c>
       <c r="E26" s="0" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="F26" s="0" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3138,22 +3284,22 @@
         <v>0</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F27" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G27" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H27" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I27" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J27" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3174,19 +3320,19 @@
         <v>0,1,2</v>
       </c>
       <c r="E28" s="0" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="F28" s="0" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="G28" s="0" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="H28" s="0" t="s">
-        <v>155</v>
+        <v>173</v>
       </c>
       <c r="I28" s="0" t="s">
-        <v>156</v>
+        <v>174</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3207,10 +3353,10 @@
         <v>0</v>
       </c>
       <c r="E29" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F29" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3231,22 +3377,22 @@
         <v>1</v>
       </c>
       <c r="E30" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F30" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G30" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H30" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I30" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J30" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3267,25 +3413,25 @@
         <v>1</v>
       </c>
       <c r="E31" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F31" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G31" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H31" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I31" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J31" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="K31" s="0" t="s">
-        <v>160</v>
+        <v>176</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3306,7 +3452,7 @@
         <v>0,1,2,3</v>
       </c>
       <c r="E32" s="0" t="s">
-        <v>145</v>
+        <v>177</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3327,10 +3473,10 @@
         <v>0</v>
       </c>
       <c r="E33" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F33" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3351,10 +3497,10 @@
         <v>0</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F34" s="0" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3375,34 +3521,34 @@
         <v>1,2</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>162</v>
+        <v>143</v>
       </c>
       <c r="F35" s="0" t="s">
-        <v>163</v>
+        <v>140</v>
       </c>
       <c r="G35" s="0" t="s">
-        <v>164</v>
+        <v>179</v>
       </c>
       <c r="H35" s="0" t="s">
-        <v>165</v>
+        <v>180</v>
       </c>
       <c r="I35" s="0" t="s">
-        <v>166</v>
+        <v>181</v>
       </c>
       <c r="J35" s="0" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="K35" s="0" t="s">
-        <v>167</v>
+        <v>141</v>
       </c>
       <c r="L35" s="0" t="s">
-        <v>168</v>
+        <v>182</v>
       </c>
       <c r="M35" s="0" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="N35" s="0" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3423,34 +3569,34 @@
         <v>2,3</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>162</v>
+        <v>143</v>
       </c>
       <c r="F36" s="0" t="s">
-        <v>163</v>
+        <v>140</v>
       </c>
       <c r="G36" s="0" t="s">
-        <v>164</v>
+        <v>179</v>
       </c>
       <c r="H36" s="0" t="s">
-        <v>165</v>
+        <v>180</v>
       </c>
       <c r="I36" s="0" t="s">
-        <v>166</v>
+        <v>181</v>
       </c>
       <c r="J36" s="0" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="K36" s="0" t="s">
-        <v>167</v>
+        <v>141</v>
       </c>
       <c r="L36" s="0" t="s">
-        <v>168</v>
+        <v>182</v>
       </c>
       <c r="M36" s="0" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="N36" s="0" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3471,22 +3617,22 @@
         <v>1</v>
       </c>
       <c r="E37" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F37" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G37" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H37" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I37" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J37" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3507,10 +3653,10 @@
         <v>1</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="F38" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3549,22 +3695,22 @@
         <v>1</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F40" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G40" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H40" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I40" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J40" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3585,22 +3731,22 @@
         <v>1</v>
       </c>
       <c r="E41" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F41" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G41" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H41" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I41" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J41" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3621,10 +3767,10 @@
         <v>1</v>
       </c>
       <c r="E42" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F42" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3645,22 +3791,22 @@
         <v>1</v>
       </c>
       <c r="E43" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F43" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G43" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H43" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I43" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J43" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3681,25 +3827,25 @@
         <v>0,1</v>
       </c>
       <c r="E44" s="0" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="F44" s="0" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="G44" s="0" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="H44" s="0" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="I44" s="0" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="J44" s="0" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="K44" s="0" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3720,22 +3866,22 @@
         <v>1</v>
       </c>
       <c r="E45" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F45" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G45" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H45" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I45" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J45" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3756,10 +3902,10 @@
         <v>1</v>
       </c>
       <c r="E46" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="F46" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3780,28 +3926,28 @@
         <v>0,1</v>
       </c>
       <c r="E47" s="0" t="s">
-        <v>171</v>
+        <v>185</v>
       </c>
       <c r="F47" s="0" t="s">
-        <v>172</v>
+        <v>186</v>
       </c>
       <c r="G47" s="0" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="H47" s="0" t="s">
-        <v>174</v>
+        <v>188</v>
       </c>
       <c r="I47" s="0" t="s">
-        <v>175</v>
+        <v>189</v>
       </c>
       <c r="J47" s="0" t="s">
-        <v>176</v>
+        <v>190</v>
       </c>
       <c r="K47" s="0" t="s">
-        <v>177</v>
+        <v>191</v>
       </c>
       <c r="L47" s="0" t="s">
-        <v>178</v>
+        <v>192</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3822,16 +3968,16 @@
         <v>1</v>
       </c>
       <c r="E48" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="F48" s="0" t="s">
-        <v>179</v>
+        <v>193</v>
       </c>
       <c r="G48" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="H48" s="0" t="s">
-        <v>160</v>
+        <v>176</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3867,13 +4013,19 @@
       </c>
       <c r="D50" s="0" t="str">
         <f aca="false">LibManager!E50</f>
-        <v>0,1</v>
+        <v>0,5</v>
       </c>
       <c r="E50" s="0" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="F50" s="0" t="s">
-        <v>180</v>
+        <v>144</v>
+      </c>
+      <c r="G50" s="0" t="s">
+        <v>140</v>
+      </c>
+      <c r="H50" s="0" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3894,22 +4046,22 @@
         <v>0</v>
       </c>
       <c r="E51" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F51" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G51" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H51" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I51" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J51" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3930,10 +4082,10 @@
         <v>1</v>
       </c>
       <c r="E52" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F52" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3954,22 +4106,22 @@
         <v>1</v>
       </c>
       <c r="E53" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F53" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G53" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H53" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I53" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J53" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3990,31 +4142,31 @@
         <v>1,3</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="F54" s="0" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="G54" s="0" t="s">
-        <v>183</v>
+        <v>196</v>
       </c>
       <c r="H54" s="0" t="s">
-        <v>184</v>
+        <v>197</v>
       </c>
       <c r="I54" s="0" t="s">
-        <v>185</v>
+        <v>198</v>
       </c>
       <c r="J54" s="0" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="K54" s="0" t="s">
-        <v>162</v>
+        <v>143</v>
       </c>
       <c r="L54" s="0" t="s">
-        <v>163</v>
+        <v>140</v>
       </c>
       <c r="M54" s="0" t="s">
-        <v>164</v>
+        <v>179</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4035,22 +4187,22 @@
         <v>0</v>
       </c>
       <c r="E55" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F55" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G55" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H55" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I55" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J55" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4071,22 +4223,22 @@
         <v>0</v>
       </c>
       <c r="E56" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F56" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G56" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H56" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I56" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J56" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4107,22 +4259,22 @@
         <v>0</v>
       </c>
       <c r="E57" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F57" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G57" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H57" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I57" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J57" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4143,22 +4295,22 @@
         <v>1</v>
       </c>
       <c r="E58" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F58" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G58" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H58" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I58" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J58" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4179,10 +4331,10 @@
         <v>1</v>
       </c>
       <c r="E59" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F59" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4203,22 +4355,22 @@
         <v>0</v>
       </c>
       <c r="E60" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F60" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G60" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H60" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I60" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J60" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4239,22 +4391,22 @@
         <v>2</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F61" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G61" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H61" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I61" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J61" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4275,22 +4427,22 @@
         <v>1</v>
       </c>
       <c r="E62" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F62" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G62" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H62" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I62" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J62" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4311,25 +4463,25 @@
         <v>0,2</v>
       </c>
       <c r="E63" s="0" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="F63" s="0" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="G63" s="0" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="H63" s="0" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="I63" s="0" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="J63" s="0" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="K63" s="0" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4350,22 +4502,22 @@
         <v>1</v>
       </c>
       <c r="E64" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F64" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G64" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H64" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I64" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J64" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4386,16 +4538,16 @@
         <v>1</v>
       </c>
       <c r="E65" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F65" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G65" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="H65" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4416,16 +4568,16 @@
         <v>0</v>
       </c>
       <c r="E66" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F66" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G66" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H66" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4446,25 +4598,25 @@
         <v>0</v>
       </c>
       <c r="E67" s="0" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F67" s="0" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G67" s="0" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H67" s="0" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="I67" s="0" t="s">
-        <v>160</v>
+        <v>176</v>
       </c>
       <c r="J67" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="K67" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4485,7 +4637,7 @@
         <v>0</v>
       </c>
       <c r="E68" s="0" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4502,97 +4654,133 @@
         <v>3</v>
       </c>
       <c r="D69" s="0" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="E69" s="0" t="s">
-        <v>162</v>
+        <v>143</v>
       </c>
       <c r="F69" s="0" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="G69" s="0" t="s">
-        <v>163</v>
+        <v>140</v>
       </c>
       <c r="H69" s="0" t="s">
-        <v>167</v>
+        <v>141</v>
       </c>
       <c r="I69" s="0" t="s">
-        <v>168</v>
+        <v>182</v>
       </c>
       <c r="J69" s="0" t="s">
-        <v>164</v>
+        <v>179</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="0" t="n">
+      <c r="A70" s="0" t="str">
         <f aca="false">LibManager!A70</f>
-        <v>0</v>
+        <v>ResizeBilinear</v>
       </c>
       <c r="B70" s="0" t="n">
         <f aca="false">LibManager!B70</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C70" s="0" t="n">
         <f aca="false">LibManager!C70</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D70" s="0" t="n">
         <f aca="false">LibManager!E70</f>
         <v>0</v>
       </c>
+      <c r="E70" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="F70" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="G70" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="H70" s="0" t="s">
+        <v>125</v>
+      </c>
+      <c r="I70" s="0" t="s">
+        <v>176</v>
+      </c>
+      <c r="J70" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="K70" s="0" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="0" t="n">
+      <c r="A71" s="0" t="str">
         <f aca="false">LibManager!A71</f>
-        <v>0</v>
+        <v>ChannelWiseQuantizedConvolution</v>
       </c>
       <c r="B71" s="0" t="n">
         <f aca="false">LibManager!B71</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C71" s="0" t="n">
         <f aca="false">LibManager!C71</f>
-        <v>0</v>
-      </c>
-      <c r="D71" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="D71" s="0" t="str">
         <f aca="false">LibManager!E71</f>
-        <v>0</v>
+        <v>0,3</v>
+      </c>
+      <c r="E71" s="0" t="s">
+        <v>128</v>
+      </c>
+      <c r="F71" s="0" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="0" t="n">
+      <c r="A72" s="0" t="str">
         <f aca="false">LibManager!A72</f>
-        <v>0</v>
+        <v>ConvTranspose</v>
       </c>
       <c r="B72" s="0" t="n">
         <f aca="false">LibManager!B72</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C72" s="0" t="n">
         <f aca="false">LibManager!C72</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D72" s="0" t="n">
         <f aca="false">LibManager!E72</f>
         <v>0</v>
       </c>
+      <c r="E72" s="0" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="0" t="n">
+      <c r="A73" s="0" t="str">
         <f aca="false">LibManager!A73</f>
-        <v>0</v>
+        <v>#NonMaxSuppression</v>
       </c>
       <c r="B73" s="0" t="n">
         <f aca="false">LibManager!B73</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C73" s="0" t="n">
         <f aca="false">LibManager!C73</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D73" s="0" t="n">
         <f aca="false">LibManager!E73</f>
         <v>0</v>
+      </c>
+      <c r="E73" s="0" t="s">
+        <v>146</v>
+      </c>
+      <c r="F73" s="0" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] Fix bug convolution doesn't support small features. Add bestImpl call at convolution.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -859,15 +859,15 @@
   <dimension ref="A1:K1048576"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="72.16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="32.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="7.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="7.8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="1" width="48.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="13.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="13.82"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="12" style="1" width="11.8"/>
   </cols>
   <sheetData>
@@ -1182,7 +1182,7 @@
         <v>34</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>22</v>

</xml_diff>

<commit_message>
[dnn-library] RWQSLS works only onn single-thread.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1028" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1028" uniqueCount="221">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -327,6 +327,9 @@
   </si>
   <si>
     <t xml:space="preserve">0,5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#Threaded, #Vectorized</t>
   </si>
   <si>
     <t xml:space="preserve">invalid,invalid,invalid,invalid,invalid,invalid,invalid</t>
@@ -2486,27 +2489,27 @@
         <v>101</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>34</v>
+        <v>102</v>
       </c>
       <c r="G50" s="1" t="s">
         <v>12</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="I50" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J50" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K50" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B51" s="1" t="n">
         <v>1</v>
@@ -2535,7 +2538,7 @@
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B52" s="1" t="n">
         <v>1</v>
@@ -2567,7 +2570,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B53" s="1" t="n">
         <v>1</v>
@@ -2599,7 +2602,7 @@
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B54" s="1" t="n">
         <v>1</v>
@@ -2608,10 +2611,10 @@
         <v>4</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G54" s="1" t="s">
         <v>12</v>
@@ -2631,7 +2634,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B55" s="1" t="n">
         <v>1</v>
@@ -2663,7 +2666,7 @@
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B56" s="1" t="n">
         <v>1</v>
@@ -2672,7 +2675,7 @@
         <v>4</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E56" s="1" t="n">
         <v>0</v>
@@ -2698,7 +2701,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B57" s="1" t="n">
         <v>1</v>
@@ -2733,7 +2736,7 @@
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B58" s="1" t="n">
         <v>1</v>
@@ -2742,7 +2745,7 @@
         <v>1</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E58" s="1" t="n">
         <v>1</v>
@@ -2765,7 +2768,7 @@
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B59" s="1" t="n">
         <v>1</v>
@@ -2797,7 +2800,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B60" s="1" t="n">
         <v>1</v>
@@ -2832,7 +2835,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B61" s="1" t="n">
         <v>2</v>
@@ -2841,7 +2844,7 @@
         <v>1</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E61" s="1" t="n">
         <v>2</v>
@@ -2867,7 +2870,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B62" s="1" t="n">
         <v>1</v>
@@ -2876,7 +2879,7 @@
         <v>1</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E62" s="1" t="n">
         <v>1</v>
@@ -2902,7 +2905,7 @@
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B63" s="1" t="n">
         <v>2</v>
@@ -2914,7 +2917,7 @@
         <v>18</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F63" s="1" t="s">
         <v>20</v>
@@ -2937,7 +2940,7 @@
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B64" s="1" t="n">
         <v>1</v>
@@ -2946,7 +2949,7 @@
         <v>1</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E64" s="1" t="n">
         <v>1</v>
@@ -2969,7 +2972,7 @@
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B65" s="1" t="n">
         <v>1</v>
@@ -2978,7 +2981,7 @@
         <v>1</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E65" s="1" t="n">
         <v>1</v>
@@ -3001,7 +3004,7 @@
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B66" s="1" t="n">
         <v>1</v>
@@ -3010,7 +3013,7 @@
         <v>1</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E66" s="1" t="n">
         <v>0</v>
@@ -3033,7 +3036,7 @@
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B67" s="1" t="n">
         <v>1</v>
@@ -3042,7 +3045,7 @@
         <v>1</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E67" s="1" t="n">
         <v>0</v>
@@ -3065,7 +3068,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B68" s="1" t="n">
         <v>1</v>
@@ -3094,7 +3097,7 @@
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B69" s="1" t="n">
         <v>1</v>
@@ -3103,10 +3106,10 @@
         <v>3</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G69" s="1" t="s">
         <v>12</v>
@@ -3126,7 +3129,7 @@
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B70" s="1" t="n">
         <v>1</v>
@@ -3135,7 +3138,7 @@
         <v>1</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E70" s="1" t="n">
         <v>0</v>
@@ -3158,7 +3161,7 @@
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B71" s="1" t="n">
         <v>1</v>
@@ -3176,21 +3179,21 @@
         <v>12</v>
       </c>
       <c r="H71" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I71" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J71" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="K71" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B72" s="1" t="n">
         <v>1</v>
@@ -3222,7 +3225,7 @@
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B73" s="1" t="n">
         <v>2</v>
@@ -3231,7 +3234,7 @@
         <v>2</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E73" s="1" t="n">
         <v>0</v>
@@ -3318,22 +3321,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3350,22 +3353,22 @@
         <v>1</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3382,25 +3385,25 @@
         <v>19</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3417,22 +3420,22 @@
         <v>0</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3449,22 +3452,22 @@
         <v>25</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3481,22 +3484,22 @@
         <v>1</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3513,22 +3516,22 @@
         <v>0</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3545,67 +3548,67 @@
         <v>19</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="R9" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="S9" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T9" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V9" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="W9" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="X9" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="Y9" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3622,22 +3625,22 @@
         <v>38</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3654,22 +3657,22 @@
         <v>0</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3686,22 +3689,22 @@
         <v>0</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3718,22 +3721,22 @@
         <v>1</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3750,28 +3753,28 @@
         <v>19</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3788,19 +3791,19 @@
         <v>25</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3817,19 +3820,19 @@
         <v>47</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3846,19 +3849,19 @@
         <v>47</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3875,19 +3878,19 @@
         <v>47</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3904,16 +3907,16 @@
         <v>25</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3930,10 +3933,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3950,10 +3953,10 @@
         <v>1</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3970,10 +3973,10 @@
         <v>19</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3990,19 +3993,19 @@
         <v>25</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4019,19 +4022,19 @@
         <v>25</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4048,19 +4051,19 @@
         <v>25</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4077,10 +4080,10 @@
         <v>25</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4097,22 +4100,22 @@
         <v>0</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4129,19 +4132,19 @@
         <v>25</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4158,10 +4161,10 @@
         <v>0</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4178,22 +4181,22 @@
         <v>1</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4210,25 +4213,25 @@
         <v>1</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4245,7 +4248,7 @@
         <v>69</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4262,10 +4265,10 @@
         <v>0</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4282,10 +4285,10 @@
         <v>0</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4302,34 +4305,34 @@
         <v>47</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="L35" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="M35" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4346,34 +4349,34 @@
         <v>76</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K36" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="L36" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="M36" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="N36" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4390,22 +4393,22 @@
         <v>1</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4422,10 +4425,10 @@
         <v>1</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4456,22 +4459,22 @@
         <v>1</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4488,22 +4491,22 @@
         <v>1</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J41" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4520,10 +4523,10 @@
         <v>1</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4540,22 +4543,22 @@
         <v>1</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4572,25 +4575,25 @@
         <v>19</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4607,22 +4610,22 @@
         <v>1</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I45" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4639,10 +4642,10 @@
         <v>1</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4659,28 +4662,28 @@
         <v>19</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I47" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="J47" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="K47" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="L47" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4697,16 +4700,16 @@
         <v>1</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4737,21 +4740,21 @@
         <v>101</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B51" s="1" t="n">
         <v>1</v>
@@ -4763,27 +4766,27 @@
         <v>0</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J51" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B52" s="1" t="n">
         <v>1</v>
@@ -4795,15 +4798,15 @@
         <v>1</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B53" s="1" t="n">
         <v>1</v>
@@ -4815,27 +4818,27 @@
         <v>1</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I53" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J53" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B54" s="1" t="n">
         <v>1</v>
@@ -4844,39 +4847,39 @@
         <v>4</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="I54" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J54" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="K54" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L54" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="M54" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B55" s="1" t="n">
         <v>1</v>
@@ -4888,27 +4891,27 @@
         <v>0</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I55" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J55" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B56" s="1" t="n">
         <v>1</v>
@@ -4920,27 +4923,27 @@
         <v>0</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I56" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J56" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B57" s="1" t="n">
         <v>1</v>
@@ -4952,27 +4955,27 @@
         <v>0</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I57" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J57" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B58" s="1" t="n">
         <v>1</v>
@@ -4984,27 +4987,27 @@
         <v>1</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J58" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B59" s="1" t="n">
         <v>1</v>
@@ -5016,15 +5019,15 @@
         <v>1</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B60" s="1" t="n">
         <v>1</v>
@@ -5036,27 +5039,27 @@
         <v>0</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I60" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J60" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B61" s="1" t="n">
         <v>2</v>
@@ -5068,27 +5071,27 @@
         <v>2</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I61" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J61" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B62" s="1" t="n">
         <v>1</v>
@@ -5100,27 +5103,27 @@
         <v>1</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I62" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J62" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B63" s="1" t="n">
         <v>2</v>
@@ -5129,33 +5132,33 @@
         <v>1</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I63" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="J63" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K63" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B64" s="1" t="n">
         <v>1</v>
@@ -5167,27 +5170,27 @@
         <v>1</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I64" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J64" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B65" s="1" t="n">
         <v>1</v>
@@ -5199,21 +5202,21 @@
         <v>1</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G65" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="H65" s="1" t="s">
         <v>144</v>
-      </c>
-      <c r="H65" s="1" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B66" s="1" t="n">
         <v>1</v>
@@ -5225,21 +5228,21 @@
         <v>0</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B67" s="1" t="n">
         <v>1</v>
@@ -5251,30 +5254,30 @@
         <v>0</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H67" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="I67" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="J67" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="I67" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="J67" s="1" t="s">
+      <c r="K67" s="1" t="s">
         <v>144</v>
-      </c>
-      <c r="K67" s="1" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B68" s="1" t="n">
         <v>1</v>
@@ -5286,12 +5289,12 @@
         <v>0</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B69" s="1" t="n">
         <v>1</v>
@@ -5300,30 +5303,30 @@
         <v>3</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="I69" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="J69" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B70" s="1" t="n">
         <v>1</v>
@@ -5335,30 +5338,30 @@
         <v>0</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G70" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H70" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="I70" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="J70" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="I70" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="J70" s="1" t="s">
+      <c r="K70" s="1" t="s">
         <v>144</v>
-      </c>
-      <c r="K70" s="1" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B71" s="1" t="n">
         <v>1</v>
@@ -5370,15 +5373,15 @@
         <v>38</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B72" s="1" t="n">
         <v>1</v>
@@ -5390,12 +5393,12 @@
         <v>0</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B73" s="1" t="n">
         <v>2</v>
@@ -5407,10 +5410,10 @@
         <v>0</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] Add bestImpl call at RowwiseQuantizedSparseLengthsWeightedSum.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1028" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1028" uniqueCount="220">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -327,9 +327,6 @@
   </si>
   <si>
     <t xml:space="preserve">0,5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#Threaded, #Vectorized</t>
   </si>
   <si>
     <t xml:space="preserve">invalid,invalid,invalid,invalid,invalid,invalid,invalid</t>
@@ -2489,27 +2486,27 @@
         <v>101</v>
       </c>
       <c r="F50" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G50" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="H50" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="G50" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="H50" s="1" t="s">
+      <c r="I50" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="J50" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="K50" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="I50" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="J50" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="K50" s="1" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B51" s="1" t="n">
         <v>1</v>
@@ -2538,7 +2535,7 @@
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B52" s="1" t="n">
         <v>1</v>
@@ -2570,7 +2567,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B53" s="1" t="n">
         <v>1</v>
@@ -2602,7 +2599,7 @@
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B54" s="1" t="n">
         <v>1</v>
@@ -2611,10 +2608,10 @@
         <v>4</v>
       </c>
       <c r="E54" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="F54" s="1" t="s">
         <v>109</v>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>110</v>
       </c>
       <c r="G54" s="1" t="s">
         <v>12</v>
@@ -2634,7 +2631,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B55" s="1" t="n">
         <v>1</v>
@@ -2666,7 +2663,7 @@
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B56" s="1" t="n">
         <v>1</v>
@@ -2675,7 +2672,7 @@
         <v>4</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E56" s="1" t="n">
         <v>0</v>
@@ -2701,7 +2698,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B57" s="1" t="n">
         <v>1</v>
@@ -2736,16 +2733,16 @@
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B58" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="B58" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C58" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>116</v>
       </c>
       <c r="E58" s="1" t="n">
         <v>1</v>
@@ -2768,7 +2765,7 @@
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B59" s="1" t="n">
         <v>1</v>
@@ -2800,7 +2797,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B60" s="1" t="n">
         <v>1</v>
@@ -2835,7 +2832,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B61" s="1" t="n">
         <v>2</v>
@@ -2844,7 +2841,7 @@
         <v>1</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E61" s="1" t="n">
         <v>2</v>
@@ -2870,16 +2867,16 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B62" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C62" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="B62" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C62" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D62" s="1" t="s">
-        <v>121</v>
       </c>
       <c r="E62" s="1" t="n">
         <v>1</v>
@@ -2905,7 +2902,7 @@
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B63" s="1" t="n">
         <v>2</v>
@@ -2917,7 +2914,7 @@
         <v>18</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F63" s="1" t="s">
         <v>20</v>
@@ -2940,16 +2937,16 @@
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B64" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C64" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" s="1" t="s">
         <v>124</v>
-      </c>
-      <c r="B64" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C64" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D64" s="1" t="s">
-        <v>125</v>
       </c>
       <c r="E64" s="1" t="n">
         <v>1</v>
@@ -2972,16 +2969,16 @@
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B65" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C65" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" s="1" t="s">
         <v>126</v>
-      </c>
-      <c r="B65" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C65" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D65" s="1" t="s">
-        <v>127</v>
       </c>
       <c r="E65" s="1" t="n">
         <v>1</v>
@@ -3004,16 +3001,16 @@
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B66" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C66" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="B66" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C66" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>129</v>
       </c>
       <c r="E66" s="1" t="n">
         <v>0</v>
@@ -3036,16 +3033,16 @@
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B67" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C67" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" s="1" t="s">
         <v>130</v>
-      </c>
-      <c r="B67" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C67" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D67" s="1" t="s">
-        <v>131</v>
       </c>
       <c r="E67" s="1" t="n">
         <v>0</v>
@@ -3068,7 +3065,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B68" s="1" t="n">
         <v>1</v>
@@ -3097,7 +3094,7 @@
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B69" s="1" t="n">
         <v>1</v>
@@ -3106,10 +3103,10 @@
         <v>3</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G69" s="1" t="s">
         <v>12</v>
@@ -3129,7 +3126,7 @@
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B70" s="1" t="n">
         <v>1</v>
@@ -3138,7 +3135,7 @@
         <v>1</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E70" s="1" t="n">
         <v>0</v>
@@ -3161,7 +3158,7 @@
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B71" s="1" t="n">
         <v>1</v>
@@ -3179,21 +3176,21 @@
         <v>12</v>
       </c>
       <c r="H71" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="I71" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="J71" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="K71" s="1" t="s">
         <v>136</v>
-      </c>
-      <c r="I71" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="J71" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="K71" s="1" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B72" s="1" t="n">
         <v>1</v>
@@ -3225,7 +3222,7 @@
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B73" s="1" t="n">
         <v>2</v>
@@ -3234,7 +3231,7 @@
         <v>2</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E73" s="1" t="n">
         <v>0</v>
@@ -3321,22 +3318,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3353,22 +3350,22 @@
         <v>1</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3385,25 +3382,25 @@
         <v>19</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="I4" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="J4" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="K4" s="1" t="s">
         <v>152</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3420,22 +3417,22 @@
         <v>0</v>
       </c>
       <c r="E5" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="I5" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="J5" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3452,22 +3449,22 @@
         <v>25</v>
       </c>
       <c r="E6" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="I6" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="J6" s="1" t="s">
         <v>158</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3484,22 +3481,22 @@
         <v>1</v>
       </c>
       <c r="E7" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="I7" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="J7" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3516,22 +3513,22 @@
         <v>0</v>
       </c>
       <c r="E8" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="H8" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="I8" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="J8" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3548,67 +3545,67 @@
         <v>19</v>
       </c>
       <c r="E9" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="H9" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="I9" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="J9" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="K9" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="K9" s="1" t="s">
+      <c r="L9" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="L9" s="1" t="s">
+      <c r="M9" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="M9" s="1" t="s">
+      <c r="N9" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="N9" s="1" t="s">
+      <c r="O9" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="O9" s="1" t="s">
+      <c r="P9" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="P9" s="1" t="s">
+      <c r="Q9" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="Q9" s="1" t="s">
+      <c r="R9" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="R9" s="1" t="s">
+      <c r="S9" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="S9" s="1" t="s">
+      <c r="T9" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="T9" s="1" t="s">
+      <c r="U9" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="U9" s="1" t="s">
+      <c r="V9" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="V9" s="1" t="s">
+      <c r="W9" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="W9" s="1" t="s">
+      <c r="X9" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="X9" s="1" t="s">
+      <c r="Y9" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="Y9" s="1" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3625,22 +3622,22 @@
         <v>38</v>
       </c>
       <c r="E10" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="H10" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="G10" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="H10" s="1" t="s">
+      <c r="I10" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="J10" s="1" t="s">
         <v>184</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3657,22 +3654,22 @@
         <v>0</v>
       </c>
       <c r="E11" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="H11" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="I11" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="J11" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3689,22 +3686,22 @@
         <v>0</v>
       </c>
       <c r="E12" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="H12" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H12" s="1" t="s">
+      <c r="I12" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I12" s="1" t="s">
+      <c r="J12" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3721,22 +3718,22 @@
         <v>1</v>
       </c>
       <c r="E13" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G13" s="1" t="s">
+      <c r="H13" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H13" s="1" t="s">
+      <c r="I13" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I13" s="1" t="s">
+      <c r="J13" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3753,28 +3750,28 @@
         <v>19</v>
       </c>
       <c r="E14" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="G14" s="1" t="s">
+      <c r="H14" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="I14" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="I14" s="1" t="s">
+      <c r="J14" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="J14" s="1" t="s">
+      <c r="K14" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="K14" s="1" t="s">
+      <c r="L14" s="1" t="s">
         <v>192</v>
-      </c>
-      <c r="L14" s="1" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3791,19 +3788,19 @@
         <v>25</v>
       </c>
       <c r="E15" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="G15" s="1" t="s">
-        <v>156</v>
-      </c>
       <c r="H15" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="I15" s="1" t="s">
         <v>194</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3820,19 +3817,19 @@
         <v>47</v>
       </c>
       <c r="E16" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="F16" s="1" t="s">
-        <v>182</v>
-      </c>
       <c r="G16" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3849,19 +3846,19 @@
         <v>47</v>
       </c>
       <c r="E17" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="F17" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="F17" s="1" t="s">
-        <v>182</v>
-      </c>
       <c r="G17" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3878,19 +3875,19 @@
         <v>47</v>
       </c>
       <c r="E18" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="F18" s="1" t="s">
-        <v>182</v>
-      </c>
       <c r="G18" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3907,16 +3904,16 @@
         <v>25</v>
       </c>
       <c r="E19" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="G19" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="G19" s="1" t="s">
-        <v>156</v>
-      </c>
       <c r="H19" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3933,10 +3930,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>141</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3953,10 +3950,10 @@
         <v>1</v>
       </c>
       <c r="E21" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>141</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3973,10 +3970,10 @@
         <v>19</v>
       </c>
       <c r="E22" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>181</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3993,19 +3990,19 @@
         <v>25</v>
       </c>
       <c r="E23" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="F23" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="F23" s="1" t="s">
+      <c r="G23" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="G23" s="1" t="s">
-        <v>156</v>
-      </c>
       <c r="H23" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="I23" s="1" t="s">
         <v>194</v>
-      </c>
-      <c r="I23" s="1" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4022,19 +4019,19 @@
         <v>25</v>
       </c>
       <c r="E24" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="F24" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="F24" s="1" t="s">
+      <c r="G24" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="G24" s="1" t="s">
-        <v>156</v>
-      </c>
       <c r="H24" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="I24" s="1" t="s">
         <v>194</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4051,19 +4048,19 @@
         <v>25</v>
       </c>
       <c r="E25" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="F25" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="F25" s="1" t="s">
+      <c r="G25" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="G25" s="1" t="s">
-        <v>156</v>
-      </c>
       <c r="H25" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="I25" s="1" t="s">
         <v>194</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4080,10 +4077,10 @@
         <v>25</v>
       </c>
       <c r="E26" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="F26" s="1" t="s">
         <v>154</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4100,22 +4097,22 @@
         <v>0</v>
       </c>
       <c r="E27" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F27" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F27" s="1" t="s">
+      <c r="G27" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G27" s="1" t="s">
+      <c r="H27" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H27" s="1" t="s">
+      <c r="I27" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I27" s="1" t="s">
+      <c r="J27" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="J27" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4132,19 +4129,19 @@
         <v>25</v>
       </c>
       <c r="E28" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="F28" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="G28" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="G28" s="1" t="s">
-        <v>156</v>
-      </c>
       <c r="H28" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="I28" s="1" t="s">
         <v>194</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4161,10 +4158,10 @@
         <v>0</v>
       </c>
       <c r="E29" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F29" s="1" t="s">
         <v>141</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4181,22 +4178,22 @@
         <v>1</v>
       </c>
       <c r="E30" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F30" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="G30" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G30" s="1" t="s">
+      <c r="H30" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H30" s="1" t="s">
+      <c r="I30" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I30" s="1" t="s">
+      <c r="J30" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="J30" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4213,25 +4210,25 @@
         <v>1</v>
       </c>
       <c r="E31" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F31" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F31" s="1" t="s">
+      <c r="G31" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G31" s="1" t="s">
+      <c r="H31" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H31" s="1" t="s">
+      <c r="I31" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I31" s="1" t="s">
+      <c r="J31" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="J31" s="1" t="s">
-        <v>146</v>
-      </c>
       <c r="K31" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4248,7 +4245,7 @@
         <v>69</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4265,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="E33" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F33" s="1" t="s">
         <v>141</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4285,10 +4282,10 @@
         <v>0</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4305,34 +4302,34 @@
         <v>47</v>
       </c>
       <c r="E35" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="J35" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="F35" s="1" t="s">
+      <c r="K35" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="G35" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="H35" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="I35" s="1" t="s">
+      <c r="L35" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="J35" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="K35" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="L35" s="1" t="s">
+      <c r="M35" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="M35" s="1" t="s">
+      <c r="N35" s="1" t="s">
         <v>204</v>
-      </c>
-      <c r="N35" s="1" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4349,34 +4346,34 @@
         <v>76</v>
       </c>
       <c r="E36" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="J36" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="F36" s="1" t="s">
+      <c r="K36" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="G36" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="H36" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="I36" s="1" t="s">
+      <c r="L36" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="J36" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="K36" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="L36" s="1" t="s">
+      <c r="M36" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="M36" s="1" t="s">
+      <c r="N36" s="1" t="s">
         <v>204</v>
-      </c>
-      <c r="N36" s="1" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4393,22 +4390,22 @@
         <v>1</v>
       </c>
       <c r="E37" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F37" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F37" s="1" t="s">
+      <c r="G37" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G37" s="1" t="s">
+      <c r="H37" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H37" s="1" t="s">
+      <c r="I37" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I37" s="1" t="s">
+      <c r="J37" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="J37" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4425,10 +4422,10 @@
         <v>1</v>
       </c>
       <c r="E38" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F38" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4459,22 +4456,22 @@
         <v>1</v>
       </c>
       <c r="E40" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F40" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F40" s="1" t="s">
+      <c r="G40" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G40" s="1" t="s">
+      <c r="H40" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H40" s="1" t="s">
+      <c r="I40" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I40" s="1" t="s">
+      <c r="J40" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="J40" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4491,22 +4488,22 @@
         <v>1</v>
       </c>
       <c r="E41" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F41" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F41" s="1" t="s">
+      <c r="G41" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G41" s="1" t="s">
+      <c r="H41" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H41" s="1" t="s">
+      <c r="I41" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I41" s="1" t="s">
+      <c r="J41" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="J41" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4523,10 +4520,10 @@
         <v>1</v>
       </c>
       <c r="E42" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F42" s="1" t="s">
         <v>141</v>
-      </c>
-      <c r="F42" s="1" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4543,22 +4540,22 @@
         <v>1</v>
       </c>
       <c r="E43" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F43" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F43" s="1" t="s">
+      <c r="G43" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G43" s="1" t="s">
+      <c r="H43" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H43" s="1" t="s">
+      <c r="I43" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I43" s="1" t="s">
+      <c r="J43" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="J43" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4575,25 +4572,25 @@
         <v>19</v>
       </c>
       <c r="E44" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="F44" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="F44" s="1" t="s">
+      <c r="G44" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="G44" s="1" t="s">
+      <c r="H44" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="H44" s="1" t="s">
+      <c r="I44" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="I44" s="1" t="s">
+      <c r="J44" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="J44" s="1" t="s">
+      <c r="K44" s="1" t="s">
         <v>152</v>
-      </c>
-      <c r="K44" s="1" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4610,22 +4607,22 @@
         <v>1</v>
       </c>
       <c r="E45" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F45" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F45" s="1" t="s">
+      <c r="G45" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G45" s="1" t="s">
+      <c r="H45" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H45" s="1" t="s">
+      <c r="I45" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I45" s="1" t="s">
+      <c r="J45" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="J45" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4642,10 +4639,10 @@
         <v>1</v>
       </c>
       <c r="E46" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="F46" s="1" t="s">
         <v>144</v>
-      </c>
-      <c r="F46" s="1" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4662,28 +4659,28 @@
         <v>19</v>
       </c>
       <c r="E47" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="F47" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="F47" s="1" t="s">
+      <c r="G47" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="G47" s="1" t="s">
+      <c r="H47" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="H47" s="1" t="s">
+      <c r="I47" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I47" s="1" t="s">
+      <c r="J47" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="J47" s="1" t="s">
+      <c r="K47" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="K47" s="1" t="s">
+      <c r="L47" s="1" t="s">
         <v>212</v>
-      </c>
-      <c r="L47" s="1" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4700,16 +4697,16 @@
         <v>1</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4740,21 +4737,21 @@
         <v>101</v>
       </c>
       <c r="E50" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="F50" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="F50" s="1" t="s">
-        <v>165</v>
-      </c>
       <c r="G50" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="H50" s="1" t="s">
         <v>161</v>
-      </c>
-      <c r="H50" s="1" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B51" s="1" t="n">
         <v>1</v>
@@ -4766,27 +4763,27 @@
         <v>0</v>
       </c>
       <c r="E51" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F51" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F51" s="1" t="s">
+      <c r="G51" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G51" s="1" t="s">
+      <c r="H51" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H51" s="1" t="s">
+      <c r="I51" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I51" s="1" t="s">
+      <c r="J51" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="J51" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B52" s="1" t="n">
         <v>1</v>
@@ -4798,15 +4795,15 @@
         <v>1</v>
       </c>
       <c r="E52" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F52" s="1" t="s">
         <v>141</v>
-      </c>
-      <c r="F52" s="1" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B53" s="1" t="n">
         <v>1</v>
@@ -4818,27 +4815,27 @@
         <v>1</v>
       </c>
       <c r="E53" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F53" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F53" s="1" t="s">
+      <c r="G53" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G53" s="1" t="s">
+      <c r="H53" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H53" s="1" t="s">
+      <c r="I53" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I53" s="1" t="s">
+      <c r="J53" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="J53" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B54" s="1" t="n">
         <v>1</v>
@@ -4847,39 +4844,39 @@
         <v>4</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E54" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="F54" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="F54" s="1" t="s">
+      <c r="G54" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="G54" s="1" t="s">
+      <c r="H54" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="H54" s="1" t="s">
+      <c r="I54" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="I54" s="1" t="s">
+      <c r="J54" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="J54" s="1" t="s">
-        <v>220</v>
-      </c>
       <c r="K54" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="L54" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="M54" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B55" s="1" t="n">
         <v>1</v>
@@ -4891,27 +4888,27 @@
         <v>0</v>
       </c>
       <c r="E55" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F55" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F55" s="1" t="s">
+      <c r="G55" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G55" s="1" t="s">
+      <c r="H55" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H55" s="1" t="s">
+      <c r="I55" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I55" s="1" t="s">
+      <c r="J55" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="J55" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B56" s="1" t="n">
         <v>1</v>
@@ -4923,27 +4920,27 @@
         <v>0</v>
       </c>
       <c r="E56" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F56" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F56" s="1" t="s">
+      <c r="G56" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G56" s="1" t="s">
+      <c r="H56" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H56" s="1" t="s">
+      <c r="I56" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I56" s="1" t="s">
+      <c r="J56" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="J56" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B57" s="1" t="n">
         <v>1</v>
@@ -4955,27 +4952,27 @@
         <v>0</v>
       </c>
       <c r="E57" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F57" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F57" s="1" t="s">
+      <c r="G57" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G57" s="1" t="s">
+      <c r="H57" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H57" s="1" t="s">
+      <c r="I57" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I57" s="1" t="s">
+      <c r="J57" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="J57" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B58" s="1" t="n">
         <v>1</v>
@@ -4987,27 +4984,27 @@
         <v>1</v>
       </c>
       <c r="E58" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F58" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F58" s="1" t="s">
+      <c r="G58" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G58" s="1" t="s">
+      <c r="H58" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H58" s="1" t="s">
+      <c r="I58" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I58" s="1" t="s">
+      <c r="J58" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="J58" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B59" s="1" t="n">
         <v>1</v>
@@ -5019,15 +5016,15 @@
         <v>1</v>
       </c>
       <c r="E59" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F59" s="1" t="s">
         <v>141</v>
-      </c>
-      <c r="F59" s="1" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B60" s="1" t="n">
         <v>1</v>
@@ -5039,27 +5036,27 @@
         <v>0</v>
       </c>
       <c r="E60" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F60" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F60" s="1" t="s">
+      <c r="G60" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G60" s="1" t="s">
+      <c r="H60" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H60" s="1" t="s">
+      <c r="I60" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I60" s="1" t="s">
+      <c r="J60" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="J60" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B61" s="1" t="n">
         <v>2</v>
@@ -5071,27 +5068,27 @@
         <v>2</v>
       </c>
       <c r="E61" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F61" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F61" s="1" t="s">
+      <c r="G61" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G61" s="1" t="s">
+      <c r="H61" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H61" s="1" t="s">
+      <c r="I61" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I61" s="1" t="s">
+      <c r="J61" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="J61" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B62" s="1" t="n">
         <v>1</v>
@@ -5103,27 +5100,27 @@
         <v>1</v>
       </c>
       <c r="E62" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F62" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F62" s="1" t="s">
+      <c r="G62" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G62" s="1" t="s">
+      <c r="H62" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H62" s="1" t="s">
+      <c r="I62" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I62" s="1" t="s">
+      <c r="J62" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="J62" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B63" s="1" t="n">
         <v>2</v>
@@ -5132,33 +5129,33 @@
         <v>1</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E63" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="F63" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="F63" s="1" t="s">
+      <c r="G63" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="G63" s="1" t="s">
+      <c r="H63" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="H63" s="1" t="s">
+      <c r="I63" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="I63" s="1" t="s">
+      <c r="J63" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="J63" s="1" t="s">
+      <c r="K63" s="1" t="s">
         <v>152</v>
-      </c>
-      <c r="K63" s="1" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B64" s="1" t="n">
         <v>1</v>
@@ -5170,27 +5167,27 @@
         <v>1</v>
       </c>
       <c r="E64" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F64" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F64" s="1" t="s">
+      <c r="G64" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G64" s="1" t="s">
+      <c r="H64" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H64" s="1" t="s">
+      <c r="I64" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="I64" s="1" t="s">
+      <c r="J64" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="J64" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B65" s="1" t="n">
         <v>1</v>
@@ -5202,21 +5199,21 @@
         <v>1</v>
       </c>
       <c r="E65" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F65" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F65" s="1" t="s">
-        <v>142</v>
-      </c>
       <c r="G65" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B66" s="1" t="n">
         <v>1</v>
@@ -5228,21 +5225,21 @@
         <v>0</v>
       </c>
       <c r="E66" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F66" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F66" s="1" t="s">
+      <c r="G66" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G66" s="1" t="s">
+      <c r="H66" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="H66" s="1" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B67" s="1" t="n">
         <v>1</v>
@@ -5254,30 +5251,30 @@
         <v>0</v>
       </c>
       <c r="E67" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F67" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F67" s="1" t="s">
+      <c r="G67" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G67" s="1" t="s">
+      <c r="H67" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="I67" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="J67" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="K67" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="H67" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="I67" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="J67" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="K67" s="1" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B68" s="1" t="n">
         <v>1</v>
@@ -5289,12 +5286,12 @@
         <v>0</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B69" s="1" t="n">
         <v>1</v>
@@ -5303,30 +5300,30 @@
         <v>3</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E69" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="F69" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="F69" s="1" t="s">
-        <v>165</v>
-      </c>
       <c r="G69" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="H69" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="H69" s="1" t="s">
-        <v>162</v>
-      </c>
       <c r="I69" s="1" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="J69" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B70" s="1" t="n">
         <v>1</v>
@@ -5338,30 +5335,30 @@
         <v>0</v>
       </c>
       <c r="E70" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F70" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F70" s="1" t="s">
+      <c r="G70" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G70" s="1" t="s">
+      <c r="H70" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="I70" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="J70" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="K70" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="H70" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="I70" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="J70" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="K70" s="1" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B71" s="1" t="n">
         <v>1</v>
@@ -5373,15 +5370,15 @@
         <v>38</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B72" s="1" t="n">
         <v>1</v>
@@ -5393,12 +5390,12 @@
         <v>0</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B73" s="1" t="n">
         <v>2</v>
@@ -5410,10 +5407,10 @@
         <v>0</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] [SW-3241] Add LIB Constraints phase - add graph phase to add constraints for lib   with lowest pririty compared to Graph and Jit - gather Lib Copy implementations - customize lib dispatch
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="736" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="200">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -113,7 +113,7 @@
     <t xml:space="preserve">Copy</t>
   </si>
   <si>
-    <t xml:space="preserve">TensorsAligned</t>
+    <t xml:space="preserve">Threaded, Vectorized, Tensorized</t>
   </si>
   <si>
     <t xml:space="preserve">CrossEntropyLoss</t>
@@ -1046,17 +1046,14 @@
       <c r="C12" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="E12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="G12" s="1" t="s">
-        <v>8</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] Add new Operators. SW-3502 Add support for AvgPool3D SW-1857 Add support for NonMaxSuppressionInst.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="200">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -62,33 +62,33 @@
     <t xml:space="preserve">Kernels, Strides, Pads</t>
   </si>
   <si>
+    <t xml:space="preserve">Threaded</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BatchOneHot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BatchedAdd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,1,2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BatchedReduceAdd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Axis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Checksum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ConvertTo</t>
+  </si>
+  <si>
     <t xml:space="preserve">0,1</t>
   </si>
   <si>
-    <t xml:space="preserve">Threaded</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BatchOneHot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BatchedAdd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0,1,2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BatchedReduceAdd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Axis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Checksum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ConvertTo</t>
-  </si>
-  <si>
     <t xml:space="preserve">Threaded, Vectorized</t>
   </si>
   <si>
@@ -377,7 +377,7 @@
     <t xml:space="preserve">ConvTranspose</t>
   </si>
   <si>
-    <t xml:space="preserve">#NonMaxSuppression</t>
+    <t xml:space="preserve">NonMaxSuppression</t>
   </si>
   <si>
     <t xml:space="preserve">CenterPointBox, MaxOutputBoxesPerClass, IouThreshold, ScoreThreshold, IsTFVersion4</t>
@@ -401,15 +401,174 @@
     <t xml:space="preserve">Int16QTy</t>
   </si>
   <si>
+    <t xml:space="preserve">FloatTy,FloatTy,FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,Float16Ty,Float16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int8QTy,Int8QTy,Int8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int8QTy,Int8QTy,Int32QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int16QTy,Int16QTy,Int16QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int16QTy,Int16QTy,Int32QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,Float16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32ITy,Float16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32ITy,FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32ITy,Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int64ITy,Float16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int64ITy,FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int64ITy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,BoolTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,BoolTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int64ITy,BoolTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32ITy,BoolTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BoolTy,FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BoolTy,Float16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BoolTy,Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BoolTy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BoolTy,BoolTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,Float16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int8QTy,Int8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int8QTy,Int32QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int16QTy,Int16QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int16QTy,Int32QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,Int8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,UInt8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,Int16QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FloatTy,Int32QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,Int8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,UInt8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,Int16QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Float16Ty,Int32QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32ITy,Int32ITy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int64ITy,Int64ITy,Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32ITy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int64ITy,Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int8QTy,Int8QTy,Int8QTy,Int32QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#Float16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int8QTy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UInt8QTy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int16QTy,Int32ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int8QTy,Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UInt8QTy,Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int16QTy,Int64ITy</t>
+  </si>
+  <si>
     <t xml:space="preserve">FloatTy, FloatTy</t>
   </si>
   <si>
     <t xml:space="preserve">Float16Ty, Float16Ty</t>
   </si>
   <si>
-    <t xml:space="preserve">Int8QTy,Int8QTy</t>
-  </si>
-  <si>
     <t xml:space="preserve">UInt8QTy,Int8QTy</t>
   </si>
   <si>
@@ -417,165 +576,6 @@
   </si>
   <si>
     <t xml:space="preserve">UInt8QTy,UInt8QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int64ITy,Int64ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FloatTy,FloatTy,FloatTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Float16Ty,Float16Ty,Float16Ty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int8QTy,Int8QTy,Int8QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int8QTy,Int8QTy,Int32QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int16QTy,Int16QTy,Int16QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int16QTy,Int16QTy,Int32QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Float16Ty,FloatTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Float16Ty,Int32ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Float16Ty,Int64ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FloatTy,Float16Ty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FloatTy,Int32ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FloatTy,Int64ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int32ITy,Float16Ty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int32ITy,FloatTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int32ITy,Int64ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int64ITy,Float16Ty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int64ITy,FloatTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int64ITy,Int32ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FloatTy,BoolTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Float16Ty,BoolTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int64ITy,BoolTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int32ITy,BoolTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BoolTy,FloatTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BoolTy,Float16Ty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BoolTy,Int64ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BoolTy,Int32ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BoolTy,BoolTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FloatTy,FloatTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Float16Ty,Float16Ty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int8QTy,Int32QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int16QTy,Int16QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int16QTy,Int32QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FloatTy,Int8QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FloatTy,UInt8QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FloatTy,Int16QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FloatTy,Int32QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Float16Ty,Int8QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Float16Ty,UInt8QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Float16Ty,Int16QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Float16Ty,Int32QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int32ITy,Int32ITy,Int32ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int64ITy,Int64ITy,Int64ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int32ITy,Int32ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int32QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int8QTy,Int8QTy,Int8QTy,Int32QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#Float16Ty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int8QTy,Int32ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UInt8QTy,Int32ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int16QTy,Int32ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int8QTy,Int64ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UInt8QTy,Int64ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int16QTy,Int64ITy</t>
   </si>
   <si>
     <t xml:space="preserve">Int8QTy,FloatTy</t>
@@ -880,11 +880,11 @@
       <c r="D4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>8</v>
@@ -892,7 +892,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>1</v>
@@ -904,7 +904,7 @@
         <v>0</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>8</v>
@@ -912,19 +912,19 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>17</v>
-      </c>
       <c r="F6" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>8</v>
@@ -932,22 +932,22 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>19</v>
-      </c>
       <c r="E7" s="1" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>8</v>
@@ -955,7 +955,7 @@
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0</v>
@@ -972,16 +972,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="B9" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>13</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>22</v>
@@ -1030,7 +1030,7 @@
         <v>0</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>8</v>
@@ -1070,7 +1070,7 @@
         <v>1</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>8</v>
@@ -1087,10 +1087,10 @@
         <v>1</v>
       </c>
       <c r="E14" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="G14" s="1" t="s">
         <v>8</v>
@@ -1107,7 +1107,7 @@
         <v>2</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>22</v>
@@ -1187,7 +1187,7 @@
         <v>2</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>22</v>
@@ -1227,7 +1227,7 @@
         <v>1</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G21" s="1" t="s">
         <v>8</v>
@@ -1244,7 +1244,7 @@
         <v>1</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>22</v>
@@ -1264,7 +1264,7 @@
         <v>2</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>22</v>
@@ -1284,7 +1284,7 @@
         <v>2</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>22</v>
@@ -1304,7 +1304,7 @@
         <v>2</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>22</v>
@@ -1324,7 +1324,7 @@
         <v>2</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>22</v>
@@ -1347,7 +1347,7 @@
         <v>0</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G27" s="1" t="s">
         <v>8</v>
@@ -1364,7 +1364,7 @@
         <v>2</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>22</v>
@@ -1413,7 +1413,7 @@
         <v>1</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G30" s="1" t="s">
         <v>8</v>
@@ -1430,7 +1430,7 @@
         <v>1</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E31" s="1" t="n">
         <v>1</v>
@@ -1516,7 +1516,7 @@
         <v>35</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G35" s="1" t="s">
         <v>8</v>
@@ -1536,7 +1536,7 @@
         <v>62</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G36" s="1" t="s">
         <v>8</v>
@@ -1559,7 +1559,7 @@
         <v>1</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G37" s="1" t="s">
         <v>8</v>
@@ -1596,7 +1596,7 @@
         <v>67</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G39" s="1" t="s">
         <v>8</v>
@@ -1616,7 +1616,7 @@
         <v>1</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G40" s="1" t="s">
         <v>8</v>
@@ -1636,7 +1636,7 @@
         <v>1</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G41" s="1" t="s">
         <v>8</v>
@@ -1702,10 +1702,10 @@
         <v>12</v>
       </c>
       <c r="E44" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F44" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="G44" s="1" t="s">
         <v>8</v>
@@ -1751,7 +1751,7 @@
         <v>1</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G46" s="1" t="s">
         <v>8</v>
@@ -1768,10 +1768,10 @@
         <v>1</v>
       </c>
       <c r="E47" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F47" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="F47" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="G47" s="1" t="s">
         <v>8</v>
@@ -1791,7 +1791,7 @@
         <v>1</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G48" s="1" t="s">
         <v>8</v>
@@ -1868,7 +1868,7 @@
         <v>1</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G52" s="1" t="s">
         <v>8</v>
@@ -1951,7 +1951,7 @@
         <v>0</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G56" s="1" t="s">
         <v>8</v>
@@ -2014,7 +2014,7 @@
         <v>1</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G59" s="1" t="s">
         <v>8</v>
@@ -2060,7 +2060,7 @@
         <v>2</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G61" s="1" t="s">
         <v>8</v>
@@ -2106,7 +2106,7 @@
         <v>104</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G63" s="1" t="s">
         <v>8</v>
@@ -2435,34 +2435,22 @@
       <c r="C4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>13</v>
+      <c r="D4" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>1</v>
@@ -2494,39 +2482,39 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>17</v>
-      </c>
       <c r="E6" s="1" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>1</v>
@@ -2558,7 +2546,7 @@
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0</v>
@@ -2590,79 +2578,79 @@
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="E9" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="L9" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="M9" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="N9" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="O9" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="P9" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="Q9" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="K9" s="1" t="s">
+      <c r="R9" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="L9" s="1" t="s">
+      <c r="S9" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="M9" s="1" t="s">
+      <c r="T9" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="N9" s="1" t="s">
+      <c r="U9" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="O9" s="1" t="s">
+      <c r="V9" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="P9" s="1" t="s">
+      <c r="W9" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="Q9" s="1" t="s">
+      <c r="X9" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="R9" s="1" t="s">
+      <c r="Y9" s="1" t="s">
         <v>152</v>
-      </c>
-      <c r="S9" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="T9" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="U9" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="V9" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="W9" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="X9" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="Y9" s="1" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2679,22 +2667,22 @@
         <v>26</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>128</v>
+        <v>155</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2804,31 +2792,31 @@
         <v>1</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E14" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="K14" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="L14" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="K14" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="L14" s="1" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2842,22 +2830,22 @@
         <v>2</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2874,19 +2862,19 @@
         <v>35</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>128</v>
+        <v>155</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>132</v>
+        <v>170</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2903,19 +2891,19 @@
         <v>35</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>128</v>
+        <v>155</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>132</v>
+        <v>170</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2932,19 +2920,19 @@
         <v>35</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>128</v>
+        <v>155</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>132</v>
+        <v>170</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2958,19 +2946,19 @@
         <v>2</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3024,13 +3012,13 @@
         <v>1</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3044,22 +3032,22 @@
         <v>2</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3073,22 +3061,22 @@
         <v>2</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3102,22 +3090,22 @@
         <v>2</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3131,13 +3119,13 @@
         <v>2</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3183,22 +3171,22 @@
         <v>2</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3285,7 +3273,7 @@
         <v>125</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3302,7 +3290,7 @@
         <v>55</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3342,7 +3330,7 @@
         <v>120</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3359,34 +3347,34 @@
         <v>35</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="G35" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="J35" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="K35" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="L35" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="M35" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="N35" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="H35" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="I35" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="J35" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="K35" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="L35" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="M35" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="N35" s="1" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3403,34 +3391,34 @@
         <v>62</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="G36" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="J36" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="K36" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="L36" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="M36" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="N36" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="H36" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="I36" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="J36" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="K36" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="L36" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="M36" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="N36" s="1" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3626,28 +3614,28 @@
         <v>1</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>126</v>
+        <v>180</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>127</v>
+        <v>181</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>128</v>
+        <v>155</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>129</v>
+        <v>182</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>130</v>
+        <v>183</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>131</v>
+        <v>184</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>132</v>
+        <v>170</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3713,7 +3701,7 @@
         <v>1</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>185</v>
@@ -3763,7 +3751,7 @@
         <v>125</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3794,16 +3782,16 @@
         <v>85</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3922,13 +3910,13 @@
         <v>199</v>
       </c>
       <c r="K54" s="1" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="L54" s="1" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="M54" s="1" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4189,25 +4177,25 @@
         <v>104</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>126</v>
+        <v>180</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>127</v>
+        <v>181</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>128</v>
+        <v>155</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>129</v>
+        <v>182</v>
       </c>
       <c r="I63" s="1" t="s">
-        <v>130</v>
+        <v>183</v>
       </c>
       <c r="J63" s="1" t="s">
-        <v>131</v>
+        <v>184</v>
       </c>
       <c r="K63" s="1" t="s">
-        <v>132</v>
+        <v>170</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4320,7 +4308,7 @@
         <v>125</v>
       </c>
       <c r="I67" s="1" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="J67" s="1" t="s">
         <v>124</v>
@@ -4360,22 +4348,22 @@
         <v>104</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="I69" s="1" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="J69" s="1" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4404,7 +4392,7 @@
         <v>125</v>
       </c>
       <c r="I70" s="1" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="J70" s="1" t="s">
         <v>124</v>
@@ -4427,10 +4415,10 @@
         <v>26</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>128</v>
+        <v>155</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4461,13 +4449,13 @@
         <v>2</v>
       </c>
       <c r="D73" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>146</v>
+        <v>124</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>149</v>
+        <v>123</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] [SW-4093] Remove scalar ConvertTo implementation
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
@@ -89,21 +89,24 @@
     <t xml:space="preserve">0,1</t>
   </si>
   <si>
+    <t xml:space="preserve">Vectorized</t>
+  </si>
+  <si>
+    <t xml:space="preserve">custom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Convolution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kernels, Strides, Pads, Group, Dilation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,3</t>
+  </si>
+  <si>
     <t xml:space="preserve">Threaded, Vectorized</t>
   </si>
   <si>
-    <t xml:space="preserve">custom</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Convolution</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kernels, Strides, Pads, Group, Dilation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0,3</t>
-  </si>
-  <si>
     <t xml:space="preserve">Convolution3D</t>
   </si>
   <si>
@@ -171,9 +174,6 @@
   </si>
   <si>
     <t xml:space="preserve">HasEndOffset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vectorized</t>
   </si>
   <si>
     <t xml:space="preserve">ExtractTensor</t>
@@ -1007,7 +1007,7 @@
         <v>26</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>23</v>
@@ -1015,7 +1015,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>1</v>
@@ -1024,7 +1024,7 @@
         <v>3</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E11" s="1" t="n">
         <v>0</v>
@@ -1038,7 +1038,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>1</v>
@@ -1050,7 +1050,7 @@
         <v>0</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>23</v>
@@ -1058,7 +1058,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>1</v>
@@ -1078,7 +1078,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>1</v>
@@ -1098,7 +1098,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>1</v>
@@ -1110,7 +1110,7 @@
         <v>16</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>23</v>
@@ -1118,7 +1118,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>1</v>
@@ -1127,10 +1127,10 @@
         <v>2</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>23</v>
@@ -1138,19 +1138,19 @@
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C17" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>35</v>
-      </c>
       <c r="F17" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>23</v>
@@ -1158,7 +1158,7 @@
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>1</v>
@@ -1167,10 +1167,10 @@
         <v>2</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G18" s="1" t="s">
         <v>23</v>
@@ -1178,7 +1178,7 @@
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>1</v>
@@ -1190,7 +1190,7 @@
         <v>16</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>23</v>
@@ -1198,7 +1198,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>1</v>
@@ -1215,7 +1215,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>1</v>
@@ -1235,7 +1235,7 @@
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>1</v>
@@ -1247,7 +1247,7 @@
         <v>21</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G22" s="1" t="s">
         <v>8</v>
@@ -1255,7 +1255,7 @@
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>1</v>
@@ -1267,7 +1267,7 @@
         <v>16</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G23" s="1" t="s">
         <v>23</v>
@@ -1275,7 +1275,7 @@
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>1</v>
@@ -1287,7 +1287,7 @@
         <v>16</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G24" s="1" t="s">
         <v>23</v>
@@ -1295,7 +1295,7 @@
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>1</v>
@@ -1307,7 +1307,7 @@
         <v>16</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G25" s="1" t="s">
         <v>23</v>
@@ -1315,7 +1315,7 @@
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>1</v>
@@ -1327,7 +1327,7 @@
         <v>16</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G26" s="1" t="s">
         <v>23</v>
@@ -1335,7 +1335,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>1</v>
@@ -1355,7 +1355,7 @@
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>1</v>
@@ -1367,7 +1367,7 @@
         <v>16</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G28" s="1" t="s">
         <v>23</v>
@@ -1375,7 +1375,7 @@
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B29" s="1" t="n">
         <v>1</v>
@@ -1384,13 +1384,13 @@
         <v>4</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E29" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="G29" s="1" t="s">
         <v>23</v>
@@ -1453,7 +1453,7 @@
         <v>55</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G32" s="1" t="s">
         <v>8</v>
@@ -1493,7 +1493,7 @@
         <v>0</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G34" s="1" t="s">
         <v>8</v>
@@ -1513,7 +1513,7 @@
         <v>60</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>13</v>
@@ -1659,7 +1659,7 @@
         <v>1</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G42" s="1" t="s">
         <v>8</v>
@@ -1682,7 +1682,7 @@
         <v>1</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G43" s="1" t="s">
         <v>8</v>
@@ -1831,7 +1831,7 @@
         <v>85</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G50" s="1" t="s">
         <v>23</v>
@@ -1888,7 +1888,7 @@
         <v>1</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G53" s="1" t="s">
         <v>8</v>
@@ -1928,7 +1928,7 @@
         <v>0</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G55" s="1" t="s">
         <v>8</v>
@@ -1974,7 +1974,7 @@
         <v>0</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G57" s="1" t="s">
         <v>8</v>
@@ -2037,7 +2037,7 @@
         <v>0</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G60" s="1" t="s">
         <v>8</v>
@@ -2687,7 +2687,7 @@
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>1</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>1</v>
@@ -2751,7 +2751,7 @@
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>1</v>
@@ -2783,7 +2783,7 @@
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>1</v>
@@ -2821,7 +2821,7 @@
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>1</v>
@@ -2850,7 +2850,7 @@
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>1</v>
@@ -2859,7 +2859,7 @@
         <v>2</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>153</v>
@@ -2879,16 +2879,16 @@
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="B17" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C17" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>35</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>153</v>
@@ -2908,7 +2908,7 @@
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>1</v>
@@ -2917,7 +2917,7 @@
         <v>2</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>153</v>
@@ -2937,7 +2937,7 @@
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>1</v>
@@ -2963,7 +2963,7 @@
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>1</v>
@@ -2983,7 +2983,7 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>1</v>
@@ -3003,7 +3003,7 @@
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>1</v>
@@ -3023,7 +3023,7 @@
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>1</v>
@@ -3052,7 +3052,7 @@
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>1</v>
@@ -3081,7 +3081,7 @@
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>1</v>
@@ -3110,7 +3110,7 @@
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>1</v>
@@ -3130,7 +3130,7 @@
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>1</v>
@@ -3162,7 +3162,7 @@
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>1</v>
@@ -3191,7 +3191,7 @@
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B29" s="1" t="n">
         <v>1</v>
@@ -3344,7 +3344,7 @@
         <v>2</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>136</v>

</xml_diff>

<commit_message>
[dnn-library] [SW-4097] Removing scalar version from element binary instructions Keeping the threaded one as generic (the vectorized one doesn't work for all the possible element kinds)
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -1110,7 +1110,7 @@
         <v>16</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>23</v>
@@ -1190,7 +1190,7 @@
         <v>16</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>23</v>
@@ -1270,7 +1270,7 @@
         <v>16</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G23" s="1" t="s">
         <v>23</v>
@@ -1290,7 +1290,7 @@
         <v>16</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G24" s="1" t="s">
         <v>23</v>
@@ -1310,7 +1310,7 @@
         <v>16</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G25" s="1" t="s">
         <v>23</v>
@@ -1330,7 +1330,7 @@
         <v>16</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G26" s="1" t="s">
         <v>23</v>
@@ -1370,7 +1370,7 @@
         <v>16</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G28" s="1" t="s">
         <v>23</v>

</xml_diff>

<commit_message>
[dnn-library] [SW-4081] Removing element compare least optimized generic implementations removed scalar kept threaded and vectorized(which is not generic as it doesn't work for all the possible elem kinds)
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -1130,7 +1130,7 @@
         <v>36</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>23</v>
@@ -1150,7 +1150,7 @@
         <v>36</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>23</v>
@@ -1170,7 +1170,7 @@
         <v>36</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G18" s="1" t="s">
         <v>23</v>

</xml_diff>

<commit_message>
[dnn-library] [SW-4131] Remove least optimized implementations for the SoftMax operator
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -1879,10 +1879,10 @@
         <v>1</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>8</v>
+        <v>23</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] [SW-4081] cleaning up non optimized generic versions for maxsplat, sparse2dense and transpose
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -254,7 +254,7 @@
     <t xml:space="preserve">Value</t>
   </si>
   <si>
-    <t xml:space="preserve">Threaded,Vectorized,Aligned32Bytes</t>
+    <t xml:space="preserve">Aligned32Bytes</t>
   </si>
   <si>
     <t xml:space="preserve">Modulo</t>
@@ -1919,7 +1919,7 @@
         <v>0</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G55" s="1" t="s">
         <v>8</v>
@@ -2068,7 +2068,7 @@
         <v>1</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="G62" s="1" t="s">
         <v>23</v>

</xml_diff>

<commit_message>
[dnn-library] [SW-4219] Operator BatchOneHot has multiple implementations and no custom impl selector
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="197">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -621,13 +621,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -644,8 +643,78 @@
       <name val="Arial"/>
       <family val="0"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="24"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="10"/>
+      <color rgb="FF808080"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF006600"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF996600"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFCC0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -654,12 +723,48 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCFFCC"/>
+        <bgColor rgb="FFCCFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCCCC"/>
+        <bgColor rgb="FFDDDDDD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCC0000"/>
+        <bgColor rgb="FF800000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF000000"/>
+        <bgColor rgb="FF003300"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF808080"/>
+        <bgColor rgb="FF969696"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFDDDDDD"/>
-        <bgColor rgb="FFCCFFCC"/>
+        <bgColor rgb="FFFFCCCC"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -667,8 +772,23 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="20">
+  <cellStyleXfs count="36">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -692,6 +812,54 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="6" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="7" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="8" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -702,33 +870,49 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="22">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="false"/>
     <cellStyle name="Comma" xfId="15" builtinId="3" customBuiltin="false"/>
     <cellStyle name="Comma [0]" xfId="16" builtinId="6" customBuiltin="false"/>
     <cellStyle name="Currency" xfId="17" builtinId="4" customBuiltin="false"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7" customBuiltin="false"/>
     <cellStyle name="Percent" xfId="19" builtinId="5" customBuiltin="false"/>
+    <cellStyle name="Heading" xfId="20" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Heading 1" xfId="21" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Heading 2" xfId="22" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Text" xfId="23" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Note" xfId="24" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Footnote" xfId="25" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Status" xfId="26" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Good" xfId="27" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Neutral" xfId="28" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Bad" xfId="29" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Warning" xfId="30" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Error" xfId="31" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Accent" xfId="32" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Accent 1" xfId="33" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Accent 2" xfId="34" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Accent 3" xfId="35" builtinId="53" customBuiltin="true"/>
   </cellStyles>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
       <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FFCC0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF006600"/>
       <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF996600"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFC0C0C0"/>
@@ -756,7 +940,7 @@
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFFFCCCC"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -894,9 +1078,6 @@
       <c r="E5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="G5" s="1" t="s">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
[dnn-library] [SW-4238] Operator SparseLengthsWeightedSum has multiple implementations and no custom impl selector
Keeping threaded and scalar.
Threaded seems to have problems under certain conditions. So I added a custom implementation selector that always selects the scalar version.
I Created SW-4292 to address this.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
@@ -287,76 +287,76 @@
     <t xml:space="preserve">1,3</t>
   </si>
   <si>
+    <t xml:space="preserve">SparseToDense</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SparseToDenseMask</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mask</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Splat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Syncopy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SyncOffset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tanh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TensorView</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TopK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transpose</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shuffle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MaxPoolWithArgMax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BatchedReduceMin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Axes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CumSum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exclusive, Reverse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SpaceToDepth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BlockSize</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ResizeNearest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RszScale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LengthsRangeFill</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SparseLengthsSum</t>
+  </si>
+  <si>
     <t xml:space="preserve">#Threaded</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SparseToDense</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SparseToDenseMask</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mask</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Splat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Syncopy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SyncOffset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tanh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TensorView</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TopK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Transpose</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shuffle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MaxPoolWithArgMax</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0,2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BatchedReduceMin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Axes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CumSum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exclusive, Reverse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SpaceToDepth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BlockSize</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ResizeNearest</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RszScale</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LengthsRangeFill</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SparseLengthsSum</t>
   </si>
   <si>
     <t xml:space="preserve">ResizeBilinear</t>
@@ -621,12 +621,13 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -643,78 +644,8 @@
       <name val="Arial"/>
       <family val="0"/>
     </font>
-    <font>
-      <b val="true"/>
-      <sz val="24"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="18"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF333333"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <i val="true"/>
-      <sz val="10"/>
-      <color rgb="FF808080"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF006600"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF996600"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FFCC0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="9">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -723,48 +654,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFCCFFCC"/>
-        <bgColor rgb="FFCCFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCCCC"/>
-        <bgColor rgb="FFDDDDDD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFCC0000"/>
-        <bgColor rgb="FF800000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF000000"/>
-        <bgColor rgb="FF003300"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF808080"/>
-        <bgColor rgb="FF969696"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFDDDDDD"/>
-        <bgColor rgb="FFFFCCCC"/>
+        <bgColor rgb="FFCCFFCC"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -772,23 +667,8 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin">
-        <color rgb="FF808080"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF808080"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF808080"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="36">
+  <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -812,54 +692,6 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="5" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="6" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="7" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="8" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -870,49 +702,33 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="22">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="false"/>
     <cellStyle name="Comma" xfId="15" builtinId="3" customBuiltin="false"/>
     <cellStyle name="Comma [0]" xfId="16" builtinId="6" customBuiltin="false"/>
     <cellStyle name="Currency" xfId="17" builtinId="4" customBuiltin="false"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7" customBuiltin="false"/>
     <cellStyle name="Percent" xfId="19" builtinId="5" customBuiltin="false"/>
-    <cellStyle name="Heading" xfId="20" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Heading 1" xfId="21" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Heading 2" xfId="22" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Text" xfId="23" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Note" xfId="24" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Footnote" xfId="25" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Status" xfId="26" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Good" xfId="27" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Neutral" xfId="28" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Bad" xfId="29" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Warning" xfId="30" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Error" xfId="31" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Accent" xfId="32" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Accent 1" xfId="33" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Accent 2" xfId="34" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Accent 3" xfId="35" builtinId="53" customBuiltin="true"/>
   </cellStyles>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
       <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFCC0000"/>
+      <rgbColor rgb="FFFF0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF006600"/>
+      <rgbColor rgb="FF008000"/>
       <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF996600"/>
+      <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFC0C0C0"/>
@@ -940,7 +756,7 @@
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCCCC"/>
+      <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -2047,15 +1863,15 @@
         <v>87</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>8</v>
+        <v>23</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B55" s="1" t="n">
         <v>1</v>
@@ -2075,7 +1891,7 @@
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B56" s="1" t="n">
         <v>1</v>
@@ -2084,7 +1900,7 @@
         <v>4</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E56" s="1" t="n">
         <v>0</v>
@@ -2098,7 +1914,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B57" s="1" t="n">
         <v>1</v>
@@ -2118,16 +1934,16 @@
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B58" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" s="1" t="s">
         <v>93</v>
-      </c>
-      <c r="B58" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C58" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>94</v>
       </c>
       <c r="E58" s="1" t="n">
         <v>1</v>
@@ -2138,7 +1954,7 @@
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B59" s="1" t="n">
         <v>1</v>
@@ -2155,7 +1971,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B60" s="1" t="n">
         <v>1</v>
@@ -2175,7 +1991,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B61" s="1" t="n">
         <v>2</v>
@@ -2184,7 +2000,7 @@
         <v>1</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E61" s="1" t="n">
         <v>2</v>
@@ -2198,16 +2014,16 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B62" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C62" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" s="1" t="s">
         <v>98</v>
-      </c>
-      <c r="B62" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C62" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D62" s="1" t="s">
-        <v>99</v>
       </c>
       <c r="E62" s="1" t="n">
         <v>1</v>
@@ -2221,7 +2037,7 @@
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B63" s="1" t="n">
         <v>2</v>
@@ -2233,7 +2049,7 @@
         <v>12</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F63" s="1" t="s">
         <v>13</v>
@@ -2244,16 +2060,16 @@
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B64" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C64" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" s="1" t="s">
         <v>102</v>
-      </c>
-      <c r="B64" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C64" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D64" s="1" t="s">
-        <v>103</v>
       </c>
       <c r="E64" s="1" t="n">
         <v>1</v>
@@ -2264,16 +2080,16 @@
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B65" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C65" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="B65" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C65" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D65" s="1" t="s">
-        <v>105</v>
       </c>
       <c r="E65" s="1" t="n">
         <v>1</v>
@@ -2284,16 +2100,16 @@
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B66" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C66" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="B66" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C66" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>107</v>
       </c>
       <c r="E66" s="1" t="n">
         <v>0</v>
@@ -2304,16 +2120,16 @@
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B67" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C67" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="B67" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C67" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D67" s="1" t="s">
-        <v>109</v>
       </c>
       <c r="E67" s="1" t="n">
         <v>0</v>
@@ -2324,7 +2140,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B68" s="1" t="n">
         <v>1</v>
@@ -2341,7 +2157,7 @@
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B69" s="1" t="n">
         <v>1</v>
@@ -2350,10 +2166,10 @@
         <v>3</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>88</v>
+        <v>111</v>
       </c>
       <c r="G69" s="1" t="s">
         <v>8</v>
@@ -2370,7 +2186,7 @@
         <v>1</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E70" s="1" t="n">
         <v>0</v>
@@ -4490,7 +4306,7 @@
         <v>1</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>177</v>
@@ -4679,7 +4495,7 @@
         <v>3</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>133</v>

</xml_diff>

<commit_message>
[dnn-library] [SW-4231] Operator IntLookupTable has multiple implementations and no custom impl selector
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="641" uniqueCount="197">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -621,13 +621,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -644,8 +643,78 @@
       <name val="Arial"/>
       <family val="0"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="24"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="10"/>
+      <color rgb="FF808080"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF006600"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF996600"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFCC0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -654,12 +723,48 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCFFCC"/>
+        <bgColor rgb="FFCCFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCCCC"/>
+        <bgColor rgb="FFDDDDDD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCC0000"/>
+        <bgColor rgb="FF800000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF000000"/>
+        <bgColor rgb="FF003300"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF808080"/>
+        <bgColor rgb="FF969696"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFDDDDDD"/>
-        <bgColor rgb="FFCCFFCC"/>
+        <bgColor rgb="FFFFCCCC"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -667,8 +772,23 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="20">
+  <cellStyleXfs count="36">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -692,6 +812,54 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="6" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="7" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="8" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -702,33 +870,49 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="22">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="false"/>
     <cellStyle name="Comma" xfId="15" builtinId="3" customBuiltin="false"/>
     <cellStyle name="Comma [0]" xfId="16" builtinId="6" customBuiltin="false"/>
     <cellStyle name="Currency" xfId="17" builtinId="4" customBuiltin="false"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7" customBuiltin="false"/>
     <cellStyle name="Percent" xfId="19" builtinId="5" customBuiltin="false"/>
+    <cellStyle name="Heading" xfId="20" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Heading 1" xfId="21" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Heading 2" xfId="22" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Text" xfId="23" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Note" xfId="24" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Footnote" xfId="25" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Status" xfId="26" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Good" xfId="27" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Neutral" xfId="28" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Bad" xfId="29" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Warning" xfId="30" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Error" xfId="31" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Accent" xfId="32" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Accent 1" xfId="33" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Accent 2" xfId="34" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="Accent 3" xfId="35" builtinId="53" customBuiltin="true"/>
   </cellStyles>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
       <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FFCC0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF006600"/>
       <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF996600"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFC0C0C0"/>
@@ -756,7 +940,7 @@
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFFFCCCC"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -1565,9 +1749,6 @@
       <c r="E39" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="F39" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="G39" s="1" t="s">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
[dnn-library] [SW-4243] Operator SparseLengthsSum has multiple implementations and no custom impl selector
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="196">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -354,9 +354,6 @@
   </si>
   <si>
     <t xml:space="preserve">SparseLengthsSum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#Threaded</t>
   </si>
   <si>
     <t xml:space="preserve">ResizeBilinear</t>
@@ -2316,16 +2313,13 @@
       <c r="E69" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="F69" s="1" t="s">
-        <v>111</v>
-      </c>
       <c r="G69" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B70" s="1" t="n">
         <v>1</v>
@@ -2345,7 +2339,7 @@
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B71" s="1" t="n">
         <v>1</v>
@@ -2365,7 +2359,7 @@
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B72" s="1" t="n">
         <v>1</v>
@@ -2385,16 +2379,16 @@
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B73" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C73" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D73" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="B73" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C73" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="D73" s="1" t="s">
-        <v>116</v>
       </c>
       <c r="E73" s="1" t="n">
         <v>0</v>
@@ -2472,22 +2466,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2507,22 +2501,22 @@
         <v>1</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2542,13 +2536,13 @@
         <v>0</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2568,22 +2562,22 @@
         <v>0</v>
       </c>
       <c r="E5" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="I5" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="J5" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2603,22 +2597,22 @@
         <v>16</v>
       </c>
       <c r="E6" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="I6" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="J6" s="1" t="s">
         <v>127</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2638,22 +2632,22 @@
         <v>1</v>
       </c>
       <c r="E7" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="I7" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="J7" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2673,22 +2667,22 @@
         <v>0</v>
       </c>
       <c r="E8" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="H8" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="I8" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="J8" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2708,67 +2702,67 @@
         <v>21</v>
       </c>
       <c r="E9" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="H9" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="I9" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="J9" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="K9" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="K9" s="1" t="s">
+      <c r="L9" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="L9" s="1" t="s">
+      <c r="M9" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="M9" s="1" t="s">
+      <c r="N9" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="N9" s="1" t="s">
+      <c r="O9" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="O9" s="1" t="s">
+      <c r="P9" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="P9" s="1" t="s">
+      <c r="Q9" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="Q9" s="1" t="s">
+      <c r="R9" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="R9" s="1" t="s">
+      <c r="S9" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="S9" s="1" t="s">
+      <c r="T9" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="T9" s="1" t="s">
+      <c r="U9" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="U9" s="1" t="s">
+      <c r="V9" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="V9" s="1" t="s">
+      <c r="W9" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="W9" s="1" t="s">
+      <c r="X9" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="X9" s="1" t="s">
+      <c r="Y9" s="1" t="s">
         <v>148</v>
-      </c>
-      <c r="Y9" s="1" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2788,22 +2782,22 @@
         <v>26</v>
       </c>
       <c r="E10" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="H10" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="H10" s="1" t="s">
+      <c r="I10" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="J10" s="1" t="s">
         <v>154</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2823,22 +2817,22 @@
         <v>0</v>
       </c>
       <c r="E11" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="H11" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="I11" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="J11" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2858,22 +2852,22 @@
         <v>0</v>
       </c>
       <c r="E12" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="H12" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H12" s="1" t="s">
+      <c r="I12" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I12" s="1" t="s">
+      <c r="J12" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2893,22 +2887,22 @@
         <v>1</v>
       </c>
       <c r="E13" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G13" s="1" t="s">
+      <c r="H13" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H13" s="1" t="s">
+      <c r="I13" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I13" s="1" t="s">
+      <c r="J13" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2928,28 +2922,28 @@
         <v>21</v>
       </c>
       <c r="E14" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="G14" s="1" t="s">
+      <c r="H14" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="I14" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="I14" s="1" t="s">
+      <c r="J14" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="J14" s="1" t="s">
+      <c r="K14" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="K14" s="1" t="s">
+      <c r="L14" s="1" t="s">
         <v>162</v>
-      </c>
-      <c r="L14" s="1" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2969,19 +2963,19 @@
         <v>16</v>
       </c>
       <c r="E15" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="G15" s="1" t="s">
-        <v>125</v>
-      </c>
       <c r="H15" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="I15" s="1" t="s">
         <v>164</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3001,19 +2995,19 @@
         <v>35</v>
       </c>
       <c r="E16" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="G16" s="1" t="s">
-        <v>152</v>
-      </c>
       <c r="H16" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="I16" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3033,19 +3027,19 @@
         <v>35</v>
       </c>
       <c r="E17" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="F17" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="G17" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="G17" s="1" t="s">
-        <v>152</v>
-      </c>
       <c r="H17" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="I17" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3065,19 +3059,19 @@
         <v>35</v>
       </c>
       <c r="E18" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="G18" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="G18" s="1" t="s">
-        <v>152</v>
-      </c>
       <c r="H18" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="I18" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="I18" s="1" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3097,16 +3091,16 @@
         <v>16</v>
       </c>
       <c r="E19" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="G19" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="G19" s="1" t="s">
-        <v>125</v>
-      </c>
       <c r="H19" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3126,10 +3120,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3149,10 +3143,10 @@
         <v>1</v>
       </c>
       <c r="E21" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3172,10 +3166,10 @@
         <v>21</v>
       </c>
       <c r="E22" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>150</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3195,19 +3189,19 @@
         <v>16</v>
       </c>
       <c r="E23" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F23" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="F23" s="1" t="s">
+      <c r="G23" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="G23" s="1" t="s">
-        <v>125</v>
-      </c>
       <c r="H23" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="I23" s="1" t="s">
         <v>164</v>
-      </c>
-      <c r="I23" s="1" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3227,19 +3221,19 @@
         <v>16</v>
       </c>
       <c r="E24" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F24" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="F24" s="1" t="s">
+      <c r="G24" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="G24" s="1" t="s">
-        <v>125</v>
-      </c>
       <c r="H24" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="I24" s="1" t="s">
         <v>164</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3259,19 +3253,19 @@
         <v>16</v>
       </c>
       <c r="E25" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F25" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="F25" s="1" t="s">
+      <c r="G25" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="G25" s="1" t="s">
-        <v>125</v>
-      </c>
       <c r="H25" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="I25" s="1" t="s">
         <v>164</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3291,10 +3285,10 @@
         <v>16</v>
       </c>
       <c r="E26" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F26" s="1" t="s">
         <v>123</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3314,22 +3308,22 @@
         <v>0</v>
       </c>
       <c r="E27" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F27" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F27" s="1" t="s">
+      <c r="G27" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G27" s="1" t="s">
+      <c r="H27" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H27" s="1" t="s">
+      <c r="I27" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I27" s="1" t="s">
+      <c r="J27" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J27" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3349,19 +3343,19 @@
         <v>16</v>
       </c>
       <c r="E28" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F28" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="G28" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="G28" s="1" t="s">
-        <v>125</v>
-      </c>
       <c r="H28" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="I28" s="1" t="s">
         <v>164</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3381,10 +3375,10 @@
         <v>0</v>
       </c>
       <c r="E29" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F29" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3404,22 +3398,22 @@
         <v>1</v>
       </c>
       <c r="E30" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F30" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="G30" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G30" s="1" t="s">
+      <c r="H30" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H30" s="1" t="s">
+      <c r="I30" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I30" s="1" t="s">
+      <c r="J30" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J30" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3439,25 +3433,25 @@
         <v>1</v>
       </c>
       <c r="E31" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F31" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F31" s="1" t="s">
+      <c r="G31" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G31" s="1" t="s">
+      <c r="H31" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H31" s="1" t="s">
+      <c r="I31" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I31" s="1" t="s">
+      <c r="J31" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="J31" s="1" t="s">
-        <v>122</v>
-      </c>
       <c r="K31" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3477,7 +3471,7 @@
         <v>54</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3497,10 +3491,10 @@
         <v>0</v>
       </c>
       <c r="E33" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F33" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3520,10 +3514,10 @@
         <v>0</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3543,34 +3537,34 @@
         <v>35</v>
       </c>
       <c r="E35" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="J35" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="F35" s="1" t="s">
+      <c r="K35" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="G35" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="H35" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="I35" s="1" t="s">
+      <c r="L35" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="J35" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="K35" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="L35" s="1" t="s">
+      <c r="M35" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="M35" s="1" t="s">
+      <c r="N35" s="1" t="s">
         <v>175</v>
-      </c>
-      <c r="N35" s="1" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3590,34 +3584,34 @@
         <v>60</v>
       </c>
       <c r="E36" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="J36" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="F36" s="1" t="s">
+      <c r="K36" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="G36" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="H36" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="I36" s="1" t="s">
+      <c r="L36" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="J36" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="K36" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="L36" s="1" t="s">
+      <c r="M36" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="M36" s="1" t="s">
+      <c r="N36" s="1" t="s">
         <v>175</v>
-      </c>
-      <c r="N36" s="1" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3637,22 +3631,22 @@
         <v>1</v>
       </c>
       <c r="E37" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F37" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F37" s="1" t="s">
+      <c r="G37" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G37" s="1" t="s">
+      <c r="H37" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H37" s="1" t="s">
+      <c r="I37" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I37" s="1" t="s">
+      <c r="J37" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J37" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3672,10 +3666,10 @@
         <v>1</v>
       </c>
       <c r="E38" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="F38" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3712,22 +3706,22 @@
         <v>1</v>
       </c>
       <c r="E40" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F40" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F40" s="1" t="s">
+      <c r="G40" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G40" s="1" t="s">
+      <c r="H40" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H40" s="1" t="s">
+      <c r="I40" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I40" s="1" t="s">
+      <c r="J40" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J40" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3747,22 +3741,22 @@
         <v>1</v>
       </c>
       <c r="E41" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F41" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F41" s="1" t="s">
+      <c r="G41" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G41" s="1" t="s">
+      <c r="H41" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H41" s="1" t="s">
+      <c r="I41" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I41" s="1" t="s">
+      <c r="J41" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J41" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3782,10 +3776,10 @@
         <v>1</v>
       </c>
       <c r="E42" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F42" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="F42" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3805,22 +3799,22 @@
         <v>1</v>
       </c>
       <c r="E43" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F43" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F43" s="1" t="s">
+      <c r="G43" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G43" s="1" t="s">
+      <c r="H43" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H43" s="1" t="s">
+      <c r="I43" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I43" s="1" t="s">
+      <c r="J43" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J43" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3840,25 +3834,25 @@
         <v>21</v>
       </c>
       <c r="E44" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="F44" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="F44" s="1" t="s">
+      <c r="G44" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="H44" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="G44" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="H44" s="1" t="s">
+      <c r="I44" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="I44" s="1" t="s">
+      <c r="J44" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="J44" s="1" t="s">
-        <v>181</v>
-      </c>
       <c r="K44" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3878,22 +3872,22 @@
         <v>1</v>
       </c>
       <c r="E45" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F45" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F45" s="1" t="s">
+      <c r="G45" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G45" s="1" t="s">
+      <c r="H45" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H45" s="1" t="s">
+      <c r="I45" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I45" s="1" t="s">
+      <c r="J45" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J45" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3913,10 +3907,10 @@
         <v>1</v>
       </c>
       <c r="E46" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F46" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="F46" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3936,28 +3930,28 @@
         <v>21</v>
       </c>
       <c r="E47" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="F47" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="F47" s="1" t="s">
+      <c r="G47" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="G47" s="1" t="s">
+      <c r="H47" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="H47" s="1" t="s">
+      <c r="I47" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="I47" s="1" t="s">
+      <c r="J47" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="J47" s="1" t="s">
+      <c r="K47" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="K47" s="1" t="s">
+      <c r="L47" s="1" t="s">
         <v>188</v>
-      </c>
-      <c r="L47" s="1" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3977,16 +3971,16 @@
         <v>1</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4023,16 +4017,16 @@
         <v>82</v>
       </c>
       <c r="E50" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="F50" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="F50" s="1" t="s">
-        <v>134</v>
-      </c>
       <c r="G50" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="H50" s="1" t="s">
         <v>130</v>
-      </c>
-      <c r="H50" s="1" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4052,22 +4046,22 @@
         <v>0</v>
       </c>
       <c r="E51" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F51" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F51" s="1" t="s">
+      <c r="G51" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G51" s="1" t="s">
+      <c r="H51" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H51" s="1" t="s">
+      <c r="I51" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I51" s="1" t="s">
+      <c r="J51" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J51" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4087,10 +4081,10 @@
         <v>1</v>
       </c>
       <c r="E52" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F52" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="F52" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4110,22 +4104,22 @@
         <v>1</v>
       </c>
       <c r="E53" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F53" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F53" s="1" t="s">
+      <c r="G53" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G53" s="1" t="s">
+      <c r="H53" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H53" s="1" t="s">
+      <c r="I53" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I53" s="1" t="s">
+      <c r="J53" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J53" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4145,31 +4139,31 @@
         <v>87</v>
       </c>
       <c r="E54" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="F54" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="F54" s="1" t="s">
+      <c r="G54" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="G54" s="1" t="s">
+      <c r="H54" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="H54" s="1" t="s">
+      <c r="I54" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="I54" s="1" t="s">
+      <c r="J54" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="J54" s="1" t="s">
-        <v>196</v>
-      </c>
       <c r="K54" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="L54" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="M54" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4189,22 +4183,22 @@
         <v>0</v>
       </c>
       <c r="E55" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F55" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F55" s="1" t="s">
+      <c r="G55" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G55" s="1" t="s">
+      <c r="H55" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H55" s="1" t="s">
+      <c r="I55" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I55" s="1" t="s">
+      <c r="J55" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J55" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4224,22 +4218,22 @@
         <v>0</v>
       </c>
       <c r="E56" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F56" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F56" s="1" t="s">
+      <c r="G56" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G56" s="1" t="s">
+      <c r="H56" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H56" s="1" t="s">
+      <c r="I56" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I56" s="1" t="s">
+      <c r="J56" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J56" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4259,22 +4253,22 @@
         <v>0</v>
       </c>
       <c r="E57" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F57" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F57" s="1" t="s">
+      <c r="G57" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G57" s="1" t="s">
+      <c r="H57" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H57" s="1" t="s">
+      <c r="I57" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I57" s="1" t="s">
+      <c r="J57" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J57" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4294,22 +4288,22 @@
         <v>1</v>
       </c>
       <c r="E58" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F58" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F58" s="1" t="s">
+      <c r="G58" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G58" s="1" t="s">
+      <c r="H58" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H58" s="1" t="s">
+      <c r="I58" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I58" s="1" t="s">
+      <c r="J58" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J58" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4329,10 +4323,10 @@
         <v>1</v>
       </c>
       <c r="E59" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F59" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="F59" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4352,22 +4346,22 @@
         <v>0</v>
       </c>
       <c r="E60" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F60" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F60" s="1" t="s">
+      <c r="G60" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G60" s="1" t="s">
+      <c r="H60" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H60" s="1" t="s">
+      <c r="I60" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I60" s="1" t="s">
+      <c r="J60" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J60" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4387,22 +4381,22 @@
         <v>2</v>
       </c>
       <c r="E61" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F61" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F61" s="1" t="s">
+      <c r="G61" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G61" s="1" t="s">
+      <c r="H61" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H61" s="1" t="s">
+      <c r="I61" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I61" s="1" t="s">
+      <c r="J61" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J61" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4422,22 +4416,22 @@
         <v>1</v>
       </c>
       <c r="E62" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F62" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F62" s="1" t="s">
+      <c r="G62" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G62" s="1" t="s">
+      <c r="H62" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H62" s="1" t="s">
+      <c r="I62" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I62" s="1" t="s">
+      <c r="J62" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J62" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4457,25 +4451,25 @@
         <v>100</v>
       </c>
       <c r="E63" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="F63" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="F63" s="1" t="s">
+      <c r="G63" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="H63" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="G63" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="H63" s="1" t="s">
+      <c r="I63" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="I63" s="1" t="s">
+      <c r="J63" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="J63" s="1" t="s">
-        <v>181</v>
-      </c>
       <c r="K63" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4495,22 +4489,22 @@
         <v>1</v>
       </c>
       <c r="E64" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F64" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F64" s="1" t="s">
+      <c r="G64" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G64" s="1" t="s">
+      <c r="H64" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H64" s="1" t="s">
+      <c r="I64" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I64" s="1" t="s">
+      <c r="J64" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J64" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4530,16 +4524,16 @@
         <v>1</v>
       </c>
       <c r="E65" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F65" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F65" s="1" t="s">
-        <v>118</v>
-      </c>
       <c r="G65" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4559,16 +4553,16 @@
         <v>0</v>
       </c>
       <c r="E66" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F66" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F66" s="1" t="s">
+      <c r="G66" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G66" s="1" t="s">
+      <c r="H66" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="H66" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4588,25 +4582,25 @@
         <v>0</v>
       </c>
       <c r="E67" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F67" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F67" s="1" t="s">
+      <c r="G67" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G67" s="1" t="s">
+      <c r="H67" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I67" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="J67" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="K67" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="H67" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="I67" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="J67" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="K67" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4626,7 +4620,7 @@
         <v>0</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4646,22 +4640,22 @@
         <v>100</v>
       </c>
       <c r="E69" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="F69" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="F69" s="1" t="s">
-        <v>134</v>
-      </c>
       <c r="G69" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="H69" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="H69" s="1" t="s">
-        <v>131</v>
-      </c>
       <c r="I69" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="J69" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4681,25 +4675,25 @@
         <v>0</v>
       </c>
       <c r="E70" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F70" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F70" s="1" t="s">
+      <c r="G70" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G70" s="1" t="s">
+      <c r="H70" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I70" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="J70" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="K70" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="H70" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="I70" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="J70" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="K70" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4719,10 +4713,10 @@
         <v>26</v>
       </c>
       <c r="E71" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="F71" s="1" t="s">
         <v>152</v>
-      </c>
-      <c r="F71" s="1" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4742,7 +4736,7 @@
         <v>0</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4762,10 +4756,10 @@
         <v>2</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] [SW-4230] Adding custom impl selector for InsertTensor apparently a custom selector is required, because the threaded version is not generic (it sometime calls the scalar one)
There are 2 conditions that make the threaded version call the scalar version. So moving these conditions to the selector instead of the implementation, and keeping both versions
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
@@ -618,12 +618,13 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -640,78 +641,8 @@
       <name val="Arial"/>
       <family val="0"/>
     </font>
-    <font>
-      <b val="true"/>
-      <sz val="24"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="18"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF333333"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <i val="true"/>
-      <sz val="10"/>
-      <color rgb="FF808080"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF006600"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF996600"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FFCC0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="9">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -720,48 +651,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFCCFFCC"/>
-        <bgColor rgb="FFCCFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCCCC"/>
-        <bgColor rgb="FFDDDDDD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFCC0000"/>
-        <bgColor rgb="FF800000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF000000"/>
-        <bgColor rgb="FF003300"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF808080"/>
-        <bgColor rgb="FF969696"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFDDDDDD"/>
-        <bgColor rgb="FFFFCCCC"/>
+        <bgColor rgb="FFCCFFCC"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -769,23 +664,8 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin">
-        <color rgb="FF808080"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF808080"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF808080"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="36">
+  <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -809,54 +689,6 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="5" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="6" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="7" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="8" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -867,49 +699,33 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="22">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="false"/>
     <cellStyle name="Comma" xfId="15" builtinId="3" customBuiltin="false"/>
     <cellStyle name="Comma [0]" xfId="16" builtinId="6" customBuiltin="false"/>
     <cellStyle name="Currency" xfId="17" builtinId="4" customBuiltin="false"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7" customBuiltin="false"/>
     <cellStyle name="Percent" xfId="19" builtinId="5" customBuiltin="false"/>
-    <cellStyle name="Heading" xfId="20" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Heading 1" xfId="21" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Heading 2" xfId="22" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Text" xfId="23" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Note" xfId="24" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Footnote" xfId="25" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Status" xfId="26" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Good" xfId="27" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Neutral" xfId="28" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Bad" xfId="29" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Warning" xfId="30" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Error" xfId="31" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Accent" xfId="32" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Accent 1" xfId="33" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Accent 2" xfId="34" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Accent 3" xfId="35" builtinId="53" customBuiltin="true"/>
   </cellStyles>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
       <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFCC0000"/>
+      <rgbColor rgb="FFFF0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF006600"/>
+      <rgbColor rgb="FF008000"/>
       <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF996600"/>
+      <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFC0C0C0"/>
@@ -937,7 +753,7 @@
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCCCC"/>
+      <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -1692,7 +1508,7 @@
         <v>13</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>8</v>
+        <v>23</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] [SW-4218] Adding custom impl selector for AvgPool if input tensor has 5 dims => scalar version is called from the threaded implementation
removing this condition from the implementation, and moving it to the impl selection class ( and setting ?custom? instead of ?default? in the implSel column of the table)
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -65,6 +65,9 @@
     <t xml:space="preserve">Threaded</t>
   </si>
   <si>
+    <t xml:space="preserve">custom</t>
+  </si>
+  <si>
     <t xml:space="preserve">BatchOneHot</t>
   </si>
   <si>
@@ -90,9 +93,6 @@
   </si>
   <si>
     <t xml:space="preserve">Vectorized</t>
-  </si>
-  <si>
-    <t xml:space="preserve">custom</t>
   </si>
   <si>
     <t xml:space="preserve">Convolution</t>
@@ -875,12 +875,12 @@
         <v>13</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>1</v>
@@ -897,7 +897,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>1</v>
@@ -906,7 +906,7 @@
         <v>2</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>8</v>
@@ -914,7 +914,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>1</v>
@@ -923,7 +923,7 @@
         <v>1</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>1</v>
@@ -934,7 +934,7 @@
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0</v>
@@ -951,7 +951,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>1</v>
@@ -960,13 +960,13 @@
         <v>1</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -986,10 +986,10 @@
         <v>26</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1029,7 +1029,7 @@
         <v>30</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1060,7 +1060,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G14" s="1" t="s">
         <v>8</v>
@@ -1077,13 +1077,13 @@
         <v>2</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1100,10 +1100,10 @@
         <v>35</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1120,10 +1120,10 @@
         <v>35</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1140,10 +1140,10 @@
         <v>35</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1157,13 +1157,13 @@
         <v>2</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1211,7 +1211,7 @@
         <v>1</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G22" s="1" t="s">
         <v>8</v>
@@ -1228,13 +1228,13 @@
         <v>2</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1248,13 +1248,13 @@
         <v>2</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1268,13 +1268,13 @@
         <v>2</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1288,13 +1288,13 @@
         <v>2</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1325,13 +1325,13 @@
         <v>2</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1351,10 +1351,10 @@
         <v>0</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1388,7 +1388,7 @@
         <v>1</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E31" s="1" t="n">
         <v>1</v>
@@ -1411,7 +1411,7 @@
         <v>54</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G32" s="1" t="s">
         <v>8</v>
@@ -1508,7 +1508,7 @@
         <v>13</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1596,10 +1596,10 @@
         <v>1</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1636,7 +1636,7 @@
         <v>12</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G44" s="1" t="s">
         <v>8</v>
@@ -1662,7 +1662,7 @@
         <v>75</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1696,7 +1696,7 @@
         <v>1</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G47" s="1" t="s">
         <v>8</v>
@@ -1736,7 +1736,7 @@
         <v>75</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1753,10 +1753,10 @@
         <v>82</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1807,10 +1807,10 @@
         <v>1</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1830,7 +1830,7 @@
         <v>13</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1990,7 +1990,7 @@
         <v>75</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2404,7 +2404,7 @@
         <v>2</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>122</v>
@@ -2509,7 +2509,7 @@
         <v>1</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>128</v>
@@ -2729,7 +2729,7 @@
         <v>1</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>155</v>
@@ -2770,7 +2770,7 @@
         <v>2</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>122</v>
@@ -2898,7 +2898,7 @@
         <v>2</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>122</v>
@@ -2973,7 +2973,7 @@
         <v>1</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>149</v>
@@ -2996,7 +2996,7 @@
         <v>2</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>122</v>
@@ -3028,7 +3028,7 @@
         <v>2</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>122</v>
@@ -3060,7 +3060,7 @@
         <v>2</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>122</v>
@@ -3092,7 +3092,7 @@
         <v>2</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>122</v>
@@ -3150,7 +3150,7 @@
         <v>2</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>122</v>
@@ -3641,7 +3641,7 @@
         <v>1</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>176</v>
@@ -3737,7 +3737,7 @@
         <v>1</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>181</v>

</xml_diff>

<commit_message>
[dnn-library] [SW-2466] Fix Flip tests. [SW-4244] ArgMax support 5 and 6 dimensions. [SW-2475] ArgMax scale must be positive. [SW-4315] ArgMax use in test same subtest naming combination. [SW-3473] ResizeNearest test int32/0 fixed. [SW-4418] Create tests regressions for ResizeNearest.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="626" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="625" uniqueCount="198">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -56,6 +56,9 @@
     <t xml:space="preserve">Axis, KeepDims</t>
   </si>
   <si>
+    <t xml:space="preserve">0,1</t>
+  </si>
+  <si>
     <t xml:space="preserve">AvgPool</t>
   </si>
   <si>
@@ -89,9 +92,6 @@
     <t xml:space="preserve">ConvertTo</t>
   </si>
   <si>
-    <t xml:space="preserve">0,1</t>
-  </si>
-  <si>
     <t xml:space="preserve">Vectorized</t>
   </si>
   <si>
@@ -389,6 +389,18 @@
     <t xml:space="preserve">Int16QTy</t>
   </si>
   <si>
+    <t xml:space="preserve">Int64ITy,FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32ITy,FloatTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int64ITy,Int8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int32ITy,Int8QTy</t>
+  </si>
+  <si>
     <t xml:space="preserve">FloatTy,FloatTy,FloatTy</t>
   </si>
   <si>
@@ -428,16 +440,10 @@
     <t xml:space="preserve">Int32ITy,Float16Ty</t>
   </si>
   <si>
-    <t xml:space="preserve">Int32ITy,FloatTy</t>
-  </si>
-  <si>
     <t xml:space="preserve">Int32ITy,Int64ITy</t>
   </si>
   <si>
     <t xml:space="preserve">Int64ITy,Float16Ty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int64ITy,FloatTy</t>
   </si>
   <si>
     <t xml:space="preserve">Int64ITy,Int32ITy</t>
@@ -618,12 +624,13 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -640,78 +647,8 @@
       <name val="Arial"/>
       <family val="0"/>
     </font>
-    <font>
-      <b val="true"/>
-      <sz val="24"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="18"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF333333"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <i val="true"/>
-      <sz val="10"/>
-      <color rgb="FF808080"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF006600"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF996600"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FFCC0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="9">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -720,48 +657,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFCCFFCC"/>
-        <bgColor rgb="FFCCFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCCCC"/>
-        <bgColor rgb="FFDDDDDD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFCC0000"/>
-        <bgColor rgb="FF800000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF000000"/>
-        <bgColor rgb="FF003300"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF808080"/>
-        <bgColor rgb="FF969696"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFDDDDDD"/>
-        <bgColor rgb="FFFFCCCC"/>
+        <bgColor rgb="FFCCFFCC"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -769,23 +670,8 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin">
-        <color rgb="FF808080"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF808080"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF808080"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="36">
+  <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -809,54 +695,6 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="5" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="6" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="7" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="8" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -867,49 +705,33 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="22">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="false"/>
     <cellStyle name="Comma" xfId="15" builtinId="3" customBuiltin="false"/>
     <cellStyle name="Comma [0]" xfId="16" builtinId="6" customBuiltin="false"/>
     <cellStyle name="Currency" xfId="17" builtinId="4" customBuiltin="false"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7" customBuiltin="false"/>
     <cellStyle name="Percent" xfId="19" builtinId="5" customBuiltin="false"/>
-    <cellStyle name="Heading" xfId="20" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Heading 1" xfId="21" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Heading 2" xfId="22" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Text" xfId="23" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Note" xfId="24" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Footnote" xfId="25" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Status" xfId="26" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Good" xfId="27" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Neutral" xfId="28" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Bad" xfId="29" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Warning" xfId="30" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Error" xfId="31" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Accent" xfId="32" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Accent 1" xfId="33" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Accent 2" xfId="34" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="Accent 3" xfId="35" builtinId="53" customBuiltin="true"/>
   </cellStyles>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
       <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFCC0000"/>
+      <rgbColor rgb="FFFF0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF006600"/>
+      <rgbColor rgb="FF008000"/>
       <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF996600"/>
+      <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFC0C0C0"/>
@@ -937,7 +759,7 @@
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCCCC"/>
+      <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -1032,8 +854,8 @@
       <c r="D3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="1" t="n">
-        <v>1</v>
+      <c r="E3" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>8</v>
@@ -1041,7 +863,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>1</v>
@@ -1050,21 +872,21 @@
         <v>1</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>1</v>
@@ -1081,7 +903,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>1</v>
@@ -1090,7 +912,7 @@
         <v>2</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>8</v>
@@ -1098,7 +920,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>1</v>
@@ -1107,7 +929,7 @@
         <v>1</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>1</v>
@@ -1118,7 +940,7 @@
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0</v>
@@ -1135,7 +957,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>1</v>
@@ -1144,13 +966,13 @@
         <v>1</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>23</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1173,7 +995,7 @@
         <v>23</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1213,7 +1035,7 @@
         <v>30</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1244,7 +1066,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="G14" s="1" t="s">
         <v>8</v>
@@ -1261,13 +1083,13 @@
         <v>2</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>23</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1287,7 +1109,7 @@
         <v>23</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1307,7 +1129,7 @@
         <v>23</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1327,7 +1149,7 @@
         <v>23</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1341,13 +1163,13 @@
         <v>2</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>23</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1395,7 +1217,7 @@
         <v>1</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="G22" s="1" t="s">
         <v>8</v>
@@ -1412,13 +1234,13 @@
         <v>2</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>23</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1432,13 +1254,13 @@
         <v>2</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>23</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1452,13 +1274,13 @@
         <v>2</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>23</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1472,13 +1294,13 @@
         <v>2</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>23</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1509,13 +1331,13 @@
         <v>2</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>23</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1538,7 +1360,7 @@
         <v>23</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1572,7 +1394,7 @@
         <v>1</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E31" s="1" t="n">
         <v>1</v>
@@ -1689,10 +1511,10 @@
         <v>1</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1783,7 +1605,7 @@
         <v>23</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1817,10 +1639,10 @@
         <v>1</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="G44" s="1" t="s">
         <v>8</v>
@@ -1846,7 +1668,7 @@
         <v>75</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1880,7 +1702,7 @@
         <v>1</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="G47" s="1" t="s">
         <v>8</v>
@@ -1920,7 +1742,7 @@
         <v>75</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1940,7 +1762,7 @@
         <v>23</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1994,7 +1816,7 @@
         <v>23</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2011,10 +1833,10 @@
         <v>87</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2171,7 +1993,7 @@
         <v>75</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2185,7 +2007,7 @@
         <v>1</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>100</v>
@@ -2492,23 +2314,19 @@
         <v>1</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>121</v>
-      </c>
+        <v>125</v>
+      </c>
+      <c r="I3" s="0"/>
+      <c r="J3" s="0"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="str">
@@ -2585,25 +2403,25 @@
         <v>2</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2690,70 +2508,70 @@
         <v>1</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>138</v>
+        <v>122</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="R9" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="S9" s="1" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="T9" s="1" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="V9" s="1" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="W9" s="1" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="X9" s="1" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="Y9" s="1" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2773,22 +2591,22 @@
         <v>26</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2910,31 +2728,31 @@
         <v>1</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2951,22 +2769,22 @@
         <v>2</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2986,19 +2804,19 @@
         <v>35</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3018,19 +2836,19 @@
         <v>35</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3050,19 +2868,19 @@
         <v>35</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3079,19 +2897,19 @@
         <v>2</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3154,13 +2972,13 @@
         <v>1</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3177,22 +2995,22 @@
         <v>2</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3209,22 +3027,22 @@
         <v>2</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3241,22 +3059,22 @@
         <v>2</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3273,13 +3091,13 @@
         <v>2</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3331,22 +3149,22 @@
         <v>2</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3442,7 +3260,7 @@
         <v>121</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3462,7 +3280,7 @@
         <v>54</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3508,7 +3326,7 @@
         <v>116</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3528,34 +3346,34 @@
         <v>35</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="L35" s="1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="M35" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3575,34 +3393,34 @@
         <v>60</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="K36" s="1" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="L36" s="1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="M36" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="N36" s="1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3822,28 +3640,28 @@
         <v>1</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3918,31 +3736,31 @@
         <v>1</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="I47" s="1" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="J47" s="1" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="K47" s="1" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="L47" s="1" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3965,13 +3783,13 @@
         <v>118</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="G48" s="1" t="s">
         <v>121</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4008,16 +3826,16 @@
         <v>82</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="F50" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="G50" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="G50" s="1" t="s">
-        <v>129</v>
-      </c>
       <c r="H50" s="1" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4130,31 +3948,31 @@
         <v>87</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="I54" s="1" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="J54" s="1" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="K54" s="1" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="L54" s="1" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="M54" s="1" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4442,25 +4260,25 @@
         <v>100</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="I63" s="1" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="J63" s="1" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="K63" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4585,7 +4403,7 @@
         <v>121</v>
       </c>
       <c r="I67" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="J67" s="1" t="s">
         <v>120</v>
@@ -4631,22 +4449,22 @@
         <v>100</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="F69" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="G69" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="G69" s="1" t="s">
-        <v>129</v>
-      </c>
       <c r="H69" s="1" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="I69" s="1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="J69" s="1" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4678,7 +4496,7 @@
         <v>121</v>
       </c>
       <c r="I70" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="J70" s="1" t="s">
         <v>120</v>
@@ -4704,10 +4522,10 @@
         <v>26</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] [SW-4213] Do FullyConnected vectorized version generic. [SW-4214] FullyConnected vectorized version pass Operator.FCCmd/0_ test. [SW-4462] ETSOC backend for FullyConnected elements types is accordingly with Glow Interpreter. Asm code has been refactored and moved outside header to specific asm file for fullyconnect.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="625" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="196">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -185,9 +185,6 @@
     <t xml:space="preserve">FullyConnected</t>
   </si>
   <si>
-    <t xml:space="preserve">0,1,2,3</t>
-  </si>
-  <si>
     <t xml:space="preserve">FusedRowwiseQuantizedSparseLengthsSum</t>
   </si>
   <si>
@@ -533,7 +530,7 @@
     <t xml:space="preserve">Int32QTy</t>
   </si>
   <si>
-    <t xml:space="preserve">Int8QTy,Int8QTy,Int8QTy,Int32QTy</t>
+    <t xml:space="preserve">Int8QTy,FloatTy</t>
   </si>
   <si>
     <t xml:space="preserve">#Float16Ty</t>
@@ -570,9 +567,6 @@
   </si>
   <si>
     <t xml:space="preserve">UInt8QTy,UInt8QTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int8QTy,FloatTy</t>
   </si>
   <si>
     <t xml:space="preserve">UInt8QTy,FloatTy</t>
@@ -1414,10 +1408,7 @@
         <v>3</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G32" s="1" t="s">
         <v>8</v>
@@ -1425,7 +1416,7 @@
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B33" s="1" t="n">
         <v>1</v>
@@ -1442,7 +1433,7 @@
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B34" s="1" t="n">
         <v>1</v>
@@ -1459,16 +1450,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D35" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="B35" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C35" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>58</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>35</v>
@@ -1479,16 +1470,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C36" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="B36" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C36" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>60</v>
       </c>
       <c r="G36" s="1" t="s">
         <v>8</v>
@@ -1496,16 +1487,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B37" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="B37" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C37" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>62</v>
       </c>
       <c r="E37" s="1" t="n">
         <v>1</v>
@@ -1519,7 +1510,7 @@
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B38" s="1" t="n">
         <v>1</v>
@@ -1536,16 +1527,16 @@
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B39" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E39" s="1" t="s">
         <v>64</v>
-      </c>
-      <c r="B39" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C39" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>65</v>
       </c>
       <c r="G39" s="1" t="s">
         <v>8</v>
@@ -1553,7 +1544,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B40" s="1" t="n">
         <v>1</v>
@@ -1570,7 +1561,7 @@
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B41" s="1" t="n">
         <v>1</v>
@@ -1587,16 +1578,16 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B42" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C42" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="B42" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C42" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>69</v>
       </c>
       <c r="E42" s="1" t="n">
         <v>1</v>
@@ -1610,16 +1601,16 @@
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B43" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D43" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="B43" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C43" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>71</v>
       </c>
       <c r="E43" s="1" t="n">
         <v>1</v>
@@ -1630,7 +1621,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B44" s="1" t="n">
         <v>1</v>
@@ -1650,22 +1641,22 @@
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B45" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B45" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C45" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D45" s="1" t="s">
+      <c r="E45" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F45" s="1" t="s">
         <v>74</v>
-      </c>
-      <c r="E45" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>75</v>
       </c>
       <c r="G45" s="1" t="s">
         <v>15</v>
@@ -1673,16 +1664,16 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B46" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="1" t="s">
         <v>76</v>
-      </c>
-      <c r="B46" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C46" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D46" s="1" t="s">
-        <v>77</v>
       </c>
       <c r="E46" s="1" t="n">
         <v>1</v>
@@ -1693,7 +1684,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B47" s="1" t="n">
         <v>1</v>
@@ -1710,7 +1701,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B48" s="1" t="n">
         <v>1</v>
@@ -1727,7 +1718,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B49" s="1" t="n">
         <v>1</v>
@@ -1736,10 +1727,10 @@
         <v>5</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G49" s="1" t="s">
         <v>15</v>
@@ -1747,7 +1738,7 @@
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B50" s="1" t="n">
         <v>1</v>
@@ -1756,7 +1747,7 @@
         <v>6</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>23</v>
@@ -1767,7 +1758,7 @@
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B51" s="1" t="n">
         <v>1</v>
@@ -1784,7 +1775,7 @@
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B52" s="1" t="n">
         <v>1</v>
@@ -1801,7 +1792,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B53" s="1" t="n">
         <v>1</v>
@@ -1821,7 +1812,7 @@
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B54" s="1" t="n">
         <v>1</v>
@@ -1830,7 +1821,7 @@
         <v>4</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F54" s="1" t="s">
         <v>14</v>
@@ -1841,7 +1832,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B55" s="1" t="n">
         <v>1</v>
@@ -1858,7 +1849,7 @@
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B56" s="1" t="n">
         <v>1</v>
@@ -1867,7 +1858,7 @@
         <v>4</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E56" s="1" t="n">
         <v>0</v>
@@ -1878,7 +1869,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B57" s="1" t="n">
         <v>1</v>
@@ -1887,7 +1878,7 @@
         <v>0</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E57" s="1" t="n">
         <v>0</v>
@@ -1898,16 +1889,16 @@
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B58" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="B58" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C58" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>93</v>
       </c>
       <c r="E58" s="1" t="n">
         <v>1</v>
@@ -1918,7 +1909,7 @@
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B59" s="1" t="n">
         <v>1</v>
@@ -1935,7 +1926,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B60" s="1" t="n">
         <v>1</v>
@@ -1955,7 +1946,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B61" s="1" t="n">
         <v>2</v>
@@ -1964,7 +1955,7 @@
         <v>1</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E61" s="1" t="n">
         <v>2</v>
@@ -1975,22 +1966,22 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B62" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C62" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B62" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C62" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D62" s="1" t="s">
-        <v>98</v>
-      </c>
       <c r="E62" s="1" t="n">
         <v>1</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G62" s="1" t="s">
         <v>15</v>
@@ -1998,7 +1989,7 @@
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B63" s="1" t="n">
         <v>2</v>
@@ -2010,7 +2001,7 @@
         <v>13</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G63" s="1" t="s">
         <v>8</v>
@@ -2018,16 +2009,16 @@
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B64" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C64" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" s="1" t="s">
         <v>101</v>
-      </c>
-      <c r="B64" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C64" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D64" s="1" t="s">
-        <v>102</v>
       </c>
       <c r="E64" s="1" t="n">
         <v>1</v>
@@ -2038,16 +2029,16 @@
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B65" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C65" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="B65" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C65" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D65" s="1" t="s">
-        <v>104</v>
       </c>
       <c r="E65" s="1" t="n">
         <v>1</v>
@@ -2058,16 +2049,16 @@
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B66" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C66" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" s="1" t="s">
         <v>105</v>
-      </c>
-      <c r="B66" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C66" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>106</v>
       </c>
       <c r="E66" s="1" t="n">
         <v>0</v>
@@ -2078,16 +2069,16 @@
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B67" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C67" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" s="1" t="s">
         <v>107</v>
-      </c>
-      <c r="B67" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C67" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D67" s="1" t="s">
-        <v>108</v>
       </c>
       <c r="E67" s="1" t="n">
         <v>0</v>
@@ -2098,7 +2089,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B68" s="1" t="n">
         <v>1</v>
@@ -2115,7 +2106,7 @@
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B69" s="1" t="n">
         <v>1</v>
@@ -2124,7 +2115,7 @@
         <v>3</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G69" s="1" t="s">
         <v>8</v>
@@ -2132,7 +2123,7 @@
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B70" s="1" t="n">
         <v>1</v>
@@ -2141,7 +2132,7 @@
         <v>1</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E70" s="1" t="n">
         <v>0</v>
@@ -2152,7 +2143,7 @@
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B71" s="1" t="n">
         <v>1</v>
@@ -2172,7 +2163,7 @@
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B72" s="1" t="n">
         <v>1</v>
@@ -2192,16 +2183,16 @@
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B73" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C73" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D73" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="B73" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C73" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="D73" s="1" t="s">
-        <v>115</v>
       </c>
       <c r="E73" s="1" t="n">
         <v>0</v>
@@ -2279,22 +2270,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2314,16 +2305,16 @@
         <v>1</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>124</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>125</v>
       </c>
       <c r="I3" s="0"/>
       <c r="J3" s="0"/>
@@ -2345,13 +2336,13 @@
         <v>0</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2371,22 +2362,22 @@
         <v>0</v>
       </c>
       <c r="E5" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="I5" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="J5" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2406,22 +2397,22 @@
         <v>18</v>
       </c>
       <c r="E6" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="I6" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="J6" s="1" t="s">
         <v>130</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2441,22 +2432,22 @@
         <v>1</v>
       </c>
       <c r="E7" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="I7" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="J7" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2476,22 +2467,22 @@
         <v>0</v>
       </c>
       <c r="E8" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="H8" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="I8" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="J8" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2511,67 +2502,67 @@
         <v>11</v>
       </c>
       <c r="E9" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="H9" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="I9" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="J9" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="K9" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="K9" s="1" t="s">
+      <c r="L9" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="M9" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="L9" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="M9" s="1" t="s">
+      <c r="N9" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="N9" s="1" t="s">
+      <c r="O9" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="P9" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="O9" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="P9" s="1" t="s">
+      <c r="Q9" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="Q9" s="1" t="s">
+      <c r="R9" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="R9" s="1" t="s">
+      <c r="S9" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="S9" s="1" t="s">
+      <c r="T9" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="T9" s="1" t="s">
+      <c r="U9" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="U9" s="1" t="s">
+      <c r="V9" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="V9" s="1" t="s">
+      <c r="W9" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="W9" s="1" t="s">
+      <c r="X9" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="X9" s="1" t="s">
+      <c r="Y9" s="1" t="s">
         <v>149</v>
-      </c>
-      <c r="Y9" s="1" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2591,22 +2582,22 @@
         <v>26</v>
       </c>
       <c r="E10" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="H10" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="H10" s="1" t="s">
+      <c r="I10" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="J10" s="1" t="s">
         <v>155</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2626,22 +2617,22 @@
         <v>0</v>
       </c>
       <c r="E11" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="H11" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="I11" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="J11" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2661,22 +2652,22 @@
         <v>0</v>
       </c>
       <c r="E12" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="H12" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H12" s="1" t="s">
+      <c r="I12" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I12" s="1" t="s">
+      <c r="J12" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2696,22 +2687,22 @@
         <v>1</v>
       </c>
       <c r="E13" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G13" s="1" t="s">
+      <c r="H13" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H13" s="1" t="s">
+      <c r="I13" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I13" s="1" t="s">
+      <c r="J13" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2731,28 +2722,28 @@
         <v>11</v>
       </c>
       <c r="E14" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="G14" s="1" t="s">
+      <c r="H14" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="I14" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="I14" s="1" t="s">
+      <c r="J14" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="J14" s="1" t="s">
+      <c r="K14" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="K14" s="1" t="s">
+      <c r="L14" s="1" t="s">
         <v>163</v>
-      </c>
-      <c r="L14" s="1" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2772,19 +2763,19 @@
         <v>18</v>
       </c>
       <c r="E15" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="G15" s="1" t="s">
-        <v>128</v>
-      </c>
       <c r="H15" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="I15" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2804,19 +2795,19 @@
         <v>35</v>
       </c>
       <c r="E16" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="G16" s="1" t="s">
-        <v>153</v>
-      </c>
       <c r="H16" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="I16" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2836,19 +2827,19 @@
         <v>35</v>
       </c>
       <c r="E17" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F17" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="G17" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="G17" s="1" t="s">
-        <v>153</v>
-      </c>
       <c r="H17" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="I17" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2868,19 +2859,19 @@
         <v>35</v>
       </c>
       <c r="E18" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="G18" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="G18" s="1" t="s">
-        <v>153</v>
-      </c>
       <c r="H18" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="I18" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="I18" s="1" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2900,16 +2891,16 @@
         <v>18</v>
       </c>
       <c r="E19" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="G19" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="G19" s="1" t="s">
-        <v>128</v>
-      </c>
       <c r="H19" s="1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2929,10 +2920,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2952,10 +2943,10 @@
         <v>1</v>
       </c>
       <c r="E21" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2975,10 +2966,10 @@
         <v>11</v>
       </c>
       <c r="E22" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2998,19 +2989,19 @@
         <v>18</v>
       </c>
       <c r="E23" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="F23" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="F23" s="1" t="s">
+      <c r="G23" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="G23" s="1" t="s">
-        <v>128</v>
-      </c>
       <c r="H23" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="I23" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="I23" s="1" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3030,19 +3021,19 @@
         <v>18</v>
       </c>
       <c r="E24" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="F24" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="F24" s="1" t="s">
+      <c r="G24" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="G24" s="1" t="s">
-        <v>128</v>
-      </c>
       <c r="H24" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="I24" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3062,19 +3053,19 @@
         <v>18</v>
       </c>
       <c r="E25" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="F25" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="F25" s="1" t="s">
+      <c r="G25" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="G25" s="1" t="s">
-        <v>128</v>
-      </c>
       <c r="H25" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="I25" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3094,10 +3085,10 @@
         <v>18</v>
       </c>
       <c r="E26" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="F26" s="1" t="s">
         <v>126</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3117,22 +3108,22 @@
         <v>0</v>
       </c>
       <c r="E27" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F27" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F27" s="1" t="s">
+      <c r="G27" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G27" s="1" t="s">
+      <c r="H27" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H27" s="1" t="s">
+      <c r="I27" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I27" s="1" t="s">
+      <c r="J27" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="J27" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3152,19 +3143,19 @@
         <v>18</v>
       </c>
       <c r="E28" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="F28" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="G28" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="G28" s="1" t="s">
-        <v>128</v>
-      </c>
       <c r="H28" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="I28" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3184,10 +3175,10 @@
         <v>0</v>
       </c>
       <c r="E29" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F29" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3207,22 +3198,22 @@
         <v>1</v>
       </c>
       <c r="E30" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F30" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="G30" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G30" s="1" t="s">
+      <c r="H30" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H30" s="1" t="s">
+      <c r="I30" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I30" s="1" t="s">
+      <c r="J30" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="J30" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3242,25 +3233,25 @@
         <v>1</v>
       </c>
       <c r="E31" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F31" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F31" s="1" t="s">
+      <c r="G31" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G31" s="1" t="s">
+      <c r="H31" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H31" s="1" t="s">
+      <c r="I31" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I31" s="1" t="s">
+      <c r="J31" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="J31" s="1" t="s">
-        <v>121</v>
-      </c>
       <c r="K31" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3277,10 +3268,28 @@
         <v>3</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>54</v>
+        <v>26</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>170</v>
+        <v>150</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="K32" s="1" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3300,10 +3309,10 @@
         <v>0</v>
       </c>
       <c r="E33" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F33" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3323,10 +3332,10 @@
         <v>0</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3346,34 +3355,34 @@
         <v>35</v>
       </c>
       <c r="E35" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="J35" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="F35" s="1" t="s">
+      <c r="K35" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="G35" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="H35" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="I35" s="1" t="s">
+      <c r="L35" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="J35" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="K35" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="L35" s="1" t="s">
+      <c r="M35" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="M35" s="1" t="s">
+      <c r="N35" s="1" t="s">
         <v>176</v>
-      </c>
-      <c r="N35" s="1" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3390,37 +3399,37 @@
         <v>2</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E36" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="J36" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="F36" s="1" t="s">
+      <c r="K36" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="G36" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="H36" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="I36" s="1" t="s">
+      <c r="L36" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="J36" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="K36" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="L36" s="1" t="s">
+      <c r="M36" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="M36" s="1" t="s">
+      <c r="N36" s="1" t="s">
         <v>176</v>
-      </c>
-      <c r="N36" s="1" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3440,22 +3449,22 @@
         <v>1</v>
       </c>
       <c r="E37" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F37" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F37" s="1" t="s">
+      <c r="G37" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G37" s="1" t="s">
+      <c r="H37" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H37" s="1" t="s">
+      <c r="I37" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I37" s="1" t="s">
+      <c r="J37" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="J37" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3475,10 +3484,10 @@
         <v>1</v>
       </c>
       <c r="E38" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F38" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3495,7 +3504,7 @@
         <v>2</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3515,22 +3524,22 @@
         <v>1</v>
       </c>
       <c r="E40" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F40" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F40" s="1" t="s">
+      <c r="G40" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G40" s="1" t="s">
+      <c r="H40" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H40" s="1" t="s">
+      <c r="I40" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I40" s="1" t="s">
+      <c r="J40" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="J40" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3550,22 +3559,22 @@
         <v>1</v>
       </c>
       <c r="E41" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F41" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F41" s="1" t="s">
+      <c r="G41" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G41" s="1" t="s">
+      <c r="H41" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H41" s="1" t="s">
+      <c r="I41" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I41" s="1" t="s">
+      <c r="J41" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="J41" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3585,10 +3594,10 @@
         <v>1</v>
       </c>
       <c r="E42" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F42" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="F42" s="1" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3608,22 +3617,22 @@
         <v>1</v>
       </c>
       <c r="E43" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F43" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F43" s="1" t="s">
+      <c r="G43" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G43" s="1" t="s">
+      <c r="H43" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H43" s="1" t="s">
+      <c r="I43" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I43" s="1" t="s">
+      <c r="J43" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="J43" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3643,25 +3652,25 @@
         <v>11</v>
       </c>
       <c r="E44" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="F44" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="F44" s="1" t="s">
+      <c r="G44" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="H44" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="G44" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="H44" s="1" t="s">
+      <c r="I44" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="I44" s="1" t="s">
+      <c r="J44" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="J44" s="1" t="s">
-        <v>182</v>
-      </c>
       <c r="K44" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3681,22 +3690,22 @@
         <v>1</v>
       </c>
       <c r="E45" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F45" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F45" s="1" t="s">
+      <c r="G45" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G45" s="1" t="s">
+      <c r="H45" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H45" s="1" t="s">
+      <c r="I45" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I45" s="1" t="s">
+      <c r="J45" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="J45" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3716,10 +3725,10 @@
         <v>1</v>
       </c>
       <c r="E46" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="F46" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="F46" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3739,28 +3748,28 @@
         <v>11</v>
       </c>
       <c r="E47" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="G47" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="F47" s="1" t="s">
+      <c r="H47" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="G47" s="1" t="s">
+      <c r="I47" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="H47" s="1" t="s">
+      <c r="J47" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="I47" s="1" t="s">
+      <c r="K47" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="J47" s="1" t="s">
+      <c r="L47" s="1" t="s">
         <v>188</v>
-      </c>
-      <c r="K47" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="L47" s="1" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3780,16 +3789,16 @@
         <v>1</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3806,7 +3815,7 @@
         <v>5</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3823,19 +3832,19 @@
         <v>6</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E50" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F50" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="F50" s="1" t="s">
-        <v>137</v>
-      </c>
       <c r="G50" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="H50" s="1" t="s">
         <v>133</v>
-      </c>
-      <c r="H50" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3855,22 +3864,22 @@
         <v>0</v>
       </c>
       <c r="E51" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F51" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F51" s="1" t="s">
+      <c r="G51" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G51" s="1" t="s">
+      <c r="H51" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H51" s="1" t="s">
+      <c r="I51" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I51" s="1" t="s">
+      <c r="J51" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="J51" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3890,10 +3899,10 @@
         <v>1</v>
       </c>
       <c r="E52" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F52" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="F52" s="1" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3913,22 +3922,22 @@
         <v>1</v>
       </c>
       <c r="E53" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F53" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F53" s="1" t="s">
+      <c r="G53" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G53" s="1" t="s">
+      <c r="H53" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H53" s="1" t="s">
+      <c r="I53" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I53" s="1" t="s">
+      <c r="J53" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="J53" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3945,34 +3954,34 @@
         <v>4</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E54" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="G54" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="F54" s="1" t="s">
+      <c r="H54" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="G54" s="1" t="s">
+      <c r="I54" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="H54" s="1" t="s">
+      <c r="J54" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="I54" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="J54" s="1" t="s">
-        <v>197</v>
-      </c>
       <c r="K54" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L54" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="M54" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3992,22 +4001,22 @@
         <v>0</v>
       </c>
       <c r="E55" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F55" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F55" s="1" t="s">
+      <c r="G55" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G55" s="1" t="s">
+      <c r="H55" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H55" s="1" t="s">
+      <c r="I55" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I55" s="1" t="s">
+      <c r="J55" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="J55" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4027,22 +4036,22 @@
         <v>0</v>
       </c>
       <c r="E56" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F56" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F56" s="1" t="s">
+      <c r="G56" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G56" s="1" t="s">
+      <c r="H56" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H56" s="1" t="s">
+      <c r="I56" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I56" s="1" t="s">
+      <c r="J56" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="J56" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4062,22 +4071,22 @@
         <v>0</v>
       </c>
       <c r="E57" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F57" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F57" s="1" t="s">
+      <c r="G57" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G57" s="1" t="s">
+      <c r="H57" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H57" s="1" t="s">
+      <c r="I57" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I57" s="1" t="s">
+      <c r="J57" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="J57" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4097,22 +4106,22 @@
         <v>1</v>
       </c>
       <c r="E58" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F58" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F58" s="1" t="s">
+      <c r="G58" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G58" s="1" t="s">
+      <c r="H58" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H58" s="1" t="s">
+      <c r="I58" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I58" s="1" t="s">
+      <c r="J58" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="J58" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4132,10 +4141,10 @@
         <v>1</v>
       </c>
       <c r="E59" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F59" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="F59" s="1" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4155,22 +4164,22 @@
         <v>0</v>
       </c>
       <c r="E60" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F60" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F60" s="1" t="s">
+      <c r="G60" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G60" s="1" t="s">
+      <c r="H60" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H60" s="1" t="s">
+      <c r="I60" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I60" s="1" t="s">
+      <c r="J60" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="J60" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4190,22 +4199,22 @@
         <v>2</v>
       </c>
       <c r="E61" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F61" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F61" s="1" t="s">
+      <c r="G61" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G61" s="1" t="s">
+      <c r="H61" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H61" s="1" t="s">
+      <c r="I61" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I61" s="1" t="s">
+      <c r="J61" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="J61" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4225,22 +4234,22 @@
         <v>1</v>
       </c>
       <c r="E62" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F62" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F62" s="1" t="s">
+      <c r="G62" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G62" s="1" t="s">
+      <c r="H62" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H62" s="1" t="s">
+      <c r="I62" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I62" s="1" t="s">
+      <c r="J62" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="J62" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4257,28 +4266,28 @@
         <v>1</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E63" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="F63" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="F63" s="1" t="s">
+      <c r="G63" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="H63" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="G63" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="H63" s="1" t="s">
+      <c r="I63" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="I63" s="1" t="s">
+      <c r="J63" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="J63" s="1" t="s">
-        <v>182</v>
-      </c>
       <c r="K63" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4298,22 +4307,22 @@
         <v>1</v>
       </c>
       <c r="E64" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F64" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F64" s="1" t="s">
+      <c r="G64" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G64" s="1" t="s">
+      <c r="H64" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H64" s="1" t="s">
+      <c r="I64" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I64" s="1" t="s">
+      <c r="J64" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="J64" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4333,16 +4342,16 @@
         <v>1</v>
       </c>
       <c r="E65" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F65" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F65" s="1" t="s">
-        <v>117</v>
-      </c>
       <c r="G65" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4362,16 +4371,16 @@
         <v>0</v>
       </c>
       <c r="E66" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F66" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F66" s="1" t="s">
+      <c r="G66" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G66" s="1" t="s">
+      <c r="H66" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="H66" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4391,25 +4400,25 @@
         <v>0</v>
       </c>
       <c r="E67" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F67" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F67" s="1" t="s">
+      <c r="G67" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G67" s="1" t="s">
+      <c r="H67" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="I67" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="J67" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="K67" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="H67" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="I67" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="J67" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="K67" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4429,7 +4438,7 @@
         <v>0</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4446,25 +4455,25 @@
         <v>3</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E69" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F69" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="F69" s="1" t="s">
-        <v>137</v>
-      </c>
       <c r="G69" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="H69" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="H69" s="1" t="s">
-        <v>134</v>
-      </c>
       <c r="I69" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="J69" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4484,25 +4493,25 @@
         <v>0</v>
       </c>
       <c r="E70" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F70" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F70" s="1" t="s">
+      <c r="G70" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G70" s="1" t="s">
+      <c r="H70" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="I70" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="J70" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="K70" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="H70" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="I70" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="J70" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="K70" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4522,10 +4531,10 @@
         <v>26</v>
       </c>
       <c r="E71" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="F71" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="F71" s="1" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4545,7 +4554,7 @@
         <v>0</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4565,10 +4574,10 @@
         <v>2</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] [SW-5037] Adding network operators test
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="198">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -62,7 +62,7 @@
     <t xml:space="preserve">AvgPool</t>
   </si>
   <si>
-    <t xml:space="preserve">Kernels, Strides, Pads</t>
+    <t xml:space="preserve">Kernels, Strides, Pads,Layout,CountIncludePads</t>
   </si>
   <si>
     <t xml:space="preserve">Threaded</t>
@@ -239,6 +239,9 @@
     <t xml:space="preserve">MaxPool</t>
   </si>
   <si>
+    <t xml:space="preserve">Kernels, Strides, Pads,Layout</t>
+  </si>
+  <si>
     <t xml:space="preserve">MaxSplat</t>
   </si>
   <si>
@@ -318,6 +321,9 @@
   </si>
   <si>
     <t xml:space="preserve">MaxPoolWithArgMax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kernels, Strides, Pads, Layout</t>
   </si>
   <si>
     <t xml:space="preserve">0,2</t>
@@ -1630,7 +1636,7 @@
         <v>1</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>13</v>
+        <v>72</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>11</v>
@@ -1641,7 +1647,7 @@
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B45" s="1" t="n">
         <v>1</v>
@@ -1650,13 +1656,13 @@
         <v>1</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E45" s="1" t="n">
         <v>1</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G45" s="1" t="s">
         <v>15</v>
@@ -1664,7 +1670,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B46" s="1" t="n">
         <v>1</v>
@@ -1673,7 +1679,7 @@
         <v>1</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E46" s="1" t="n">
         <v>1</v>
@@ -1684,7 +1690,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B47" s="1" t="n">
         <v>1</v>
@@ -1701,7 +1707,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B48" s="1" t="n">
         <v>1</v>
@@ -1718,7 +1724,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B49" s="1" t="n">
         <v>1</v>
@@ -1730,7 +1736,7 @@
         <v>64</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G49" s="1" t="s">
         <v>15</v>
@@ -1738,7 +1744,7 @@
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B50" s="1" t="n">
         <v>1</v>
@@ -1747,7 +1753,7 @@
         <v>6</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>23</v>
@@ -1758,7 +1764,7 @@
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B51" s="1" t="n">
         <v>1</v>
@@ -1775,7 +1781,7 @@
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B52" s="1" t="n">
         <v>1</v>
@@ -1792,7 +1798,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B53" s="1" t="n">
         <v>1</v>
@@ -1812,7 +1818,7 @@
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B54" s="1" t="n">
         <v>1</v>
@@ -1821,7 +1827,7 @@
         <v>4</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F54" s="1" t="s">
         <v>14</v>
@@ -1832,7 +1838,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B55" s="1" t="n">
         <v>1</v>
@@ -1849,7 +1855,7 @@
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B56" s="1" t="n">
         <v>1</v>
@@ -1858,7 +1864,7 @@
         <v>4</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E56" s="1" t="n">
         <v>0</v>
@@ -1869,7 +1875,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B57" s="1" t="n">
         <v>1</v>
@@ -1878,7 +1884,7 @@
         <v>0</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E57" s="1" t="n">
         <v>0</v>
@@ -1889,7 +1895,7 @@
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B58" s="1" t="n">
         <v>1</v>
@@ -1898,7 +1904,7 @@
         <v>1</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E58" s="1" t="n">
         <v>1</v>
@@ -1909,7 +1915,7 @@
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B59" s="1" t="n">
         <v>1</v>
@@ -1926,7 +1932,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B60" s="1" t="n">
         <v>1</v>
@@ -1946,7 +1952,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B61" s="1" t="n">
         <v>2</v>
@@ -1955,7 +1961,7 @@
         <v>1</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E61" s="1" t="n">
         <v>2</v>
@@ -1966,7 +1972,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B62" s="1" t="n">
         <v>1</v>
@@ -1975,13 +1981,13 @@
         <v>1</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E62" s="1" t="n">
         <v>1</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G62" s="1" t="s">
         <v>15</v>
@@ -1989,7 +1995,7 @@
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B63" s="1" t="n">
         <v>2</v>
@@ -1998,10 +2004,10 @@
         <v>1</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>13</v>
+        <v>100</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G63" s="1" t="s">
         <v>8</v>
@@ -2009,7 +2015,7 @@
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B64" s="1" t="n">
         <v>1</v>
@@ -2018,7 +2024,7 @@
         <v>1</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E64" s="1" t="n">
         <v>1</v>
@@ -2029,7 +2035,7 @@
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B65" s="1" t="n">
         <v>1</v>
@@ -2038,7 +2044,7 @@
         <v>1</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E65" s="1" t="n">
         <v>1</v>
@@ -2049,7 +2055,7 @@
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B66" s="1" t="n">
         <v>1</v>
@@ -2058,7 +2064,7 @@
         <v>1</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E66" s="1" t="n">
         <v>0</v>
@@ -2069,7 +2075,7 @@
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B67" s="1" t="n">
         <v>1</v>
@@ -2078,7 +2084,7 @@
         <v>1</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E67" s="1" t="n">
         <v>0</v>
@@ -2089,7 +2095,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B68" s="1" t="n">
         <v>1</v>
@@ -2106,7 +2112,7 @@
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B69" s="1" t="n">
         <v>1</v>
@@ -2115,7 +2121,7 @@
         <v>3</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G69" s="1" t="s">
         <v>8</v>
@@ -2123,7 +2129,7 @@
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B70" s="1" t="n">
         <v>1</v>
@@ -2132,7 +2138,7 @@
         <v>1</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E70" s="1" t="n">
         <v>0</v>
@@ -2143,7 +2149,7 @@
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B71" s="1" t="n">
         <v>1</v>
@@ -2163,7 +2169,7 @@
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B72" s="1" t="n">
         <v>1</v>
@@ -2183,7 +2189,7 @@
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B73" s="1" t="n">
         <v>2</v>
@@ -2192,7 +2198,7 @@
         <v>2</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E73" s="1" t="n">
         <v>0</v>
@@ -2270,22 +2276,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2305,16 +2311,16 @@
         <v>1</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="I3" s="0"/>
       <c r="J3" s="0"/>
@@ -2336,13 +2342,13 @@
         <v>0</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2362,22 +2368,22 @@
         <v>0</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2397,22 +2403,22 @@
         <v>18</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2432,22 +2438,22 @@
         <v>1</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2467,22 +2473,22 @@
         <v>0</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2502,67 +2508,67 @@
         <v>11</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="R9" s="1" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="S9" s="1" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="T9" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="V9" s="1" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="W9" s="1" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="X9" s="1" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="Y9" s="1" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2582,22 +2588,22 @@
         <v>26</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2617,22 +2623,22 @@
         <v>0</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2652,22 +2658,22 @@
         <v>0</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2687,22 +2693,22 @@
         <v>1</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2722,28 +2728,28 @@
         <v>11</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2763,19 +2769,19 @@
         <v>18</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2795,19 +2801,19 @@
         <v>35</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2827,19 +2833,19 @@
         <v>35</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2859,19 +2865,19 @@
         <v>35</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2891,16 +2897,16 @@
         <v>18</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2920,10 +2926,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2943,10 +2949,10 @@
         <v>1</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2966,10 +2972,10 @@
         <v>11</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2989,19 +2995,19 @@
         <v>18</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3021,19 +3027,19 @@
         <v>18</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3053,19 +3059,19 @@
         <v>18</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3085,10 +3091,10 @@
         <v>18</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3108,22 +3114,22 @@
         <v>0</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3143,19 +3149,19 @@
         <v>18</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3175,10 +3181,10 @@
         <v>0</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3198,22 +3204,22 @@
         <v>1</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3233,25 +3239,25 @@
         <v>1</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3271,25 +3277,25 @@
         <v>26</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3309,10 +3315,10 @@
         <v>0</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3332,10 +3338,10 @@
         <v>0</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3355,34 +3361,34 @@
         <v>35</v>
       </c>
       <c r="E35" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="J35" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="K35" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="F35" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="G35" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="H35" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="I35" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="J35" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="K35" s="1" t="s">
-        <v>133</v>
-      </c>
       <c r="L35" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="M35" s="1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3402,34 +3408,34 @@
         <v>59</v>
       </c>
       <c r="E36" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="J36" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="K36" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="F36" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="G36" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="H36" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="I36" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="J36" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="K36" s="1" t="s">
-        <v>133</v>
-      </c>
       <c r="L36" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="M36" s="1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="N36" s="1" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3449,22 +3455,22 @@
         <v>1</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3484,10 +3490,10 @@
         <v>1</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3524,22 +3530,22 @@
         <v>1</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3559,22 +3565,22 @@
         <v>1</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J41" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3594,10 +3600,10 @@
         <v>1</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3617,22 +3623,22 @@
         <v>1</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3652,25 +3658,25 @@
         <v>11</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3690,22 +3696,22 @@
         <v>1</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I45" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3725,10 +3731,10 @@
         <v>1</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3748,28 +3754,28 @@
         <v>11</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="I47" s="1" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="J47" s="1" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="K47" s="1" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="L47" s="1" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3789,16 +3795,16 @@
         <v>1</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3832,19 +3838,19 @@
         <v>6</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E50" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="G50" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="H50" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="F50" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="G50" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="H50" s="1" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3864,22 +3870,22 @@
         <v>0</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J51" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3899,10 +3905,10 @@
         <v>1</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3922,22 +3928,22 @@
         <v>1</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I53" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J53" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3954,34 +3960,34 @@
         <v>4</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="I54" s="1" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="J54" s="1" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="K54" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="L54" s="1" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="M54" s="1" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4001,22 +4007,22 @@
         <v>0</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I55" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J55" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4036,22 +4042,22 @@
         <v>0</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I56" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J56" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4071,22 +4077,22 @@
         <v>0</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I57" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J57" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4106,22 +4112,22 @@
         <v>1</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J58" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4141,10 +4147,10 @@
         <v>1</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4164,22 +4170,22 @@
         <v>0</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I60" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J60" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4199,22 +4205,22 @@
         <v>2</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I61" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J61" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4234,22 +4240,22 @@
         <v>1</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I62" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J62" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4266,28 +4272,28 @@
         <v>1</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="I63" s="1" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="J63" s="1" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="K63" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4307,22 +4313,22 @@
         <v>1</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I64" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J64" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4342,16 +4348,16 @@
         <v>1</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4371,16 +4377,16 @@
         <v>0</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4400,25 +4406,25 @@
         <v>0</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H67" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="I67" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="J67" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="K67" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="I67" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="J67" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="K67" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4438,7 +4444,7 @@
         <v>0</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4455,25 +4461,25 @@
         <v>3</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E69" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="F69" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="G69" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="H69" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="F69" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="G69" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="H69" s="1" t="s">
-        <v>133</v>
-      </c>
       <c r="I69" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="J69" s="1" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4493,25 +4499,25 @@
         <v>0</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G70" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H70" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="I70" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="J70" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="K70" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="I70" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="J70" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="K70" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4531,10 +4537,10 @@
         <v>26</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4554,7 +4560,7 @@
         <v>0</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4574,10 +4580,10 @@
         <v>2</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] [SW-5583] Add necessary support for new parameters introduced by Glow for Convolution and derivated Operands. New parameters FusedActivation and FusedActivationArgs.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="199">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -98,274 +98,277 @@
     <t xml:space="preserve">Convolution</t>
   </si>
   <si>
+    <t xml:space="preserve">Kernels, Strides, Pads, Group, Dilation, FusedActivation, FusedActivationArgs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Convolution3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kernels, Strides, Pads, Group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tensorized</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CrossEntropyLoss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dequantize</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementAdd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementCmpEQ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementCmpLT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementCmpLTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementDiv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementExp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementIsNaN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementLog</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementMax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementMin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementMul</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementPow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementSelect</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementSub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EmbeddingBag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HasEndOffset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ExtractTensor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Offsets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FullyConnected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FusedRowwiseQuantizedSparseLengthsSum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FusedRowwiseQuantizedSparseLengthsWeightedSum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gather</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BatchDims</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GatherRanges</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsertTensor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Offsets, Count,Axis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int8Converter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IntLookupTable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NONE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LengthsSum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LengthsToRanges</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LocalResponseNormalization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HalfWindowSize, Alpha, Beta, K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MatMul</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transposed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MaxPool</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kernels, Strides, Pads,Layout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MaxSplat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aligned32Bytes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modulo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Divisor, SignFollowDivisor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quantize</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RescaleQuantized</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RowwiseQuantizedFullyConnected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RowwiseQuantizedSparseLengthsWeightedSum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ScatterData</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sigmoid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SoftMax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SparseLengthsWeightedSum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SparseToDense</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SparseToDenseMask</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mask</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Splat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Syncopy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SyncOffset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tanh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TensorView</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TopK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transpose</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shuffle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MaxPoolWithArgMax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kernels, Strides, Pads, Layout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BatchedReduceMin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Axes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CumSum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exclusive, Reverse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SpaceToDepth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BlockSize</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ResizeNearest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RszScale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LengthsRangeFill</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SparseLengthsSum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ResizeBilinear</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ChannelWiseQuantizedConvolution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ConvTranspose</t>
+  </si>
+  <si>
     <t xml:space="preserve">Kernels, Strides, Pads, Group, Dilation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0,3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Convolution3D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kernels, Strides, Pads, Group</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Copy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tensorized</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CrossEntropyLoss</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dequantize</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementAdd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementCmpEQ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementCmpLT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementCmpLTE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementDiv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementExp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementIsNaN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementLog</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementMax</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementMin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementMul</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementPow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementSelect</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ElementSub</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EmbeddingBag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HasEndOffset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ExtractTensor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Offsets</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flip</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FullyConnected</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FusedRowwiseQuantizedSparseLengthsSum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FusedRowwiseQuantizedSparseLengthsWeightedSum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gather</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BatchDims</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GatherRanges</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsertTensor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Offsets, Count,Axis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int8Converter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IntLookupTable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NONE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LengthsSum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LengthsToRanges</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LocalResponseNormalization</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HalfWindowSize, Alpha, Beta, K</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MatMul</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Transposed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MaxPool</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kernels, Strides, Pads,Layout</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MaxSplat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aligned32Bytes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modulo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Divisor, SignFollowDivisor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quantize</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RescaleQuantized</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RowwiseQuantizedFullyConnected</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RowwiseQuantizedSparseLengthsWeightedSum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0,5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ScatterData</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sigmoid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SoftMax</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SparseLengthsWeightedSum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SparseToDense</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SparseToDenseMask</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mask</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Splat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Syncopy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SyncOffset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tanh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TensorView</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TopK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Transpose</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shuffle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MaxPoolWithArgMax</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kernels, Strides, Pads, Layout</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0,2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BatchedReduceMin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Axes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CumSum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exclusive, Reverse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SpaceToDepth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BlockSize</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ResizeNearest</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RszScale</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LengthsRangeFill</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SparseLengthsSum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ResizeBilinear</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ChannelWiseQuantizedConvolution</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ConvTranspose</t>
   </si>
   <si>
     <t xml:space="preserve">NonMaxSuppression</t>
@@ -2178,7 +2181,7 @@
         <v>3</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>25</v>
+        <v>115</v>
       </c>
       <c r="E72" s="1" t="n">
         <v>0</v>
@@ -2189,7 +2192,7 @@
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B73" s="1" t="n">
         <v>2</v>
@@ -2198,7 +2201,7 @@
         <v>2</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E73" s="1" t="n">
         <v>0</v>
@@ -2276,22 +2279,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2311,16 +2314,16 @@
         <v>1</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="I3" s="0"/>
       <c r="J3" s="0"/>
@@ -2342,13 +2345,13 @@
         <v>0</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2368,22 +2371,22 @@
         <v>0</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2403,22 +2406,22 @@
         <v>18</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2438,22 +2441,22 @@
         <v>1</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2473,22 +2476,22 @@
         <v>0</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2508,67 +2511,67 @@
         <v>11</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L9" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="N9" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="O9" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="M9" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="N9" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="O9" s="1" t="s">
-        <v>123</v>
-      </c>
       <c r="P9" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="R9" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="S9" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="T9" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="V9" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="W9" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="X9" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="Y9" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2588,22 +2591,22 @@
         <v>26</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2623,22 +2626,22 @@
         <v>0</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2658,22 +2661,22 @@
         <v>0</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2693,22 +2696,22 @@
         <v>1</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2728,28 +2731,28 @@
         <v>11</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2769,19 +2772,19 @@
         <v>18</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2801,19 +2804,19 @@
         <v>35</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2833,19 +2836,19 @@
         <v>35</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2865,19 +2868,19 @@
         <v>35</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2897,16 +2900,16 @@
         <v>18</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2926,10 +2929,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2949,10 +2952,10 @@
         <v>1</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2972,10 +2975,10 @@
         <v>11</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2995,19 +2998,19 @@
         <v>18</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3027,19 +3030,19 @@
         <v>18</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3059,19 +3062,19 @@
         <v>18</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3091,10 +3094,10 @@
         <v>18</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3114,22 +3117,22 @@
         <v>0</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3149,19 +3152,19 @@
         <v>18</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3181,10 +3184,10 @@
         <v>0</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3204,22 +3207,22 @@
         <v>1</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3239,25 +3242,25 @@
         <v>1</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3277,25 +3280,25 @@
         <v>26</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3315,10 +3318,10 @@
         <v>0</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3338,10 +3341,10 @@
         <v>0</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3361,34 +3364,34 @@
         <v>35</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="L35" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="M35" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3408,34 +3411,34 @@
         <v>59</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K36" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="L36" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="M36" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="N36" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3455,22 +3458,22 @@
         <v>1</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3490,10 +3493,10 @@
         <v>1</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3530,22 +3533,22 @@
         <v>1</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3565,22 +3568,22 @@
         <v>1</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J41" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3600,10 +3603,10 @@
         <v>1</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3623,22 +3626,22 @@
         <v>1</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3658,25 +3661,25 @@
         <v>11</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3696,22 +3699,22 @@
         <v>1</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I45" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3731,10 +3734,10 @@
         <v>1</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3754,28 +3757,28 @@
         <v>11</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I47" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="J47" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="K47" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="L47" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3795,16 +3798,16 @@
         <v>1</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3841,16 +3844,16 @@
         <v>82</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3870,22 +3873,22 @@
         <v>0</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J51" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3905,10 +3908,10 @@
         <v>1</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3928,22 +3931,22 @@
         <v>1</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I53" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J53" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3963,31 +3966,31 @@
         <v>87</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I54" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J54" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K54" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L54" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="M54" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4007,22 +4010,22 @@
         <v>0</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I55" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J55" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4042,22 +4045,22 @@
         <v>0</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I56" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J56" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4077,22 +4080,22 @@
         <v>0</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I57" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J57" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4112,22 +4115,22 @@
         <v>1</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J58" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4147,10 +4150,10 @@
         <v>1</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4170,22 +4173,22 @@
         <v>0</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I60" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J60" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4205,22 +4208,22 @@
         <v>2</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I61" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J61" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4240,22 +4243,22 @@
         <v>1</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I62" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J62" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4275,25 +4278,25 @@
         <v>101</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="I63" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J63" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="K63" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4313,22 +4316,22 @@
         <v>1</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I64" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J64" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4348,16 +4351,16 @@
         <v>1</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G65" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="H65" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="H65" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4377,16 +4380,16 @@
         <v>0</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4406,25 +4409,25 @@
         <v>0</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H67" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="I67" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="J67" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="I67" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="J67" s="1" t="s">
+      <c r="K67" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="K67" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4444,7 +4447,7 @@
         <v>0</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4464,22 +4467,22 @@
         <v>101</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I69" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J69" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4499,25 +4502,25 @@
         <v>0</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G70" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H70" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="I70" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="J70" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="I70" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="J70" s="1" t="s">
+      <c r="K70" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="K70" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4537,10 +4540,10 @@
         <v>26</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4560,7 +4563,7 @@
         <v>0</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4580,10 +4583,10 @@
         <v>2</v>
       </c>
       <c r="E73" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F73" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="F73" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] [SW-5157] Remove obsolete MatMulTransposed code
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="198">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -231,9 +231,6 @@
   </si>
   <si>
     <t xml:space="preserve">MatMul</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Transposed</t>
   </si>
   <si>
     <t xml:space="preserve">MaxPool</t>
@@ -1618,9 +1615,6 @@
       <c r="C43" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D43" s="1" t="s">
-        <v>70</v>
-      </c>
       <c r="E43" s="1" t="n">
         <v>1</v>
       </c>
@@ -1630,16 +1624,16 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B44" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="1" t="s">
         <v>71</v>
-      </c>
-      <c r="B44" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C44" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>11</v>
@@ -1650,22 +1644,22 @@
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B45" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B45" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C45" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D45" s="1" t="s">
+      <c r="E45" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F45" s="1" t="s">
         <v>74</v>
-      </c>
-      <c r="E45" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>75</v>
       </c>
       <c r="G45" s="1" t="s">
         <v>15</v>
@@ -1673,16 +1667,16 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B46" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="1" t="s">
         <v>76</v>
-      </c>
-      <c r="B46" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C46" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D46" s="1" t="s">
-        <v>77</v>
       </c>
       <c r="E46" s="1" t="n">
         <v>1</v>
@@ -1693,7 +1687,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B47" s="1" t="n">
         <v>1</v>
@@ -1710,7 +1704,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B48" s="1" t="n">
         <v>1</v>
@@ -1727,7 +1721,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B49" s="1" t="n">
         <v>1</v>
@@ -1739,7 +1733,7 @@
         <v>64</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G49" s="1" t="s">
         <v>15</v>
@@ -1747,7 +1741,7 @@
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B50" s="1" t="n">
         <v>1</v>
@@ -1756,7 +1750,7 @@
         <v>6</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>23</v>
@@ -1767,7 +1761,7 @@
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B51" s="1" t="n">
         <v>1</v>
@@ -1784,7 +1778,7 @@
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B52" s="1" t="n">
         <v>1</v>
@@ -1801,7 +1795,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B53" s="1" t="n">
         <v>1</v>
@@ -1821,7 +1815,7 @@
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B54" s="1" t="n">
         <v>1</v>
@@ -1830,7 +1824,7 @@
         <v>4</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F54" s="1" t="s">
         <v>14</v>
@@ -1841,7 +1835,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B55" s="1" t="n">
         <v>1</v>
@@ -1858,7 +1852,7 @@
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B56" s="1" t="n">
         <v>1</v>
@@ -1867,7 +1861,7 @@
         <v>4</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E56" s="1" t="n">
         <v>0</v>
@@ -1878,7 +1872,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B57" s="1" t="n">
         <v>1</v>
@@ -1887,7 +1881,7 @@
         <v>0</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E57" s="1" t="n">
         <v>0</v>
@@ -1898,16 +1892,16 @@
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B58" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="B58" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C58" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>93</v>
       </c>
       <c r="E58" s="1" t="n">
         <v>1</v>
@@ -1918,7 +1912,7 @@
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B59" s="1" t="n">
         <v>1</v>
@@ -1935,7 +1929,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B60" s="1" t="n">
         <v>1</v>
@@ -1955,7 +1949,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B61" s="1" t="n">
         <v>2</v>
@@ -1964,7 +1958,7 @@
         <v>1</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E61" s="1" t="n">
         <v>2</v>
@@ -1975,22 +1969,22 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B62" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C62" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B62" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C62" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D62" s="1" t="s">
-        <v>98</v>
-      </c>
       <c r="E62" s="1" t="n">
         <v>1</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G62" s="1" t="s">
         <v>15</v>
@@ -1998,19 +1992,19 @@
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B63" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C63" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D63" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B63" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C63" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D63" s="1" t="s">
+      <c r="E63" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="E63" s="1" t="s">
-        <v>101</v>
       </c>
       <c r="G63" s="1" t="s">
         <v>8</v>
@@ -2018,16 +2012,16 @@
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B64" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C64" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" s="1" t="s">
         <v>102</v>
-      </c>
-      <c r="B64" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C64" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D64" s="1" t="s">
-        <v>103</v>
       </c>
       <c r="E64" s="1" t="n">
         <v>1</v>
@@ -2038,16 +2032,16 @@
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B65" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C65" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="B65" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C65" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D65" s="1" t="s">
-        <v>105</v>
       </c>
       <c r="E65" s="1" t="n">
         <v>1</v>
@@ -2058,16 +2052,16 @@
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B66" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C66" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="B66" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C66" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>107</v>
       </c>
       <c r="E66" s="1" t="n">
         <v>0</v>
@@ -2078,16 +2072,16 @@
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B67" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C67" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="B67" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C67" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D67" s="1" t="s">
-        <v>109</v>
       </c>
       <c r="E67" s="1" t="n">
         <v>0</v>
@@ -2098,7 +2092,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B68" s="1" t="n">
         <v>1</v>
@@ -2115,7 +2109,7 @@
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B69" s="1" t="n">
         <v>1</v>
@@ -2124,7 +2118,7 @@
         <v>3</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G69" s="1" t="s">
         <v>8</v>
@@ -2132,7 +2126,7 @@
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B70" s="1" t="n">
         <v>1</v>
@@ -2141,7 +2135,7 @@
         <v>1</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E70" s="1" t="n">
         <v>0</v>
@@ -2152,7 +2146,7 @@
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B71" s="1" t="n">
         <v>1</v>
@@ -2172,7 +2166,7 @@
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B72" s="1" t="n">
         <v>1</v>
@@ -2181,7 +2175,7 @@
         <v>3</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E72" s="1" t="n">
         <v>0</v>
@@ -2192,16 +2186,16 @@
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B73" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C73" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D73" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="B73" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C73" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="D73" s="1" t="s">
-        <v>117</v>
       </c>
       <c r="E73" s="1" t="n">
         <v>0</v>
@@ -2279,22 +2273,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2314,16 +2308,16 @@
         <v>1</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>126</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>127</v>
       </c>
       <c r="I3" s="0"/>
       <c r="J3" s="0"/>
@@ -2345,13 +2339,13 @@
         <v>0</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2371,22 +2365,22 @@
         <v>0</v>
       </c>
       <c r="E5" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="I5" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="J5" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2406,22 +2400,22 @@
         <v>18</v>
       </c>
       <c r="E6" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="I6" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="J6" s="1" t="s">
         <v>132</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2441,22 +2435,22 @@
         <v>1</v>
       </c>
       <c r="E7" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="I7" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="J7" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2476,22 +2470,22 @@
         <v>0</v>
       </c>
       <c r="E8" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="H8" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="I8" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="J8" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2511,67 +2505,67 @@
         <v>11</v>
       </c>
       <c r="E9" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="H9" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="I9" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="J9" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="K9" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="K9" s="1" t="s">
+      <c r="L9" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="M9" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="L9" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="M9" s="1" t="s">
+      <c r="N9" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="N9" s="1" t="s">
+      <c r="O9" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="P9" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="O9" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="P9" s="1" t="s">
+      <c r="Q9" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="Q9" s="1" t="s">
+      <c r="R9" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="R9" s="1" t="s">
+      <c r="S9" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="S9" s="1" t="s">
+      <c r="T9" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="T9" s="1" t="s">
+      <c r="U9" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="U9" s="1" t="s">
+      <c r="V9" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="V9" s="1" t="s">
+      <c r="W9" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="W9" s="1" t="s">
+      <c r="X9" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="X9" s="1" t="s">
+      <c r="Y9" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="Y9" s="1" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2591,22 +2585,22 @@
         <v>26</v>
       </c>
       <c r="E10" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="H10" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="H10" s="1" t="s">
+      <c r="I10" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="J10" s="1" t="s">
         <v>157</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2626,22 +2620,22 @@
         <v>0</v>
       </c>
       <c r="E11" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="H11" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="I11" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="J11" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2661,22 +2655,22 @@
         <v>0</v>
       </c>
       <c r="E12" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="H12" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H12" s="1" t="s">
+      <c r="I12" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I12" s="1" t="s">
+      <c r="J12" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2696,22 +2690,22 @@
         <v>1</v>
       </c>
       <c r="E13" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G13" s="1" t="s">
+      <c r="H13" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H13" s="1" t="s">
+      <c r="I13" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I13" s="1" t="s">
+      <c r="J13" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2731,28 +2725,28 @@
         <v>11</v>
       </c>
       <c r="E14" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="G14" s="1" t="s">
+      <c r="H14" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="I14" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="I14" s="1" t="s">
+      <c r="J14" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="J14" s="1" t="s">
+      <c r="K14" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="K14" s="1" t="s">
+      <c r="L14" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="L14" s="1" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2772,19 +2766,19 @@
         <v>18</v>
       </c>
       <c r="E15" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="G15" s="1" t="s">
-        <v>130</v>
-      </c>
       <c r="H15" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="I15" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2804,19 +2798,19 @@
         <v>35</v>
       </c>
       <c r="E16" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="G16" s="1" t="s">
-        <v>155</v>
-      </c>
       <c r="H16" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="I16" s="1" t="s">
         <v>169</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2836,19 +2830,19 @@
         <v>35</v>
       </c>
       <c r="E17" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="F17" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="G17" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="G17" s="1" t="s">
-        <v>155</v>
-      </c>
       <c r="H17" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="I17" s="1" t="s">
         <v>169</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2868,19 +2862,19 @@
         <v>35</v>
       </c>
       <c r="E18" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="G18" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="G18" s="1" t="s">
-        <v>155</v>
-      </c>
       <c r="H18" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="I18" s="1" t="s">
         <v>169</v>
-      </c>
-      <c r="I18" s="1" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2900,16 +2894,16 @@
         <v>18</v>
       </c>
       <c r="E19" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="G19" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="G19" s="1" t="s">
-        <v>130</v>
-      </c>
       <c r="H19" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2929,10 +2923,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2952,10 +2946,10 @@
         <v>1</v>
       </c>
       <c r="E21" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2975,10 +2969,10 @@
         <v>11</v>
       </c>
       <c r="E22" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2998,19 +2992,19 @@
         <v>18</v>
       </c>
       <c r="E23" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="F23" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="F23" s="1" t="s">
+      <c r="G23" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="G23" s="1" t="s">
-        <v>130</v>
-      </c>
       <c r="H23" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="I23" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="I23" s="1" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3030,19 +3024,19 @@
         <v>18</v>
       </c>
       <c r="E24" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="F24" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="F24" s="1" t="s">
+      <c r="G24" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="G24" s="1" t="s">
-        <v>130</v>
-      </c>
       <c r="H24" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="I24" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3062,19 +3056,19 @@
         <v>18</v>
       </c>
       <c r="E25" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="F25" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="F25" s="1" t="s">
+      <c r="G25" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="G25" s="1" t="s">
-        <v>130</v>
-      </c>
       <c r="H25" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="I25" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3094,10 +3088,10 @@
         <v>18</v>
       </c>
       <c r="E26" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="F26" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3117,22 +3111,22 @@
         <v>0</v>
       </c>
       <c r="E27" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F27" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F27" s="1" t="s">
+      <c r="G27" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G27" s="1" t="s">
+      <c r="H27" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H27" s="1" t="s">
+      <c r="I27" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I27" s="1" t="s">
+      <c r="J27" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J27" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3152,19 +3146,19 @@
         <v>18</v>
       </c>
       <c r="E28" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="F28" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="G28" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="G28" s="1" t="s">
-        <v>130</v>
-      </c>
       <c r="H28" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="I28" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3184,10 +3178,10 @@
         <v>0</v>
       </c>
       <c r="E29" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F29" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3207,22 +3201,22 @@
         <v>1</v>
       </c>
       <c r="E30" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F30" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="G30" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G30" s="1" t="s">
+      <c r="H30" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H30" s="1" t="s">
+      <c r="I30" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I30" s="1" t="s">
+      <c r="J30" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J30" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3242,25 +3236,25 @@
         <v>1</v>
       </c>
       <c r="E31" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F31" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F31" s="1" t="s">
+      <c r="G31" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G31" s="1" t="s">
+      <c r="H31" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H31" s="1" t="s">
+      <c r="I31" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I31" s="1" t="s">
+      <c r="J31" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="J31" s="1" t="s">
-        <v>123</v>
-      </c>
       <c r="K31" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3280,25 +3274,25 @@
         <v>26</v>
       </c>
       <c r="E32" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="F32" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="F32" s="1" t="s">
+      <c r="G32" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="G32" s="1" t="s">
+      <c r="H32" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="H32" s="1" t="s">
+      <c r="I32" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="J32" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="I32" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="J32" s="1" t="s">
+      <c r="K32" s="1" t="s">
         <v>157</v>
-      </c>
-      <c r="K32" s="1" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3318,10 +3312,10 @@
         <v>0</v>
       </c>
       <c r="E33" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F33" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3341,10 +3335,10 @@
         <v>0</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3364,34 +3358,34 @@
         <v>35</v>
       </c>
       <c r="E35" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="J35" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="F35" s="1" t="s">
+      <c r="K35" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="G35" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="H35" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="I35" s="1" t="s">
+      <c r="L35" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="J35" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="K35" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="L35" s="1" t="s">
+      <c r="M35" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="M35" s="1" t="s">
+      <c r="N35" s="1" t="s">
         <v>178</v>
-      </c>
-      <c r="N35" s="1" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3411,34 +3405,34 @@
         <v>59</v>
       </c>
       <c r="E36" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="J36" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="F36" s="1" t="s">
+      <c r="K36" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="G36" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="H36" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="I36" s="1" t="s">
+      <c r="L36" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="J36" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="K36" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="L36" s="1" t="s">
+      <c r="M36" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="M36" s="1" t="s">
+      <c r="N36" s="1" t="s">
         <v>178</v>
-      </c>
-      <c r="N36" s="1" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3458,22 +3452,22 @@
         <v>1</v>
       </c>
       <c r="E37" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F37" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F37" s="1" t="s">
+      <c r="G37" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G37" s="1" t="s">
+      <c r="H37" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H37" s="1" t="s">
+      <c r="I37" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I37" s="1" t="s">
+      <c r="J37" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J37" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3493,10 +3487,10 @@
         <v>1</v>
       </c>
       <c r="E38" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F38" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3533,22 +3527,22 @@
         <v>1</v>
       </c>
       <c r="E40" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F40" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F40" s="1" t="s">
+      <c r="G40" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G40" s="1" t="s">
+      <c r="H40" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H40" s="1" t="s">
+      <c r="I40" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I40" s="1" t="s">
+      <c r="J40" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J40" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3568,22 +3562,22 @@
         <v>1</v>
       </c>
       <c r="E41" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F41" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F41" s="1" t="s">
+      <c r="G41" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G41" s="1" t="s">
+      <c r="H41" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H41" s="1" t="s">
+      <c r="I41" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I41" s="1" t="s">
+      <c r="J41" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J41" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3603,10 +3597,10 @@
         <v>1</v>
       </c>
       <c r="E42" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F42" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="F42" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3626,22 +3620,22 @@
         <v>1</v>
       </c>
       <c r="E43" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F43" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F43" s="1" t="s">
+      <c r="G43" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G43" s="1" t="s">
+      <c r="H43" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H43" s="1" t="s">
+      <c r="I43" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I43" s="1" t="s">
+      <c r="J43" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J43" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3661,25 +3655,25 @@
         <v>11</v>
       </c>
       <c r="E44" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="F44" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="F44" s="1" t="s">
+      <c r="G44" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="H44" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="G44" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="H44" s="1" t="s">
+      <c r="I44" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="I44" s="1" t="s">
+      <c r="J44" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="J44" s="1" t="s">
-        <v>184</v>
-      </c>
       <c r="K44" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3699,22 +3693,22 @@
         <v>1</v>
       </c>
       <c r="E45" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F45" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F45" s="1" t="s">
+      <c r="G45" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G45" s="1" t="s">
+      <c r="H45" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H45" s="1" t="s">
+      <c r="I45" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I45" s="1" t="s">
+      <c r="J45" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J45" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3734,10 +3728,10 @@
         <v>1</v>
       </c>
       <c r="E46" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="F46" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="F46" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3757,28 +3751,28 @@
         <v>11</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F47" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="G47" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="G47" s="1" t="s">
+      <c r="H47" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="H47" s="1" t="s">
+      <c r="I47" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="I47" s="1" t="s">
+      <c r="J47" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="J47" s="1" t="s">
+      <c r="K47" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="K47" s="1" t="s">
+      <c r="L47" s="1" t="s">
         <v>190</v>
-      </c>
-      <c r="L47" s="1" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3798,16 +3792,16 @@
         <v>1</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3841,19 +3835,19 @@
         <v>6</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E50" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="F50" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="F50" s="1" t="s">
-        <v>139</v>
-      </c>
       <c r="G50" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="H50" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="H50" s="1" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3873,22 +3867,22 @@
         <v>0</v>
       </c>
       <c r="E51" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F51" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F51" s="1" t="s">
+      <c r="G51" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G51" s="1" t="s">
+      <c r="H51" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H51" s="1" t="s">
+      <c r="I51" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I51" s="1" t="s">
+      <c r="J51" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J51" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3908,10 +3902,10 @@
         <v>1</v>
       </c>
       <c r="E52" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F52" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="F52" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3931,22 +3925,22 @@
         <v>1</v>
       </c>
       <c r="E53" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F53" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F53" s="1" t="s">
+      <c r="G53" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G53" s="1" t="s">
+      <c r="H53" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H53" s="1" t="s">
+      <c r="I53" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I53" s="1" t="s">
+      <c r="J53" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J53" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3963,34 +3957,34 @@
         <v>4</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E54" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="F54" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="F54" s="1" t="s">
+      <c r="G54" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="G54" s="1" t="s">
+      <c r="H54" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="H54" s="1" t="s">
+      <c r="I54" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="I54" s="1" t="s">
+      <c r="J54" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="J54" s="1" t="s">
-        <v>198</v>
-      </c>
       <c r="K54" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="L54" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="M54" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4010,22 +4004,22 @@
         <v>0</v>
       </c>
       <c r="E55" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F55" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F55" s="1" t="s">
+      <c r="G55" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G55" s="1" t="s">
+      <c r="H55" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H55" s="1" t="s">
+      <c r="I55" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I55" s="1" t="s">
+      <c r="J55" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J55" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4045,22 +4039,22 @@
         <v>0</v>
       </c>
       <c r="E56" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F56" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F56" s="1" t="s">
+      <c r="G56" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G56" s="1" t="s">
+      <c r="H56" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H56" s="1" t="s">
+      <c r="I56" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I56" s="1" t="s">
+      <c r="J56" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J56" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4080,22 +4074,22 @@
         <v>0</v>
       </c>
       <c r="E57" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F57" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F57" s="1" t="s">
+      <c r="G57" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G57" s="1" t="s">
+      <c r="H57" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H57" s="1" t="s">
+      <c r="I57" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I57" s="1" t="s">
+      <c r="J57" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J57" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4115,22 +4109,22 @@
         <v>1</v>
       </c>
       <c r="E58" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F58" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F58" s="1" t="s">
+      <c r="G58" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G58" s="1" t="s">
+      <c r="H58" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H58" s="1" t="s">
+      <c r="I58" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I58" s="1" t="s">
+      <c r="J58" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J58" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4150,10 +4144,10 @@
         <v>1</v>
       </c>
       <c r="E59" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F59" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="F59" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4173,22 +4167,22 @@
         <v>0</v>
       </c>
       <c r="E60" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F60" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F60" s="1" t="s">
+      <c r="G60" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G60" s="1" t="s">
+      <c r="H60" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H60" s="1" t="s">
+      <c r="I60" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I60" s="1" t="s">
+      <c r="J60" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J60" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4208,22 +4202,22 @@
         <v>2</v>
       </c>
       <c r="E61" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F61" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F61" s="1" t="s">
+      <c r="G61" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G61" s="1" t="s">
+      <c r="H61" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H61" s="1" t="s">
+      <c r="I61" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I61" s="1" t="s">
+      <c r="J61" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J61" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4243,22 +4237,22 @@
         <v>1</v>
       </c>
       <c r="E62" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F62" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F62" s="1" t="s">
+      <c r="G62" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G62" s="1" t="s">
+      <c r="H62" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H62" s="1" t="s">
+      <c r="I62" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I62" s="1" t="s">
+      <c r="J62" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J62" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4275,28 +4269,28 @@
         <v>1</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E63" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="F63" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="F63" s="1" t="s">
+      <c r="G63" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="H63" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="G63" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="H63" s="1" t="s">
+      <c r="I63" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="I63" s="1" t="s">
+      <c r="J63" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="J63" s="1" t="s">
-        <v>184</v>
-      </c>
       <c r="K63" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4316,22 +4310,22 @@
         <v>1</v>
       </c>
       <c r="E64" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F64" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F64" s="1" t="s">
+      <c r="G64" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G64" s="1" t="s">
+      <c r="H64" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H64" s="1" t="s">
+      <c r="I64" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I64" s="1" t="s">
+      <c r="J64" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J64" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4351,16 +4345,16 @@
         <v>1</v>
       </c>
       <c r="E65" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F65" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F65" s="1" t="s">
-        <v>119</v>
-      </c>
       <c r="G65" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4380,16 +4374,16 @@
         <v>0</v>
       </c>
       <c r="E66" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F66" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F66" s="1" t="s">
+      <c r="G66" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G66" s="1" t="s">
+      <c r="H66" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="H66" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4409,25 +4403,25 @@
         <v>0</v>
       </c>
       <c r="E67" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F67" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F67" s="1" t="s">
+      <c r="G67" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G67" s="1" t="s">
+      <c r="H67" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="I67" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="J67" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="K67" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="H67" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="I67" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="J67" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="K67" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4447,7 +4441,7 @@
         <v>0</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4464,25 +4458,25 @@
         <v>3</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E69" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="F69" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="F69" s="1" t="s">
-        <v>139</v>
-      </c>
       <c r="G69" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="H69" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="H69" s="1" t="s">
-        <v>136</v>
-      </c>
       <c r="I69" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J69" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4502,25 +4496,25 @@
         <v>0</v>
       </c>
       <c r="E70" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F70" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F70" s="1" t="s">
+      <c r="G70" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G70" s="1" t="s">
+      <c r="H70" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="I70" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="J70" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="K70" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="H70" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="I70" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="J70" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="K70" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4540,10 +4534,10 @@
         <v>26</v>
       </c>
       <c r="E71" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="F71" s="1" t="s">
         <v>155</v>
-      </c>
-      <c r="F71" s="1" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4563,7 +4557,7 @@
         <v>0</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4583,10 +4577,10 @@
         <v>2</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] [SW-5678] Deprecate CheckSum custom operator
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="197">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -84,9 +84,6 @@
   </si>
   <si>
     <t xml:space="preserve">Axis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Checksum</t>
   </si>
   <si>
     <t xml:space="preserve">ConvertTo</t>
@@ -938,46 +935,52 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C8" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="1" t="n">
-        <v>0</v>
+      <c r="E8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>22</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="B9" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>1</v>
@@ -986,56 +989,50 @@
         <v>3</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>23</v>
+        <v>27</v>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="E11" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="F11" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="G11" s="1" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1046,10 +1043,10 @@
         <v>1</v>
       </c>
       <c r="C13" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E13" s="1" t="n">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>8</v>
@@ -1063,13 +1060,16 @@
         <v>1</v>
       </c>
       <c r="C14" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>11</v>
+        <v>18</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>22</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1083,30 +1083,30 @@
         <v>2</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B16" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C16" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>35</v>
-      </c>
       <c r="F16" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>15</v>
@@ -1123,10 +1123,10 @@
         <v>2</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>15</v>
@@ -1143,16 +1143,16 @@
         <v>2</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G18" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
         <v>38</v>
       </c>
@@ -1160,16 +1160,13 @@
         <v>1</v>
       </c>
       <c r="C19" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>23</v>
+        <v>1</v>
+      </c>
+      <c r="E19" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1189,7 +1186,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
         <v>40</v>
       </c>
@@ -1199,8 +1196,8 @@
       <c r="C21" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E21" s="1" t="n">
-        <v>1</v>
+      <c r="E21" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="G21" s="1" t="s">
         <v>8</v>
@@ -1214,13 +1211,16 @@
         <v>1</v>
       </c>
       <c r="C22" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>11</v>
+        <v>18</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>22</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1237,7 +1237,7 @@
         <v>18</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G23" s="1" t="s">
         <v>15</v>
@@ -1257,7 +1257,7 @@
         <v>18</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G24" s="1" t="s">
         <v>15</v>
@@ -1277,13 +1277,13 @@
         <v>18</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G25" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
         <v>45</v>
       </c>
@@ -1291,19 +1291,16 @@
         <v>1</v>
       </c>
       <c r="C26" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>23</v>
+        <v>3</v>
+      </c>
+      <c r="E26" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
         <v>46</v>
       </c>
@@ -1311,13 +1308,16 @@
         <v>1</v>
       </c>
       <c r="C27" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="E27" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>22</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1328,44 +1328,44 @@
         <v>1</v>
       </c>
       <c r="C28" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>18</v>
+        <v>4</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E28" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G28" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B29" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C29" s="1" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E29" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B30" s="1" t="n">
         <v>1</v>
@@ -1374,7 +1374,7 @@
         <v>1</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="E30" s="1" t="n">
         <v>1</v>
@@ -1391,19 +1391,16 @@
         <v>1</v>
       </c>
       <c r="C31" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E31" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="G31" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
         <v>53</v>
       </c>
@@ -1413,8 +1410,8 @@
       <c r="C32" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E32" s="1" t="s">
-        <v>26</v>
+      <c r="E32" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="G32" s="1" t="s">
         <v>8</v>
@@ -1428,7 +1425,7 @@
         <v>1</v>
       </c>
       <c r="C33" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E33" s="1" t="n">
         <v>0</v>
@@ -1437,7 +1434,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
         <v>55</v>
       </c>
@@ -1445,10 +1442,13 @@
         <v>1</v>
       </c>
       <c r="C34" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E34" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>34</v>
       </c>
       <c r="G34" s="1" t="s">
         <v>8</v>
@@ -1456,19 +1456,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B35" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C35" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D35" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="E35" s="1" t="s">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="G35" s="1" t="s">
         <v>8</v>
@@ -1476,42 +1473,42 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B36" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C36" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>59</v>
+        <v>1</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E36" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="G36" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B37" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" s="1" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B37" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C37" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="E37" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G37" s="1" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1522,18 +1519,18 @@
         <v>1</v>
       </c>
       <c r="C38" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E38" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>63</v>
       </c>
       <c r="G38" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B39" s="1" t="n">
         <v>1</v>
@@ -1541,14 +1538,14 @@
       <c r="C39" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E39" s="1" t="s">
-        <v>64</v>
+      <c r="E39" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="G39" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
         <v>65</v>
       </c>
@@ -1556,7 +1553,7 @@
         <v>1</v>
       </c>
       <c r="C40" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E40" s="1" t="n">
         <v>1</v>
@@ -1565,47 +1562,47 @@
         <v>8</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
         <v>66</v>
       </c>
       <c r="B41" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C41" s="1" t="n">
         <v>1</v>
       </c>
+      <c r="D41" s="1" t="s">
+        <v>67</v>
+      </c>
       <c r="E41" s="1" t="n">
         <v>1</v>
       </c>
+      <c r="F41" s="1" t="s">
+        <v>22</v>
+      </c>
       <c r="G41" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B42" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E42" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="B42" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C42" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E42" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F42" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="G42" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
         <v>69</v>
       </c>
@@ -1613,18 +1610,21 @@
         <v>1</v>
       </c>
       <c r="C43" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E43" s="1" t="n">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="G43" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B44" s="1" t="n">
         <v>1</v>
@@ -1633,41 +1633,41 @@
         <v>1</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>11</v>
+        <v>72</v>
+      </c>
+      <c r="E44" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>73</v>
       </c>
       <c r="G44" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B45" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E45" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" s="1" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="B45" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C45" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="E45" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="G45" s="1" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B46" s="1" t="n">
         <v>1</v>
@@ -1675,11 +1675,8 @@
       <c r="C46" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D46" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="E46" s="1" t="n">
-        <v>1</v>
+      <c r="E46" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="G46" s="1" t="s">
         <v>8</v>
@@ -1695,8 +1692,8 @@
       <c r="C47" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E47" s="1" t="s">
-        <v>11</v>
+      <c r="E47" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="G47" s="1" t="s">
         <v>8</v>
@@ -1710,16 +1707,19 @@
         <v>1</v>
       </c>
       <c r="C48" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E48" s="1" t="n">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>73</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
         <v>79</v>
       </c>
@@ -1727,13 +1727,13 @@
         <v>1</v>
       </c>
       <c r="C49" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>74</v>
+        <v>22</v>
       </c>
       <c r="G49" s="1" t="s">
         <v>15</v>
@@ -1741,22 +1741,19 @@
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B50" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C50" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="E50" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F50" s="1" t="s">
-        <v>23</v>
+        <v>2</v>
+      </c>
+      <c r="E50" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1767,16 +1764,16 @@
         <v>1</v>
       </c>
       <c r="C51" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E51" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G51" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
         <v>83</v>
       </c>
@@ -1789,11 +1786,14 @@
       <c r="E52" s="1" t="n">
         <v>1</v>
       </c>
+      <c r="F52" s="1" t="s">
+        <v>22</v>
+      </c>
       <c r="G52" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
         <v>84</v>
       </c>
@@ -1801,39 +1801,36 @@
         <v>1</v>
       </c>
       <c r="C53" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E53" s="1" t="n">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>85</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="G53" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B54" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C54" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E54" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>14</v>
+        <v>2</v>
+      </c>
+      <c r="E54" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
         <v>87</v>
       </c>
@@ -1841,7 +1838,10 @@
         <v>1</v>
       </c>
       <c r="C55" s="1" t="n">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>88</v>
       </c>
       <c r="E55" s="1" t="n">
         <v>0</v>
@@ -1850,18 +1850,18 @@
         <v>8</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B56" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C56" s="1" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="E56" s="1" t="n">
         <v>0</v>
@@ -1870,7 +1870,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
         <v>90</v>
       </c>
@@ -1878,13 +1878,13 @@
         <v>1</v>
       </c>
       <c r="C57" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="E57" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G57" s="1" t="s">
         <v>8</v>
@@ -1892,16 +1892,13 @@
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B58" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C58" s="1" t="n">
         <v>1</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>92</v>
       </c>
       <c r="E58" s="1" t="n">
         <v>1</v>
@@ -1910,7 +1907,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
         <v>93</v>
       </c>
@@ -1920,8 +1917,11 @@
       <c r="C59" s="1" t="n">
         <v>1</v>
       </c>
+      <c r="D59" s="1" t="s">
+        <v>50</v>
+      </c>
       <c r="E59" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G59" s="1" t="s">
         <v>8</v>
@@ -1932,16 +1932,16 @@
         <v>94</v>
       </c>
       <c r="B60" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C60" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>51</v>
+        <v>94</v>
       </c>
       <c r="E60" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G60" s="1" t="s">
         <v>8</v>
@@ -1952,59 +1952,59 @@
         <v>95</v>
       </c>
       <c r="B61" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C61" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E61" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="F61" s="1" t="s">
+        <v>73</v>
       </c>
       <c r="G61" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B62" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C62" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="E62" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="G62" s="1" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="B62" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C62" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D62" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="E62" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F62" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="G62" s="1" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B63" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C63" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="E63" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
+      </c>
+      <c r="E63" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="G63" s="1" t="s">
         <v>8</v>
@@ -2012,7 +2012,7 @@
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B64" s="1" t="n">
         <v>1</v>
@@ -2021,7 +2021,7 @@
         <v>1</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E64" s="1" t="n">
         <v>1</v>
@@ -2032,7 +2032,7 @@
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B65" s="1" t="n">
         <v>1</v>
@@ -2041,10 +2041,10 @@
         <v>1</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E65" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G65" s="1" t="s">
         <v>8</v>
@@ -2052,7 +2052,7 @@
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B66" s="1" t="n">
         <v>1</v>
@@ -2061,7 +2061,7 @@
         <v>1</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E66" s="1" t="n">
         <v>0</v>
@@ -2070,18 +2070,15 @@
         <v>8</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B67" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C67" s="1" t="n">
         <v>1</v>
-      </c>
-      <c r="D67" s="1" t="s">
-        <v>108</v>
       </c>
       <c r="E67" s="1" t="n">
         <v>0</v>
@@ -2090,7 +2087,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
         <v>109</v>
       </c>
@@ -2098,10 +2095,10 @@
         <v>1</v>
       </c>
       <c r="C68" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E68" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="E68" s="1" t="s">
+        <v>99</v>
       </c>
       <c r="G68" s="1" t="s">
         <v>8</v>
@@ -2115,10 +2112,13 @@
         <v>1</v>
       </c>
       <c r="C69" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="E69" s="1" t="s">
-        <v>100</v>
+        <v>1</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E69" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="G69" s="1" t="s">
         <v>8</v>
@@ -2132,13 +2132,13 @@
         <v>1</v>
       </c>
       <c r="C70" s="1" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="E70" s="1" t="n">
-        <v>0</v>
+        <v>24</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="G70" s="1" t="s">
         <v>8</v>
@@ -2152,13 +2152,13 @@
         <v>1</v>
       </c>
       <c r="C71" s="1" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E71" s="1" t="s">
-        <v>26</v>
+        <v>113</v>
+      </c>
+      <c r="E71" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="G71" s="1" t="s">
         <v>8</v>
@@ -2166,16 +2166,16 @@
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B72" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C72" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E72" s="1" t="n">
         <v>0</v>
@@ -2184,26 +2184,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="B73" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C73" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="D73" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="E73" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G73" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2221,7 +2202,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Y83"/>
+  <dimension ref="A1:Y82"/>
   <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44.99"/>
@@ -2273,22 +2254,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2308,16 +2289,16 @@
         <v>1</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>125</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>126</v>
       </c>
       <c r="I3" s="0"/>
       <c r="J3" s="0"/>
@@ -2339,13 +2320,13 @@
         <v>0</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2365,22 +2346,22 @@
         <v>0</v>
       </c>
       <c r="E5" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="I5" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="J5" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2400,22 +2381,22 @@
         <v>18</v>
       </c>
       <c r="E6" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="I6" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="J6" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2435,63 +2416,108 @@
         <v>1</v>
       </c>
       <c r="E7" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="I7" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="J7" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="str">
         <f aca="false">LibManager!A8</f>
-        <v>Checksum</v>
+        <v>ConvertTo</v>
       </c>
       <c r="B8" s="1" t="n">
         <f aca="false">LibManager!B8</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C8" s="1" t="n">
         <f aca="false">LibManager!C8</f>
         <v>1</v>
       </c>
-      <c r="D8" s="1" t="n">
-        <v>0</v>
+      <c r="D8" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>118</v>
+        <v>133</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>121</v>
+        <v>136</v>
       </c>
       <c r="J8" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="O8" s="1" t="s">
         <v>122</v>
+      </c>
+      <c r="P8" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="Q8" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="R8" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="S8" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="T8" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="U8" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="V8" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="W8" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="X8" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="Y8" s="1" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="str">
         <f aca="false">LibManager!A9</f>
-        <v>ConvertTo</v>
+        <v>Convolution</v>
       </c>
       <c r="B9" s="1" t="n">
         <f aca="false">LibManager!B9</f>
@@ -2499,79 +2525,34 @@
       </c>
       <c r="C9" s="1" t="n">
         <f aca="false">LibManager!C9</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>133</v>
+        <v>151</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>134</v>
+        <v>152</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>135</v>
+        <v>153</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>136</v>
+        <v>154</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>137</v>
+        <v>155</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="K9" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="L9" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="M9" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="N9" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="O9" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="P9" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="Q9" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="R9" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="S9" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="T9" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="U9" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="V9" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="W9" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="X9" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="Y9" s="1" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="str">
         <f aca="false">LibManager!A10</f>
-        <v>Convolution</v>
+        <v>Convolution3D</v>
       </c>
       <c r="B10" s="1" t="n">
         <f aca="false">LibManager!B10</f>
@@ -2581,32 +2562,32 @@
         <f aca="false">LibManager!C10</f>
         <v>3</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>26</v>
+      <c r="D10" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>152</v>
+        <v>116</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>153</v>
+        <v>117</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>154</v>
+        <v>118</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>155</v>
+        <v>119</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>156</v>
+        <v>120</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>157</v>
+        <v>121</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="str">
         <f aca="false">LibManager!A11</f>
-        <v>Convolution3D</v>
+        <v>Copy</v>
       </c>
       <c r="B11" s="1" t="n">
         <f aca="false">LibManager!B11</f>
@@ -2614,34 +2595,34 @@
       </c>
       <c r="C11" s="1" t="n">
         <f aca="false">LibManager!C11</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D11" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E11" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="H11" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="I11" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="J11" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="str">
         <f aca="false">LibManager!A12</f>
-        <v>Copy</v>
+        <v>CrossEntropyLoss</v>
       </c>
       <c r="B12" s="1" t="n">
         <f aca="false">LibManager!B12</f>
@@ -2649,34 +2630,34 @@
       </c>
       <c r="C12" s="1" t="n">
         <f aca="false">LibManager!C12</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D12" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="H12" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H12" s="1" t="s">
+      <c r="I12" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I12" s="1" t="s">
+      <c r="J12" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="str">
         <f aca="false">LibManager!A13</f>
-        <v>CrossEntropyLoss</v>
+        <v>Dequantize</v>
       </c>
       <c r="B13" s="1" t="n">
         <f aca="false">LibManager!B13</f>
@@ -2684,34 +2665,40 @@
       </c>
       <c r="C13" s="1" t="n">
         <f aca="false">LibManager!C13</f>
-        <v>2</v>
-      </c>
-      <c r="D13" s="1" t="n">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>117</v>
+        <v>157</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>118</v>
+        <v>158</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>119</v>
+        <v>159</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>121</v>
+        <v>161</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>122</v>
+        <v>162</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="str">
         <f aca="false">LibManager!A14</f>
-        <v>Dequantize</v>
+        <v>ElementAdd</v>
       </c>
       <c r="B14" s="1" t="n">
         <f aca="false">LibManager!B14</f>
@@ -2719,40 +2706,31 @@
       </c>
       <c r="C14" s="1" t="n">
         <f aca="false">LibManager!C14</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>158</v>
+        <v>126</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>159</v>
+        <v>127</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>160</v>
+        <v>128</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="K14" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="L14" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="str">
         <f aca="false">LibManager!A15</f>
-        <v>ElementAdd</v>
+        <v>ElementCmpEQ</v>
       </c>
       <c r="B15" s="1" t="n">
         <f aca="false">LibManager!B15</f>
@@ -2763,28 +2741,28 @@
         <v>2</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>127</v>
+        <v>151</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>128</v>
+        <v>152</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>129</v>
+        <v>153</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="str">
         <f aca="false">LibManager!A16</f>
-        <v>ElementCmpEQ</v>
+        <v>ElementCmpLT</v>
       </c>
       <c r="B16" s="1" t="n">
         <f aca="false">LibManager!B16</f>
@@ -2795,28 +2773,28 @@
         <v>2</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E16" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="G16" s="1" t="s">
-        <v>154</v>
-      </c>
       <c r="H16" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="I16" s="1" t="s">
         <v>168</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="str">
         <f aca="false">LibManager!A17</f>
-        <v>ElementCmpLT</v>
+        <v>ElementCmpLTE</v>
       </c>
       <c r="B17" s="1" t="n">
         <f aca="false">LibManager!B17</f>
@@ -2827,28 +2805,28 @@
         <v>2</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E17" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="F17" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="G17" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="G17" s="1" t="s">
-        <v>154</v>
-      </c>
       <c r="H17" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="I17" s="1" t="s">
         <v>168</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="str">
         <f aca="false">LibManager!A18</f>
-        <v>ElementCmpLTE</v>
+        <v>ElementDiv</v>
       </c>
       <c r="B18" s="1" t="n">
         <f aca="false">LibManager!B18</f>
@@ -2859,28 +2837,25 @@
         <v>2</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>152</v>
+        <v>126</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>153</v>
+        <v>127</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>154</v>
+        <v>128</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="I18" s="1" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="str">
         <f aca="false">LibManager!A19</f>
-        <v>ElementDiv</v>
+        <v>ElementExp</v>
       </c>
       <c r="B19" s="1" t="n">
         <f aca="false">LibManager!B19</f>
@@ -2888,28 +2863,22 @@
       </c>
       <c r="C19" s="1" t="n">
         <f aca="false">LibManager!C19</f>
-        <v>2</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>18</v>
+        <v>1</v>
+      </c>
+      <c r="D19" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>167</v>
+        <v>117</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="str">
         <f aca="false">LibManager!A20</f>
-        <v>ElementExp</v>
+        <v>ElementIsNaN</v>
       </c>
       <c r="B20" s="1" t="n">
         <f aca="false">LibManager!B20</f>
@@ -2923,16 +2892,16 @@
         <v>1</v>
       </c>
       <c r="E20" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="str">
         <f aca="false">LibManager!A21</f>
-        <v>ElementIsNaN</v>
+        <v>ElementLog</v>
       </c>
       <c r="B21" s="1" t="n">
         <f aca="false">LibManager!B21</f>
@@ -2942,20 +2911,20 @@
         <f aca="false">LibManager!C21</f>
         <v>1</v>
       </c>
-      <c r="D21" s="1" t="n">
-        <v>1</v>
+      <c r="D21" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>117</v>
+        <v>151</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>118</v>
+        <v>152</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="str">
         <f aca="false">LibManager!A22</f>
-        <v>ElementLog</v>
+        <v>ElementMax</v>
       </c>
       <c r="B22" s="1" t="n">
         <f aca="false">LibManager!B22</f>
@@ -2963,22 +2932,31 @@
       </c>
       <c r="C22" s="1" t="n">
         <f aca="false">LibManager!C22</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>152</v>
+        <v>126</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>153</v>
+        <v>127</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="str">
         <f aca="false">LibManager!A23</f>
-        <v>ElementMax</v>
+        <v>ElementMin</v>
       </c>
       <c r="B23" s="1" t="n">
         <f aca="false">LibManager!B23</f>
@@ -2992,25 +2970,25 @@
         <v>18</v>
       </c>
       <c r="E23" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="F23" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="F23" s="1" t="s">
+      <c r="G23" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="G23" s="1" t="s">
-        <v>129</v>
-      </c>
       <c r="H23" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="I23" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="I23" s="1" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="str">
         <f aca="false">LibManager!A24</f>
-        <v>ElementMin</v>
+        <v>ElementMul</v>
       </c>
       <c r="B24" s="1" t="n">
         <f aca="false">LibManager!B24</f>
@@ -3024,25 +3002,25 @@
         <v>18</v>
       </c>
       <c r="E24" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="F24" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="F24" s="1" t="s">
+      <c r="G24" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="G24" s="1" t="s">
-        <v>129</v>
-      </c>
       <c r="H24" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="I24" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="str">
         <f aca="false">LibManager!A25</f>
-        <v>ElementMul</v>
+        <v>ElementPow</v>
       </c>
       <c r="B25" s="1" t="n">
         <f aca="false">LibManager!B25</f>
@@ -3056,25 +3034,16 @@
         <v>18</v>
       </c>
       <c r="E25" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="F25" s="1" t="s">
         <v>127</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="H25" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="str">
         <f aca="false">LibManager!A26</f>
-        <v>ElementPow</v>
+        <v>ElementSelect</v>
       </c>
       <c r="B26" s="1" t="n">
         <f aca="false">LibManager!B26</f>
@@ -3082,22 +3051,34 @@
       </c>
       <c r="C26" s="1" t="n">
         <f aca="false">LibManager!C26</f>
-        <v>2</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>18</v>
+        <v>3</v>
+      </c>
+      <c r="D26" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>128</v>
+        <v>117</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="str">
         <f aca="false">LibManager!A27</f>
-        <v>ElementSelect</v>
+        <v>ElementSub</v>
       </c>
       <c r="B27" s="1" t="n">
         <f aca="false">LibManager!B27</f>
@@ -3105,34 +3086,31 @@
       </c>
       <c r="C27" s="1" t="n">
         <f aca="false">LibManager!C27</f>
-        <v>3</v>
-      </c>
-      <c r="D27" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>119</v>
+        <v>128</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>120</v>
+        <v>165</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="J27" s="1" t="s">
-        <v>122</v>
+        <v>166</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="str">
         <f aca="false">LibManager!A28</f>
-        <v>ElementSub</v>
+        <v>EmbeddingBag</v>
       </c>
       <c r="B28" s="1" t="n">
         <f aca="false">LibManager!B28</f>
@@ -3140,31 +3118,22 @@
       </c>
       <c r="C28" s="1" t="n">
         <f aca="false">LibManager!C28</f>
-        <v>2</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>18</v>
+        <v>4</v>
+      </c>
+      <c r="D28" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="G28" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="H28" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>167</v>
+        <v>117</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="str">
         <f aca="false">LibManager!A29</f>
-        <v>EmbeddingBag</v>
+        <v>ExtractTensor</v>
       </c>
       <c r="B29" s="1" t="n">
         <f aca="false">LibManager!B29</f>
@@ -3172,22 +3141,34 @@
       </c>
       <c r="C29" s="1" t="n">
         <f aca="false">LibManager!C29</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D29" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E29" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F29" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F29" s="1" t="s">
+      <c r="G29" s="1" t="s">
         <v>118</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="str">
         <f aca="false">LibManager!A30</f>
-        <v>ExtractTensor</v>
+        <v>Flip</v>
       </c>
       <c r="B30" s="1" t="n">
         <f aca="false">LibManager!B30</f>
@@ -3201,28 +3182,31 @@
         <v>1</v>
       </c>
       <c r="E30" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F30" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="G30" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G30" s="1" t="s">
+      <c r="H30" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H30" s="1" t="s">
+      <c r="I30" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I30" s="1" t="s">
+      <c r="J30" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="J30" s="1" t="s">
-        <v>122</v>
+      <c r="K30" s="1" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="str">
         <f aca="false">LibManager!A31</f>
-        <v>Flip</v>
+        <v>FullyConnected</v>
       </c>
       <c r="B31" s="1" t="n">
         <f aca="false">LibManager!B31</f>
@@ -3230,37 +3214,37 @@
       </c>
       <c r="C31" s="1" t="n">
         <f aca="false">LibManager!C31</f>
-        <v>1</v>
-      </c>
-      <c r="D31" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>117</v>
+        <v>151</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>118</v>
+        <v>152</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>119</v>
+        <v>153</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>120</v>
+        <v>154</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>121</v>
+        <v>170</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>122</v>
+        <v>155</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>170</v>
+        <v>156</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="str">
         <f aca="false">LibManager!A32</f>
-        <v>FullyConnected</v>
+        <v>FusedRowwiseQuantizedSparseLengthsSum</v>
       </c>
       <c r="B32" s="1" t="n">
         <f aca="false">LibManager!B32</f>
@@ -3270,35 +3254,20 @@
         <f aca="false">LibManager!C32</f>
         <v>3</v>
       </c>
-      <c r="D32" s="1" t="s">
-        <v>26</v>
+      <c r="D32" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>152</v>
+        <v>116</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="G32" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="H32" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="I32" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="J32" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="K32" s="1" t="s">
-        <v>157</v>
+        <v>117</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="str">
         <f aca="false">LibManager!A33</f>
-        <v>FusedRowwiseQuantizedSparseLengthsSum</v>
+        <v>FusedRowwiseQuantizedSparseLengthsWeightedSum</v>
       </c>
       <c r="B33" s="1" t="n">
         <f aca="false">LibManager!B33</f>
@@ -3306,22 +3275,22 @@
       </c>
       <c r="C33" s="1" t="n">
         <f aca="false">LibManager!C33</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D33" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>118</v>
+        <v>171</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="str">
         <f aca="false">LibManager!A34</f>
-        <v>FusedRowwiseQuantizedSparseLengthsWeightedSum</v>
+        <v>Gather</v>
       </c>
       <c r="B34" s="1" t="n">
         <f aca="false">LibManager!B34</f>
@@ -3329,116 +3298,128 @@
       </c>
       <c r="C34" s="1" t="n">
         <f aca="false">LibManager!C34</f>
-        <v>4</v>
-      </c>
-      <c r="D34" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>34</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="F34" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="G34" s="1" t="s">
         <v>172</v>
+      </c>
+      <c r="H34" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="J34" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="K34" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="L34" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="M34" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="N34" s="1" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="str">
         <f aca="false">LibManager!A35</f>
-        <v>Gather</v>
+        <v>GatherRanges</v>
       </c>
       <c r="B35" s="1" t="n">
         <f aca="false">LibManager!B35</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C35" s="1" t="n">
         <f aca="false">LibManager!C35</f>
         <v>2</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="E35" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="J35" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="F35" s="1" t="s">
+      <c r="K35" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="G35" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="H35" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="I35" s="1" t="s">
+      <c r="L35" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="J35" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="K35" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="L35" s="1" t="s">
+      <c r="M35" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="M35" s="1" t="s">
+      <c r="N35" s="1" t="s">
         <v>177</v>
-      </c>
-      <c r="N35" s="1" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="str">
         <f aca="false">LibManager!A36</f>
-        <v>GatherRanges</v>
+        <v>InsertTensor</v>
       </c>
       <c r="B36" s="1" t="n">
         <f aca="false">LibManager!B36</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C36" s="1" t="n">
         <f aca="false">LibManager!C36</f>
-        <v>2</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>59</v>
+        <v>1</v>
+      </c>
+      <c r="D36" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>137</v>
+        <v>116</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>134</v>
+        <v>117</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>173</v>
+        <v>118</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>174</v>
+        <v>119</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>175</v>
+        <v>120</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="K36" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="L36" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="M36" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="N36" s="1" t="s">
-        <v>178</v>
+        <v>121</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="str">
         <f aca="false">LibManager!A37</f>
-        <v>InsertTensor</v>
+        <v>Int8Converter</v>
       </c>
       <c r="B37" s="1" t="n">
         <f aca="false">LibManager!B37</f>
@@ -3452,28 +3433,16 @@
         <v>1</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="G37" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="H37" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="I37" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="J37" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="str">
         <f aca="false">LibManager!A38</f>
-        <v>Int8Converter</v>
+        <v>IntLookupTable</v>
       </c>
       <c r="B38" s="1" t="n">
         <f aca="false">LibManager!B38</f>
@@ -3481,22 +3450,16 @@
       </c>
       <c r="C38" s="1" t="n">
         <f aca="false">LibManager!C38</f>
-        <v>1</v>
-      </c>
-      <c r="D38" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E38" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>120</v>
+        <v>2</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="str">
         <f aca="false">LibManager!A39</f>
-        <v>IntLookupTable</v>
+        <v>LengthsSum</v>
       </c>
       <c r="B39" s="1" t="n">
         <f aca="false">LibManager!B39</f>
@@ -3506,14 +3469,32 @@
         <f aca="false">LibManager!C39</f>
         <v>2</v>
       </c>
-      <c r="D39" s="1" t="s">
-        <v>64</v>
+      <c r="D39" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="G39" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="H39" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="I39" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="J39" s="1" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="str">
         <f aca="false">LibManager!A40</f>
-        <v>LengthsSum</v>
+        <v>LengthsToRanges</v>
       </c>
       <c r="B40" s="1" t="n">
         <f aca="false">LibManager!B40</f>
@@ -3521,38 +3502,38 @@
       </c>
       <c r="C40" s="1" t="n">
         <f aca="false">LibManager!C40</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D40" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E40" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F40" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F40" s="1" t="s">
+      <c r="G40" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G40" s="1" t="s">
+      <c r="H40" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H40" s="1" t="s">
+      <c r="I40" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I40" s="1" t="s">
+      <c r="J40" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J40" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="str">
         <f aca="false">LibManager!A41</f>
-        <v>LengthsToRanges</v>
+        <v>LocalResponseNormalization</v>
       </c>
       <c r="B41" s="1" t="n">
         <f aca="false">LibManager!B41</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C41" s="1" t="n">
         <f aca="false">LibManager!C41</f>
@@ -3562,51 +3543,51 @@
         <v>1</v>
       </c>
       <c r="E41" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F41" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="F41" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="G41" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="H41" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="I41" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="J41" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="str">
         <f aca="false">LibManager!A42</f>
-        <v>LocalResponseNormalization</v>
+        <v>MatMul</v>
       </c>
       <c r="B42" s="1" t="n">
         <f aca="false">LibManager!B42</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C42" s="1" t="n">
         <f aca="false">LibManager!C42</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D42" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E42" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F42" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F42" s="1" t="s">
+      <c r="G42" s="1" t="s">
         <v>118</v>
+      </c>
+      <c r="H42" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="I42" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="J42" s="1" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="str">
         <f aca="false">LibManager!A43</f>
-        <v>MatMul</v>
+        <v>MaxPool</v>
       </c>
       <c r="B43" s="1" t="n">
         <f aca="false">LibManager!B43</f>
@@ -3614,34 +3595,37 @@
       </c>
       <c r="C43" s="1" t="n">
         <f aca="false">LibManager!C43</f>
-        <v>2</v>
-      </c>
-      <c r="D43" s="1" t="n">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>117</v>
+        <v>178</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>118</v>
+        <v>179</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>119</v>
+        <v>153</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>120</v>
+        <v>180</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>121</v>
+        <v>181</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>122</v>
+        <v>182</v>
+      </c>
+      <c r="K43" s="1" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="str">
         <f aca="false">LibManager!A44</f>
-        <v>MaxPool</v>
+        <v>MaxSplat</v>
       </c>
       <c r="B44" s="1" t="n">
         <f aca="false">LibManager!B44</f>
@@ -3651,35 +3635,32 @@
         <f aca="false">LibManager!C44</f>
         <v>1</v>
       </c>
-      <c r="D44" s="1" t="s">
-        <v>11</v>
+      <c r="D44" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>179</v>
+        <v>116</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>180</v>
+        <v>117</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>154</v>
+        <v>118</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>181</v>
+        <v>119</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>182</v>
+        <v>120</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="K44" s="1" t="s">
-        <v>169</v>
+        <v>121</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="str">
         <f aca="false">LibManager!A45</f>
-        <v>MaxSplat</v>
+        <v>Modulo</v>
       </c>
       <c r="B45" s="1" t="n">
         <f aca="false">LibManager!B45</f>
@@ -3693,28 +3674,16 @@
         <v>1</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="G45" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="H45" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="I45" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="J45" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="str">
         <f aca="false">LibManager!A46</f>
-        <v>Modulo</v>
+        <v>Quantize</v>
       </c>
       <c r="B46" s="1" t="n">
         <f aca="false">LibManager!B46</f>
@@ -3724,20 +3693,38 @@
         <f aca="false">LibManager!C46</f>
         <v>1</v>
       </c>
-      <c r="D46" s="1" t="n">
-        <v>1</v>
+      <c r="D46" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>120</v>
+        <v>170</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>121</v>
+        <v>183</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="H46" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="I46" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="J46" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="K46" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="L46" s="1" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="str">
         <f aca="false">LibManager!A47</f>
-        <v>Quantize</v>
+        <v>RescaleQuantized</v>
       </c>
       <c r="B47" s="1" t="n">
         <f aca="false">LibManager!B47</f>
@@ -3747,38 +3734,26 @@
         <f aca="false">LibManager!C47</f>
         <v>1</v>
       </c>
-      <c r="D47" s="1" t="s">
-        <v>11</v>
+      <c r="D47" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>171</v>
+        <v>118</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>185</v>
+        <v>121</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="I47" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="J47" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="K47" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="L47" s="1" t="s">
-        <v>190</v>
+        <v>169</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="str">
         <f aca="false">LibManager!A48</f>
-        <v>RescaleQuantized</v>
+        <v>RowwiseQuantizedFullyConnected</v>
       </c>
       <c r="B48" s="1" t="n">
         <f aca="false">LibManager!B48</f>
@@ -3786,28 +3761,16 @@
       </c>
       <c r="C48" s="1" t="n">
         <f aca="false">LibManager!C48</f>
-        <v>1</v>
-      </c>
-      <c r="D48" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E48" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="F48" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="G48" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="H48" s="1" t="s">
-        <v>170</v>
+        <v>5</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="str">
         <f aca="false">LibManager!A49</f>
-        <v>RowwiseQuantizedFullyConnected</v>
+        <v>RowwiseQuantizedSparseLengthsWeightedSum</v>
       </c>
       <c r="B49" s="1" t="n">
         <f aca="false">LibManager!B49</f>
@@ -3815,16 +3778,28 @@
       </c>
       <c r="C49" s="1" t="n">
         <f aca="false">LibManager!C49</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>64</v>
+        <v>80</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="G49" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="H49" s="1" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="str">
         <f aca="false">LibManager!A50</f>
-        <v>RowwiseQuantizedSparseLengthsWeightedSum</v>
+        <v>ScatterData</v>
       </c>
       <c r="B50" s="1" t="n">
         <f aca="false">LibManager!B50</f>
@@ -3832,28 +3807,34 @@
       </c>
       <c r="C50" s="1" t="n">
         <f aca="false">LibManager!C50</f>
-        <v>6</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>81</v>
+        <v>2</v>
+      </c>
+      <c r="D50" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>137</v>
+        <v>116</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>138</v>
+        <v>117</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>134</v>
+        <v>118</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>135</v>
+        <v>119</v>
+      </c>
+      <c r="I50" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="J50" s="1" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="str">
         <f aca="false">LibManager!A51</f>
-        <v>ScatterData</v>
+        <v>Sigmoid</v>
       </c>
       <c r="B51" s="1" t="n">
         <f aca="false">LibManager!B51</f>
@@ -3861,34 +3842,22 @@
       </c>
       <c r="C51" s="1" t="n">
         <f aca="false">LibManager!C51</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D51" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E51" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F51" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="F51" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="G51" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="H51" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="I51" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="J51" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="str">
         <f aca="false">LibManager!A52</f>
-        <v>Sigmoid</v>
+        <v>SoftMax</v>
       </c>
       <c r="B52" s="1" t="n">
         <f aca="false">LibManager!B52</f>
@@ -3902,16 +3871,28 @@
         <v>1</v>
       </c>
       <c r="E52" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F52" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F52" s="1" t="s">
+      <c r="G52" s="1" t="s">
         <v>118</v>
+      </c>
+      <c r="H52" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="I52" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="J52" s="1" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="str">
         <f aca="false">LibManager!A53</f>
-        <v>SoftMax</v>
+        <v>SparseLengthsWeightedSum</v>
       </c>
       <c r="B53" s="1" t="n">
         <f aca="false">LibManager!B53</f>
@@ -3919,34 +3900,43 @@
       </c>
       <c r="C53" s="1" t="n">
         <f aca="false">LibManager!C53</f>
-        <v>1</v>
-      </c>
-      <c r="D53" s="1" t="n">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>85</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>117</v>
+        <v>191</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>118</v>
+        <v>192</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>119</v>
+        <v>193</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>120</v>
+        <v>194</v>
       </c>
       <c r="I53" s="1" t="s">
-        <v>121</v>
+        <v>195</v>
       </c>
       <c r="J53" s="1" t="s">
-        <v>122</v>
+        <v>196</v>
+      </c>
+      <c r="K53" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="L53" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="M53" s="1" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="str">
         <f aca="false">LibManager!A54</f>
-        <v>SparseLengthsWeightedSum</v>
+        <v>SparseToDense</v>
       </c>
       <c r="B54" s="1" t="n">
         <f aca="false">LibManager!B54</f>
@@ -3954,43 +3944,34 @@
       </c>
       <c r="C54" s="1" t="n">
         <f aca="false">LibManager!C54</f>
-        <v>4</v>
-      </c>
-      <c r="D54" s="1" t="s">
-        <v>86</v>
+        <v>2</v>
+      </c>
+      <c r="D54" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>192</v>
+        <v>116</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>193</v>
+        <v>117</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>194</v>
+        <v>118</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>195</v>
+        <v>119</v>
       </c>
       <c r="I54" s="1" t="s">
-        <v>196</v>
+        <v>120</v>
       </c>
       <c r="J54" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="K54" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="L54" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="M54" s="1" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="str">
         <f aca="false">LibManager!A55</f>
-        <v>SparseToDense</v>
+        <v>SparseToDenseMask</v>
       </c>
       <c r="B55" s="1" t="n">
         <f aca="false">LibManager!B55</f>
@@ -3998,34 +3979,34 @@
       </c>
       <c r="C55" s="1" t="n">
         <f aca="false">LibManager!C55</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D55" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E55" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F55" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F55" s="1" t="s">
+      <c r="G55" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G55" s="1" t="s">
+      <c r="H55" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H55" s="1" t="s">
+      <c r="I55" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I55" s="1" t="s">
+      <c r="J55" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J55" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="str">
         <f aca="false">LibManager!A56</f>
-        <v>SparseToDenseMask</v>
+        <v>Splat</v>
       </c>
       <c r="B56" s="1" t="n">
         <f aca="false">LibManager!B56</f>
@@ -4033,34 +4014,34 @@
       </c>
       <c r="C56" s="1" t="n">
         <f aca="false">LibManager!C56</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D56" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E56" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F56" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F56" s="1" t="s">
+      <c r="G56" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G56" s="1" t="s">
+      <c r="H56" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H56" s="1" t="s">
+      <c r="I56" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I56" s="1" t="s">
+      <c r="J56" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J56" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="str">
         <f aca="false">LibManager!A57</f>
-        <v>Splat</v>
+        <v>Syncopy</v>
       </c>
       <c r="B57" s="1" t="n">
         <f aca="false">LibManager!B57</f>
@@ -4068,34 +4049,34 @@
       </c>
       <c r="C57" s="1" t="n">
         <f aca="false">LibManager!C57</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D57" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E57" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F57" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F57" s="1" t="s">
+      <c r="G57" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G57" s="1" t="s">
+      <c r="H57" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H57" s="1" t="s">
+      <c r="I57" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I57" s="1" t="s">
+      <c r="J57" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J57" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="str">
         <f aca="false">LibManager!A58</f>
-        <v>Syncopy</v>
+        <v>Tanh</v>
       </c>
       <c r="B58" s="1" t="n">
         <f aca="false">LibManager!B58</f>
@@ -4109,28 +4090,16 @@
         <v>1</v>
       </c>
       <c r="E58" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F58" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="F58" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="G58" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="H58" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="I58" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="J58" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="str">
         <f aca="false">LibManager!A59</f>
-        <v>Tanh</v>
+        <v>TensorView</v>
       </c>
       <c r="B59" s="1" t="n">
         <f aca="false">LibManager!B59</f>
@@ -4141,162 +4110,174 @@
         <v>1</v>
       </c>
       <c r="D59" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E59" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F59" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F59" s="1" t="s">
+      <c r="G59" s="1" t="s">
         <v>118</v>
+      </c>
+      <c r="H59" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="I59" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="J59" s="1" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="str">
         <f aca="false">LibManager!A60</f>
-        <v>TensorView</v>
+        <v>TopK</v>
       </c>
       <c r="B60" s="1" t="n">
         <f aca="false">LibManager!B60</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C60" s="1" t="n">
         <f aca="false">LibManager!C60</f>
         <v>1</v>
       </c>
       <c r="D60" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E60" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F60" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F60" s="1" t="s">
+      <c r="G60" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G60" s="1" t="s">
+      <c r="H60" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H60" s="1" t="s">
+      <c r="I60" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I60" s="1" t="s">
+      <c r="J60" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J60" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="str">
         <f aca="false">LibManager!A61</f>
-        <v>TopK</v>
+        <v>Transpose</v>
       </c>
       <c r="B61" s="1" t="n">
         <f aca="false">LibManager!B61</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C61" s="1" t="n">
         <f aca="false">LibManager!C61</f>
         <v>1</v>
       </c>
       <c r="D61" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E61" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F61" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F61" s="1" t="s">
+      <c r="G61" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G61" s="1" t="s">
+      <c r="H61" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H61" s="1" t="s">
+      <c r="I61" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I61" s="1" t="s">
+      <c r="J61" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J61" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="str">
         <f aca="false">LibManager!A62</f>
-        <v>Transpose</v>
+        <v>MaxPoolWithArgMax</v>
       </c>
       <c r="B62" s="1" t="n">
         <f aca="false">LibManager!B62</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C62" s="1" t="n">
         <f aca="false">LibManager!C62</f>
         <v>1</v>
       </c>
-      <c r="D62" s="1" t="n">
-        <v>1</v>
+      <c r="D62" s="1" t="s">
+        <v>99</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>117</v>
+        <v>178</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>118</v>
+        <v>179</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>119</v>
+        <v>153</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>120</v>
+        <v>180</v>
       </c>
       <c r="I62" s="1" t="s">
-        <v>121</v>
+        <v>181</v>
       </c>
       <c r="J62" s="1" t="s">
-        <v>122</v>
+        <v>182</v>
+      </c>
+      <c r="K62" s="1" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="str">
         <f aca="false">LibManager!A63</f>
-        <v>MaxPoolWithArgMax</v>
+        <v>BatchedReduceMin</v>
       </c>
       <c r="B63" s="1" t="n">
         <f aca="false">LibManager!B63</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C63" s="1" t="n">
         <f aca="false">LibManager!C63</f>
         <v>1</v>
       </c>
-      <c r="D63" s="1" t="s">
-        <v>100</v>
+      <c r="D63" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>179</v>
+        <v>116</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>180</v>
+        <v>117</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>154</v>
+        <v>118</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>181</v>
+        <v>119</v>
       </c>
       <c r="I63" s="1" t="s">
-        <v>182</v>
+        <v>120</v>
       </c>
       <c r="J63" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="K63" s="1" t="s">
-        <v>169</v>
+        <v>121</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="str">
         <f aca="false">LibManager!A64</f>
-        <v>BatchedReduceMin</v>
+        <v>CumSum</v>
       </c>
       <c r="B64" s="1" t="n">
         <f aca="false">LibManager!B64</f>
@@ -4310,28 +4291,22 @@
         <v>1</v>
       </c>
       <c r="E64" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F64" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F64" s="1" t="s">
-        <v>118</v>
-      </c>
       <c r="G64" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="H64" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="H64" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="I64" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="J64" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="str">
         <f aca="false">LibManager!A65</f>
-        <v>CumSum</v>
+        <v>SpaceToDepth</v>
       </c>
       <c r="B65" s="1" t="n">
         <f aca="false">LibManager!B65</f>
@@ -4342,25 +4317,25 @@
         <v>1</v>
       </c>
       <c r="D65" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E65" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F65" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F65" s="1" t="s">
+      <c r="G65" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G65" s="1" t="s">
-        <v>121</v>
-      </c>
       <c r="H65" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="str">
         <f aca="false">LibManager!A66</f>
-        <v>SpaceToDepth</v>
+        <v>ResizeNearest</v>
       </c>
       <c r="B66" s="1" t="n">
         <f aca="false">LibManager!B66</f>
@@ -4374,22 +4349,31 @@
         <v>0</v>
       </c>
       <c r="E66" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F66" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F66" s="1" t="s">
+      <c r="G66" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G66" s="1" t="s">
+      <c r="H66" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I66" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="J66" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="K66" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="H66" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="str">
         <f aca="false">LibManager!A67</f>
-        <v>ResizeNearest</v>
+        <v>LengthsRangeFill</v>
       </c>
       <c r="B67" s="1" t="n">
         <f aca="false">LibManager!B67</f>
@@ -4403,31 +4387,13 @@
         <v>0</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="F67" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="G67" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="H67" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="I67" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="J67" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="K67" s="1" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="str">
         <f aca="false">LibManager!A68</f>
-        <v>LengthsRangeFill</v>
+        <v>SparseLengthsSum</v>
       </c>
       <c r="B68" s="1" t="n">
         <f aca="false">LibManager!B68</f>
@@ -4435,19 +4401,34 @@
       </c>
       <c r="C68" s="1" t="n">
         <f aca="false">LibManager!C68</f>
-        <v>1</v>
-      </c>
-      <c r="D68" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="D68" s="1" t="s">
+        <v>99</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>121</v>
+        <v>136</v>
+      </c>
+      <c r="F68" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="G68" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="H68" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="I68" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="J68" s="1" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="1" t="str">
         <f aca="false">LibManager!A69</f>
-        <v>SparseLengthsSum</v>
+        <v>ResizeBilinear</v>
       </c>
       <c r="B69" s="1" t="n">
         <f aca="false">LibManager!B69</f>
@@ -4455,34 +4436,37 @@
       </c>
       <c r="C69" s="1" t="n">
         <f aca="false">LibManager!C69</f>
-        <v>3</v>
-      </c>
-      <c r="D69" s="1" t="s">
-        <v>100</v>
+        <v>1</v>
+      </c>
+      <c r="D69" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>137</v>
+        <v>116</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>138</v>
+        <v>117</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>134</v>
+        <v>118</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="I69" s="1" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="J69" s="1" t="s">
-        <v>173</v>
+        <v>120</v>
+      </c>
+      <c r="K69" s="1" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="str">
         <f aca="false">LibManager!A70</f>
-        <v>ResizeBilinear</v>
+        <v>ChannelWiseQuantizedConvolution</v>
       </c>
       <c r="B70" s="1" t="n">
         <f aca="false">LibManager!B70</f>
@@ -4490,37 +4474,22 @@
       </c>
       <c r="C70" s="1" t="n">
         <f aca="false">LibManager!C70</f>
-        <v>1</v>
-      </c>
-      <c r="D70" s="1" t="n">
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>117</v>
+        <v>153</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="G70" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="H70" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="I70" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="J70" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="K70" s="1" t="s">
-        <v>120</v>
+        <v>154</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="str">
         <f aca="false">LibManager!A71</f>
-        <v>ChannelWiseQuantizedConvolution</v>
+        <v>ConvTranspose</v>
       </c>
       <c r="B71" s="1" t="n">
         <f aca="false">LibManager!B71</f>
@@ -4528,59 +4497,53 @@
       </c>
       <c r="C71" s="1" t="n">
         <f aca="false">LibManager!C71</f>
-        <v>7</v>
-      </c>
-      <c r="D71" s="1" t="s">
-        <v>26</v>
+        <v>3</v>
+      </c>
+      <c r="D71" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="F71" s="1" t="s">
-        <v>155</v>
+        <v>116</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="str">
         <f aca="false">LibManager!A72</f>
-        <v>ConvTranspose</v>
+        <v>NonMaxSuppression</v>
       </c>
       <c r="B72" s="1" t="n">
         <f aca="false">LibManager!B72</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C72" s="1" t="n">
         <f aca="false">LibManager!C72</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D72" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>117</v>
+        <v>120</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="1" t="str">
+      <c r="A73" s="1" t="n">
         <f aca="false">LibManager!A73</f>
-        <v>NonMaxSuppression</v>
+        <v>0</v>
       </c>
       <c r="B73" s="1" t="n">
         <f aca="false">LibManager!B73</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C73" s="1" t="n">
         <f aca="false">LibManager!C73</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D73" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E73" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="F73" s="1" t="s">
-        <v>120</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4715,9 +4678,6 @@
         <f aca="false">LibManager!C81</f>
         <v>0</v>
       </c>
-      <c r="D81" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="1" t="n">
@@ -4730,20 +4690,6 @@
       </c>
       <c r="C82" s="1" t="n">
         <f aca="false">LibManager!C82</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A83" s="1" t="n">
-        <f aca="false">LibManager!A83</f>
-        <v>0</v>
-      </c>
-      <c r="B83" s="1" t="n">
-        <f aca="false">LibManager!B83</f>
-        <v>0</v>
-      </c>
-      <c r="C83" s="1" t="n">
-        <f aca="false">LibManager!C83</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[dnn-library] [SW-6339] The Touch Operator instruction has been added to dnnlib. libManager.xlsx has been update with Touch instruction. clang re-applied to some src/*.cpp
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="611" uniqueCount="198">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -371,6 +371,9 @@
     <t xml:space="preserve">CenterPointBox, MaxOutputBoxesPerClass, IouThreshold, ScoreThreshold, IsTFVersion4</t>
   </si>
   <si>
+    <t xml:space="preserve">Touch</t>
+  </si>
+  <si>
     <t xml:space="preserve">FloatTy</t>
   </si>
   <si>
@@ -606,6 +609,12 @@
   </si>
   <si>
     <t xml:space="preserve">Int16QTy, Int64ITy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BFloat16Ty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BoolTy</t>
   </si>
 </sst>
 </file>
@@ -2154,6 +2163,23 @@
         <v>8</v>
       </c>
     </row>
+    <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B73" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C73" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
@@ -2224,22 +2250,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2259,16 +2285,16 @@
         <v>1</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="I3" s="0"/>
       <c r="J3" s="0"/>
@@ -2290,13 +2316,13 @@
         <v>0</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2316,22 +2342,22 @@
         <v>0</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2351,22 +2377,22 @@
         <v>18</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2386,22 +2412,22 @@
         <v>1</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2421,67 +2447,67 @@
         <v>11</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="L8" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="O8" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="M8" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="N8" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="O8" s="1" t="s">
-        <v>122</v>
-      </c>
       <c r="P8" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="R8" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="S8" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="T8" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="U8" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="V8" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="W8" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="X8" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="Y8" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2501,22 +2527,22 @@
         <v>25</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2536,22 +2562,22 @@
         <v>0</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2571,22 +2597,22 @@
         <v>0</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2606,22 +2632,22 @@
         <v>1</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2641,28 +2667,28 @@
         <v>11</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2682,19 +2708,19 @@
         <v>0</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H14" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I14" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2714,19 +2740,19 @@
         <v>34</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2746,19 +2772,19 @@
         <v>34</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2778,19 +2804,19 @@
         <v>34</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2810,16 +2836,16 @@
         <v>0</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2839,10 +2865,10 @@
         <v>1</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2862,10 +2888,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2885,10 +2911,10 @@
         <v>11</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2908,19 +2934,19 @@
         <v>0</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H22" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I22" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="I22" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2940,19 +2966,19 @@
         <v>0</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H23" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I23" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="I23" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2972,19 +2998,19 @@
         <v>0</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H24" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I24" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3004,10 +3030,10 @@
         <v>0</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3027,22 +3053,22 @@
         <v>0</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3062,19 +3088,19 @@
         <v>0</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H27" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I27" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="I27" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3094,10 +3120,10 @@
         <v>0</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3117,22 +3143,22 @@
         <v>1</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3152,25 +3178,25 @@
         <v>1</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3190,25 +3216,25 @@
         <v>25</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3228,10 +3254,10 @@
         <v>0</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3251,10 +3277,10 @@
         <v>0</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3274,34 +3300,34 @@
         <v>34</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="K34" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="L34" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="M34" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="N34" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3321,34 +3347,34 @@
         <v>58</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="L35" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="M35" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3368,22 +3394,22 @@
         <v>1</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3403,10 +3429,10 @@
         <v>1</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3443,22 +3469,22 @@
         <v>1</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3478,22 +3504,22 @@
         <v>1</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3513,10 +3539,10 @@
         <v>1</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3536,22 +3562,22 @@
         <v>1</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3571,25 +3597,25 @@
         <v>11</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K43" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3609,22 +3635,22 @@
         <v>1</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3644,10 +3670,10 @@
         <v>1</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3667,28 +3693,28 @@
         <v>11</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="I46" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="J46" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K46" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="L46" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3708,16 +3734,16 @@
         <v>1</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3754,16 +3780,16 @@
         <v>80</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3783,22 +3809,22 @@
         <v>0</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I50" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J50" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3818,10 +3844,10 @@
         <v>1</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3841,22 +3867,22 @@
         <v>1</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I52" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J52" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3876,31 +3902,31 @@
         <v>85</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="I53" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="J53" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="K53" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="L53" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="M53" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3920,22 +3946,22 @@
         <v>0</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I54" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J54" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3955,22 +3981,22 @@
         <v>0</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I55" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J55" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3990,22 +4016,22 @@
         <v>0</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I56" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J56" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4025,22 +4051,22 @@
         <v>1</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I57" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J57" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4060,10 +4086,10 @@
         <v>1</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4083,22 +4109,22 @@
         <v>0</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I59" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J59" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4118,22 +4144,22 @@
         <v>2</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I60" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J60" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4153,22 +4179,22 @@
         <v>1</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I61" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J61" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4188,25 +4214,25 @@
         <v>99</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I62" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J62" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K62" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4226,22 +4252,22 @@
         <v>1</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I63" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J63" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4261,16 +4287,16 @@
         <v>1</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G64" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="H64" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="H64" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4290,16 +4316,16 @@
         <v>0</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4319,25 +4345,25 @@
         <v>0</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H66" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="I66" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="J66" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I66" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="J66" s="1" t="s">
+      <c r="K66" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="K66" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4357,7 +4383,7 @@
         <v>0</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4377,22 +4403,22 @@
         <v>99</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H68" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I68" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J68" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4412,25 +4438,25 @@
         <v>0</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H69" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="I69" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="J69" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I69" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="J69" s="1" t="s">
+      <c r="K69" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="K69" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4450,10 +4476,10 @@
         <v>25</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4473,7 +4499,7 @@
         <v>0</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4493,20 +4519,20 @@
         <v>2</v>
       </c>
       <c r="E72" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="F72" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="F72" s="1" t="s">
-        <v>119</v>
-      </c>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="1" t="n">
+      <c r="A73" s="1" t="str">
         <f aca="false">LibManager!A73</f>
-        <v>0</v>
+        <v>Touch</v>
       </c>
       <c r="B73" s="1" t="n">
         <f aca="false">LibManager!B73</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C73" s="1" t="n">
         <f aca="false">LibManager!C73</f>
@@ -4514,6 +4540,36 @@
       </c>
       <c r="D73" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="E73" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="G73" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="H73" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="I73" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="J73" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="K73" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="L73" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="M73" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="N73" s="1" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] Fix. Touch has to be handle in the same way alloc and dealloc does.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="611" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="195">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -371,9 +371,6 @@
     <t xml:space="preserve">CenterPointBox, MaxOutputBoxesPerClass, IouThreshold, ScoreThreshold, IsTFVersion4</t>
   </si>
   <si>
-    <t xml:space="preserve">Touch</t>
-  </si>
-  <si>
     <t xml:space="preserve">FloatTy</t>
   </si>
   <si>
@@ -609,12 +606,6 @@
   </si>
   <si>
     <t xml:space="preserve">Int16QTy, Int64ITy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BFloat16Ty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BoolTy</t>
   </si>
 </sst>
 </file>
@@ -2163,23 +2154,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="B73" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C73" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E73" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G73" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
@@ -2198,7 +2173,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Y82"/>
+  <dimension ref="A1:Y81"/>
   <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44.99"/>
@@ -2250,22 +2225,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2285,16 +2260,16 @@
         <v>1</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>125</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>126</v>
       </c>
       <c r="I3" s="0"/>
       <c r="J3" s="0"/>
@@ -2316,13 +2291,13 @@
         <v>0</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2342,22 +2317,22 @@
         <v>0</v>
       </c>
       <c r="E5" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="I5" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="J5" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2377,22 +2352,22 @@
         <v>18</v>
       </c>
       <c r="E6" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="I6" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="J6" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2412,22 +2387,22 @@
         <v>1</v>
       </c>
       <c r="E7" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="I7" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="J7" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2447,67 +2422,67 @@
         <v>11</v>
       </c>
       <c r="E8" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="H8" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="I8" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="J8" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="J8" s="1" t="s">
+      <c r="K8" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="K8" s="1" t="s">
+      <c r="L8" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="M8" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="L8" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="M8" s="1" t="s">
+      <c r="N8" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="N8" s="1" t="s">
+      <c r="O8" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="P8" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="O8" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="P8" s="1" t="s">
+      <c r="Q8" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="Q8" s="1" t="s">
+      <c r="R8" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="R8" s="1" t="s">
+      <c r="S8" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="S8" s="1" t="s">
+      <c r="T8" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="T8" s="1" t="s">
+      <c r="U8" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="U8" s="1" t="s">
+      <c r="V8" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="V8" s="1" t="s">
+      <c r="W8" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="W8" s="1" t="s">
+      <c r="X8" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="X8" s="1" t="s">
+      <c r="Y8" s="1" t="s">
         <v>150</v>
-      </c>
-      <c r="Y8" s="1" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2527,22 +2502,22 @@
         <v>25</v>
       </c>
       <c r="E9" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="H9" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="I9" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="J9" s="1" t="s">
         <v>156</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2562,22 +2537,22 @@
         <v>0</v>
       </c>
       <c r="E10" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="H10" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H10" s="1" t="s">
+      <c r="I10" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="J10" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2597,22 +2572,22 @@
         <v>0</v>
       </c>
       <c r="E11" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="H11" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="I11" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="J11" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2632,22 +2607,22 @@
         <v>1</v>
       </c>
       <c r="E12" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="H12" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H12" s="1" t="s">
+      <c r="I12" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I12" s="1" t="s">
+      <c r="J12" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2667,28 +2642,28 @@
         <v>11</v>
       </c>
       <c r="E13" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="G13" s="1" t="s">
+      <c r="H13" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="H13" s="1" t="s">
+      <c r="I13" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="I13" s="1" t="s">
+      <c r="J13" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="J13" s="1" t="s">
+      <c r="K13" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="K13" s="1" t="s">
+      <c r="L13" s="1" t="s">
         <v>164</v>
-      </c>
-      <c r="L13" s="1" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2708,19 +2683,19 @@
         <v>0</v>
       </c>
       <c r="E14" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G14" s="1" t="s">
+      <c r="H14" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="I14" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2740,19 +2715,19 @@
         <v>34</v>
       </c>
       <c r="E15" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="G15" s="1" t="s">
-        <v>154</v>
-      </c>
       <c r="H15" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="I15" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2772,19 +2747,19 @@
         <v>34</v>
       </c>
       <c r="E16" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="G16" s="1" t="s">
-        <v>154</v>
-      </c>
       <c r="H16" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="I16" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2804,19 +2779,19 @@
         <v>34</v>
       </c>
       <c r="E17" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="F17" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="G17" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="G17" s="1" t="s">
-        <v>154</v>
-      </c>
       <c r="H17" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="I17" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2836,16 +2811,16 @@
         <v>0</v>
       </c>
       <c r="E18" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="G18" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="H18" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2865,10 +2840,10 @@
         <v>1</v>
       </c>
       <c r="E19" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2888,10 +2863,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2911,10 +2886,10 @@
         <v>11</v>
       </c>
       <c r="E21" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>152</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2934,19 +2909,19 @@
         <v>0</v>
       </c>
       <c r="E22" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F22" s="1" t="s">
+      <c r="G22" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G22" s="1" t="s">
+      <c r="H22" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="I22" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="H22" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="I22" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2966,19 +2941,19 @@
         <v>0</v>
       </c>
       <c r="E23" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F23" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F23" s="1" t="s">
+      <c r="G23" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G23" s="1" t="s">
+      <c r="H23" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="I23" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="H23" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="I23" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2998,19 +2973,19 @@
         <v>0</v>
       </c>
       <c r="E24" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F24" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F24" s="1" t="s">
+      <c r="G24" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G24" s="1" t="s">
+      <c r="H24" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="I24" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="H24" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3030,10 +3005,10 @@
         <v>0</v>
       </c>
       <c r="E25" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F25" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3053,22 +3028,22 @@
         <v>0</v>
       </c>
       <c r="E26" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F26" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F26" s="1" t="s">
+      <c r="G26" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G26" s="1" t="s">
+      <c r="H26" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H26" s="1" t="s">
+      <c r="I26" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I26" s="1" t="s">
+      <c r="J26" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J26" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3088,19 +3063,19 @@
         <v>0</v>
       </c>
       <c r="E27" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F27" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F27" s="1" t="s">
+      <c r="G27" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G27" s="1" t="s">
+      <c r="H27" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="I27" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="H27" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="I27" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3120,10 +3095,10 @@
         <v>0</v>
       </c>
       <c r="E28" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F28" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3143,22 +3118,22 @@
         <v>1</v>
       </c>
       <c r="E29" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F29" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F29" s="1" t="s">
+      <c r="G29" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G29" s="1" t="s">
+      <c r="H29" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H29" s="1" t="s">
+      <c r="I29" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I29" s="1" t="s">
+      <c r="J29" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J29" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3178,25 +3153,25 @@
         <v>1</v>
       </c>
       <c r="E30" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F30" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="G30" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G30" s="1" t="s">
+      <c r="H30" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H30" s="1" t="s">
+      <c r="I30" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I30" s="1" t="s">
+      <c r="J30" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="J30" s="1" t="s">
-        <v>122</v>
-      </c>
       <c r="K30" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3216,25 +3191,25 @@
         <v>25</v>
       </c>
       <c r="E31" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="F31" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="F31" s="1" t="s">
+      <c r="G31" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="G31" s="1" t="s">
+      <c r="H31" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="H31" s="1" t="s">
+      <c r="I31" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="J31" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="I31" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="J31" s="1" t="s">
+      <c r="K31" s="1" t="s">
         <v>156</v>
-      </c>
-      <c r="K31" s="1" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3254,10 +3229,10 @@
         <v>0</v>
       </c>
       <c r="E32" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F32" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3277,10 +3252,10 @@
         <v>0</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3300,34 +3275,34 @@
         <v>34</v>
       </c>
       <c r="E34" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="H34" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="J34" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="F34" s="1" t="s">
+      <c r="K34" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="G34" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="H34" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="I34" s="1" t="s">
+      <c r="L34" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="J34" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="K34" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="L34" s="1" t="s">
+      <c r="M34" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="M34" s="1" t="s">
+      <c r="N34" s="1" t="s">
         <v>175</v>
-      </c>
-      <c r="N34" s="1" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3347,34 +3322,34 @@
         <v>58</v>
       </c>
       <c r="E35" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="J35" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="F35" s="1" t="s">
+      <c r="K35" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="G35" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="H35" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="I35" s="1" t="s">
+      <c r="L35" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="J35" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="K35" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="L35" s="1" t="s">
+      <c r="M35" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="M35" s="1" t="s">
+      <c r="N35" s="1" t="s">
         <v>175</v>
-      </c>
-      <c r="N35" s="1" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3394,22 +3369,22 @@
         <v>1</v>
       </c>
       <c r="E36" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F36" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F36" s="1" t="s">
+      <c r="G36" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G36" s="1" t="s">
+      <c r="H36" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H36" s="1" t="s">
+      <c r="I36" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I36" s="1" t="s">
+      <c r="J36" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J36" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3429,10 +3404,10 @@
         <v>1</v>
       </c>
       <c r="E37" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="F37" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3469,22 +3444,22 @@
         <v>1</v>
       </c>
       <c r="E39" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F39" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F39" s="1" t="s">
+      <c r="G39" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G39" s="1" t="s">
+      <c r="H39" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H39" s="1" t="s">
+      <c r="I39" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I39" s="1" t="s">
+      <c r="J39" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J39" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3504,22 +3479,22 @@
         <v>1</v>
       </c>
       <c r="E40" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F40" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F40" s="1" t="s">
+      <c r="G40" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G40" s="1" t="s">
+      <c r="H40" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H40" s="1" t="s">
+      <c r="I40" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I40" s="1" t="s">
+      <c r="J40" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J40" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3539,10 +3514,10 @@
         <v>1</v>
       </c>
       <c r="E41" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F41" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="F41" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3562,22 +3537,22 @@
         <v>1</v>
       </c>
       <c r="E42" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F42" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F42" s="1" t="s">
+      <c r="G42" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G42" s="1" t="s">
+      <c r="H42" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H42" s="1" t="s">
+      <c r="I42" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I42" s="1" t="s">
+      <c r="J42" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J42" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3597,25 +3572,25 @@
         <v>11</v>
       </c>
       <c r="E43" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="F43" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="F43" s="1" t="s">
+      <c r="G43" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="H43" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="G43" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="H43" s="1" t="s">
+      <c r="I43" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="I43" s="1" t="s">
+      <c r="J43" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="J43" s="1" t="s">
-        <v>181</v>
-      </c>
       <c r="K43" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3635,22 +3610,22 @@
         <v>1</v>
       </c>
       <c r="E44" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F44" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F44" s="1" t="s">
+      <c r="G44" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G44" s="1" t="s">
+      <c r="H44" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H44" s="1" t="s">
+      <c r="I44" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I44" s="1" t="s">
+      <c r="J44" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J44" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3670,10 +3645,10 @@
         <v>1</v>
       </c>
       <c r="E45" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F45" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3693,28 +3668,28 @@
         <v>11</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F46" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="G46" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="G46" s="1" t="s">
+      <c r="H46" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="H46" s="1" t="s">
+      <c r="I46" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="I46" s="1" t="s">
+      <c r="J46" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="J46" s="1" t="s">
+      <c r="K46" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="K46" s="1" t="s">
+      <c r="L46" s="1" t="s">
         <v>187</v>
-      </c>
-      <c r="L46" s="1" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3734,16 +3709,16 @@
         <v>1</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3780,16 +3755,16 @@
         <v>80</v>
       </c>
       <c r="E49" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="F49" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="F49" s="1" t="s">
-        <v>138</v>
-      </c>
       <c r="G49" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="H49" s="1" t="s">
         <v>134</v>
-      </c>
-      <c r="H49" s="1" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3809,22 +3784,22 @@
         <v>0</v>
       </c>
       <c r="E50" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F50" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F50" s="1" t="s">
+      <c r="G50" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G50" s="1" t="s">
+      <c r="H50" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H50" s="1" t="s">
+      <c r="I50" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I50" s="1" t="s">
+      <c r="J50" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J50" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3844,10 +3819,10 @@
         <v>1</v>
       </c>
       <c r="E51" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F51" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="F51" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3867,22 +3842,22 @@
         <v>1</v>
       </c>
       <c r="E52" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F52" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F52" s="1" t="s">
+      <c r="G52" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G52" s="1" t="s">
+      <c r="H52" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H52" s="1" t="s">
+      <c r="I52" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I52" s="1" t="s">
+      <c r="J52" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J52" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3902,31 +3877,31 @@
         <v>85</v>
       </c>
       <c r="E53" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="F53" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="F53" s="1" t="s">
+      <c r="G53" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="G53" s="1" t="s">
+      <c r="H53" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="H53" s="1" t="s">
+      <c r="I53" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="I53" s="1" t="s">
+      <c r="J53" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="J53" s="1" t="s">
-        <v>195</v>
-      </c>
       <c r="K53" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="L53" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="M53" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3946,22 +3921,22 @@
         <v>0</v>
       </c>
       <c r="E54" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F54" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F54" s="1" t="s">
+      <c r="G54" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G54" s="1" t="s">
+      <c r="H54" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H54" s="1" t="s">
+      <c r="I54" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I54" s="1" t="s">
+      <c r="J54" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J54" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3981,22 +3956,22 @@
         <v>0</v>
       </c>
       <c r="E55" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F55" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F55" s="1" t="s">
+      <c r="G55" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G55" s="1" t="s">
+      <c r="H55" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H55" s="1" t="s">
+      <c r="I55" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I55" s="1" t="s">
+      <c r="J55" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J55" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4016,22 +3991,22 @@
         <v>0</v>
       </c>
       <c r="E56" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F56" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F56" s="1" t="s">
+      <c r="G56" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G56" s="1" t="s">
+      <c r="H56" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H56" s="1" t="s">
+      <c r="I56" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I56" s="1" t="s">
+      <c r="J56" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J56" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4051,22 +4026,22 @@
         <v>1</v>
       </c>
       <c r="E57" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F57" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F57" s="1" t="s">
+      <c r="G57" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G57" s="1" t="s">
+      <c r="H57" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H57" s="1" t="s">
+      <c r="I57" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I57" s="1" t="s">
+      <c r="J57" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J57" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4086,10 +4061,10 @@
         <v>1</v>
       </c>
       <c r="E58" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F58" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="F58" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4109,22 +4084,22 @@
         <v>0</v>
       </c>
       <c r="E59" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F59" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F59" s="1" t="s">
+      <c r="G59" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G59" s="1" t="s">
+      <c r="H59" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H59" s="1" t="s">
+      <c r="I59" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I59" s="1" t="s">
+      <c r="J59" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J59" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4144,22 +4119,22 @@
         <v>2</v>
       </c>
       <c r="E60" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F60" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F60" s="1" t="s">
+      <c r="G60" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G60" s="1" t="s">
+      <c r="H60" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H60" s="1" t="s">
+      <c r="I60" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I60" s="1" t="s">
+      <c r="J60" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J60" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4179,22 +4154,22 @@
         <v>1</v>
       </c>
       <c r="E61" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F61" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F61" s="1" t="s">
+      <c r="G61" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G61" s="1" t="s">
+      <c r="H61" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H61" s="1" t="s">
+      <c r="I61" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I61" s="1" t="s">
+      <c r="J61" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J61" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4214,25 +4189,25 @@
         <v>99</v>
       </c>
       <c r="E62" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="F62" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="F62" s="1" t="s">
+      <c r="G62" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="H62" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="G62" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="H62" s="1" t="s">
+      <c r="I62" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="I62" s="1" t="s">
+      <c r="J62" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="J62" s="1" t="s">
-        <v>181</v>
-      </c>
       <c r="K62" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4252,22 +4227,22 @@
         <v>1</v>
       </c>
       <c r="E63" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F63" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F63" s="1" t="s">
+      <c r="G63" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G63" s="1" t="s">
+      <c r="H63" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H63" s="1" t="s">
+      <c r="I63" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I63" s="1" t="s">
+      <c r="J63" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="J63" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4287,16 +4262,16 @@
         <v>1</v>
       </c>
       <c r="E64" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F64" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F64" s="1" t="s">
-        <v>118</v>
-      </c>
       <c r="G64" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4316,16 +4291,16 @@
         <v>0</v>
       </c>
       <c r="E65" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F65" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F65" s="1" t="s">
+      <c r="G65" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G65" s="1" t="s">
+      <c r="H65" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="H65" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4345,25 +4320,25 @@
         <v>0</v>
       </c>
       <c r="E66" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F66" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F66" s="1" t="s">
+      <c r="G66" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G66" s="1" t="s">
+      <c r="H66" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I66" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="J66" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="K66" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="H66" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="I66" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="J66" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="K66" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4383,7 +4358,7 @@
         <v>0</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4403,22 +4378,22 @@
         <v>99</v>
       </c>
       <c r="E68" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="F68" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="F68" s="1" t="s">
-        <v>138</v>
-      </c>
       <c r="G68" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="H68" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="H68" s="1" t="s">
-        <v>135</v>
-      </c>
       <c r="I68" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="J68" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4438,25 +4413,25 @@
         <v>0</v>
       </c>
       <c r="E69" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F69" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F69" s="1" t="s">
+      <c r="G69" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G69" s="1" t="s">
+      <c r="H69" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I69" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="J69" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="K69" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="H69" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="I69" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="J69" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="K69" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4476,10 +4451,10 @@
         <v>25</v>
       </c>
       <c r="E70" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="F70" s="1" t="s">
         <v>154</v>
-      </c>
-      <c r="F70" s="1" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4499,7 +4474,7 @@
         <v>0</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4519,20 +4494,20 @@
         <v>2</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F72" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="1" t="str">
+      <c r="A73" s="1" t="n">
         <f aca="false">LibManager!A73</f>
-        <v>Touch</v>
+        <v>0</v>
       </c>
       <c r="B73" s="1" t="n">
         <f aca="false">LibManager!B73</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C73" s="1" t="n">
         <f aca="false">LibManager!C73</f>
@@ -4540,36 +4515,6 @@
       </c>
       <c r="D73" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="E73" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="F73" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="G73" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="H73" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="I73" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="J73" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="K73" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="L73" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="M73" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="N73" s="1" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4687,9 +4632,6 @@
         <f aca="false">LibManager!C80</f>
         <v>0</v>
       </c>
-      <c r="D80" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="1" t="n">
@@ -4702,20 +4644,6 @@
       </c>
       <c r="C81" s="1" t="n">
         <f aca="false">LibManager!C81</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A82" s="1" t="n">
-        <f aca="false">LibManager!A82</f>
-        <v>0</v>
-      </c>
-      <c r="B82" s="1" t="n">
-        <f aca="false">LibManager!B82</f>
-        <v>0</v>
-      </c>
-      <c r="C82" s="1" t="n">
-        <f aca="false">LibManager!C82</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[dnn-library] [SW-6517] Updated libManager.xlsl and regenerated the inlining stubs
On the "instances" tab from libManager.xlsl, changed the SoftMax row
so it contains only three types: FloatTy, Float16Ty and BFloat16.

Those are the only types supported by the SoftMax implementation from
the Glow interpreter and are the only ones for which should be
instanciated. Moreover, our implementation did not work for types other
that the three here mentioned.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="596" uniqueCount="196">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -588,6 +588,9 @@
   </si>
   <si>
     <t xml:space="preserve">UInt8QTy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BFloat16Ty</t>
   </si>
   <si>
     <t xml:space="preserve">FloatTy, Int64ITy</t>
@@ -3848,16 +3851,7 @@
         <v>117</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="H52" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="I52" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="J52" s="1" t="s">
-        <v>121</v>
+        <v>189</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3877,22 +3871,22 @@
         <v>85</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="I53" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="J53" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="K53" s="1" t="s">
         <v>136</v>

</xml_diff>

<commit_message>
[dnn-library] [SW-3816] Remove unused scalar code for convolution
Removed the implementation selector for convolution, since we will
always want to run the vectorized code from now on. Also the old unused
code has been removed.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="596" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="196">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -968,11 +968,8 @@
       <c r="E9" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F9" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="G9" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] [SW-8540] Fix element kind usage in FRQSL(W)S
- FRQSL(W)S was using wrong element kind when handling scales, offsets
  and weights.

- Enable FRQSLWS support with Float16Ty output.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="195">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -528,9 +528,6 @@
   </si>
   <si>
     <t xml:space="preserve">Int8QTy,FloatTy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#Float16Ty</t>
   </si>
   <si>
     <t xml:space="preserve">Int8QTy,Int32ITy</t>
@@ -3255,7 +3252,7 @@
         <v>116</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>169</v>
+        <v>117</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3281,13 +3278,13 @@
         <v>133</v>
       </c>
       <c r="G34" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="H34" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="H34" s="1" t="s">
+      <c r="I34" s="1" t="s">
         <v>171</v>
-      </c>
-      <c r="I34" s="1" t="s">
-        <v>172</v>
       </c>
       <c r="J34" s="1" t="s">
         <v>137</v>
@@ -3296,13 +3293,13 @@
         <v>134</v>
       </c>
       <c r="L34" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="M34" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="M34" s="1" t="s">
+      <c r="N34" s="1" t="s">
         <v>174</v>
-      </c>
-      <c r="N34" s="1" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3328,13 +3325,13 @@
         <v>133</v>
       </c>
       <c r="G35" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="H35" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="H35" s="1" t="s">
+      <c r="I35" s="1" t="s">
         <v>171</v>
-      </c>
-      <c r="I35" s="1" t="s">
-        <v>172</v>
       </c>
       <c r="J35" s="1" t="s">
         <v>137</v>
@@ -3343,13 +3340,13 @@
         <v>134</v>
       </c>
       <c r="L35" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="M35" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="M35" s="1" t="s">
+      <c r="N35" s="1" t="s">
         <v>174</v>
-      </c>
-      <c r="N35" s="1" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3572,22 +3569,22 @@
         <v>11</v>
       </c>
       <c r="E43" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="F43" s="1" t="s">
         <v>176</v>
-      </c>
-      <c r="F43" s="1" t="s">
-        <v>177</v>
       </c>
       <c r="G43" s="1" t="s">
         <v>153</v>
       </c>
       <c r="H43" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="I43" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="I43" s="1" t="s">
+      <c r="J43" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="J43" s="1" t="s">
-        <v>180</v>
       </c>
       <c r="K43" s="1" t="s">
         <v>166</v>
@@ -3671,25 +3668,25 @@
         <v>168</v>
       </c>
       <c r="F46" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="G46" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="G46" s="1" t="s">
+      <c r="H46" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="H46" s="1" t="s">
+      <c r="I46" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="I46" s="1" t="s">
+      <c r="J46" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="J46" s="1" t="s">
+      <c r="K46" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="K46" s="1" t="s">
+      <c r="L46" s="1" t="s">
         <v>186</v>
-      </c>
-      <c r="L46" s="1" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3712,7 +3709,7 @@
         <v>118</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="G47" s="1" t="s">
         <v>121</v>
@@ -3848,7 +3845,7 @@
         <v>117</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3868,22 +3865,22 @@
         <v>85</v>
       </c>
       <c r="E53" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="F53" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="F53" s="1" t="s">
+      <c r="G53" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="G53" s="1" t="s">
+      <c r="H53" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="H53" s="1" t="s">
+      <c r="I53" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="I53" s="1" t="s">
+      <c r="J53" s="1" t="s">
         <v>194</v>
-      </c>
-      <c r="J53" s="1" t="s">
-        <v>195</v>
       </c>
       <c r="K53" s="1" t="s">
         <v>136</v>
@@ -3892,7 +3889,7 @@
         <v>133</v>
       </c>
       <c r="M53" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4180,22 +4177,22 @@
         <v>99</v>
       </c>
       <c r="E62" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="F62" s="1" t="s">
         <v>176</v>
-      </c>
-      <c r="F62" s="1" t="s">
-        <v>177</v>
       </c>
       <c r="G62" s="1" t="s">
         <v>153</v>
       </c>
       <c r="H62" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="I62" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="I62" s="1" t="s">
+      <c r="J62" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="J62" s="1" t="s">
-        <v>180</v>
       </c>
       <c r="K62" s="1" t="s">
         <v>166</v>
@@ -4381,10 +4378,10 @@
         <v>134</v>
       </c>
       <c r="I68" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="J68" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] Fixed broken paths on libManager.py
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="195">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -982,8 +982,8 @@
       <c r="D10" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E10" s="1" t="n">
-        <v>0</v>
+      <c r="E10" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>8</v>
@@ -2530,26 +2530,26 @@
         <f aca="false">LibManager!C10</f>
         <v>3</v>
       </c>
-      <c r="D10" s="1" t="n">
-        <v>0</v>
+      <c r="D10" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>116</v>
+        <v>151</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>117</v>
+        <v>152</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>118</v>
+        <v>153</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>119</v>
+        <v>154</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>120</v>
+        <v>155</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>121</v>
+        <v>156</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] [SW-11149] Updated libManager.xlsx cacheState.xlsx
BatchedReduceAdd, EmbeddingBag, FullyConnected, MatMul needed to
be updated on the cacheState.xlsx:

- L1 state changed from dirty to untouched
- L2 state changed from dirty to untouched
- Enabled global store for destination tensor

The ElementErf operator was missing on both spreadsheets.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="196">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -135,6 +135,9 @@
   </si>
   <si>
     <t xml:space="preserve">ElementDiv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ElementErf</t>
   </si>
   <si>
     <t xml:space="preserve">ElementExp</t>
@@ -1171,7 +1174,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
         <v>40</v>
       </c>
@@ -1181,8 +1184,8 @@
       <c r="C21" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E21" s="1" t="s">
-        <v>11</v>
+      <c r="E21" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="G21" s="1" t="s">
         <v>8</v>
@@ -1196,10 +1199,10 @@
         <v>1</v>
       </c>
       <c r="C22" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E22" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="G22" s="1" t="s">
         <v>8</v>
@@ -1256,7 +1259,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
         <v>45</v>
       </c>
@@ -1264,7 +1267,7 @@
         <v>1</v>
       </c>
       <c r="C26" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E26" s="1" t="n">
         <v>0</v>
@@ -1273,7 +1276,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
         <v>46</v>
       </c>
@@ -1281,7 +1284,7 @@
         <v>1</v>
       </c>
       <c r="C27" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E27" s="1" t="n">
         <v>0</v>
@@ -1298,33 +1301,30 @@
         <v>1</v>
       </c>
       <c r="C28" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B29" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D28" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E28" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="1" t="s">
+      <c r="D29" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B29" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C29" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>50</v>
-      </c>
       <c r="E29" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G29" s="1" t="s">
         <v>8</v>
@@ -1332,16 +1332,16 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B30" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="B30" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C30" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>20</v>
       </c>
       <c r="E30" s="1" t="n">
         <v>1</v>
@@ -1358,16 +1358,19 @@
         <v>1</v>
       </c>
       <c r="C31" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>25</v>
+        <v>1</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E31" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="G31" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
         <v>53</v>
       </c>
@@ -1377,8 +1380,8 @@
       <c r="C32" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E32" s="1" t="n">
-        <v>0</v>
+      <c r="E32" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="G32" s="1" t="s">
         <v>8</v>
@@ -1392,7 +1395,7 @@
         <v>1</v>
       </c>
       <c r="C33" s="1" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E33" s="1" t="n">
         <v>0</v>
@@ -1401,7 +1404,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
         <v>55</v>
       </c>
@@ -1409,13 +1412,10 @@
         <v>1</v>
       </c>
       <c r="C34" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>34</v>
+        <v>4</v>
+      </c>
+      <c r="E34" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="G34" s="1" t="s">
         <v>8</v>
@@ -1423,16 +1423,19 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D35" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B35" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C35" s="1" t="n">
-        <v>2</v>
-      </c>
       <c r="E35" s="1" t="s">
-        <v>58</v>
+        <v>34</v>
       </c>
       <c r="G35" s="1" t="s">
         <v>8</v>
@@ -1440,42 +1443,42 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C36" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B36" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C36" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" s="1" t="s">
+      <c r="G36" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E36" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F36" s="1" t="s">
+      <c r="B37" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E37" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G36" s="1" t="s">
+      <c r="G37" s="1" t="s">
         <v>15</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="B37" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C37" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E37" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G37" s="1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1486,33 +1489,33 @@
         <v>1</v>
       </c>
       <c r="C38" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E38" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E38" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="G38" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="1" t="s">
+      <c r="B39" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E39" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B39" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C39" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E39" s="1" t="n">
-        <v>1</v>
-      </c>
       <c r="G39" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
         <v>65</v>
       </c>
@@ -1520,7 +1523,7 @@
         <v>1</v>
       </c>
       <c r="C40" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E40" s="1" t="n">
         <v>1</v>
@@ -1529,47 +1532,47 @@
         <v>8</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
         <v>66</v>
       </c>
       <c r="B41" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C41" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D41" s="1" t="s">
+      <c r="E41" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="E41" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F41" s="1" t="s">
+      <c r="B42" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C42" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E42" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="G41" s="1" t="s">
+      <c r="G42" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B42" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C42" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E42" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G42" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
         <v>69</v>
       </c>
@@ -1577,73 +1580,73 @@
         <v>1</v>
       </c>
       <c r="C43" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D43" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E43" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="E43" s="1" t="s">
+      <c r="B44" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E44" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G43" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="B44" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C44" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D44" s="1" t="s">
+      <c r="G44" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E44" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F44" s="1" t="s">
+      <c r="B45" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="G44" s="1" t="s">
+      <c r="E45" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="G45" s="1" t="s">
         <v>15</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B45" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C45" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="E45" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G45" s="1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B46" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B46" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C46" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E46" s="1" t="s">
-        <v>11</v>
+      <c r="E46" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="G46" s="1" t="s">
         <v>8</v>
@@ -1659,8 +1662,8 @@
       <c r="C47" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E47" s="1" t="n">
-        <v>1</v>
+      <c r="E47" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="G47" s="1" t="s">
         <v>8</v>
@@ -1674,19 +1677,16 @@
         <v>1</v>
       </c>
       <c r="C48" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="E48" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="F48" s="1" t="s">
-        <v>73</v>
+        <v>1</v>
+      </c>
+      <c r="E48" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
         <v>79</v>
       </c>
@@ -1694,13 +1694,13 @@
         <v>1</v>
       </c>
       <c r="C49" s="1" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>80</v>
+        <v>64</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>22</v>
+        <v>74</v>
       </c>
       <c r="G49" s="1" t="s">
         <v>15</v>
@@ -1708,19 +1708,22 @@
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B50" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="E50" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="B50" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C50" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E50" s="1" t="n">
-        <v>0</v>
+      <c r="F50" s="1" t="s">
+        <v>22</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1731,16 +1734,16 @@
         <v>1</v>
       </c>
       <c r="C51" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E51" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G51" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
         <v>83</v>
       </c>
@@ -1753,14 +1756,11 @@
       <c r="E52" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="F52" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="G52" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
         <v>84</v>
       </c>
@@ -1768,36 +1768,39 @@
         <v>1</v>
       </c>
       <c r="C53" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E53" s="1" t="s">
-        <v>85</v>
+        <v>1</v>
+      </c>
+      <c r="E53" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="G53" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B54" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C54" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E54" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B54" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C54" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E54" s="1" t="n">
-        <v>0</v>
+      <c r="F54" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
         <v>87</v>
       </c>
@@ -1805,31 +1808,28 @@
         <v>1</v>
       </c>
       <c r="C55" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E55" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B56" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C56" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D55" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="E55" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G55" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="1" t="s">
+      <c r="D56" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="B56" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C56" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D56" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="E56" s="1" t="n">
         <v>0</v>
       </c>
@@ -1837,7 +1837,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
         <v>90</v>
       </c>
@@ -1845,13 +1845,13 @@
         <v>1</v>
       </c>
       <c r="C57" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="E57" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G57" s="1" t="s">
         <v>8</v>
@@ -1859,14 +1859,17 @@
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B58" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="B58" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C58" s="1" t="n">
-        <v>1</v>
-      </c>
       <c r="E58" s="1" t="n">
         <v>1</v>
       </c>
@@ -1874,7 +1877,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
         <v>93</v>
       </c>
@@ -1884,11 +1887,8 @@
       <c r="C59" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D59" s="1" t="s">
-        <v>50</v>
-      </c>
       <c r="E59" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G59" s="1" t="s">
         <v>8</v>
@@ -1899,16 +1899,16 @@
         <v>94</v>
       </c>
       <c r="B60" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C60" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>94</v>
+        <v>51</v>
       </c>
       <c r="E60" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G60" s="1" t="s">
         <v>8</v>
@@ -1919,59 +1919,59 @@
         <v>95</v>
       </c>
       <c r="B61" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C61" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D61" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="E61" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G61" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="E61" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F61" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="G61" s="1" t="s">
+      <c r="B62" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C62" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E62" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="G62" s="1" t="s">
         <v>15</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="B62" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C62" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D62" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="E62" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="G62" s="1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B63" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C63" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E63" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="B63" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C63" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D63" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="E63" s="1" t="n">
-        <v>1</v>
       </c>
       <c r="G63" s="1" t="s">
         <v>8</v>
@@ -1979,16 +1979,16 @@
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B64" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C64" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" s="1" t="s">
         <v>102</v>
-      </c>
-      <c r="B64" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C64" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D64" s="1" t="s">
-        <v>103</v>
       </c>
       <c r="E64" s="1" t="n">
         <v>1</v>
@@ -1999,19 +1999,19 @@
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B65" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C65" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="B65" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C65" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D65" s="1" t="s">
-        <v>105</v>
-      </c>
       <c r="E65" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G65" s="1" t="s">
         <v>8</v>
@@ -2019,34 +2019,37 @@
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B66" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C66" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="B66" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C66" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D66" s="1" t="s">
+      <c r="E66" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="E66" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G66" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="1" t="s">
+      <c r="B67" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C67" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B67" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C67" s="1" t="n">
-        <v>1</v>
-      </c>
       <c r="E67" s="1" t="n">
         <v>0</v>
       </c>
@@ -2054,7 +2057,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
         <v>109</v>
       </c>
@@ -2062,10 +2065,10 @@
         <v>1</v>
       </c>
       <c r="C68" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="E68" s="1" t="s">
-        <v>99</v>
+        <v>1</v>
+      </c>
+      <c r="E68" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="G68" s="1" t="s">
         <v>8</v>
@@ -2079,13 +2082,10 @@
         <v>1</v>
       </c>
       <c r="C69" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D69" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="E69" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="E69" s="1" t="s">
+        <v>100</v>
       </c>
       <c r="G69" s="1" t="s">
         <v>8</v>
@@ -2099,13 +2099,13 @@
         <v>1</v>
       </c>
       <c r="C70" s="1" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E70" s="1" t="s">
-        <v>25</v>
+        <v>108</v>
+      </c>
+      <c r="E70" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="G70" s="1" t="s">
         <v>8</v>
@@ -2119,13 +2119,13 @@
         <v>1</v>
       </c>
       <c r="C71" s="1" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="E71" s="1" t="n">
-        <v>0</v>
+        <v>24</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="G71" s="1" t="s">
         <v>8</v>
@@ -2133,25 +2133,44 @@
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B72" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C72" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D72" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="B72" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C72" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="D72" s="1" t="s">
+      <c r="E72" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="E72" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G72" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+      <c r="B73" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C73" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="E73" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
@@ -2170,7 +2189,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Y81"/>
+  <dimension ref="A1:Y82"/>
   <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44.99"/>
@@ -2222,22 +2241,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2257,16 +2276,16 @@
         <v>1</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="I3" s="0"/>
       <c r="J3" s="0"/>
@@ -2288,13 +2307,13 @@
         <v>0</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2314,22 +2333,22 @@
         <v>0</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2349,22 +2368,22 @@
         <v>18</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2384,22 +2403,22 @@
         <v>1</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2419,67 +2438,67 @@
         <v>11</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="L8" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="O8" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="M8" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="N8" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="O8" s="1" t="s">
-        <v>122</v>
-      </c>
       <c r="P8" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="R8" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="S8" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="T8" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="U8" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="V8" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="W8" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="X8" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="Y8" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2499,22 +2518,22 @@
         <v>25</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2534,22 +2553,22 @@
         <v>25</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2569,22 +2588,22 @@
         <v>0</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2604,22 +2623,22 @@
         <v>1</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2639,28 +2658,28 @@
         <v>11</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2680,19 +2699,19 @@
         <v>0</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H14" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I14" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2712,19 +2731,19 @@
         <v>34</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2744,19 +2763,19 @@
         <v>34</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2776,19 +2795,19 @@
         <v>34</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2808,22 +2827,22 @@
         <v>0</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="str">
         <f aca="false">LibManager!A19</f>
-        <v>ElementExp</v>
+        <v>ElementErf</v>
       </c>
       <c r="B19" s="1" t="n">
         <f aca="false">LibManager!B19</f>
@@ -2837,16 +2856,16 @@
         <v>1</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="str">
         <f aca="false">LibManager!A20</f>
-        <v>ElementIsNaN</v>
+        <v>ElementExp</v>
       </c>
       <c r="B20" s="1" t="n">
         <f aca="false">LibManager!B20</f>
@@ -2860,16 +2879,16 @@
         <v>1</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="str">
         <f aca="false">LibManager!A21</f>
-        <v>ElementLog</v>
+        <v>ElementIsNaN</v>
       </c>
       <c r="B21" s="1" t="n">
         <f aca="false">LibManager!B21</f>
@@ -2879,20 +2898,20 @@
         <f aca="false">LibManager!C21</f>
         <v>1</v>
       </c>
-      <c r="D21" s="1" t="s">
-        <v>11</v>
+      <c r="D21" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>151</v>
+        <v>117</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>152</v>
+        <v>118</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="str">
         <f aca="false">LibManager!A22</f>
-        <v>ElementMax</v>
+        <v>ElementLog</v>
       </c>
       <c r="B22" s="1" t="n">
         <f aca="false">LibManager!B22</f>
@@ -2900,31 +2919,22 @@
       </c>
       <c r="C22" s="1" t="n">
         <f aca="false">LibManager!C22</f>
-        <v>2</v>
-      </c>
-      <c r="D22" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="H22" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="I22" s="1" t="s">
-        <v>119</v>
+        <v>153</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="str">
         <f aca="false">LibManager!A23</f>
-        <v>ElementMin</v>
+        <v>ElementMax</v>
       </c>
       <c r="B23" s="1" t="n">
         <f aca="false">LibManager!B23</f>
@@ -2938,25 +2948,25 @@
         <v>0</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H23" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I23" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="I23" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="str">
         <f aca="false">LibManager!A24</f>
-        <v>ElementMul</v>
+        <v>ElementMin</v>
       </c>
       <c r="B24" s="1" t="n">
         <f aca="false">LibManager!B24</f>
@@ -2970,25 +2980,25 @@
         <v>0</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H24" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I24" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="str">
         <f aca="false">LibManager!A25</f>
-        <v>ElementPow</v>
+        <v>ElementMul</v>
       </c>
       <c r="B25" s="1" t="n">
         <f aca="false">LibManager!B25</f>
@@ -3002,16 +3012,25 @@
         <v>0</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="str">
         <f aca="false">LibManager!A26</f>
-        <v>ElementSelect</v>
+        <v>ElementPow</v>
       </c>
       <c r="B26" s="1" t="n">
         <f aca="false">LibManager!B26</f>
@@ -3019,34 +3038,22 @@
       </c>
       <c r="C26" s="1" t="n">
         <f aca="false">LibManager!C26</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D26" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="G26" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="H26" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="I26" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="J26" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="str">
         <f aca="false">LibManager!A27</f>
-        <v>ElementSub</v>
+        <v>ElementSelect</v>
       </c>
       <c r="B27" s="1" t="n">
         <f aca="false">LibManager!B27</f>
@@ -3054,31 +3061,34 @@
       </c>
       <c r="C27" s="1" t="n">
         <f aca="false">LibManager!C27</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D27" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H27" s="1" t="s">
         <v>120</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="str">
         <f aca="false">LibManager!A28</f>
-        <v>EmbeddingBag</v>
+        <v>ElementSub</v>
       </c>
       <c r="B28" s="1" t="n">
         <f aca="false">LibManager!B28</f>
@@ -3086,22 +3096,31 @@
       </c>
       <c r="C28" s="1" t="n">
         <f aca="false">LibManager!C28</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D28" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="str">
         <f aca="false">LibManager!A29</f>
-        <v>ExtractTensor</v>
+        <v>EmbeddingBag</v>
       </c>
       <c r="B29" s="1" t="n">
         <f aca="false">LibManager!B29</f>
@@ -3109,34 +3128,22 @@
       </c>
       <c r="C29" s="1" t="n">
         <f aca="false">LibManager!C29</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D29" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="G29" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="H29" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="I29" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="J29" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="str">
         <f aca="false">LibManager!A30</f>
-        <v>Flip</v>
+        <v>ExtractTensor</v>
       </c>
       <c r="B30" s="1" t="n">
         <f aca="false">LibManager!B30</f>
@@ -3150,31 +3157,28 @@
         <v>1</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="K30" s="1" t="s">
-        <v>167</v>
+        <v>122</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="str">
         <f aca="false">LibManager!A31</f>
-        <v>FullyConnected</v>
+        <v>Flip</v>
       </c>
       <c r="B31" s="1" t="n">
         <f aca="false">LibManager!B31</f>
@@ -3182,37 +3186,37 @@
       </c>
       <c r="C31" s="1" t="n">
         <f aca="false">LibManager!C31</f>
-        <v>3</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>25</v>
+        <v>1</v>
+      </c>
+      <c r="D31" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>151</v>
+        <v>117</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>152</v>
+        <v>118</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>153</v>
+        <v>119</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>154</v>
+        <v>120</v>
       </c>
       <c r="I31" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="K31" s="1" t="s">
         <v>168</v>
-      </c>
-      <c r="J31" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="K31" s="1" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="str">
         <f aca="false">LibManager!A32</f>
-        <v>FusedRowwiseQuantizedSparseLengthsSum</v>
+        <v>FullyConnected</v>
       </c>
       <c r="B32" s="1" t="n">
         <f aca="false">LibManager!B32</f>
@@ -3222,20 +3226,35 @@
         <f aca="false">LibManager!C32</f>
         <v>3</v>
       </c>
-      <c r="D32" s="1" t="n">
-        <v>0</v>
+      <c r="D32" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>117</v>
+        <v>153</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="K32" s="1" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="str">
         <f aca="false">LibManager!A33</f>
-        <v>FusedRowwiseQuantizedSparseLengthsWeightedSum</v>
+        <v>FusedRowwiseQuantizedSparseLengthsSum</v>
       </c>
       <c r="B33" s="1" t="n">
         <f aca="false">LibManager!B33</f>
@@ -3243,22 +3262,22 @@
       </c>
       <c r="C33" s="1" t="n">
         <f aca="false">LibManager!C33</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D33" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="str">
         <f aca="false">LibManager!A34</f>
-        <v>Gather</v>
+        <v>FusedRowwiseQuantizedSparseLengthsWeightedSum</v>
       </c>
       <c r="B34" s="1" t="n">
         <f aca="false">LibManager!B34</f>
@@ -3266,128 +3285,116 @@
       </c>
       <c r="C34" s="1" t="n">
         <f aca="false">LibManager!C34</f>
-        <v>2</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>34</v>
+        <v>4</v>
+      </c>
+      <c r="D34" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>136</v>
+        <v>117</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="G34" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="H34" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="I34" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="J34" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="K34" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="L34" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="M34" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="N34" s="1" t="s">
-        <v>174</v>
+        <v>118</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="str">
         <f aca="false">LibManager!A35</f>
-        <v>GatherRanges</v>
+        <v>Gather</v>
       </c>
       <c r="B35" s="1" t="n">
         <f aca="false">LibManager!B35</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C35" s="1" t="n">
         <f aca="false">LibManager!C35</f>
         <v>2</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>58</v>
+        <v>34</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="L35" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="M35" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="str">
         <f aca="false">LibManager!A36</f>
-        <v>InsertTensor</v>
+        <v>GatherRanges</v>
       </c>
       <c r="B36" s="1" t="n">
         <f aca="false">LibManager!B36</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C36" s="1" t="n">
         <f aca="false">LibManager!C36</f>
-        <v>1</v>
-      </c>
-      <c r="D36" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>59</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>116</v>
+        <v>137</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>117</v>
+        <v>134</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>118</v>
+        <v>170</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>119</v>
+        <v>171</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>120</v>
+        <v>172</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>121</v>
+        <v>138</v>
+      </c>
+      <c r="K36" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="L36" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="M36" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="N36" s="1" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="str">
         <f aca="false">LibManager!A37</f>
-        <v>Int8Converter</v>
+        <v>InsertTensor</v>
       </c>
       <c r="B37" s="1" t="n">
         <f aca="false">LibManager!B37</f>
@@ -3401,16 +3408,28 @@
         <v>1</v>
       </c>
       <c r="E37" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F37" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F37" s="1" t="s">
+      <c r="G37" s="1" t="s">
         <v>119</v>
+      </c>
+      <c r="H37" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="I37" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="J37" s="1" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="str">
         <f aca="false">LibManager!A38</f>
-        <v>IntLookupTable</v>
+        <v>Int8Converter</v>
       </c>
       <c r="B38" s="1" t="n">
         <f aca="false">LibManager!B38</f>
@@ -3418,16 +3437,22 @@
       </c>
       <c r="C38" s="1" t="n">
         <f aca="false">LibManager!C38</f>
-        <v>2</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>63</v>
+        <v>1</v>
+      </c>
+      <c r="D38" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="str">
         <f aca="false">LibManager!A39</f>
-        <v>LengthsSum</v>
+        <v>IntLookupTable</v>
       </c>
       <c r="B39" s="1" t="n">
         <f aca="false">LibManager!B39</f>
@@ -3437,32 +3462,14 @@
         <f aca="false">LibManager!C39</f>
         <v>2</v>
       </c>
-      <c r="D39" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="F39" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="G39" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="H39" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="I39" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="J39" s="1" t="s">
-        <v>121</v>
+      <c r="D39" s="1" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="str">
         <f aca="false">LibManager!A40</f>
-        <v>LengthsToRanges</v>
+        <v>LengthsSum</v>
       </c>
       <c r="B40" s="1" t="n">
         <f aca="false">LibManager!B40</f>
@@ -3470,38 +3477,38 @@
       </c>
       <c r="C40" s="1" t="n">
         <f aca="false">LibManager!C40</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D40" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="str">
         <f aca="false">LibManager!A41</f>
-        <v>LocalResponseNormalization</v>
+        <v>LengthsToRanges</v>
       </c>
       <c r="B41" s="1" t="n">
         <f aca="false">LibManager!B41</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C41" s="1" t="n">
         <f aca="false">LibManager!C41</f>
@@ -3511,51 +3518,51 @@
         <v>1</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="H41" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="I41" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="J41" s="1" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="str">
         <f aca="false">LibManager!A42</f>
-        <v>MatMul</v>
+        <v>LocalResponseNormalization</v>
       </c>
       <c r="B42" s="1" t="n">
         <f aca="false">LibManager!B42</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C42" s="1" t="n">
         <f aca="false">LibManager!C42</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D42" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="G42" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="H42" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="I42" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="J42" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="str">
         <f aca="false">LibManager!A43</f>
-        <v>MaxPool</v>
+        <v>MatMul</v>
       </c>
       <c r="B43" s="1" t="n">
         <f aca="false">LibManager!B43</f>
@@ -3563,37 +3570,34 @@
       </c>
       <c r="C43" s="1" t="n">
         <f aca="false">LibManager!C43</f>
-        <v>1</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>11</v>
+        <v>2</v>
+      </c>
+      <c r="D43" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>175</v>
+        <v>117</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>176</v>
+        <v>118</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>153</v>
+        <v>119</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>177</v>
+        <v>120</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>178</v>
+        <v>121</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="K43" s="1" t="s">
-        <v>166</v>
+        <v>122</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="str">
         <f aca="false">LibManager!A44</f>
-        <v>MaxSplat</v>
+        <v>MaxPool</v>
       </c>
       <c r="B44" s="1" t="n">
         <f aca="false">LibManager!B44</f>
@@ -3603,32 +3607,35 @@
         <f aca="false">LibManager!C44</f>
         <v>1</v>
       </c>
-      <c r="D44" s="1" t="n">
-        <v>1</v>
+      <c r="D44" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>116</v>
+        <v>176</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>117</v>
+        <v>177</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>119</v>
+        <v>178</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>120</v>
+        <v>179</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>121</v>
+        <v>180</v>
+      </c>
+      <c r="K44" s="1" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="str">
         <f aca="false">LibManager!A45</f>
-        <v>Modulo</v>
+        <v>MaxSplat</v>
       </c>
       <c r="B45" s="1" t="n">
         <f aca="false">LibManager!B45</f>
@@ -3642,16 +3649,28 @@
         <v>1</v>
       </c>
       <c r="E45" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="G45" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="F45" s="1" t="s">
+      <c r="H45" s="1" t="s">
         <v>120</v>
+      </c>
+      <c r="I45" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="J45" s="1" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="str">
         <f aca="false">LibManager!A46</f>
-        <v>Quantize</v>
+        <v>Modulo</v>
       </c>
       <c r="B46" s="1" t="n">
         <f aca="false">LibManager!B46</f>
@@ -3661,38 +3680,20 @@
         <f aca="false">LibManager!C46</f>
         <v>1</v>
       </c>
-      <c r="D46" s="1" t="s">
-        <v>11</v>
+      <c r="D46" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>168</v>
+        <v>120</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="G46" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="H46" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="I46" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="J46" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="K46" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="L46" s="1" t="s">
-        <v>186</v>
+        <v>121</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="str">
         <f aca="false">LibManager!A47</f>
-        <v>RescaleQuantized</v>
+        <v>Quantize</v>
       </c>
       <c r="B47" s="1" t="n">
         <f aca="false">LibManager!B47</f>
@@ -3702,26 +3703,38 @@
         <f aca="false">LibManager!C47</f>
         <v>1</v>
       </c>
-      <c r="D47" s="1" t="n">
-        <v>1</v>
+      <c r="D47" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>118</v>
+        <v>169</v>
       </c>
       <c r="F47" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="H47" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="I47" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="J47" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="K47" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="L47" s="1" t="s">
         <v>187</v>
-      </c>
-      <c r="G47" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="H47" s="1" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="str">
         <f aca="false">LibManager!A48</f>
-        <v>RowwiseQuantizedFullyConnected</v>
+        <v>RescaleQuantized</v>
       </c>
       <c r="B48" s="1" t="n">
         <f aca="false">LibManager!B48</f>
@@ -3729,16 +3742,28 @@
       </c>
       <c r="C48" s="1" t="n">
         <f aca="false">LibManager!C48</f>
-        <v>5</v>
-      </c>
-      <c r="D48" s="1" t="s">
-        <v>63</v>
+        <v>1</v>
+      </c>
+      <c r="D48" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="G48" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="H48" s="1" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="str">
         <f aca="false">LibManager!A49</f>
-        <v>RowwiseQuantizedSparseLengthsWeightedSum</v>
+        <v>RowwiseQuantizedFullyConnected</v>
       </c>
       <c r="B49" s="1" t="n">
         <f aca="false">LibManager!B49</f>
@@ -3746,28 +3771,16 @@
       </c>
       <c r="C49" s="1" t="n">
         <f aca="false">LibManager!C49</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="E49" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="F49" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="G49" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="H49" s="1" t="s">
-        <v>134</v>
+        <v>64</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="str">
         <f aca="false">LibManager!A50</f>
-        <v>ScatterData</v>
+        <v>RowwiseQuantizedSparseLengthsWeightedSum</v>
       </c>
       <c r="B50" s="1" t="n">
         <f aca="false">LibManager!B50</f>
@@ -3775,34 +3788,28 @@
       </c>
       <c r="C50" s="1" t="n">
         <f aca="false">LibManager!C50</f>
-        <v>2</v>
-      </c>
-      <c r="D50" s="1" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>81</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>116</v>
+        <v>137</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>117</v>
+        <v>138</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>118</v>
+        <v>134</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="I50" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="J50" s="1" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="str">
         <f aca="false">LibManager!A51</f>
-        <v>Sigmoid</v>
+        <v>ScatterData</v>
       </c>
       <c r="B51" s="1" t="n">
         <f aca="false">LibManager!B51</f>
@@ -3810,22 +3817,34 @@
       </c>
       <c r="C51" s="1" t="n">
         <f aca="false">LibManager!C51</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D51" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
+      </c>
+      <c r="G51" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="H51" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="I51" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="J51" s="1" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="str">
         <f aca="false">LibManager!A52</f>
-        <v>SoftMax</v>
+        <v>Sigmoid</v>
       </c>
       <c r="B52" s="1" t="n">
         <f aca="false">LibManager!B52</f>
@@ -3839,19 +3858,16 @@
         <v>1</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="G52" s="1" t="s">
-        <v>188</v>
+        <v>118</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="str">
         <f aca="false">LibManager!A53</f>
-        <v>SparseLengthsWeightedSum</v>
+        <v>SoftMax</v>
       </c>
       <c r="B53" s="1" t="n">
         <f aca="false">LibManager!B53</f>
@@ -3859,43 +3875,25 @@
       </c>
       <c r="C53" s="1" t="n">
         <f aca="false">LibManager!C53</f>
-        <v>4</v>
-      </c>
-      <c r="D53" s="1" t="s">
-        <v>85</v>
+        <v>1</v>
+      </c>
+      <c r="D53" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="E53" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="G53" s="1" t="s">
         <v>189</v>
-      </c>
-      <c r="F53" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="G53" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="H53" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="I53" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="J53" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="K53" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="L53" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="M53" s="1" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="str">
         <f aca="false">LibManager!A54</f>
-        <v>SparseToDense</v>
+        <v>SparseLengthsWeightedSum</v>
       </c>
       <c r="B54" s="1" t="n">
         <f aca="false">LibManager!B54</f>
@@ -3903,34 +3901,43 @@
       </c>
       <c r="C54" s="1" t="n">
         <f aca="false">LibManager!C54</f>
-        <v>2</v>
-      </c>
-      <c r="D54" s="1" t="n">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>86</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>116</v>
+        <v>190</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>117</v>
+        <v>191</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>118</v>
+        <v>192</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>119</v>
+        <v>193</v>
       </c>
       <c r="I54" s="1" t="s">
-        <v>120</v>
+        <v>194</v>
       </c>
       <c r="J54" s="1" t="s">
-        <v>121</v>
+        <v>195</v>
+      </c>
+      <c r="K54" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="L54" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="M54" s="1" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="str">
         <f aca="false">LibManager!A55</f>
-        <v>SparseToDenseMask</v>
+        <v>SparseToDense</v>
       </c>
       <c r="B55" s="1" t="n">
         <f aca="false">LibManager!B55</f>
@@ -3938,34 +3945,34 @@
       </c>
       <c r="C55" s="1" t="n">
         <f aca="false">LibManager!C55</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D55" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I55" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J55" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="str">
         <f aca="false">LibManager!A56</f>
-        <v>Splat</v>
+        <v>SparseToDenseMask</v>
       </c>
       <c r="B56" s="1" t="n">
         <f aca="false">LibManager!B56</f>
@@ -3973,34 +3980,34 @@
       </c>
       <c r="C56" s="1" t="n">
         <f aca="false">LibManager!C56</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D56" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I56" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J56" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="str">
         <f aca="false">LibManager!A57</f>
-        <v>Syncopy</v>
+        <v>Splat</v>
       </c>
       <c r="B57" s="1" t="n">
         <f aca="false">LibManager!B57</f>
@@ -4008,34 +4015,34 @@
       </c>
       <c r="C57" s="1" t="n">
         <f aca="false">LibManager!C57</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D57" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I57" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J57" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="str">
         <f aca="false">LibManager!A58</f>
-        <v>Tanh</v>
+        <v>Syncopy</v>
       </c>
       <c r="B58" s="1" t="n">
         <f aca="false">LibManager!B58</f>
@@ -4049,16 +4056,28 @@
         <v>1</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
+      </c>
+      <c r="G58" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="H58" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="I58" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="J58" s="1" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="str">
         <f aca="false">LibManager!A59</f>
-        <v>TensorView</v>
+        <v>Tanh</v>
       </c>
       <c r="B59" s="1" t="n">
         <f aca="false">LibManager!B59</f>
@@ -4069,174 +4088,162 @@
         <v>1</v>
       </c>
       <c r="D59" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="G59" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="H59" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="I59" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="J59" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="str">
         <f aca="false">LibManager!A60</f>
-        <v>TopK</v>
+        <v>TensorView</v>
       </c>
       <c r="B60" s="1" t="n">
         <f aca="false">LibManager!B60</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C60" s="1" t="n">
         <f aca="false">LibManager!C60</f>
         <v>1</v>
       </c>
       <c r="D60" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I60" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J60" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="str">
         <f aca="false">LibManager!A61</f>
-        <v>Transpose</v>
+        <v>TopK</v>
       </c>
       <c r="B61" s="1" t="n">
         <f aca="false">LibManager!B61</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C61" s="1" t="n">
         <f aca="false">LibManager!C61</f>
         <v>1</v>
       </c>
       <c r="D61" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I61" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J61" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="str">
         <f aca="false">LibManager!A62</f>
-        <v>MaxPoolWithArgMax</v>
+        <v>Transpose</v>
       </c>
       <c r="B62" s="1" t="n">
         <f aca="false">LibManager!B62</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C62" s="1" t="n">
         <f aca="false">LibManager!C62</f>
         <v>1</v>
       </c>
-      <c r="D62" s="1" t="s">
-        <v>99</v>
+      <c r="D62" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>175</v>
+        <v>117</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>176</v>
+        <v>118</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>153</v>
+        <v>119</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>177</v>
+        <v>120</v>
       </c>
       <c r="I62" s="1" t="s">
-        <v>178</v>
+        <v>121</v>
       </c>
       <c r="J62" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="K62" s="1" t="s">
-        <v>166</v>
+        <v>122</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="str">
         <f aca="false">LibManager!A63</f>
-        <v>BatchedReduceMin</v>
+        <v>MaxPoolWithArgMax</v>
       </c>
       <c r="B63" s="1" t="n">
         <f aca="false">LibManager!B63</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C63" s="1" t="n">
         <f aca="false">LibManager!C63</f>
         <v>1</v>
       </c>
-      <c r="D63" s="1" t="n">
-        <v>1</v>
+      <c r="D63" s="1" t="s">
+        <v>100</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>116</v>
+        <v>176</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>117</v>
+        <v>177</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>119</v>
+        <v>178</v>
       </c>
       <c r="I63" s="1" t="s">
-        <v>120</v>
+        <v>179</v>
       </c>
       <c r="J63" s="1" t="s">
-        <v>121</v>
+        <v>180</v>
+      </c>
+      <c r="K63" s="1" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="str">
         <f aca="false">LibManager!A64</f>
-        <v>CumSum</v>
+        <v>BatchedReduceMin</v>
       </c>
       <c r="B64" s="1" t="n">
         <f aca="false">LibManager!B64</f>
@@ -4250,22 +4257,28 @@
         <v>1</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G64" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="H64" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H64" s="1" t="s">
-        <v>119</v>
+      <c r="I64" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="J64" s="1" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="str">
         <f aca="false">LibManager!A65</f>
-        <v>SpaceToDepth</v>
+        <v>CumSum</v>
       </c>
       <c r="B65" s="1" t="n">
         <f aca="false">LibManager!B65</f>
@@ -4276,25 +4289,25 @@
         <v>1</v>
       </c>
       <c r="D65" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="str">
         <f aca="false">LibManager!A66</f>
-        <v>ResizeNearest</v>
+        <v>SpaceToDepth</v>
       </c>
       <c r="B66" s="1" t="n">
         <f aca="false">LibManager!B66</f>
@@ -4308,31 +4321,22 @@
         <v>0</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="I66" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="J66" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="K66" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="str">
         <f aca="false">LibManager!A67</f>
-        <v>LengthsRangeFill</v>
+        <v>ResizeNearest</v>
       </c>
       <c r="B67" s="1" t="n">
         <f aca="false">LibManager!B67</f>
@@ -4346,13 +4350,31 @@
         <v>0</v>
       </c>
       <c r="E67" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F67" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="G67" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="H67" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="I67" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="J67" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="K67" s="1" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="str">
         <f aca="false">LibManager!A68</f>
-        <v>SparseLengthsSum</v>
+        <v>LengthsRangeFill</v>
       </c>
       <c r="B68" s="1" t="n">
         <f aca="false">LibManager!B68</f>
@@ -4360,34 +4382,19 @@
       </c>
       <c r="C68" s="1" t="n">
         <f aca="false">LibManager!C68</f>
-        <v>3</v>
-      </c>
-      <c r="D68" s="1" t="s">
-        <v>99</v>
+        <v>1</v>
+      </c>
+      <c r="D68" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="F68" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="G68" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="H68" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="I68" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="J68" s="1" t="s">
-        <v>169</v>
+        <v>121</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="1" t="str">
         <f aca="false">LibManager!A69</f>
-        <v>ResizeBilinear</v>
+        <v>SparseLengthsSum</v>
       </c>
       <c r="B69" s="1" t="n">
         <f aca="false">LibManager!B69</f>
@@ -4395,37 +4402,34 @@
       </c>
       <c r="C69" s="1" t="n">
         <f aca="false">LibManager!C69</f>
-        <v>1</v>
-      </c>
-      <c r="D69" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>100</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>116</v>
+        <v>137</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>117</v>
+        <v>138</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>118</v>
+        <v>134</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="I69" s="1" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="J69" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="K69" s="1" t="s">
-        <v>119</v>
+        <v>170</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="str">
         <f aca="false">LibManager!A70</f>
-        <v>ChannelWiseQuantizedConvolution</v>
+        <v>ResizeBilinear</v>
       </c>
       <c r="B70" s="1" t="n">
         <f aca="false">LibManager!B70</f>
@@ -4433,22 +4437,37 @@
       </c>
       <c r="C70" s="1" t="n">
         <f aca="false">LibManager!C70</f>
-        <v>7</v>
-      </c>
-      <c r="D70" s="1" t="s">
-        <v>25</v>
+        <v>1</v>
+      </c>
+      <c r="D70" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>153</v>
+        <v>117</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>154</v>
+        <v>118</v>
+      </c>
+      <c r="G70" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="H70" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="I70" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="J70" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="K70" s="1" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="str">
         <f aca="false">LibManager!A71</f>
-        <v>ConvTranspose</v>
+        <v>ChannelWiseQuantizedConvolution</v>
       </c>
       <c r="B71" s="1" t="n">
         <f aca="false">LibManager!B71</f>
@@ -4456,53 +4475,59 @@
       </c>
       <c r="C71" s="1" t="n">
         <f aca="false">LibManager!C71</f>
-        <v>3</v>
-      </c>
-      <c r="D71" s="1" t="n">
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>116</v>
+        <v>154</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="str">
         <f aca="false">LibManager!A72</f>
-        <v>NonMaxSuppression</v>
+        <v>ConvTranspose</v>
       </c>
       <c r="B72" s="1" t="n">
         <f aca="false">LibManager!B72</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C72" s="1" t="n">
         <f aca="false">LibManager!C72</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D72" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="F72" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="1" t="n">
+      <c r="A73" s="1" t="str">
         <f aca="false">LibManager!A73</f>
-        <v>0</v>
+        <v>NonMaxSuppression</v>
       </c>
       <c r="B73" s="1" t="n">
         <f aca="false">LibManager!B73</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C73" s="1" t="n">
         <f aca="false">LibManager!C73</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D73" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="E73" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4620,6 +4645,9 @@
         <f aca="false">LibManager!C80</f>
         <v>0</v>
       </c>
+      <c r="D80" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="1" t="n">
@@ -4632,6 +4660,20 @@
       </c>
       <c r="C81" s="1" t="n">
         <f aca="false">LibManager!C81</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A82" s="1" t="n">
+        <f aca="false">LibManager!A82</f>
+        <v>0</v>
+      </c>
+      <c r="B82" s="1" t="n">
+        <f aca="false">LibManager!B82</f>
+        <v>0</v>
+      </c>
+      <c r="C82" s="1" t="n">
+        <f aca="false">LibManager!C82</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[dnn-library] Executed libmanager script. It updates the automatic files as excel provided.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="196">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -2628,18 +2628,6 @@
       <c r="F12" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G12" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="I12" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>122</v>
-      </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="str">
@@ -3518,23 +3506,9 @@
         <v>1</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="F41" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="G41" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="H41" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="I41" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="J41" s="1" t="s">
-        <v>122</v>
-      </c>
+      <c r="I41" s="0"/>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="str">

</xml_diff>

<commit_message>
[dnn-library] [SW-11228] New splat implementation
A new Splat implementation that is simple to the point of being just a
memset-like mechanism using vector code.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="197">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -294,6 +294,9 @@
   </si>
   <si>
     <t xml:space="preserve">Splat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ValueBits</t>
   </si>
   <si>
     <t xml:space="preserve">Syncopy</t>
@@ -1848,7 +1851,7 @@
         <v>0</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="E57" s="1" t="n">
         <v>0</v>
@@ -1859,7 +1862,7 @@
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B58" s="1" t="n">
         <v>1</v>
@@ -1868,7 +1871,7 @@
         <v>1</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E58" s="1" t="n">
         <v>1</v>
@@ -1879,7 +1882,7 @@
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B59" s="1" t="n">
         <v>1</v>
@@ -1896,7 +1899,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B60" s="1" t="n">
         <v>1</v>
@@ -1916,7 +1919,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B61" s="1" t="n">
         <v>2</v>
@@ -1925,7 +1928,7 @@
         <v>1</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E61" s="1" t="n">
         <v>2</v>
@@ -1936,7 +1939,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B62" s="1" t="n">
         <v>1</v>
@@ -1945,7 +1948,7 @@
         <v>1</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E62" s="1" t="n">
         <v>1</v>
@@ -1959,7 +1962,7 @@
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B63" s="1" t="n">
         <v>2</v>
@@ -1968,10 +1971,10 @@
         <v>1</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G63" s="1" t="s">
         <v>8</v>
@@ -1979,7 +1982,7 @@
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B64" s="1" t="n">
         <v>1</v>
@@ -1988,7 +1991,7 @@
         <v>1</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E64" s="1" t="n">
         <v>1</v>
@@ -1999,7 +2002,7 @@
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B65" s="1" t="n">
         <v>1</v>
@@ -2008,7 +2011,7 @@
         <v>1</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E65" s="1" t="n">
         <v>1</v>
@@ -2019,7 +2022,7 @@
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B66" s="1" t="n">
         <v>1</v>
@@ -2028,7 +2031,7 @@
         <v>1</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E66" s="1" t="n">
         <v>0</v>
@@ -2039,7 +2042,7 @@
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B67" s="1" t="n">
         <v>1</v>
@@ -2048,7 +2051,7 @@
         <v>1</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E67" s="1" t="n">
         <v>0</v>
@@ -2059,7 +2062,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B68" s="1" t="n">
         <v>1</v>
@@ -2076,7 +2079,7 @@
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B69" s="1" t="n">
         <v>1</v>
@@ -2085,7 +2088,7 @@
         <v>3</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G69" s="1" t="s">
         <v>8</v>
@@ -2093,7 +2096,7 @@
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B70" s="1" t="n">
         <v>1</v>
@@ -2102,7 +2105,7 @@
         <v>1</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E70" s="1" t="n">
         <v>0</v>
@@ -2113,7 +2116,7 @@
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B71" s="1" t="n">
         <v>1</v>
@@ -2133,7 +2136,7 @@
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B72" s="1" t="n">
         <v>1</v>
@@ -2142,7 +2145,7 @@
         <v>3</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E72" s="1" t="n">
         <v>0</v>
@@ -2153,7 +2156,7 @@
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B73" s="1" t="n">
         <v>2</v>
@@ -2162,7 +2165,7 @@
         <v>2</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E73" s="1" t="n">
         <v>0</v>
@@ -2241,22 +2244,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2276,16 +2279,16 @@
         <v>1</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="I3" s="0"/>
       <c r="J3" s="0"/>
@@ -2307,13 +2310,13 @@
         <v>0</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2333,22 +2336,22 @@
         <v>0</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2368,22 +2371,22 @@
         <v>18</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2403,22 +2406,22 @@
         <v>1</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2438,67 +2441,67 @@
         <v>11</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L8" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="O8" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="M8" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="N8" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="O8" s="1" t="s">
-        <v>123</v>
-      </c>
       <c r="P8" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="R8" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="S8" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="T8" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="U8" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="V8" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="W8" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="X8" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="Y8" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2518,22 +2521,22 @@
         <v>25</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2553,22 +2556,22 @@
         <v>25</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2588,22 +2591,22 @@
         <v>0</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2623,10 +2626,10 @@
         <v>1</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2646,28 +2649,28 @@
         <v>11</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2687,19 +2690,19 @@
         <v>0</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H14" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="I14" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2719,19 +2722,19 @@
         <v>34</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2751,19 +2754,19 @@
         <v>34</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2783,19 +2786,19 @@
         <v>34</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2815,16 +2818,16 @@
         <v>0</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2844,10 +2847,10 @@
         <v>1</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2867,10 +2870,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2890,10 +2893,10 @@
         <v>1</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2913,10 +2916,10 @@
         <v>11</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2936,19 +2939,19 @@
         <v>0</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H23" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="I23" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="I23" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2968,19 +2971,19 @@
         <v>0</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H24" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="I24" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3000,19 +3003,19 @@
         <v>0</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H25" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="I25" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3032,10 +3035,10 @@
         <v>0</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3055,22 +3058,22 @@
         <v>0</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3090,19 +3093,19 @@
         <v>0</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H28" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="I28" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3122,10 +3125,10 @@
         <v>0</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3145,22 +3148,22 @@
         <v>1</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3180,25 +3183,25 @@
         <v>1</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3218,25 +3221,25 @@
         <v>25</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3256,10 +3259,10 @@
         <v>0</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3279,10 +3282,10 @@
         <v>0</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3302,34 +3305,34 @@
         <v>34</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="L35" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="M35" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3349,34 +3352,34 @@
         <v>59</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K36" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="L36" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="M36" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="N36" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3396,22 +3399,22 @@
         <v>1</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3431,10 +3434,10 @@
         <v>1</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3471,22 +3474,22 @@
         <v>1</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3506,7 +3509,7 @@
         <v>1</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I41" s="0"/>
     </row>
@@ -3527,10 +3530,10 @@
         <v>1</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3550,22 +3553,22 @@
         <v>1</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3585,25 +3588,25 @@
         <v>11</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3623,22 +3626,22 @@
         <v>1</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I45" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3658,10 +3661,10 @@
         <v>1</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3681,28 +3684,28 @@
         <v>11</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="I47" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="J47" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K47" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="L47" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3722,16 +3725,16 @@
         <v>1</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3768,16 +3771,16 @@
         <v>81</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3797,22 +3800,22 @@
         <v>0</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J51" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3832,10 +3835,10 @@
         <v>1</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3855,13 +3858,13 @@
         <v>1</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3881,31 +3884,31 @@
         <v>86</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="I54" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="J54" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="K54" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L54" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="M54" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3925,22 +3928,22 @@
         <v>0</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I55" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J55" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3960,22 +3963,22 @@
         <v>0</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I56" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J56" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3995,22 +3998,22 @@
         <v>0</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I57" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J57" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4030,22 +4033,22 @@
         <v>1</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J58" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4065,10 +4068,10 @@
         <v>1</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4088,22 +4091,22 @@
         <v>0</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I60" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J60" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4123,22 +4126,22 @@
         <v>2</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I61" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J61" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4158,22 +4161,22 @@
         <v>1</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I62" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J62" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4190,28 +4193,28 @@
         <v>1</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I63" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J63" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K63" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4231,22 +4234,22 @@
         <v>1</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I64" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J64" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4266,16 +4269,16 @@
         <v>1</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G65" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="H65" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="H65" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4295,16 +4298,16 @@
         <v>0</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4324,25 +4327,25 @@
         <v>0</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H67" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="I67" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="J67" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="I67" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="J67" s="1" t="s">
+      <c r="K67" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="K67" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4362,7 +4365,7 @@
         <v>0</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4379,25 +4382,25 @@
         <v>3</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I69" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J69" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4417,25 +4420,25 @@
         <v>0</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G70" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H70" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="I70" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="J70" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="I70" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="J70" s="1" t="s">
+      <c r="K70" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="K70" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4455,10 +4458,10 @@
         <v>25</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4478,7 +4481,7 @@
         <v>0</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4498,10 +4501,10 @@
         <v>2</v>
       </c>
       <c r="E73" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F73" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="F73" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] [SW-11122] New simpler maxplat implementation
The previous version was converting the source tensor to float
for applying the max operation between float elements, but a
better approach was possible by instead converting the splat
value to the source tensor type and operating with that type.

While I was at it I also did an experiment of reworking the
partitionLoop infrastructure so the caller can avoid passing
the compute operation as a function pointer, potentially messing
with the inlining of the function. The new alternative kernel
dispatching mechanism uses a preprocessor parameter for passing
the compute function name.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="196">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -242,7 +242,7 @@
     <t xml:space="preserve">MaxSplat</t>
   </si>
   <si>
-    <t xml:space="preserve">Value</t>
+    <t xml:space="preserve">ValueBits</t>
   </si>
   <si>
     <t xml:space="preserve">Aligned32Bytes</t>
@@ -294,9 +294,6 @@
   </si>
   <si>
     <t xml:space="preserve">Splat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ValueBits</t>
   </si>
   <si>
     <t xml:space="preserve">Syncopy</t>
@@ -1851,7 +1848,7 @@
         <v>0</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="E57" s="1" t="n">
         <v>0</v>
@@ -1862,16 +1859,16 @@
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B58" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="B58" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C58" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>93</v>
       </c>
       <c r="E58" s="1" t="n">
         <v>1</v>
@@ -1882,7 +1879,7 @@
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B59" s="1" t="n">
         <v>1</v>
@@ -1899,7 +1896,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B60" s="1" t="n">
         <v>1</v>
@@ -1919,7 +1916,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B61" s="1" t="n">
         <v>2</v>
@@ -1928,7 +1925,7 @@
         <v>1</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E61" s="1" t="n">
         <v>2</v>
@@ -1939,16 +1936,16 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B62" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C62" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" s="1" t="s">
         <v>97</v>
-      </c>
-      <c r="B62" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C62" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D62" s="1" t="s">
-        <v>98</v>
       </c>
       <c r="E62" s="1" t="n">
         <v>1</v>
@@ -1962,19 +1959,19 @@
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B63" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C63" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D63" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B63" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C63" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D63" s="1" t="s">
+      <c r="E63" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="E63" s="1" t="s">
-        <v>101</v>
       </c>
       <c r="G63" s="1" t="s">
         <v>8</v>
@@ -1982,16 +1979,16 @@
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B64" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C64" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" s="1" t="s">
         <v>102</v>
-      </c>
-      <c r="B64" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C64" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D64" s="1" t="s">
-        <v>103</v>
       </c>
       <c r="E64" s="1" t="n">
         <v>1</v>
@@ -2002,16 +1999,16 @@
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B65" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C65" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="B65" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C65" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D65" s="1" t="s">
-        <v>105</v>
       </c>
       <c r="E65" s="1" t="n">
         <v>1</v>
@@ -2022,16 +2019,16 @@
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B66" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C66" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="B66" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C66" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>107</v>
       </c>
       <c r="E66" s="1" t="n">
         <v>0</v>
@@ -2042,16 +2039,16 @@
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B67" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C67" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="B67" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C67" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D67" s="1" t="s">
-        <v>109</v>
       </c>
       <c r="E67" s="1" t="n">
         <v>0</v>
@@ -2062,7 +2059,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B68" s="1" t="n">
         <v>1</v>
@@ -2079,7 +2076,7 @@
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B69" s="1" t="n">
         <v>1</v>
@@ -2088,7 +2085,7 @@
         <v>3</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G69" s="1" t="s">
         <v>8</v>
@@ -2096,7 +2093,7 @@
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B70" s="1" t="n">
         <v>1</v>
@@ -2105,7 +2102,7 @@
         <v>1</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E70" s="1" t="n">
         <v>0</v>
@@ -2116,7 +2113,7 @@
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B71" s="1" t="n">
         <v>1</v>
@@ -2136,7 +2133,7 @@
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B72" s="1" t="n">
         <v>1</v>
@@ -2145,7 +2142,7 @@
         <v>3</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E72" s="1" t="n">
         <v>0</v>
@@ -2156,16 +2153,16 @@
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B73" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C73" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D73" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="B73" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C73" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="D73" s="1" t="s">
-        <v>117</v>
       </c>
       <c r="E73" s="1" t="n">
         <v>0</v>
@@ -2244,22 +2241,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2279,16 +2276,16 @@
         <v>1</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>126</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>127</v>
       </c>
       <c r="I3" s="0"/>
       <c r="J3" s="0"/>
@@ -2310,13 +2307,13 @@
         <v>0</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2336,22 +2333,22 @@
         <v>0</v>
       </c>
       <c r="E5" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="I5" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="J5" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2371,22 +2368,22 @@
         <v>18</v>
       </c>
       <c r="E6" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="I6" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="J6" s="1" t="s">
         <v>132</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2406,22 +2403,22 @@
         <v>1</v>
       </c>
       <c r="E7" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="I7" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="J7" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2441,67 +2438,67 @@
         <v>11</v>
       </c>
       <c r="E8" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="H8" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="I8" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="J8" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="J8" s="1" t="s">
+      <c r="K8" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="K8" s="1" t="s">
+      <c r="L8" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="M8" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="L8" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="M8" s="1" t="s">
+      <c r="N8" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="N8" s="1" t="s">
+      <c r="O8" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="P8" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="O8" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="P8" s="1" t="s">
+      <c r="Q8" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="Q8" s="1" t="s">
+      <c r="R8" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="R8" s="1" t="s">
+      <c r="S8" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="S8" s="1" t="s">
+      <c r="T8" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="T8" s="1" t="s">
+      <c r="U8" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="U8" s="1" t="s">
+      <c r="V8" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="V8" s="1" t="s">
+      <c r="W8" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="W8" s="1" t="s">
+      <c r="X8" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="X8" s="1" t="s">
+      <c r="Y8" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="Y8" s="1" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2521,22 +2518,22 @@
         <v>25</v>
       </c>
       <c r="E9" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="H9" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="I9" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="J9" s="1" t="s">
         <v>157</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2556,22 +2553,22 @@
         <v>25</v>
       </c>
       <c r="E10" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="H10" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="H10" s="1" t="s">
+      <c r="I10" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="J10" s="1" t="s">
         <v>157</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2591,22 +2588,22 @@
         <v>0</v>
       </c>
       <c r="E11" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="H11" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="I11" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="J11" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2626,10 +2623,10 @@
         <v>1</v>
       </c>
       <c r="E12" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2649,28 +2646,28 @@
         <v>11</v>
       </c>
       <c r="E13" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="G13" s="1" t="s">
+      <c r="H13" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="H13" s="1" t="s">
+      <c r="I13" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="I13" s="1" t="s">
+      <c r="J13" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="J13" s="1" t="s">
+      <c r="K13" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="K13" s="1" t="s">
+      <c r="L13" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="L13" s="1" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2690,19 +2687,19 @@
         <v>0</v>
       </c>
       <c r="E14" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G14" s="1" t="s">
+      <c r="H14" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I14" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2722,19 +2719,19 @@
         <v>34</v>
       </c>
       <c r="E15" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="G15" s="1" t="s">
-        <v>155</v>
-      </c>
       <c r="H15" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="I15" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2754,19 +2751,19 @@
         <v>34</v>
       </c>
       <c r="E16" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="G16" s="1" t="s">
-        <v>155</v>
-      </c>
       <c r="H16" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="I16" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2786,19 +2783,19 @@
         <v>34</v>
       </c>
       <c r="E17" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="F17" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="G17" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="G17" s="1" t="s">
-        <v>155</v>
-      </c>
       <c r="H17" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="I17" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2818,16 +2815,16 @@
         <v>0</v>
       </c>
       <c r="E18" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="G18" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="H18" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2847,10 +2844,10 @@
         <v>1</v>
       </c>
       <c r="E19" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2870,10 +2867,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2893,10 +2890,10 @@
         <v>1</v>
       </c>
       <c r="E21" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2916,10 +2913,10 @@
         <v>11</v>
       </c>
       <c r="E22" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2939,19 +2936,19 @@
         <v>0</v>
       </c>
       <c r="E23" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F23" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F23" s="1" t="s">
+      <c r="G23" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G23" s="1" t="s">
+      <c r="H23" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I23" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="H23" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="I23" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2971,19 +2968,19 @@
         <v>0</v>
       </c>
       <c r="E24" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F24" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F24" s="1" t="s">
+      <c r="G24" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G24" s="1" t="s">
+      <c r="H24" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I24" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="H24" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3003,19 +3000,19 @@
         <v>0</v>
       </c>
       <c r="E25" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F25" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F25" s="1" t="s">
+      <c r="G25" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G25" s="1" t="s">
+      <c r="H25" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I25" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="H25" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3035,10 +3032,10 @@
         <v>0</v>
       </c>
       <c r="E26" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F26" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3058,22 +3055,22 @@
         <v>0</v>
       </c>
       <c r="E27" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F27" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F27" s="1" t="s">
+      <c r="G27" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G27" s="1" t="s">
+      <c r="H27" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H27" s="1" t="s">
+      <c r="I27" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I27" s="1" t="s">
+      <c r="J27" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J27" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3093,19 +3090,19 @@
         <v>0</v>
       </c>
       <c r="E28" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F28" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="G28" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G28" s="1" t="s">
+      <c r="H28" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I28" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="H28" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3125,10 +3122,10 @@
         <v>0</v>
       </c>
       <c r="E29" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F29" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3148,22 +3145,22 @@
         <v>1</v>
       </c>
       <c r="E30" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F30" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="G30" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G30" s="1" t="s">
+      <c r="H30" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H30" s="1" t="s">
+      <c r="I30" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I30" s="1" t="s">
+      <c r="J30" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J30" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3183,25 +3180,25 @@
         <v>1</v>
       </c>
       <c r="E31" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F31" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F31" s="1" t="s">
+      <c r="G31" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G31" s="1" t="s">
+      <c r="H31" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H31" s="1" t="s">
+      <c r="I31" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I31" s="1" t="s">
+      <c r="J31" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="J31" s="1" t="s">
-        <v>123</v>
-      </c>
       <c r="K31" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3221,25 +3218,25 @@
         <v>25</v>
       </c>
       <c r="E32" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="F32" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="F32" s="1" t="s">
+      <c r="G32" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="G32" s="1" t="s">
+      <c r="H32" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="H32" s="1" t="s">
+      <c r="I32" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="J32" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="I32" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="J32" s="1" t="s">
+      <c r="K32" s="1" t="s">
         <v>157</v>
-      </c>
-      <c r="K32" s="1" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3259,10 +3256,10 @@
         <v>0</v>
       </c>
       <c r="E33" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F33" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3282,10 +3279,10 @@
         <v>0</v>
       </c>
       <c r="E34" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F34" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3305,34 +3302,34 @@
         <v>34</v>
       </c>
       <c r="E35" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="J35" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="F35" s="1" t="s">
+      <c r="K35" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="G35" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="H35" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="I35" s="1" t="s">
+      <c r="L35" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="J35" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="K35" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="L35" s="1" t="s">
+      <c r="M35" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="M35" s="1" t="s">
+      <c r="N35" s="1" t="s">
         <v>175</v>
-      </c>
-      <c r="N35" s="1" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3352,34 +3349,34 @@
         <v>59</v>
       </c>
       <c r="E36" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="J36" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="F36" s="1" t="s">
+      <c r="K36" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="G36" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="H36" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="I36" s="1" t="s">
+      <c r="L36" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="J36" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="K36" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="L36" s="1" t="s">
+      <c r="M36" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="M36" s="1" t="s">
+      <c r="N36" s="1" t="s">
         <v>175</v>
-      </c>
-      <c r="N36" s="1" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3399,22 +3396,22 @@
         <v>1</v>
       </c>
       <c r="E37" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F37" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F37" s="1" t="s">
+      <c r="G37" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G37" s="1" t="s">
+      <c r="H37" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H37" s="1" t="s">
+      <c r="I37" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I37" s="1" t="s">
+      <c r="J37" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J37" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3434,10 +3431,10 @@
         <v>1</v>
       </c>
       <c r="E38" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F38" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3474,22 +3471,22 @@
         <v>1</v>
       </c>
       <c r="E40" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F40" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F40" s="1" t="s">
+      <c r="G40" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G40" s="1" t="s">
+      <c r="H40" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H40" s="1" t="s">
+      <c r="I40" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I40" s="1" t="s">
+      <c r="J40" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J40" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3509,7 +3506,7 @@
         <v>1</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="I41" s="0"/>
     </row>
@@ -3530,10 +3527,10 @@
         <v>1</v>
       </c>
       <c r="E42" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F42" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="F42" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3553,22 +3550,22 @@
         <v>1</v>
       </c>
       <c r="E43" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F43" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F43" s="1" t="s">
+      <c r="G43" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G43" s="1" t="s">
+      <c r="H43" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H43" s="1" t="s">
+      <c r="I43" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I43" s="1" t="s">
+      <c r="J43" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J43" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3588,25 +3585,25 @@
         <v>11</v>
       </c>
       <c r="E44" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="F44" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="F44" s="1" t="s">
+      <c r="G44" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="H44" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="G44" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="H44" s="1" t="s">
+      <c r="I44" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="I44" s="1" t="s">
+      <c r="J44" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="J44" s="1" t="s">
-        <v>181</v>
-      </c>
       <c r="K44" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3626,22 +3623,22 @@
         <v>1</v>
       </c>
       <c r="E45" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F45" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F45" s="1" t="s">
+      <c r="G45" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G45" s="1" t="s">
+      <c r="H45" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H45" s="1" t="s">
+      <c r="I45" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I45" s="1" t="s">
+      <c r="J45" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J45" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3661,10 +3658,10 @@
         <v>1</v>
       </c>
       <c r="E46" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="F46" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="F46" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3684,28 +3681,28 @@
         <v>11</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F47" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="G47" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="G47" s="1" t="s">
+      <c r="H47" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="H47" s="1" t="s">
+      <c r="I47" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="I47" s="1" t="s">
+      <c r="J47" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="J47" s="1" t="s">
+      <c r="K47" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="K47" s="1" t="s">
+      <c r="L47" s="1" t="s">
         <v>187</v>
-      </c>
-      <c r="L47" s="1" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3725,16 +3722,16 @@
         <v>1</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3771,16 +3768,16 @@
         <v>81</v>
       </c>
       <c r="E50" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="F50" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="F50" s="1" t="s">
-        <v>139</v>
-      </c>
       <c r="G50" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="H50" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="H50" s="1" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3800,22 +3797,22 @@
         <v>0</v>
       </c>
       <c r="E51" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F51" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F51" s="1" t="s">
+      <c r="G51" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G51" s="1" t="s">
+      <c r="H51" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H51" s="1" t="s">
+      <c r="I51" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I51" s="1" t="s">
+      <c r="J51" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J51" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3835,10 +3832,10 @@
         <v>1</v>
       </c>
       <c r="E52" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F52" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="F52" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3858,13 +3855,13 @@
         <v>1</v>
       </c>
       <c r="E53" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F53" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F53" s="1" t="s">
-        <v>119</v>
-      </c>
       <c r="G53" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3884,31 +3881,31 @@
         <v>86</v>
       </c>
       <c r="E54" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="F54" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="F54" s="1" t="s">
+      <c r="G54" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="G54" s="1" t="s">
+      <c r="H54" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="H54" s="1" t="s">
+      <c r="I54" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="I54" s="1" t="s">
+      <c r="J54" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="J54" s="1" t="s">
-        <v>196</v>
-      </c>
       <c r="K54" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="L54" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="M54" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3928,22 +3925,22 @@
         <v>0</v>
       </c>
       <c r="E55" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F55" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F55" s="1" t="s">
+      <c r="G55" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G55" s="1" t="s">
+      <c r="H55" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H55" s="1" t="s">
+      <c r="I55" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I55" s="1" t="s">
+      <c r="J55" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J55" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3963,22 +3960,22 @@
         <v>0</v>
       </c>
       <c r="E56" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F56" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F56" s="1" t="s">
+      <c r="G56" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G56" s="1" t="s">
+      <c r="H56" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H56" s="1" t="s">
+      <c r="I56" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I56" s="1" t="s">
+      <c r="J56" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J56" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3998,22 +3995,22 @@
         <v>0</v>
       </c>
       <c r="E57" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F57" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F57" s="1" t="s">
+      <c r="G57" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G57" s="1" t="s">
+      <c r="H57" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H57" s="1" t="s">
+      <c r="I57" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I57" s="1" t="s">
+      <c r="J57" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J57" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4033,22 +4030,22 @@
         <v>1</v>
       </c>
       <c r="E58" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F58" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F58" s="1" t="s">
+      <c r="G58" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G58" s="1" t="s">
+      <c r="H58" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H58" s="1" t="s">
+      <c r="I58" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I58" s="1" t="s">
+      <c r="J58" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J58" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4068,10 +4065,10 @@
         <v>1</v>
       </c>
       <c r="E59" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F59" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="F59" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4091,22 +4088,22 @@
         <v>0</v>
       </c>
       <c r="E60" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F60" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F60" s="1" t="s">
+      <c r="G60" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G60" s="1" t="s">
+      <c r="H60" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H60" s="1" t="s">
+      <c r="I60" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I60" s="1" t="s">
+      <c r="J60" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J60" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4126,22 +4123,22 @@
         <v>2</v>
       </c>
       <c r="E61" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F61" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F61" s="1" t="s">
+      <c r="G61" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G61" s="1" t="s">
+      <c r="H61" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H61" s="1" t="s">
+      <c r="I61" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I61" s="1" t="s">
+      <c r="J61" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J61" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4161,22 +4158,22 @@
         <v>1</v>
       </c>
       <c r="E62" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F62" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F62" s="1" t="s">
+      <c r="G62" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G62" s="1" t="s">
+      <c r="H62" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H62" s="1" t="s">
+      <c r="I62" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I62" s="1" t="s">
+      <c r="J62" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J62" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4193,28 +4190,28 @@
         <v>1</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E63" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="F63" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="F63" s="1" t="s">
+      <c r="G63" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="H63" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="G63" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="H63" s="1" t="s">
+      <c r="I63" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="I63" s="1" t="s">
+      <c r="J63" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="J63" s="1" t="s">
-        <v>181</v>
-      </c>
       <c r="K63" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4234,22 +4231,22 @@
         <v>1</v>
       </c>
       <c r="E64" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F64" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F64" s="1" t="s">
+      <c r="G64" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G64" s="1" t="s">
+      <c r="H64" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H64" s="1" t="s">
+      <c r="I64" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I64" s="1" t="s">
+      <c r="J64" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J64" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4269,16 +4266,16 @@
         <v>1</v>
       </c>
       <c r="E65" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F65" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F65" s="1" t="s">
-        <v>119</v>
-      </c>
       <c r="G65" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4298,16 +4295,16 @@
         <v>0</v>
       </c>
       <c r="E66" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F66" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F66" s="1" t="s">
+      <c r="G66" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G66" s="1" t="s">
+      <c r="H66" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="H66" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4327,25 +4324,25 @@
         <v>0</v>
       </c>
       <c r="E67" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F67" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F67" s="1" t="s">
+      <c r="G67" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G67" s="1" t="s">
+      <c r="H67" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="I67" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="J67" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="K67" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="H67" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="I67" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="J67" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="K67" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4365,7 +4362,7 @@
         <v>0</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4382,25 +4379,25 @@
         <v>3</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E69" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="F69" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="F69" s="1" t="s">
-        <v>139</v>
-      </c>
       <c r="G69" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="H69" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="H69" s="1" t="s">
-        <v>136</v>
-      </c>
       <c r="I69" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="J69" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4420,25 +4417,25 @@
         <v>0</v>
       </c>
       <c r="E70" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F70" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F70" s="1" t="s">
+      <c r="G70" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G70" s="1" t="s">
+      <c r="H70" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="I70" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="J70" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="K70" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="H70" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="I70" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="J70" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="K70" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4458,10 +4455,10 @@
         <v>25</v>
       </c>
       <c r="E71" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="F71" s="1" t="s">
         <v>155</v>
-      </c>
-      <c r="F71" s="1" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4481,7 +4478,7 @@
         <v>0</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4501,10 +4498,10 @@
         <v>2</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] [SW-13621] Support Quantized-weights in EmbeddingBag - Preliminary sequential implementation
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="198">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -173,6 +173,9 @@
     <t xml:space="preserve">HasEndOffset</t>
   </si>
   <si>
+    <t xml:space="preserve">0,2</t>
+  </si>
+  <si>
     <t xml:space="preserve">ExtractTensor</t>
   </si>
   <si>
@@ -321,9 +324,6 @@
   </si>
   <si>
     <t xml:space="preserve">Kernels, Strides, Pads, Layout</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0,2</t>
   </si>
   <si>
     <t xml:space="preserve">BatchedReduceMin</t>
@@ -1329,8 +1329,8 @@
       <c r="D29" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="E29" s="1" t="n">
-        <v>0</v>
+      <c r="E29" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="G29" s="1" t="s">
         <v>8</v>
@@ -1338,7 +1338,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B30" s="1" t="n">
         <v>1</v>
@@ -1347,7 +1347,7 @@
         <v>1</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E30" s="1" t="n">
         <v>1</v>
@@ -1358,7 +1358,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B31" s="1" t="n">
         <v>1</v>
@@ -1378,7 +1378,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B32" s="1" t="n">
         <v>1</v>
@@ -1395,7 +1395,7 @@
     </row>
     <row r="33" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B33" s="1" t="n">
         <v>1</v>
@@ -1412,7 +1412,7 @@
     </row>
     <row r="34" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B34" s="1" t="n">
         <v>1</v>
@@ -1429,7 +1429,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B35" s="1" t="n">
         <v>1</v>
@@ -1438,7 +1438,7 @@
         <v>2</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>34</v>
@@ -1449,7 +1449,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B36" s="1" t="n">
         <v>2</v>
@@ -1458,7 +1458,7 @@
         <v>2</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G36" s="1" t="s">
         <v>8</v>
@@ -1466,7 +1466,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B37" s="1" t="n">
         <v>1</v>
@@ -1475,7 +1475,7 @@
         <v>1</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E37" s="1" t="n">
         <v>1</v>
@@ -1489,7 +1489,7 @@
     </row>
     <row r="38" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B38" s="1" t="n">
         <v>1</v>
@@ -1506,7 +1506,7 @@
     </row>
     <row r="39" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B39" s="1" t="n">
         <v>1</v>
@@ -1515,7 +1515,7 @@
         <v>2</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G39" s="1" t="s">
         <v>8</v>
@@ -1523,7 +1523,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B40" s="1" t="n">
         <v>1</v>
@@ -1540,7 +1540,7 @@
     </row>
     <row r="41" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B41" s="1" t="n">
         <v>1</v>
@@ -1557,7 +1557,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B42" s="1" t="n">
         <v>2</v>
@@ -1566,7 +1566,7 @@
         <v>1</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E42" s="1" t="n">
         <v>1</v>
@@ -1580,7 +1580,7 @@
     </row>
     <row r="43" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B43" s="1" t="n">
         <v>1</v>
@@ -1597,7 +1597,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B44" s="1" t="n">
         <v>1</v>
@@ -1606,7 +1606,7 @@
         <v>1</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>11</v>
@@ -1617,7 +1617,7 @@
     </row>
     <row r="45" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B45" s="1" t="n">
         <v>1</v>
@@ -1626,13 +1626,13 @@
         <v>1</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E45" s="1" t="n">
         <v>1</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G45" s="1" t="s">
         <v>15</v>
@@ -1640,7 +1640,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B46" s="1" t="n">
         <v>1</v>
@@ -1649,7 +1649,7 @@
         <v>1</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E46" s="1" t="n">
         <v>1</v>
@@ -1660,7 +1660,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B47" s="1" t="n">
         <v>1</v>
@@ -1677,7 +1677,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B48" s="1" t="n">
         <v>1</v>
@@ -1694,7 +1694,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B49" s="1" t="n">
         <v>1</v>
@@ -1703,10 +1703,10 @@
         <v>5</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G49" s="1" t="s">
         <v>15</v>
@@ -1714,7 +1714,7 @@
     </row>
     <row r="50" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B50" s="1" t="n">
         <v>1</v>
@@ -1723,7 +1723,7 @@
         <v>6</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>22</v>
@@ -1734,7 +1734,7 @@
     </row>
     <row r="51" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B51" s="1" t="n">
         <v>1</v>
@@ -1751,7 +1751,7 @@
     </row>
     <row r="52" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B52" s="1" t="n">
         <v>1</v>
@@ -1768,7 +1768,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B53" s="1" t="n">
         <v>1</v>
@@ -1788,7 +1788,7 @@
     </row>
     <row r="54" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B54" s="1" t="n">
         <v>1</v>
@@ -1797,7 +1797,7 @@
         <v>4</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F54" s="1" t="s">
         <v>14</v>
@@ -1808,7 +1808,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B55" s="1" t="n">
         <v>1</v>
@@ -1825,7 +1825,7 @@
     </row>
     <row r="56" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B56" s="1" t="n">
         <v>1</v>
@@ -1834,7 +1834,7 @@
         <v>4</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E56" s="1" t="n">
         <v>0</v>
@@ -1845,7 +1845,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B57" s="1" t="n">
         <v>1</v>
@@ -1854,7 +1854,7 @@
         <v>0</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E57" s="1" t="n">
         <v>0</v>
@@ -1865,7 +1865,7 @@
     </row>
     <row r="58" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B58" s="1" t="n">
         <v>1</v>
@@ -1874,7 +1874,7 @@
         <v>1</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E58" s="1" t="n">
         <v>1</v>
@@ -1885,7 +1885,7 @@
     </row>
     <row r="59" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B59" s="1" t="n">
         <v>1</v>
@@ -1902,7 +1902,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B60" s="1" t="n">
         <v>1</v>
@@ -1911,7 +1911,7 @@
         <v>1</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E60" s="1" t="n">
         <v>0</v>
@@ -1922,7 +1922,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B61" s="1" t="n">
         <v>2</v>
@@ -1931,7 +1931,7 @@
         <v>1</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E61" s="1" t="n">
         <v>2</v>
@@ -1942,7 +1942,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B62" s="1" t="n">
         <v>1</v>
@@ -1951,13 +1951,13 @@
         <v>1</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E62" s="1" t="n">
         <v>1</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G62" s="1" t="s">
         <v>15</v>
@@ -1965,7 +1965,7 @@
     </row>
     <row r="63" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B63" s="1" t="n">
         <v>2</v>
@@ -1974,10 +1974,10 @@
         <v>1</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G63" s="1" t="s">
         <v>8</v>
@@ -2091,7 +2091,7 @@
         <v>3</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F69" s="1" t="s">
         <v>14</v>
@@ -2203,6 +2203,7 @@
     <row r="75" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="76" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="77" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048575" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
@@ -2227,7 +2228,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44.99"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="10.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.64"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="19.99"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="21.17"/>
@@ -3148,14 +3149,17 @@
         <f aca="false">LibManager!C29</f>
         <v>4</v>
       </c>
-      <c r="D29" s="1" t="n">
-        <v>0</v>
+      <c r="D29" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>119</v>
+        <v>154</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>120</v>
+        <v>155</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3376,7 +3380,7 @@
         <v>2</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>139</v>
@@ -3481,7 +3485,7 @@
         <v>2</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3777,7 +3781,7 @@
         <v>5</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3794,7 +3798,7 @@
         <v>6</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E50" s="1" t="s">
         <v>139</v>
@@ -3907,7 +3911,7 @@
         <v>4</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>192</v>
@@ -4219,7 +4223,7 @@
         <v>1</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>178</v>
@@ -4408,7 +4412,7 @@
         <v>3</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>139</v>

</xml_diff>

<commit_message>
[dnn-library] [SW-13621] dequantie data instead of weights - There is an occupied semantics case here. wegihts go into "data" for   the EB op PoV
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
@@ -173,157 +173,157 @@
     <t xml:space="preserve">HasEndOffset</t>
   </si>
   <si>
+    <t xml:space="preserve">ExtractTensor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Offsets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FullyConnected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FusedRowwiseQuantizedSparseLengthsSum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FusedRowwiseQuantizedSparseLengthsWeightedSum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gather</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BatchDims</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GatherRanges</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsertTensor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Offsets, Count,Axis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Int8Converter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IntLookupTable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NONE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LengthsSum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LengthsToRanges</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LocalResponseNormalization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HalfWindowSize, Alpha, Beta, K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MatMul</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MaxPool</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kernels, Strides, Pads,Layout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MaxSplat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ValueBits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aligned32Bytes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modulo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Divisor, SignFollowDivisor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quantize</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RescaleQuantized</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RowwiseQuantizedFullyConnected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RowwiseQuantizedSparseLengthsWeightedSum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ScatterData</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sigmoid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SoftMax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SparseLengthsWeightedSum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SparseToDense</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SparseToDenseMask</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mask</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Splat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Syncopy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SyncOffset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tanh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TensorView</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TopK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transpose</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shuffle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MaxPoolWithArgMax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kernels, Strides, Pads, Layout</t>
+  </si>
+  <si>
     <t xml:space="preserve">0,2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ExtractTensor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Offsets</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flip</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FullyConnected</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FusedRowwiseQuantizedSparseLengthsSum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FusedRowwiseQuantizedSparseLengthsWeightedSum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gather</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BatchDims</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GatherRanges</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsertTensor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Offsets, Count,Axis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int8Converter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IntLookupTable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NONE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LengthsSum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LengthsToRanges</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LocalResponseNormalization</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HalfWindowSize, Alpha, Beta, K</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MatMul</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MaxPool</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kernels, Strides, Pads,Layout</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MaxSplat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ValueBits</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aligned32Bytes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modulo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Divisor, SignFollowDivisor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quantize</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RescaleQuantized</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RowwiseQuantizedFullyConnected</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RowwiseQuantizedSparseLengthsWeightedSum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0,5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ScatterData</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sigmoid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SoftMax</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SparseLengthsWeightedSum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SparseToDense</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SparseToDenseMask</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mask</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Splat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Syncopy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SyncOffset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tanh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TensorView</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TopK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Transpose</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shuffle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MaxPoolWithArgMax</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kernels, Strides, Pads, Layout</t>
   </si>
   <si>
     <t xml:space="preserve">BatchedReduceMin</t>
@@ -1330,7 +1330,7 @@
         <v>49</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="G29" s="1" t="s">
         <v>8</v>
@@ -1338,16 +1338,16 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B30" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="B30" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C30" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>52</v>
       </c>
       <c r="E30" s="1" t="n">
         <v>1</v>
@@ -1358,7 +1358,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B31" s="1" t="n">
         <v>1</v>
@@ -1378,7 +1378,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B32" s="1" t="n">
         <v>1</v>
@@ -1395,7 +1395,7 @@
     </row>
     <row r="33" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B33" s="1" t="n">
         <v>1</v>
@@ -1412,7 +1412,7 @@
     </row>
     <row r="34" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B34" s="1" t="n">
         <v>1</v>
@@ -1429,16 +1429,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D35" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="B35" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C35" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>58</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>34</v>
@@ -1449,16 +1449,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C36" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="B36" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C36" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>60</v>
       </c>
       <c r="G36" s="1" t="s">
         <v>8</v>
@@ -1466,16 +1466,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B37" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="B37" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C37" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>62</v>
       </c>
       <c r="E37" s="1" t="n">
         <v>1</v>
@@ -1489,7 +1489,7 @@
     </row>
     <row r="38" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B38" s="1" t="n">
         <v>1</v>
@@ -1506,16 +1506,16 @@
     </row>
     <row r="39" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B39" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E39" s="1" t="s">
         <v>64</v>
-      </c>
-      <c r="B39" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C39" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>65</v>
       </c>
       <c r="G39" s="1" t="s">
         <v>8</v>
@@ -1523,7 +1523,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B40" s="1" t="n">
         <v>1</v>
@@ -1540,7 +1540,7 @@
     </row>
     <row r="41" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B41" s="1" t="n">
         <v>1</v>
@@ -1557,16 +1557,16 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B42" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C42" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="B42" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C42" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>69</v>
       </c>
       <c r="E42" s="1" t="n">
         <v>1</v>
@@ -1580,7 +1580,7 @@
     </row>
     <row r="43" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B43" s="1" t="n">
         <v>1</v>
@@ -1597,16 +1597,16 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B44" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="1" t="s">
         <v>71</v>
-      </c>
-      <c r="B44" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C44" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>11</v>
@@ -1617,22 +1617,22 @@
     </row>
     <row r="45" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B45" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B45" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C45" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D45" s="1" t="s">
+      <c r="E45" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F45" s="1" t="s">
         <v>74</v>
-      </c>
-      <c r="E45" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>75</v>
       </c>
       <c r="G45" s="1" t="s">
         <v>15</v>
@@ -1640,16 +1640,16 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B46" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="1" t="s">
         <v>76</v>
-      </c>
-      <c r="B46" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C46" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D46" s="1" t="s">
-        <v>77</v>
       </c>
       <c r="E46" s="1" t="n">
         <v>1</v>
@@ -1660,7 +1660,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B47" s="1" t="n">
         <v>1</v>
@@ -1677,7 +1677,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B48" s="1" t="n">
         <v>1</v>
@@ -1694,7 +1694,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B49" s="1" t="n">
         <v>1</v>
@@ -1703,10 +1703,10 @@
         <v>5</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G49" s="1" t="s">
         <v>15</v>
@@ -1714,7 +1714,7 @@
     </row>
     <row r="50" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B50" s="1" t="n">
         <v>1</v>
@@ -1723,7 +1723,7 @@
         <v>6</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>22</v>
@@ -1734,7 +1734,7 @@
     </row>
     <row r="51" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B51" s="1" t="n">
         <v>1</v>
@@ -1751,7 +1751,7 @@
     </row>
     <row r="52" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B52" s="1" t="n">
         <v>1</v>
@@ -1768,7 +1768,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B53" s="1" t="n">
         <v>1</v>
@@ -1788,7 +1788,7 @@
     </row>
     <row r="54" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B54" s="1" t="n">
         <v>1</v>
@@ -1797,7 +1797,7 @@
         <v>4</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F54" s="1" t="s">
         <v>14</v>
@@ -1808,7 +1808,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B55" s="1" t="n">
         <v>1</v>
@@ -1825,7 +1825,7 @@
     </row>
     <row r="56" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B56" s="1" t="n">
         <v>1</v>
@@ -1834,7 +1834,7 @@
         <v>4</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E56" s="1" t="n">
         <v>0</v>
@@ -1845,7 +1845,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B57" s="1" t="n">
         <v>1</v>
@@ -1854,7 +1854,7 @@
         <v>0</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E57" s="1" t="n">
         <v>0</v>
@@ -1865,16 +1865,16 @@
     </row>
     <row r="58" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B58" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="B58" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C58" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>93</v>
       </c>
       <c r="E58" s="1" t="n">
         <v>1</v>
@@ -1885,7 +1885,7 @@
     </row>
     <row r="59" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B59" s="1" t="n">
         <v>1</v>
@@ -1902,7 +1902,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B60" s="1" t="n">
         <v>1</v>
@@ -1911,7 +1911,7 @@
         <v>1</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E60" s="1" t="n">
         <v>0</v>
@@ -1922,7 +1922,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B61" s="1" t="n">
         <v>2</v>
@@ -1931,7 +1931,7 @@
         <v>1</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E61" s="1" t="n">
         <v>2</v>
@@ -1942,22 +1942,22 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B62" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C62" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B62" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C62" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D62" s="1" t="s">
-        <v>98</v>
-      </c>
       <c r="E62" s="1" t="n">
         <v>1</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G62" s="1" t="s">
         <v>15</v>
@@ -1965,19 +1965,19 @@
     </row>
     <row r="63" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B63" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C63" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D63" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B63" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C63" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D63" s="1" t="s">
+      <c r="E63" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="E63" s="1" t="s">
-        <v>50</v>
       </c>
       <c r="G63" s="1" t="s">
         <v>8</v>
@@ -2091,7 +2091,7 @@
         <v>3</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F69" s="1" t="s">
         <v>14</v>
@@ -3150,7 +3150,7 @@
         <v>4</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>154</v>
@@ -3380,7 +3380,7 @@
         <v>2</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>139</v>
@@ -3485,7 +3485,7 @@
         <v>2</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3781,7 +3781,7 @@
         <v>5</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3798,7 +3798,7 @@
         <v>6</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E50" s="1" t="s">
         <v>139</v>
@@ -3911,7 +3911,7 @@
         <v>4</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>192</v>
@@ -4223,7 +4223,7 @@
         <v>1</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>178</v>
@@ -4412,7 +4412,7 @@
         <v>3</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>139</v>

</xml_diff>

<commit_message>
[dnn-library] [SW-16712] Extend CumSum to support multiple dims and axis
- Extend lib implementation of CumSum to support multiple dimensions
  and accumulation axis.

- TODO: support negative axis. Needs changes in the Api.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="LibManager" sheetId="1" state="visible" r:id="rId2"/>
@@ -362,7 +362,7 @@
     <t xml:space="preserve">CumSum</t>
   </si>
   <si>
-    <t xml:space="preserve">Exclusive, Reverse</t>
+    <t xml:space="preserve">Exclusive, Reverse, Axis</t>
   </si>
   <si>
     <t xml:space="preserve">SpaceToDepth</t>

</xml_diff>

<commit_message>
[dnn-library] [SW-19566] Add Profile instruction - profile instruction traverses the input tensor and provides the min and max values to the provided offset in the output tensor as float 32 values.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="665" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="221">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -284,6 +284,12 @@
     <t xml:space="preserve">Divisor, SignFollowDivisor</t>
   </si>
   <si>
+    <t xml:space="preserve">Profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SyncOffset</t>
+  </si>
+  <si>
     <t xml:space="preserve">Quantize</t>
   </si>
   <si>
@@ -327,9 +333,6 @@
   </si>
   <si>
     <t xml:space="preserve">Syncopy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SyncOffset</t>
   </si>
   <si>
     <t xml:space="preserve">Tanh</t>
@@ -793,12 +796,12 @@
     </xf>
   </cellXfs>
   <cellStyles count="6">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="false"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3" customBuiltin="false"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6" customBuiltin="false"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4" customBuiltin="false"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7" customBuiltin="false"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5" customBuiltin="false"/>
   </cellStyles>
   <colors>
     <indexedColors>
@@ -864,12 +867,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G83"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:G84"/>
+  <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.83"/>
@@ -878,7 +881,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="32.49"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="7.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="1" width="48.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="1" width="48.35"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="13.83"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="12" style="1" width="11.84"/>
   </cols>
@@ -1901,8 +1904,11 @@
       <c r="C55" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E55" s="1" t="s">
-        <v>11</v>
+      <c r="D55" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E55" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="G55" s="1" t="s">
         <v>8</v>
@@ -1910,7 +1916,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B56" s="1" t="n">
         <v>1</v>
@@ -1918,8 +1924,8 @@
       <c r="C56" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E56" s="1" t="n">
-        <v>1</v>
+      <c r="E56" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="G56" s="1" t="s">
         <v>8</v>
@@ -1927,39 +1933,36 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B57" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C57" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B58" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="E57" s="1" t="s">
+      <c r="E58" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="F57" s="1" t="s">
+      <c r="F58" s="1" t="s">
         <v>84</v>
-      </c>
-      <c r="G57" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B58" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C58" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="E58" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="F58" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="G58" s="1" t="s">
         <v>15</v>
@@ -1973,35 +1976,38 @@
         <v>1</v>
       </c>
       <c r="C59" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E59" s="1" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>22</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B60" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C60" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E60" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G60" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B61" s="1" t="n">
         <v>1</v>
@@ -2012,34 +2018,31 @@
       <c r="E61" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="F61" s="1" t="s">
+      <c r="G61" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B62" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C62" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F62" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="G61" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="B62" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C62" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E62" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="F62" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="G62" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
         <v>97</v>
       </c>
@@ -2047,27 +2050,27 @@
         <v>1</v>
       </c>
       <c r="C63" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E63" s="1" t="n">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F63" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B64" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C64" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="D64" s="1" t="s">
-        <v>99</v>
+        <v>2</v>
       </c>
       <c r="E64" s="1" t="n">
         <v>0</v>
@@ -2076,7 +2079,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
         <v>100</v>
       </c>
@@ -2084,33 +2087,33 @@
         <v>1</v>
       </c>
       <c r="C65" s="1" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D65" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="E65" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B66" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C66" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D66" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="E65" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G65" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="B66" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C66" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>102</v>
-      </c>
       <c r="E66" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G66" s="1" t="s">
         <v>8</v>
@@ -2126,6 +2129,9 @@
       <c r="C67" s="1" t="n">
         <v>1</v>
       </c>
+      <c r="D67" s="1" t="s">
+        <v>88</v>
+      </c>
       <c r="E67" s="1" t="n">
         <v>1</v>
       </c>
@@ -2133,7 +2139,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
         <v>104</v>
       </c>
@@ -2143,11 +2149,8 @@
       <c r="C68" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D68" s="1" t="s">
-        <v>62</v>
-      </c>
       <c r="E68" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G68" s="1" t="s">
         <v>8</v>
@@ -2158,16 +2161,16 @@
         <v>105</v>
       </c>
       <c r="B69" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C69" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>105</v>
+        <v>62</v>
       </c>
       <c r="E69" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G69" s="1" t="s">
         <v>8</v>
@@ -2178,59 +2181,59 @@
         <v>106</v>
       </c>
       <c r="B70" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C70" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E70" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F70" s="1" t="s">
-        <v>84</v>
+        <v>2</v>
       </c>
       <c r="G70" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B71" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C71" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D71" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B71" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C71" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="D71" s="1" t="s">
+      <c r="E71" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="G71" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="E71" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G71" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="1" t="s">
+      <c r="B72" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C72" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D72" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="B72" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C72" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D72" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="E72" s="1" t="s">
-        <v>112</v>
+      <c r="E72" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="G72" s="1" t="s">
         <v>8</v>
@@ -2238,19 +2241,19 @@
     </row>
     <row r="73" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B73" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C73" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E73" s="1" t="s">
         <v>113</v>
-      </c>
-      <c r="B73" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C73" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D73" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="E73" s="1" t="n">
-        <v>1</v>
       </c>
       <c r="G73" s="1" t="s">
         <v>8</v>
@@ -2258,16 +2261,16 @@
     </row>
     <row r="74" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B74" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C74" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D74" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="B74" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C74" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D74" s="1" t="s">
-        <v>116</v>
       </c>
       <c r="E74" s="1" t="n">
         <v>1</v>
@@ -2278,19 +2281,19 @@
     </row>
     <row r="75" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B75" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C75" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D75" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="B75" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C75" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D75" s="1" t="s">
-        <v>118</v>
-      </c>
       <c r="E75" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G75" s="1" t="s">
         <v>8</v>
@@ -2298,34 +2301,37 @@
     </row>
     <row r="76" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B76" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C76" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D76" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="B76" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C76" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D76" s="1" t="s">
+      <c r="E76" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="E76" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G76" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="1" t="s">
+      <c r="B77" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C77" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D77" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B77" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C77" s="1" t="n">
-        <v>1</v>
-      </c>
       <c r="E77" s="1" t="n">
         <v>0</v>
       </c>
@@ -2333,7 +2339,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="1" t="s">
         <v>122</v>
       </c>
@@ -2341,16 +2347,13 @@
         <v>1</v>
       </c>
       <c r="C78" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="E78" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="F78" s="1" t="s">
-        <v>14</v>
+        <v>1</v>
+      </c>
+      <c r="E78" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="G78" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2361,16 +2364,16 @@
         <v>1</v>
       </c>
       <c r="C79" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D79" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="E79" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="E79" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F79" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="G79" s="1" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2381,13 +2384,13 @@
         <v>1</v>
       </c>
       <c r="C80" s="1" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E80" s="1" t="s">
-        <v>25</v>
+        <v>121</v>
+      </c>
+      <c r="E80" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="G80" s="1" t="s">
         <v>8</v>
@@ -2401,13 +2404,13 @@
         <v>1</v>
       </c>
       <c r="C81" s="1" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="E81" s="1" t="n">
-        <v>0</v>
+        <v>24</v>
+      </c>
+      <c r="E81" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="G81" s="1" t="s">
         <v>8</v>
@@ -2415,48 +2418,68 @@
     </row>
     <row r="82" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B82" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C82" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D82" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B82" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C82" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="D82" s="1" t="s">
+      <c r="E82" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G82" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A83" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="E82" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G82" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="1" t="s">
+      <c r="B83" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C83" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D83" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="B83" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C83" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D83" s="1" t="s">
+      <c r="E83" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G83" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="E83" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G83" s="1" t="s">
+      <c r="B84" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C84" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="E84" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" s="1" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -2465,29 +2488,29 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Y91"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:Y92"/>
+  <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44.99"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="10.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.64"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="19.99"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="21.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="24.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="24.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="24.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="24.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="1" width="17.16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="16.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="16.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="14.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="15"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1025" min="17" style="1" width="8.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="17" style="1" width="8.67"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2521,22 +2544,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2556,34 +2579,34 @@
         <v>1</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2603,13 +2626,13 @@
         <v>0</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2629,22 +2652,22 @@
         <v>0</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2664,22 +2687,22 @@
         <v>18</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2699,22 +2722,22 @@
         <v>1</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2734,67 +2757,67 @@
         <v>11</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="L8" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="O8" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="M8" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="N8" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="O8" s="1" t="s">
-        <v>137</v>
-      </c>
       <c r="P8" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="R8" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S8" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="T8" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="U8" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="V8" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="W8" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="X8" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="Y8" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2814,22 +2837,22 @@
         <v>25</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2849,22 +2872,22 @@
         <v>25</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2884,22 +2907,22 @@
         <v>0</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2919,10 +2942,10 @@
         <v>1</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2942,28 +2965,28 @@
         <v>11</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2983,19 +3006,19 @@
         <v>0</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H14" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="I14" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3029,19 +3052,19 @@
         <v>36</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3061,19 +3084,19 @@
         <v>36</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3093,19 +3116,19 @@
         <v>36</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3125,19 +3148,19 @@
         <v>36</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3157,10 +3180,10 @@
         <v>0</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3180,16 +3203,16 @@
         <v>0</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3209,10 +3232,10 @@
         <v>1</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3232,10 +3255,10 @@
         <v>1</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3255,10 +3278,10 @@
         <v>1</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3278,10 +3301,10 @@
         <v>11</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3301,19 +3324,19 @@
         <v>0</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H26" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="I26" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="I26" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3333,19 +3356,19 @@
         <v>0</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H27" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="I27" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="I27" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3365,19 +3388,19 @@
         <v>0</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H28" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="I28" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3397,10 +3420,10 @@
         <v>1</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3451,10 +3474,10 @@
         <v>0</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3474,22 +3497,22 @@
         <v>0</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3509,10 +3532,10 @@
         <v>0</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3532,19 +3555,19 @@
         <v>0</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H35" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="I35" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="I35" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3578,28 +3601,28 @@
         <v>59</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="K37" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="L37" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3619,22 +3642,22 @@
         <v>1</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3654,25 +3677,25 @@
         <v>1</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="K39" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3692,25 +3715,25 @@
         <v>25</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K40" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3730,10 +3753,10 @@
         <v>0</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3753,10 +3776,10 @@
         <v>0</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3776,34 +3799,34 @@
         <v>36</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K43" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L43" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="M43" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="N43" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3823,34 +3846,34 @@
         <v>70</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L44" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="M44" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="N44" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3870,22 +3893,22 @@
         <v>1</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I45" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3905,10 +3928,10 @@
         <v>1</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3945,22 +3968,22 @@
         <v>1</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I48" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J48" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3980,7 +4003,7 @@
         <v>1</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4000,10 +4023,10 @@
         <v>1</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4023,22 +4046,22 @@
         <v>1</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J51" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4058,25 +4081,25 @@
         <v>11</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I52" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="J52" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="K52" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4096,22 +4119,22 @@
         <v>1</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I53" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J53" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4131,57 +4154,39 @@
         <v>1</v>
       </c>
       <c r="E54" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B55" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C55" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="G55" s="1" t="s">
         <v>134</v>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="1" t="str">
-        <f aca="false">LibManager!A55</f>
-        <v>Quantize</v>
-      </c>
-      <c r="B55" s="1" t="n">
-        <f aca="false">LibManager!B55</f>
-        <v>1</v>
-      </c>
-      <c r="C55" s="1" t="n">
-        <f aca="false">LibManager!C55</f>
-        <v>1</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E55" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="F55" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="G55" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="H55" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="I55" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="J55" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="K55" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="L55" s="1" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="str">
         <f aca="false">LibManager!A56</f>
-        <v>RescaleQuantized</v>
+        <v>Quantize</v>
       </c>
       <c r="B56" s="1" t="n">
         <f aca="false">LibManager!B56</f>
@@ -4191,26 +4196,38 @@
         <f aca="false">LibManager!C56</f>
         <v>1</v>
       </c>
-      <c r="D56" s="1" t="n">
-        <v>1</v>
+      <c r="D56" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>133</v>
+        <v>194</v>
       </c>
       <c r="F56" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="H56" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="I56" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="J56" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="K56" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="L56" s="1" t="s">
         <v>212</v>
-      </c>
-      <c r="G56" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="H56" s="1" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="str">
         <f aca="false">LibManager!A57</f>
-        <v>RowwiseQuantizedFullyConnected</v>
+        <v>RescaleQuantized</v>
       </c>
       <c r="B57" s="1" t="n">
         <f aca="false">LibManager!B57</f>
@@ -4218,16 +4235,28 @@
       </c>
       <c r="C57" s="1" t="n">
         <f aca="false">LibManager!C57</f>
-        <v>5</v>
-      </c>
-      <c r="D57" s="1" t="s">
-        <v>34</v>
+        <v>1</v>
+      </c>
+      <c r="D57" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="G57" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="H57" s="1" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="str">
         <f aca="false">LibManager!A58</f>
-        <v>RowwiseQuantizedSparseLengthsWeightedSum</v>
+        <v>RowwiseQuantizedFullyConnected</v>
       </c>
       <c r="B58" s="1" t="n">
         <f aca="false">LibManager!B58</f>
@@ -4235,28 +4264,16 @@
       </c>
       <c r="C58" s="1" t="n">
         <f aca="false">LibManager!C58</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="E58" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="F58" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="G58" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="H58" s="1" t="s">
-        <v>155</v>
+        <v>34</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="str">
         <f aca="false">LibManager!A59</f>
-        <v>ScatterData</v>
+        <v>RowwiseQuantizedSparseLengthsWeightedSum</v>
       </c>
       <c r="B59" s="1" t="n">
         <f aca="false">LibManager!B59</f>
@@ -4264,34 +4281,28 @@
       </c>
       <c r="C59" s="1" t="n">
         <f aca="false">LibManager!C59</f>
-        <v>2</v>
-      </c>
-      <c r="D59" s="1" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>93</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>131</v>
+        <v>158</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>132</v>
+        <v>159</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>133</v>
+        <v>155</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="I59" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="J59" s="1" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="str">
         <f aca="false">LibManager!A60</f>
-        <v>Sigmoid</v>
+        <v>ScatterData</v>
       </c>
       <c r="B60" s="1" t="n">
         <f aca="false">LibManager!B60</f>
@@ -4299,22 +4310,34 @@
       </c>
       <c r="C60" s="1" t="n">
         <f aca="false">LibManager!C60</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D60" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="H60" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="I60" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="J60" s="1" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="str">
         <f aca="false">LibManager!A61</f>
-        <v>SoftMax</v>
+        <v>Sigmoid</v>
       </c>
       <c r="B61" s="1" t="n">
         <f aca="false">LibManager!B61</f>
@@ -4328,19 +4351,16 @@
         <v>1</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="G61" s="1" t="s">
-        <v>213</v>
+        <v>133</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="str">
         <f aca="false">LibManager!A62</f>
-        <v>SparseLengthsWeightedSum</v>
+        <v>SoftMax</v>
       </c>
       <c r="B62" s="1" t="n">
         <f aca="false">LibManager!B62</f>
@@ -4348,43 +4368,25 @@
       </c>
       <c r="C62" s="1" t="n">
         <f aca="false">LibManager!C62</f>
-        <v>4</v>
-      </c>
-      <c r="D62" s="1" t="s">
-        <v>96</v>
+        <v>1</v>
+      </c>
+      <c r="D62" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="E62" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="G62" s="1" t="s">
         <v>214</v>
-      </c>
-      <c r="F62" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="G62" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="H62" s="1" t="s">
-        <v>217</v>
-      </c>
-      <c r="I62" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="J62" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="K62" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="L62" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="M62" s="1" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="str">
         <f aca="false">LibManager!A63</f>
-        <v>SparseToDense</v>
+        <v>SparseLengthsWeightedSum</v>
       </c>
       <c r="B63" s="1" t="n">
         <f aca="false">LibManager!B63</f>
@@ -4392,34 +4394,43 @@
       </c>
       <c r="C63" s="1" t="n">
         <f aca="false">LibManager!C63</f>
-        <v>2</v>
-      </c>
-      <c r="D63" s="1" t="n">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>98</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>131</v>
+        <v>215</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>132</v>
+        <v>216</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>133</v>
+        <v>217</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>134</v>
+        <v>218</v>
       </c>
       <c r="I63" s="1" t="s">
-        <v>135</v>
+        <v>219</v>
       </c>
       <c r="J63" s="1" t="s">
-        <v>136</v>
+        <v>220</v>
+      </c>
+      <c r="K63" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="L63" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="M63" s="1" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="str">
         <f aca="false">LibManager!A64</f>
-        <v>SparseToDenseMask</v>
+        <v>SparseToDense</v>
       </c>
       <c r="B64" s="1" t="n">
         <f aca="false">LibManager!B64</f>
@@ -4427,34 +4438,34 @@
       </c>
       <c r="C64" s="1" t="n">
         <f aca="false">LibManager!C64</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D64" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I64" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J64" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="str">
         <f aca="false">LibManager!A65</f>
-        <v>Splat</v>
+        <v>SparseToDenseMask</v>
       </c>
       <c r="B65" s="1" t="n">
         <f aca="false">LibManager!B65</f>
@@ -4462,34 +4473,34 @@
       </c>
       <c r="C65" s="1" t="n">
         <f aca="false">LibManager!C65</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D65" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I65" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J65" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="str">
         <f aca="false">LibManager!A66</f>
-        <v>Syncopy</v>
+        <v>Splat</v>
       </c>
       <c r="B66" s="1" t="n">
         <f aca="false">LibManager!B66</f>
@@ -4497,34 +4508,34 @@
       </c>
       <c r="C66" s="1" t="n">
         <f aca="false">LibManager!C66</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D66" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I66" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J66" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="str">
         <f aca="false">LibManager!A67</f>
-        <v>Tanh</v>
+        <v>Syncopy</v>
       </c>
       <c r="B67" s="1" t="n">
         <f aca="false">LibManager!B67</f>
@@ -4538,16 +4549,28 @@
         <v>1</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
+      </c>
+      <c r="G67" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="H67" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="I67" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="J67" s="1" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="str">
         <f aca="false">LibManager!A68</f>
-        <v>TensorView</v>
+        <v>Tanh</v>
       </c>
       <c r="B68" s="1" t="n">
         <f aca="false">LibManager!B68</f>
@@ -4558,101 +4581,89 @@
         <v>1</v>
       </c>
       <c r="D68" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="G68" s="1" t="s">
         <v>133</v>
-      </c>
-      <c r="H68" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="I68" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="J68" s="1" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="1" t="str">
         <f aca="false">LibManager!A69</f>
-        <v>TopK</v>
+        <v>TensorView</v>
       </c>
       <c r="B69" s="1" t="n">
         <f aca="false">LibManager!B69</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C69" s="1" t="n">
         <f aca="false">LibManager!C69</f>
         <v>1</v>
       </c>
       <c r="D69" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I69" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J69" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="str">
         <f aca="false">LibManager!A70</f>
-        <v>Transpose</v>
+        <v>TopK</v>
       </c>
       <c r="B70" s="1" t="n">
         <f aca="false">LibManager!B70</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C70" s="1" t="n">
         <f aca="false">LibManager!C70</f>
         <v>1</v>
       </c>
       <c r="D70" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G70" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H70" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I70" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J70" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="str">
         <f aca="false">LibManager!A71</f>
-        <v>Trilu</v>
+        <v>Transpose</v>
       </c>
       <c r="B71" s="1" t="n">
         <f aca="false">LibManager!B71</f>
@@ -4660,107 +4671,107 @@
       </c>
       <c r="C71" s="1" t="n">
         <f aca="false">LibManager!C71</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D71" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G71" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H71" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I71" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J71" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="str">
         <f aca="false">LibManager!A72</f>
-        <v>MaxPoolWithArgMax</v>
+        <v>Trilu</v>
       </c>
       <c r="B72" s="1" t="n">
         <f aca="false">LibManager!B72</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C72" s="1" t="n">
         <f aca="false">LibManager!C72</f>
-        <v>1</v>
-      </c>
-      <c r="D72" s="1" t="s">
-        <v>112</v>
+        <v>2</v>
+      </c>
+      <c r="D72" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>200</v>
+        <v>132</v>
       </c>
       <c r="F72" s="1" t="s">
-        <v>201</v>
+        <v>133</v>
       </c>
       <c r="G72" s="1" t="s">
-        <v>172</v>
+        <v>134</v>
       </c>
       <c r="H72" s="1" t="s">
-        <v>202</v>
+        <v>135</v>
       </c>
       <c r="I72" s="1" t="s">
-        <v>203</v>
+        <v>136</v>
       </c>
       <c r="J72" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="K72" s="1" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="str">
         <f aca="false">LibManager!A73</f>
-        <v>BatchedReduceMin</v>
+        <v>MaxPoolWithArgMax</v>
       </c>
       <c r="B73" s="1" t="n">
         <f aca="false">LibManager!B73</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C73" s="1" t="n">
         <f aca="false">LibManager!C73</f>
         <v>1</v>
       </c>
-      <c r="D73" s="1" t="n">
-        <v>1</v>
+      <c r="D73" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>131</v>
+        <v>201</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>132</v>
+        <v>202</v>
       </c>
       <c r="G73" s="1" t="s">
-        <v>133</v>
+        <v>173</v>
       </c>
       <c r="H73" s="1" t="s">
-        <v>134</v>
+        <v>203</v>
       </c>
       <c r="I73" s="1" t="s">
-        <v>135</v>
+        <v>204</v>
       </c>
       <c r="J73" s="1" t="s">
-        <v>136</v>
+        <v>205</v>
+      </c>
+      <c r="K73" s="1" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="1" t="str">
         <f aca="false">LibManager!A74</f>
-        <v>CumSum</v>
+        <v>BatchedReduceMin</v>
       </c>
       <c r="B74" s="1" t="n">
         <f aca="false">LibManager!B74</f>
@@ -4774,22 +4785,28 @@
         <v>1</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F74" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G74" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="H74" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="H74" s="1" t="s">
-        <v>134</v>
+      <c r="I74" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="J74" s="1" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="1" t="str">
         <f aca="false">LibManager!A75</f>
-        <v>SpaceToDepth</v>
+        <v>CumSum</v>
       </c>
       <c r="B75" s="1" t="n">
         <f aca="false">LibManager!B75</f>
@@ -4800,25 +4817,25 @@
         <v>1</v>
       </c>
       <c r="D75" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G75" s="1" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="H75" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="1" t="str">
         <f aca="false">LibManager!A76</f>
-        <v>ResizeNearest</v>
+        <v>SpaceToDepth</v>
       </c>
       <c r="B76" s="1" t="n">
         <f aca="false">LibManager!B76</f>
@@ -4832,31 +4849,22 @@
         <v>0</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G76" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H76" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="I76" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="J76" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="K76" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="1" t="str">
         <f aca="false">LibManager!A77</f>
-        <v>LengthsRangeFill</v>
+        <v>ResizeNearest</v>
       </c>
       <c r="B77" s="1" t="n">
         <f aca="false">LibManager!B77</f>
@@ -4870,13 +4878,31 @@
         <v>0</v>
       </c>
       <c r="E77" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="F77" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="G77" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="H77" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="I77" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="J77" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="K77" s="1" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="1" t="str">
         <f aca="false">LibManager!A78</f>
-        <v>SparseLengthsSum</v>
+        <v>LengthsRangeFill</v>
       </c>
       <c r="B78" s="1" t="n">
         <f aca="false">LibManager!B78</f>
@@ -4884,34 +4910,19 @@
       </c>
       <c r="C78" s="1" t="n">
         <f aca="false">LibManager!C78</f>
-        <v>3</v>
-      </c>
-      <c r="D78" s="1" t="s">
-        <v>112</v>
+        <v>1</v>
+      </c>
+      <c r="D78" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="F78" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="G78" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="H78" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="I78" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="J78" s="1" t="s">
-        <v>194</v>
+        <v>136</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="1" t="str">
         <f aca="false">LibManager!A79</f>
-        <v>ResizeBilinear</v>
+        <v>SparseLengthsSum</v>
       </c>
       <c r="B79" s="1" t="n">
         <f aca="false">LibManager!B79</f>
@@ -4919,37 +4930,34 @@
       </c>
       <c r="C79" s="1" t="n">
         <f aca="false">LibManager!C79</f>
-        <v>1</v>
-      </c>
-      <c r="D79" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="D79" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>131</v>
+        <v>158</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>132</v>
+        <v>159</v>
       </c>
       <c r="G79" s="1" t="s">
-        <v>133</v>
+        <v>155</v>
       </c>
       <c r="H79" s="1" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="I79" s="1" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="J79" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="K79" s="1" t="s">
-        <v>134</v>
+        <v>195</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="1" t="str">
         <f aca="false">LibManager!A80</f>
-        <v>ChannelWiseQuantizedConvolution</v>
+        <v>ResizeBilinear</v>
       </c>
       <c r="B80" s="1" t="n">
         <f aca="false">LibManager!B80</f>
@@ -4957,22 +4965,37 @@
       </c>
       <c r="C80" s="1" t="n">
         <f aca="false">LibManager!C80</f>
-        <v>7</v>
-      </c>
-      <c r="D80" s="1" t="s">
-        <v>25</v>
+        <v>1</v>
+      </c>
+      <c r="D80" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>172</v>
+        <v>132</v>
       </c>
       <c r="F80" s="1" t="s">
-        <v>173</v>
+        <v>133</v>
+      </c>
+      <c r="G80" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="H80" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="I80" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="J80" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="K80" s="1" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="1" t="str">
         <f aca="false">LibManager!A81</f>
-        <v>ConvTranspose</v>
+        <v>ChannelWiseQuantizedConvolution</v>
       </c>
       <c r="B81" s="1" t="n">
         <f aca="false">LibManager!B81</f>
@@ -4980,73 +5003,79 @@
       </c>
       <c r="C81" s="1" t="n">
         <f aca="false">LibManager!C81</f>
-        <v>3</v>
-      </c>
-      <c r="D81" s="1" t="n">
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>131</v>
+        <v>173</v>
+      </c>
+      <c r="F81" s="1" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="1" t="str">
         <f aca="false">LibManager!A82</f>
-        <v>NonMaxSuppression</v>
+        <v>ConvTranspose</v>
       </c>
       <c r="B82" s="1" t="n">
         <f aca="false">LibManager!B82</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C82" s="1" t="n">
         <f aca="false">LibManager!C82</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D82" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="F82" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="1" t="str">
         <f aca="false">LibManager!A83</f>
-        <v>ETSOCGenericOp</v>
+        <v>NonMaxSuppression</v>
       </c>
       <c r="B83" s="1" t="n">
         <f aca="false">LibManager!B83</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C83" s="1" t="n">
         <f aca="false">LibManager!C83</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D83" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>131</v>
+        <v>136</v>
+      </c>
+      <c r="F83" s="1" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A84" s="1" t="n">
+      <c r="A84" s="1" t="str">
         <f aca="false">LibManager!A84</f>
-        <v>0</v>
+        <v>ETSOCGenericOp</v>
       </c>
       <c r="B84" s="1" t="n">
         <f aca="false">LibManager!B84</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C84" s="1" t="n">
         <f aca="false">LibManager!C84</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D84" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="E84" s="1" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5147,6 +5176,9 @@
         <f aca="false">LibManager!C90</f>
         <v>0</v>
       </c>
+      <c r="D90" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="91" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="1" t="n">
@@ -5162,13 +5194,27 @@
         <v>0</v>
       </c>
     </row>
+    <row r="92" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A92" s="1" t="n">
+        <f aca="false">LibManager!A92</f>
+        <v>0</v>
+      </c>
+      <c r="B92" s="1" t="n">
+        <f aca="false">LibManager!B92</f>
+        <v>0</v>
+      </c>
+      <c r="C92" s="1" t="n">
+        <f aca="false">LibManager!C92</f>
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12 &amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12 Page &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12 &amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12 Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[dnn-library] [SW-21425] Implemented OneHot in the dnnlibrary
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/libManager.xlsx
+++ b/dnn-library/scripts/libManager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="677" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="690" uniqueCount="225">
   <si>
     <t xml:space="preserve">Operator</t>
   </si>
@@ -288,6 +288,12 @@
   </si>
   <si>
     <t xml:space="preserve">Divisor, SignFollowDivisor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OneHot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Axis, Depth</t>
   </si>
   <si>
     <t xml:space="preserve">Profile</t>
@@ -983,7 +989,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G86"/>
+  <dimension ref="A1:G87"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44.84"/>
@@ -2048,13 +2054,13 @@
         <v>1</v>
       </c>
       <c r="C57" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D57" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E57" s="1" t="n">
-        <v>1</v>
+      <c r="E57" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="G57" s="1" t="s">
         <v>8</v>
@@ -2070,8 +2076,11 @@
       <c r="C58" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E58" s="1" t="s">
-        <v>11</v>
+      <c r="D58" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="E58" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="G58" s="1" t="s">
         <v>8</v>
@@ -2079,7 +2088,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B59" s="1" t="n">
         <v>1</v>
@@ -2087,8 +2096,8 @@
       <c r="C59" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E59" s="1" t="n">
-        <v>1</v>
+      <c r="E59" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="G59" s="1" t="s">
         <v>8</v>
@@ -2096,39 +2105,36 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B60" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C60" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E60" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B61" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C61" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="E60" s="1" t="s">
+      <c r="E61" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="F60" s="1" t="s">
+      <c r="F61" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="G60" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="B61" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C61" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="E61" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="F61" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="G61" s="1" t="s">
         <v>15</v>
@@ -2142,35 +2148,38 @@
         <v>1</v>
       </c>
       <c r="C62" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E62" s="1" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="E62" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>22</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B63" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C63" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E63" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G63" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B64" s="1" t="n">
         <v>1</v>
@@ -2181,34 +2190,31 @@
       <c r="E64" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="F64" s="1" t="s">
+      <c r="G64" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B65" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C65" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E65" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F65" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="G64" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="B65" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C65" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E65" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="F65" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="G65" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
         <v>101</v>
       </c>
@@ -2216,27 +2222,27 @@
         <v>1</v>
       </c>
       <c r="C66" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E66" s="1" t="n">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="E66" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="F66" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="67" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B67" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C67" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="D67" s="1" t="s">
-        <v>103</v>
+        <v>2</v>
       </c>
       <c r="E67" s="1" t="n">
         <v>0</v>
@@ -2245,7 +2251,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
         <v>104</v>
       </c>
@@ -2253,33 +2259,33 @@
         <v>1</v>
       </c>
       <c r="C68" s="1" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D68" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="E68" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B69" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C69" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="E68" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G68" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="B69" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C69" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D69" s="1" t="s">
-        <v>90</v>
-      </c>
       <c r="E69" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G69" s="1" t="s">
         <v>8</v>
@@ -2287,7 +2293,7 @@
     </row>
     <row r="70" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B70" s="1" t="n">
         <v>1</v>
@@ -2295,6 +2301,9 @@
       <c r="C70" s="1" t="n">
         <v>1</v>
       </c>
+      <c r="D70" s="1" t="s">
+        <v>92</v>
+      </c>
       <c r="E70" s="1" t="n">
         <v>1</v>
       </c>
@@ -2302,9 +2311,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B71" s="1" t="n">
         <v>1</v>
@@ -2312,11 +2321,8 @@
       <c r="C71" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D71" s="1" t="s">
-        <v>64</v>
-      </c>
       <c r="E71" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G71" s="1" t="s">
         <v>8</v>
@@ -2324,19 +2330,19 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B72" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C72" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>108</v>
+        <v>64</v>
       </c>
       <c r="E72" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G72" s="1" t="s">
         <v>8</v>
@@ -2344,10 +2350,10 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B73" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C73" s="1" t="n">
         <v>1</v>
@@ -2356,13 +2362,10 @@
         <v>110</v>
       </c>
       <c r="E73" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F73" s="1" t="s">
-        <v>86</v>
+        <v>2</v>
       </c>
       <c r="G73" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2373,7 +2376,7 @@
         <v>1</v>
       </c>
       <c r="C74" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D74" s="1" t="s">
         <v>112</v>
@@ -2381,25 +2384,28 @@
       <c r="E74" s="1" t="n">
         <v>1</v>
       </c>
+      <c r="F74" s="1" t="s">
+        <v>86</v>
+      </c>
       <c r="G74" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="75" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="1" t="s">
         <v>113</v>
       </c>
       <c r="B75" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C75" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D75" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="E75" s="1" t="s">
-        <v>115</v>
+      <c r="E75" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="G75" s="1" t="s">
         <v>8</v>
@@ -2407,19 +2413,19 @@
     </row>
     <row r="76" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B76" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C76" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D76" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="B76" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C76" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D76" s="1" t="s">
+      <c r="E76" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="E76" s="1" t="n">
-        <v>1</v>
       </c>
       <c r="G76" s="1" t="s">
         <v>8</v>
@@ -2459,7 +2465,7 @@
         <v>121</v>
       </c>
       <c r="E78" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G78" s="1" t="s">
         <v>8</v>
@@ -2485,7 +2491,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="1" t="s">
         <v>124</v>
       </c>
@@ -2495,6 +2501,9 @@
       <c r="C80" s="1" t="n">
         <v>1</v>
       </c>
+      <c r="D80" s="1" t="s">
+        <v>125</v>
+      </c>
       <c r="E80" s="1" t="n">
         <v>0</v>
       </c>
@@ -2502,61 +2511,58 @@
         <v>8</v>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B81" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C81" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="E81" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="F81" s="1" t="s">
-        <v>14</v>
+        <v>1</v>
+      </c>
+      <c r="E81" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="G81" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B82" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C82" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D82" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="E82" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F82" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="G82" s="1" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B83" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C83" s="1" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E83" s="1" t="s">
-        <v>25</v>
+        <v>125</v>
+      </c>
+      <c r="E83" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="G83" s="1" t="s">
         <v>8</v>
@@ -2564,19 +2570,19 @@
     </row>
     <row r="84" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B84" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C84" s="1" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="E84" s="1" t="n">
-        <v>0</v>
+        <v>24</v>
+      </c>
+      <c r="E84" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="G84" s="1" t="s">
         <v>8</v>
@@ -2587,10 +2593,10 @@
         <v>130</v>
       </c>
       <c r="B85" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C85" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D85" s="1" t="s">
         <v>131</v>
@@ -2602,15 +2608,15 @@
         <v>8</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="1" t="s">
         <v>132</v>
       </c>
       <c r="B86" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C86" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D86" s="1" t="s">
         <v>133</v>
@@ -2619,6 +2625,26 @@
         <v>0</v>
       </c>
       <c r="G86" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="B87" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C87" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D87" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E87" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G87" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2638,7 +2664,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Y94"/>
+  <dimension ref="A1:Y95"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44.99"/>
@@ -2690,22 +2716,22 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2725,34 +2751,34 @@
         <v>1</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2772,13 +2798,13 @@
         <v>0</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2798,22 +2824,22 @@
         <v>0</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2833,22 +2859,22 @@
         <v>18</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2868,22 +2894,22 @@
         <v>1</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2903,67 +2929,67 @@
         <v>11</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="M8" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="O8" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="P8" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="N8" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="O8" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="P8" s="1" t="s">
-        <v>145</v>
-      </c>
       <c r="Q8" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="R8" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S8" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="T8" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="U8" s="1" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="V8" s="1" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="W8" s="1" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="X8" s="1" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="Y8" s="1" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2983,22 +3009,22 @@
         <v>25</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3018,22 +3044,22 @@
         <v>25</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3053,22 +3079,22 @@
         <v>0</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3088,10 +3114,10 @@
         <v>1</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3111,28 +3137,28 @@
         <v>11</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3152,10 +3178,10 @@
         <v>0</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3175,10 +3201,10 @@
         <v>0</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3198,19 +3224,19 @@
         <v>0</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3247,19 +3273,19 @@
         <v>38</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3279,19 +3305,19 @@
         <v>38</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3311,19 +3337,19 @@
         <v>38</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3343,19 +3369,19 @@
         <v>38</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3375,10 +3401,10 @@
         <v>0</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3398,16 +3424,16 @@
         <v>0</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3427,10 +3453,10 @@
         <v>1</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3450,10 +3476,10 @@
         <v>1</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3473,10 +3499,10 @@
         <v>1</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3496,10 +3522,10 @@
         <v>11</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3519,19 +3545,19 @@
         <v>0</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3551,19 +3577,19 @@
         <v>0</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3583,19 +3609,19 @@
         <v>0</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3615,10 +3641,10 @@
         <v>1</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3672,10 +3698,10 @@
         <v>0</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3695,22 +3721,22 @@
         <v>0</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3730,10 +3756,10 @@
         <v>0</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3753,19 +3779,19 @@
         <v>0</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3802,28 +3828,28 @@
         <v>61</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="K39" s="1" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="L39" s="1" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3843,22 +3869,22 @@
         <v>1</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3878,25 +3904,25 @@
         <v>1</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J41" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="K41" s="1" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3916,25 +3942,25 @@
         <v>25</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="K42" s="1" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3954,10 +3980,10 @@
         <v>0</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3977,10 +4003,10 @@
         <v>0</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4000,34 +4026,34 @@
         <v>38</v>
       </c>
       <c r="E45" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="H45" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="I45" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="J45" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="K45" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="F45" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="G45" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="H45" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="I45" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="J45" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="K45" s="1" t="s">
-        <v>158</v>
-      </c>
       <c r="L45" s="1" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="M45" s="1" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="N45" s="1" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4047,34 +4073,34 @@
         <v>72</v>
       </c>
       <c r="E46" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="H46" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="I46" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="J46" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="K46" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="F46" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="G46" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="H46" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="I46" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="J46" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="K46" s="1" t="s">
-        <v>158</v>
-      </c>
       <c r="L46" s="1" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="M46" s="1" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="N46" s="1" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4094,22 +4120,22 @@
         <v>1</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I47" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J47" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4129,10 +4155,10 @@
         <v>1</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4169,22 +4195,22 @@
         <v>1</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I50" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J50" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4204,7 +4230,7 @@
         <v>1</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4224,10 +4250,10 @@
         <v>1</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4247,22 +4273,22 @@
         <v>1</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I53" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J53" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4282,25 +4308,25 @@
         <v>11</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="I54" s="1" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="J54" s="1" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="K54" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4320,22 +4346,22 @@
         <v>1</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I55" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J55" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4355,10 +4381,10 @@
         <v>1</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4369,66 +4395,60 @@
         <v>1</v>
       </c>
       <c r="C57" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D57" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>134</v>
+        <v>163</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>135</v>
+        <v>160</v>
       </c>
       <c r="G57" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="H57" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="I57" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="J57" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="K57" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B58" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" s="1" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="58" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="1" t="str">
-        <f aca="false">LibManager!A58</f>
-        <v>Quantize</v>
-      </c>
-      <c r="B58" s="1" t="n">
-        <f aca="false">LibManager!B58</f>
-        <v>1</v>
-      </c>
-      <c r="C58" s="1" t="n">
-        <f aca="false">LibManager!C58</f>
-        <v>1</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E58" s="1" t="s">
-        <v>196</v>
-      </c>
       <c r="F58" s="1" t="s">
-        <v>208</v>
+        <v>137</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="H58" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="I58" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="J58" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="K58" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="L58" s="1" t="s">
-        <v>214</v>
+        <v>138</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="str">
         <f aca="false">LibManager!A59</f>
-        <v>RescaleQuantized</v>
+        <v>Quantize</v>
       </c>
       <c r="B59" s="1" t="n">
         <f aca="false">LibManager!B59</f>
@@ -4438,26 +4458,38 @@
         <f aca="false">LibManager!C59</f>
         <v>1</v>
       </c>
-      <c r="D59" s="1" t="n">
-        <v>1</v>
+      <c r="D59" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>136</v>
+        <v>198</v>
       </c>
       <c r="F59" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="G59" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="H59" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="I59" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="J59" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="K59" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="G59" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="H59" s="1" t="s">
-        <v>195</v>
+      <c r="L59" s="1" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="str">
         <f aca="false">LibManager!A60</f>
-        <v>RowwiseQuantizedFullyConnected</v>
+        <v>RescaleQuantized</v>
       </c>
       <c r="B60" s="1" t="n">
         <f aca="false">LibManager!B60</f>
@@ -4465,16 +4497,28 @@
       </c>
       <c r="C60" s="1" t="n">
         <f aca="false">LibManager!C60</f>
-        <v>5</v>
-      </c>
-      <c r="D60" s="1" t="s">
-        <v>36</v>
+        <v>1</v>
+      </c>
+      <c r="D60" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="H60" s="1" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="str">
         <f aca="false">LibManager!A61</f>
-        <v>RowwiseQuantizedSparseLengthsWeightedSum</v>
+        <v>RowwiseQuantizedFullyConnected</v>
       </c>
       <c r="B61" s="1" t="n">
         <f aca="false">LibManager!B61</f>
@@ -4482,28 +4526,16 @@
       </c>
       <c r="C61" s="1" t="n">
         <f aca="false">LibManager!C61</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="E61" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="F61" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="G61" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="H61" s="1" t="s">
-        <v>158</v>
+        <v>36</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="str">
         <f aca="false">LibManager!A62</f>
-        <v>ScatterData</v>
+        <v>RowwiseQuantizedSparseLengthsWeightedSum</v>
       </c>
       <c r="B62" s="1" t="n">
         <f aca="false">LibManager!B62</f>
@@ -4511,34 +4543,28 @@
       </c>
       <c r="C62" s="1" t="n">
         <f aca="false">LibManager!C62</f>
-        <v>2</v>
-      </c>
-      <c r="D62" s="1" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>97</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>134</v>
+        <v>162</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>135</v>
+        <v>163</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>136</v>
+        <v>159</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="I62" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="J62" s="1" t="s">
-        <v>139</v>
+        <v>160</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="str">
         <f aca="false">LibManager!A63</f>
-        <v>Sigmoid</v>
+        <v>ScatterData</v>
       </c>
       <c r="B63" s="1" t="n">
         <f aca="false">LibManager!B63</f>
@@ -4546,22 +4572,34 @@
       </c>
       <c r="C63" s="1" t="n">
         <f aca="false">LibManager!C63</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D63" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
+      </c>
+      <c r="G63" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="H63" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="I63" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="J63" s="1" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="str">
         <f aca="false">LibManager!A64</f>
-        <v>SoftMax</v>
+        <v>Sigmoid</v>
       </c>
       <c r="B64" s="1" t="n">
         <f aca="false">LibManager!B64</f>
@@ -4575,19 +4613,16 @@
         <v>1</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="G64" s="1" t="s">
-        <v>216</v>
+        <v>137</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="str">
         <f aca="false">LibManager!A65</f>
-        <v>SparseLengthsWeightedSum</v>
+        <v>SoftMax</v>
       </c>
       <c r="B65" s="1" t="n">
         <f aca="false">LibManager!B65</f>
@@ -4595,43 +4630,25 @@
       </c>
       <c r="C65" s="1" t="n">
         <f aca="false">LibManager!C65</f>
-        <v>4</v>
-      </c>
-      <c r="D65" s="1" t="s">
-        <v>100</v>
+        <v>1</v>
+      </c>
+      <c r="D65" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>217</v>
+        <v>136</v>
       </c>
       <c r="F65" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="G65" s="1" t="s">
         <v>218</v>
-      </c>
-      <c r="G65" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="H65" s="1" t="s">
-        <v>220</v>
-      </c>
-      <c r="I65" s="1" t="s">
-        <v>221</v>
-      </c>
-      <c r="J65" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="K65" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="L65" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="M65" s="1" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="str">
         <f aca="false">LibManager!A66</f>
-        <v>SparseToDense</v>
+        <v>SparseLengthsWeightedSum</v>
       </c>
       <c r="B66" s="1" t="n">
         <f aca="false">LibManager!B66</f>
@@ -4639,34 +4656,43 @@
       </c>
       <c r="C66" s="1" t="n">
         <f aca="false">LibManager!C66</f>
-        <v>2</v>
-      </c>
-      <c r="D66" s="1" t="n">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>102</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>134</v>
+        <v>219</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>135</v>
+        <v>220</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>136</v>
+        <v>221</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>137</v>
+        <v>222</v>
       </c>
       <c r="I66" s="1" t="s">
-        <v>138</v>
+        <v>223</v>
       </c>
       <c r="J66" s="1" t="s">
-        <v>139</v>
+        <v>224</v>
+      </c>
+      <c r="K66" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="L66" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="M66" s="1" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="str">
         <f aca="false">LibManager!A67</f>
-        <v>SparseToDenseMask</v>
+        <v>SparseToDense</v>
       </c>
       <c r="B67" s="1" t="n">
         <f aca="false">LibManager!B67</f>
@@ -4674,34 +4700,34 @@
       </c>
       <c r="C67" s="1" t="n">
         <f aca="false">LibManager!C67</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D67" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I67" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J67" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="str">
         <f aca="false">LibManager!A68</f>
-        <v>Splat</v>
+        <v>SparseToDenseMask</v>
       </c>
       <c r="B68" s="1" t="n">
         <f aca="false">LibManager!B68</f>
@@ -4709,34 +4735,34 @@
       </c>
       <c r="C68" s="1" t="n">
         <f aca="false">LibManager!C68</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D68" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H68" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I68" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J68" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="1" t="str">
         <f aca="false">LibManager!A69</f>
-        <v>Syncopy</v>
+        <v>Splat</v>
       </c>
       <c r="B69" s="1" t="n">
         <f aca="false">LibManager!B69</f>
@@ -4744,34 +4770,34 @@
       </c>
       <c r="C69" s="1" t="n">
         <f aca="false">LibManager!C69</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D69" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I69" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J69" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="str">
         <f aca="false">LibManager!A70</f>
-        <v>Tanh</v>
+        <v>Syncopy</v>
       </c>
       <c r="B70" s="1" t="n">
         <f aca="false">LibManager!B70</f>
@@ -4785,16 +4811,28 @@
         <v>1</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
+      </c>
+      <c r="G70" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="H70" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="I70" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="J70" s="1" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="str">
         <f aca="false">LibManager!A71</f>
-        <v>TensorView</v>
+        <v>Tanh</v>
       </c>
       <c r="B71" s="1" t="n">
         <f aca="false">LibManager!B71</f>
@@ -4805,101 +4843,89 @@
         <v>1</v>
       </c>
       <c r="D71" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="G71" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="H71" s="1" t="s">
         <v>137</v>
-      </c>
-      <c r="I71" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="J71" s="1" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="str">
         <f aca="false">LibManager!A72</f>
-        <v>TopK</v>
+        <v>TensorView</v>
       </c>
       <c r="B72" s="1" t="n">
         <f aca="false">LibManager!B72</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C72" s="1" t="n">
         <f aca="false">LibManager!C72</f>
         <v>1</v>
       </c>
       <c r="D72" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F72" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G72" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H72" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I72" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J72" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="str">
         <f aca="false">LibManager!A73</f>
-        <v>Transpose</v>
+        <v>TopK</v>
       </c>
       <c r="B73" s="1" t="n">
         <f aca="false">LibManager!B73</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C73" s="1" t="n">
         <f aca="false">LibManager!C73</f>
         <v>1</v>
       </c>
       <c r="D73" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G73" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H73" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I73" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J73" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="1" t="str">
         <f aca="false">LibManager!A74</f>
-        <v>Trilu</v>
+        <v>Transpose</v>
       </c>
       <c r="B74" s="1" t="n">
         <f aca="false">LibManager!B74</f>
@@ -4907,107 +4933,107 @@
       </c>
       <c r="C74" s="1" t="n">
         <f aca="false">LibManager!C74</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D74" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F74" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G74" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H74" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I74" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J74" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="1" t="str">
         <f aca="false">LibManager!A75</f>
-        <v>MaxPoolWithArgMax</v>
+        <v>Trilu</v>
       </c>
       <c r="B75" s="1" t="n">
         <f aca="false">LibManager!B75</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C75" s="1" t="n">
         <f aca="false">LibManager!C75</f>
-        <v>1</v>
-      </c>
-      <c r="D75" s="1" t="s">
-        <v>115</v>
+        <v>2</v>
+      </c>
+      <c r="D75" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>203</v>
+        <v>136</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>204</v>
+        <v>137</v>
       </c>
       <c r="G75" s="1" t="s">
-        <v>175</v>
+        <v>138</v>
       </c>
       <c r="H75" s="1" t="s">
-        <v>205</v>
+        <v>139</v>
       </c>
       <c r="I75" s="1" t="s">
-        <v>206</v>
+        <v>140</v>
       </c>
       <c r="J75" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="K75" s="1" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="1" t="str">
         <f aca="false">LibManager!A76</f>
-        <v>BatchedReduceMin</v>
+        <v>MaxPoolWithArgMax</v>
       </c>
       <c r="B76" s="1" t="n">
         <f aca="false">LibManager!B76</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C76" s="1" t="n">
         <f aca="false">LibManager!C76</f>
         <v>1</v>
       </c>
-      <c r="D76" s="1" t="n">
-        <v>1</v>
+      <c r="D76" s="1" t="s">
+        <v>117</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>134</v>
+        <v>205</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>135</v>
+        <v>206</v>
       </c>
       <c r="G76" s="1" t="s">
-        <v>136</v>
+        <v>177</v>
       </c>
       <c r="H76" s="1" t="s">
-        <v>137</v>
+        <v>207</v>
       </c>
       <c r="I76" s="1" t="s">
-        <v>138</v>
+        <v>208</v>
       </c>
       <c r="J76" s="1" t="s">
-        <v>139</v>
+        <v>209</v>
+      </c>
+      <c r="K76" s="1" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="1" t="str">
         <f aca="false">LibManager!A77</f>
-        <v>CumSum</v>
+        <v>BatchedReduceMin</v>
       </c>
       <c r="B77" s="1" t="n">
         <f aca="false">LibManager!B77</f>
@@ -5021,22 +5047,28 @@
         <v>1</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F77" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G77" s="1" t="s">
         <v>138</v>
       </c>
       <c r="H77" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
+      </c>
+      <c r="I77" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="J77" s="1" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="1" t="str">
         <f aca="false">LibManager!A78</f>
-        <v>SpaceToDepth</v>
+        <v>CumSum</v>
       </c>
       <c r="B78" s="1" t="n">
         <f aca="false">LibManager!B78</f>
@@ -5047,25 +5079,25 @@
         <v>1</v>
       </c>
       <c r="D78" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F78" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G78" s="1" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="H78" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="1" t="str">
         <f aca="false">LibManager!A79</f>
-        <v>ResizeNearest</v>
+        <v>SpaceToDepth</v>
       </c>
       <c r="B79" s="1" t="n">
         <f aca="false">LibManager!B79</f>
@@ -5079,31 +5111,22 @@
         <v>0</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G79" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H79" s="1" t="s">
         <v>139</v>
-      </c>
-      <c r="I79" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="J79" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="K79" s="1" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="1" t="str">
         <f aca="false">LibManager!A80</f>
-        <v>LengthsRangeFill</v>
+        <v>ResizeNearest</v>
       </c>
       <c r="B80" s="1" t="n">
         <f aca="false">LibManager!B80</f>
@@ -5117,13 +5140,31 @@
         <v>0</v>
       </c>
       <c r="E80" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="F80" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="G80" s="1" t="s">
         <v>138</v>
+      </c>
+      <c r="H80" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="I80" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="J80" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="K80" s="1" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="1" t="str">
         <f aca="false">LibManager!A81</f>
-        <v>SparseLengthsSum</v>
+        <v>LengthsRangeFill</v>
       </c>
       <c r="B81" s="1" t="n">
         <f aca="false">LibManager!B81</f>
@@ -5131,34 +5172,19 @@
       </c>
       <c r="C81" s="1" t="n">
         <f aca="false">LibManager!C81</f>
-        <v>3</v>
-      </c>
-      <c r="D81" s="1" t="s">
-        <v>115</v>
+        <v>1</v>
+      </c>
+      <c r="D81" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="F81" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="G81" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="H81" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="I81" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="J81" s="1" t="s">
-        <v>197</v>
+        <v>140</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="1" t="str">
         <f aca="false">LibManager!A82</f>
-        <v>ResizeBilinear</v>
+        <v>SparseLengthsSum</v>
       </c>
       <c r="B82" s="1" t="n">
         <f aca="false">LibManager!B82</f>
@@ -5166,37 +5192,34 @@
       </c>
       <c r="C82" s="1" t="n">
         <f aca="false">LibManager!C82</f>
-        <v>1</v>
-      </c>
-      <c r="D82" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="D82" s="1" t="s">
+        <v>117</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>134</v>
+        <v>162</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>135</v>
+        <v>163</v>
       </c>
       <c r="G82" s="1" t="s">
-        <v>136</v>
+        <v>159</v>
       </c>
       <c r="H82" s="1" t="s">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="I82" s="1" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="J82" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="K82" s="1" t="s">
-        <v>137</v>
+        <v>199</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="1" t="str">
         <f aca="false">LibManager!A83</f>
-        <v>ChannelWiseQuantizedConvolution</v>
+        <v>ResizeBilinear</v>
       </c>
       <c r="B83" s="1" t="n">
         <f aca="false">LibManager!B83</f>
@@ -5204,22 +5227,37 @@
       </c>
       <c r="C83" s="1" t="n">
         <f aca="false">LibManager!C83</f>
-        <v>7</v>
-      </c>
-      <c r="D83" s="1" t="s">
-        <v>25</v>
+        <v>1</v>
+      </c>
+      <c r="D83" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>175</v>
+        <v>136</v>
       </c>
       <c r="F83" s="1" t="s">
-        <v>176</v>
+        <v>137</v>
+      </c>
+      <c r="G83" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="H83" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="I83" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="J83" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="K83" s="1" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="1" t="str">
         <f aca="false">LibManager!A84</f>
-        <v>ConvTranspose</v>
+        <v>ChannelWiseQuantizedConvolution</v>
       </c>
       <c r="B84" s="1" t="n">
         <f aca="false">LibManager!B84</f>
@@ -5227,73 +5265,79 @@
       </c>
       <c r="C84" s="1" t="n">
         <f aca="false">LibManager!C84</f>
-        <v>3</v>
-      </c>
-      <c r="D84" s="1" t="n">
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>134</v>
+        <v>177</v>
+      </c>
+      <c r="F84" s="1" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="1" t="str">
         <f aca="false">LibManager!A85</f>
-        <v>NonMaxSuppression</v>
+        <v>ConvTranspose</v>
       </c>
       <c r="B85" s="1" t="n">
         <f aca="false">LibManager!B85</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C85" s="1" t="n">
         <f aca="false">LibManager!C85</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D85" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="F85" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="1" t="str">
         <f aca="false">LibManager!A86</f>
-        <v>ETSOCGenericOp</v>
+        <v>NonMaxSuppression</v>
       </c>
       <c r="B86" s="1" t="n">
         <f aca="false">LibManager!B86</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C86" s="1" t="n">
         <f aca="false">LibManager!C86</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D86" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>134</v>
+        <v>140</v>
+      </c>
+      <c r="F86" s="1" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A87" s="1" t="n">
+      <c r="A87" s="1" t="str">
         <f aca="false">LibManager!A87</f>
-        <v>0</v>
+        <v>ETSOCGenericOp</v>
       </c>
       <c r="B87" s="1" t="n">
         <f aca="false">LibManager!B87</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C87" s="1" t="n">
         <f aca="false">LibManager!C87</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D87" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="E87" s="1" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5394,6 +5438,9 @@
         <f aca="false">LibManager!C93</f>
         <v>0</v>
       </c>
+      <c r="D93" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="1" t="n">
@@ -5406,6 +5453,20 @@
       </c>
       <c r="C94" s="1" t="n">
         <f aca="false">LibManager!C94</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A95" s="1" t="n">
+        <f aca="false">LibManager!A95</f>
+        <v>0</v>
+      </c>
+      <c r="B95" s="1" t="n">
+        <f aca="false">LibManager!B95</f>
+        <v>0</v>
+      </c>
+      <c r="C95" s="1" t="n">
+        <f aca="false">LibManager!C95</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>